<commit_message>
docs(qa): add PREM-07 webhook-delivery check (now 68 cases)
Verify on the Stripe event-destination delivery log that the checkout/subscription
events reach the Worker with a 200, the concrete plumbing check beyond the in-app
entitlement flip.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3463,9 +3463,49 @@
       <c r="I68" s="9" t="inlineStr"/>
       <c r="J68" s="7" t="inlineStr"/>
     </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>PREM-07</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>Webhook delivery succeeds (Stripe side)</t>
+        </is>
+      </c>
+      <c r="E69" s="9" t="inlineStr">
+        <is>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr"/>
+      <c r="I69" s="9" t="inlineStr"/>
+      <c r="J69" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J68"/>
-  <conditionalFormatting sqref="H2:H68">
+  <autoFilter ref="A1:J69"/>
+  <conditionalFormatting sqref="H2:H69">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3477,7 +3517,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3513,7 +3553,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>68</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3564,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$68,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$69,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3535,7 +3575,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$68,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$69,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3546,7 +3586,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$68,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$69,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3557,7 +3597,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$68,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$69,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -3568,7 +3608,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>67-COUNTA('Test Suite'!$H$2:$H$68)</f>
+        <f>68-COUNTA('Test Suite'!$H$2:$H$69)</f>
         <v/>
       </c>
     </row>
@@ -3579,7 +3619,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$68,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$69,"P1")</f>
         <v/>
       </c>
     </row>
@@ -3590,7 +3630,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$68,"P1",'Test Suite'!$H$2:$H$68,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$69,"P1",'Test Suite'!$H$2:$H$69,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(premium): cancel/manage via the Stripe Billing Portal
The standard build-vs-buy call: don't build custom cancel UI, use Stripe's hosted
Billing Portal. A /portal endpoint creates a portal session from the user's
stripe_customer_id (now captured from the webhook into a new entitlements column),
the Premium screen gets a "Manage subscription" button that opens it, and a
cancellation flows back through the existing customer.subscription.* webhook ->
entitlement reverts to free. Tenure (started_at) survives a cancel via COALESCE.

Also gave the premium panel a quiet "Back to Today" link. E2E PREM-08/09 added
(now 70). 184 client + 67 server tests green.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3503,9 +3503,89 @@
       <c r="I69" s="9" t="inlineStr"/>
       <c r="J69" s="7" t="inlineStr"/>
     </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>PREM-08</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>Manage subscription opens the billing portal</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="inlineStr">
+        <is>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="inlineStr">
+        <is>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr"/>
+      <c r="I70" s="9" t="inlineStr"/>
+      <c r="J70" s="7" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>PREM-09</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>Cancel reverts to free</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>In the portal, cancel the subscription, then return to the app.</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="inlineStr">
+        <is>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr"/>
+      <c r="I71" s="9" t="inlineStr"/>
+      <c r="J71" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J69"/>
-  <conditionalFormatting sqref="H2:H69">
+  <autoFilter ref="A1:J71"/>
+  <conditionalFormatting sqref="H2:H71">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3517,7 +3597,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3553,7 +3633,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>70</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3644,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$69,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$71,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3575,7 +3655,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$69,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$71,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3586,7 +3666,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$69,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$71,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3597,7 +3677,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$69,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$71,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -3608,7 +3688,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>68-COUNTA('Test Suite'!$H$2:$H$69)</f>
+        <f>70-COUNTA('Test Suite'!$H$2:$H$71)</f>
         <v/>
       </c>
     </row>
@@ -3619,7 +3699,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$69,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$71,"P1")</f>
         <v/>
       </c>
     </row>
@@ -3630,7 +3710,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$69,"P1",'Test Suite'!$H$2:$H$69,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$71,"P1",'Test Suite'!$H$2:$H$71,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(premium): subscription lifecycle states (renews vs cancels)
Capture cancel_at_period_end and the period-end date (read from the dahlia
subscription items, where Stripe moved current_period_end). The Premium screen now
shows "Renews <date>" when active and "Premium until <date>, then free" when a
cancel is scheduled, so a cancel-then-keep round-trip is visible in the data, not
just inferred from a timestamp. Two new D1 columns (applied live); the webhook write
COALESCEs the period so a null checkout event cannot clobber a known date.

E2E PREM-10 added (now 71). 184 client + 68 server tests green.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3566,7 +3566,7 @@
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel the subscription, then return to the app.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
@@ -3583,9 +3583,49 @@
       <c r="I71" s="9" t="inlineStr"/>
       <c r="J71" s="7" t="inlineStr"/>
     </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr"/>
+      <c r="I72" s="9" t="inlineStr"/>
+      <c r="J72" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J71"/>
-  <conditionalFormatting sqref="H2:H71">
+  <autoFilter ref="A1:J72"/>
+  <conditionalFormatting sqref="H2:H72">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3597,7 +3637,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3633,7 +3673,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>71</t>
         </is>
       </c>
     </row>
@@ -3644,7 +3684,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$71,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$72,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3655,7 +3695,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$71,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$72,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3666,7 +3706,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$71,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$72,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3677,7 +3717,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$71,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$72,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -3688,7 +3728,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>70-COUNTA('Test Suite'!$H$2:$H$71)</f>
+        <f>71-COUNTA('Test Suite'!$H$2:$H$72)</f>
         <v/>
       </c>
     </row>
@@ -3699,7 +3739,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$71,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$72,"P1")</f>
         <v/>
       </c>
     </row>
@@ -3710,7 +3750,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$71,"P1",'Test Suite'!$H$2:$H$71,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$72,"P1",'Test Suite'!$H$2:$H$72,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(lookback): show scheduled future tasks on the calendar
Deferring a task (or using "Date...") moved it off Today into the "Later" strip,
but the Lookback calendar, the natural "what's scheduled when" surface, showed
nothing on its date, so it read as "disappeared." Now future days with a scheduled
one-off get a mauve outline dot (distinct from the sage filled completion dot), and
tapping a future day lists those tasks under a "Scheduled" label. Future-dated
one-offs only; recurring stays in the Repeating drawer. scheduledByDay is pure +
unit-tested. The completion payoff stays the headline.

E2E LB-04 added. 186 client + 69 server tests green. Verified in preview.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1626,37 +1626,37 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr"/>
@@ -1666,7 +1666,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1681,22 +1681,22 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr"/>
@@ -1706,7 +1706,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1754,24 +1754,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1801,22 +1801,22 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1841,22 +1841,22 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr"/>
@@ -1866,32 +1866,32 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1921,17 +1921,17 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1961,17 +1961,17 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -1994,24 +1994,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2041,17 +2041,17 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2081,17 +2081,17 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,37 +2106,37 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr"/>
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2161,22 +2161,22 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr"/>
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2201,17 +2201,17 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2234,24 +2234,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C38" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,32 +2266,32 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2321,22 +2321,22 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr"/>
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2401,17 +2401,17 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2441,17 +2441,17 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2474,29 +2474,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr"/>
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2521,22 +2521,22 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr"/>
@@ -2546,37 +2546,37 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr"/>
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2594,24 +2594,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C47" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,17 +2641,17 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,12 +2706,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
@@ -2721,22 +2721,22 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr"/>
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2761,22 +2761,22 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr"/>
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2794,24 +2794,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C52" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,37 +2826,37 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2874,24 +2874,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,17 +2921,17 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,32 +2946,32 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -2994,24 +2994,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C57" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,37 +3026,37 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr"/>
@@ -3066,12 +3066,12 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
@@ -3081,22 +3081,22 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr"/>
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3121,22 +3121,22 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr"/>
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3154,29 +3154,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C61" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,37 +3186,37 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3241,22 +3241,22 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr"/>
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3281,17 +3281,17 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3321,22 +3321,22 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,22 +3361,22 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3394,24 +3394,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C67" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3474,29 +3474,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3521,17 +3521,17 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,17 +3561,17 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3594,24 +3594,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C72" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3623,9 +3623,49 @@
       <c r="I72" s="9" t="inlineStr"/>
       <c r="J72" s="7" t="inlineStr"/>
     </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr"/>
+      <c r="I73" s="9" t="inlineStr"/>
+      <c r="J73" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J72"/>
-  <conditionalFormatting sqref="H2:H72">
+  <autoFilter ref="A1:J73"/>
+  <conditionalFormatting sqref="H2:H73">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3637,7 +3677,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3673,7 +3713,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>72</t>
         </is>
       </c>
     </row>
@@ -3684,7 +3724,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$72,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$73,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3695,7 +3735,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$72,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$73,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3706,7 +3746,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$72,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$73,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3717,7 +3757,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$72,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$73,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -3728,7 +3768,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>71-COUNTA('Test Suite'!$H$2:$H$72)</f>
+        <f>72-COUNTA('Test Suite'!$H$2:$H$73)</f>
         <v/>
       </c>
     </row>
@@ -3739,7 +3779,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$72,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$73,"P1")</f>
         <v/>
       </c>
     </row>
@@ -3750,7 +3790,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$72,"P1",'Test Suite'!$H$2:$H$72,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$73,"P1",'Test Suite'!$H$2:$H$73,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(today): rest the day after closing it, instead of returning to the same screen
The close-the-day wrap was a complete ritual, but "Goodnight" dismissed straight
back to the identical Today (same tasks, same list), so closing the day felt like
nothing happened. Now Goodnight persists a per-day closed flag and Today becomes a
calm "You've closed today" rested screen (task list + capture hidden, dusk art,
what you finished, "it's all here tomorrow"). "Reopen today" clears it; the flag is
keyed by date so it self-clears at the next day. No tasks are reset or lost.

This completes the daily loop's emotional spine: dump, work, close, rest, tomorrow.
New storage helpers (load/saveClosedDate). E2E TOD-04 rewritten + TOD-04b added.
186 client + 69 server tests green. Verified in preview (close -> rested, survives
reload, reopen restores).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1154,24 +1154,24 @@
           <t>Today</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Close the day gently</t>
+          <t>Close the day -&gt; rested state</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Complete / close out the day.</t>
+          <t>Tap 'Close the day', read the wrap, then tap 'Goodnight'.</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Gentle close, zero guilt. Unfinished tasks are not shamed.</t>
+          <t>Wrap celebrates what you finished (zero guilt, unfinished never shamed). After Goodnight, Today becomes a calm 'You've closed today' rested screen with the task list + capture hidden. Survives reload.</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1186,7 +1186,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>TOD-05</t>
+          <t>TOD-04b</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -1201,17 +1201,17 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Undo a completion</t>
+          <t>Reopen a closed day</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Complete a task, then undo it (toggle back).</t>
+          <t>From the rested screen, tap 'Reopen today'.</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Returns to open cleanly. Counts/Lookback stay consistent.</t>
+          <t>Returns to the normal Today with all tasks intact. (A new calendar day also auto-clears the closed state.)</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1226,7 +1226,7 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>TOD-06</t>
+          <t>TOD-05</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -1234,24 +1234,24 @@
           <t>Today</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Persistence across restart</t>
+          <t>Undo a completion</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>Add tasks, fully close the app/tab, reopen.</t>
+          <t>Complete a task, then undo it (toggle back).</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Tasks are still there (local-first). Nothing lost.</t>
+          <t>Returns to open cleanly. Counts/Lookback stay consistent.</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1266,12 +1266,12 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>TOD-06</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -1281,17 +1281,17 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Persistence across restart</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>Add tasks, fully close the app/tab, reopen.</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>Tasks are still there (local-first). Nothing lost.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1306,7 +1306,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -1314,24 +1314,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -1346,7 +1346,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -1361,17 +1361,17 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1386,7 +1386,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -1401,17 +1401,17 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -1426,12 +1426,12 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
@@ -1441,17 +1441,17 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>With several tasks present, run Sort-for-me / triage.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Sensible ordering/grouping. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1466,12 +1466,12 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -1481,17 +1481,17 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage)</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>With several tasks present, run Sort-for-me / triage.</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Sensible ordering/grouping. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1506,32 +1506,32 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1546,7 +1546,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -1561,17 +1561,17 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1586,7 +1586,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1594,24 +1594,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1626,7 +1626,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -1641,17 +1641,17 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1666,37 +1666,37 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr"/>
@@ -1706,7 +1706,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1721,22 +1721,22 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr"/>
@@ -1746,7 +1746,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1761,17 +1761,17 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1794,24 +1794,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -1826,7 +1826,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1841,22 +1841,22 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr"/>
@@ -1866,7 +1866,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1881,22 +1881,22 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr"/>
@@ -1906,32 +1906,32 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1961,17 +1961,17 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2001,17 +2001,17 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2034,24 +2034,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2081,17 +2081,17 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2121,17 +2121,17 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,37 +2146,37 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr"/>
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2201,22 +2201,22 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr"/>
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2274,24 +2274,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C39" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,32 +2306,32 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2361,22 +2361,22 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr"/>
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2401,17 +2401,17 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2441,17 +2441,17 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2481,17 +2481,17 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2514,29 +2514,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr"/>
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,22 +2561,22 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr"/>
@@ -2586,37 +2586,37 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr"/>
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2634,24 +2634,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C48" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,12 +2746,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
@@ -2761,22 +2761,22 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr"/>
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2801,22 +2801,22 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr"/>
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2834,24 +2834,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C53" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,37 +2866,37 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2914,24 +2914,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C55" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,17 +2961,17 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,32 +2986,32 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3034,24 +3034,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C58" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,37 +3066,37 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr"/>
@@ -3106,12 +3106,12 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
@@ -3121,22 +3121,22 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr"/>
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3161,22 +3161,22 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3194,29 +3194,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,37 +3226,37 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr"/>
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3281,22 +3281,22 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3321,17 +3321,17 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,22 +3361,22 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,22 +3401,22 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3434,24 +3434,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C68" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,22 +3481,22 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3514,29 +3514,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C70" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,17 +3561,17 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3601,17 +3601,17 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3634,24 +3634,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C73" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3663,9 +3663,49 @@
       <c r="I73" s="9" t="inlineStr"/>
       <c r="J73" s="7" t="inlineStr"/>
     </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr"/>
+      <c r="I74" s="9" t="inlineStr"/>
+      <c r="J74" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J73"/>
-  <conditionalFormatting sqref="H2:H73">
+  <autoFilter ref="A1:J74"/>
+  <conditionalFormatting sqref="H2:H74">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3677,7 +3717,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3713,7 +3753,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>73</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3764,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$73,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$74,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3735,7 +3775,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$73,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$74,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3746,7 +3786,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$73,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$74,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3757,7 +3797,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$73,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$74,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -3768,7 +3808,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>72-COUNTA('Test Suite'!$H$2:$H$73)</f>
+        <f>73-COUNTA('Test Suite'!$H$2:$H$74)</f>
         <v/>
       </c>
     </row>
@@ -3779,7 +3819,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$73,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$74,"P1")</f>
         <v/>
       </c>
     </row>
@@ -3790,7 +3830,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$73,"P1",'Test Suite'!$H$2:$H$73,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$74,"P1",'Test Suite'!$H$2:$H$74,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(capture): surface "Sort for me" with a one-line hint
The brain-dump's main button swaps from "Break it down" (one line) to "Sort for me"
(2+ lines) by line count, clean but invisible: the founder never found Sort because
he always typed single tasks, and the placeholder ("one per line") never named the
AI-triage payoff. Now, the moment one line is typed, a quiet hint appears: "More
than one? Put each on its own line and I'll sort them for you." It shows only at
lineCount === 1, so the resting screen stays clean and it vanishes once the Sort
button itself appears. No new button, no setting.

E2E AI-05 updated. 186 client tests green. Verified in preview (1 line -> hint +
Break it down; 2 lines -> no hint + Sort for me).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -1481,17 +1481,17 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage)</t>
+          <t>Sort-for-me (triage + discoverability)</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>With several tasks present, run Sort-for-me / triage.</t>
+          <t>In the brain-dump, type 2+ things, one per line. After one line a hint should nudge 'put each on its own line'; at two lines 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Sensible ordering/grouping. Calm, never scolding.</t>
+          <t>Hint is visible at one line, so Sort is discoverable. Sort returns a sensible ordering/grouping onto Today. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix(tasks): rename Keep to Close and give Remove a calm "danger" colour
The long-press menu read poorly: "Keep" looked like a no-op (it is actually the
menu's only escape), and Remove shared the mauve accent with everything else, so the
one destructive action did not look destructive.

- Keep -> Close, moved to the right of Remove, given the prominent mauve accent the
  safe default deserves (matches the sliced-task menu, which already said "Close").
- Remove now uses a new palette token `danger` (light #A1554C, dark #D2887E), a muted
  brick: the calm stand-in for the red a delete would get, no alarm, AA-contrast on
  the menu's mauve-tint background in both schemes.
- Handler unchanged; purely label, order, and colour.

E2E TOD-07 added. 192 client tests green. Verified in preview: order Tomorrow /
Break down / Remove / Close, Close mauve, Remove brick.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1306,32 +1306,32 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>TOD-07</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Long-press a task: the action menu</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>Press and hold a task to open its menu: Tomorrow, Break down, Remove, Close.</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>Remove is the only 'danger' (brick) coloured action; Close (mauve, to the right of Remove) just dismisses with nothing lost. Tomorrow defers, Break down opens decompose.</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -1346,7 +1346,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -1354,24 +1354,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1386,7 +1386,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -1401,17 +1401,17 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -1426,7 +1426,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -1441,17 +1441,17 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1466,12 +1466,12 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -1481,17 +1481,17 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1506,12 +1506,12 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -1521,17 +1521,17 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1546,32 +1546,32 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1586,7 +1586,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1601,17 +1601,17 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1626,7 +1626,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -1634,24 +1634,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1666,7 +1666,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1681,17 +1681,17 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1706,37 +1706,37 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr"/>
@@ -1746,7 +1746,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1761,22 +1761,22 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr"/>
@@ -1786,7 +1786,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1801,17 +1801,17 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -1826,7 +1826,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1834,24 +1834,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,7 +1866,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1881,22 +1881,22 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr"/>
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1921,22 +1921,22 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr"/>
@@ -1946,32 +1946,32 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2001,17 +2001,17 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2041,17 +2041,17 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2074,24 +2074,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2121,17 +2121,17 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,37 +2186,37 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr"/>
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,22 +2241,22 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr"/>
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2281,17 +2281,17 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2314,24 +2314,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C40" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2346,32 +2346,32 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2401,22 +2401,22 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr"/>
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2441,17 +2441,17 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2481,17 +2481,17 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2521,17 +2521,17 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2554,29 +2554,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C46" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr"/>
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,22 +2601,22 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr"/>
@@ -2626,37 +2626,37 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr"/>
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2674,24 +2674,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2761,17 +2761,17 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,12 +2786,12 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
@@ -2801,22 +2801,22 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr"/>
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,22 +2841,22 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2874,24 +2874,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C54" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,37 +2906,37 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2954,24 +2954,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C56" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3001,17 +3001,17 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,32 +3026,32 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3074,24 +3074,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C59" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,37 +3106,37 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr"/>
@@ -3146,12 +3146,12 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
@@ -3161,22 +3161,22 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3201,22 +3201,22 @@
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3234,29 +3234,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr"/>
@@ -3266,37 +3266,37 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3321,22 +3321,22 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,17 +3361,17 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,22 +3401,22 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3474,24 +3474,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C69" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3521,22 +3521,22 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3554,29 +3554,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C71" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3601,17 +3601,17 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3674,24 +3674,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C74" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3703,9 +3703,49 @@
       <c r="I74" s="9" t="inlineStr"/>
       <c r="J74" s="7" t="inlineStr"/>
     </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr"/>
+      <c r="I75" s="9" t="inlineStr"/>
+      <c r="J75" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J74"/>
-  <conditionalFormatting sqref="H2:H74">
+  <autoFilter ref="A1:J75"/>
+  <conditionalFormatting sqref="H2:H75">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3717,7 +3757,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3753,7 +3793,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>74</t>
         </is>
       </c>
     </row>
@@ -3764,7 +3804,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$74,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$75,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3775,7 +3815,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$74,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$75,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3786,7 +3826,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$74,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$75,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3797,7 +3837,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$74,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$75,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -3808,7 +3848,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>73-COUNTA('Test Suite'!$H$2:$H$74)</f>
+        <f>74-COUNTA('Test Suite'!$H$2:$H$75)</f>
         <v/>
       </c>
     </row>
@@ -3819,7 +3859,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$74,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$75,"P1")</f>
         <v/>
       </c>
     </row>
@@ -3830,7 +3870,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$74,"P1",'Test Suite'!$H$2:$H$74,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$75,"P1",'Test Suite'!$H$2:$H$75,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(today): shame-free re-entry after a multi-day gap
Open after falling off for a while and every other to-do app says "47 overdue."
DoubleDone now shows a calm "Welcome back, the past is fine, here's just today" card
above Today. The single biggest retention lever for this audience.

A persisted last-open date drives it: on focus, if the last open was >= 4 calendar
days ago (isReentry, pure + unit-tested via daysBetween), the card shows; the open
stamps today so it shows once per gap and never re-nags. Decided against a full-screen
takeover (a gentle card is kinder to an RSD-sensitive user) and against any reshuffle
of old tasks (they already carry no overdue framing).

194 client tests green (+2). E2E TOD-08 added. Verified in preview (6-day gap shows
it; reopening clears it).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J75"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1346,32 +1346,32 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>TOD-08</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Shame-free re-entry after a gap</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>Simulate not opening the app for 4+ days (set localStorage 'doubledone.lastopen.v1' to a date 5+ days ago), then reload Today.</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>A calm 'Welcome back, the past is fine, here's just today' card appears above Today, never '47 overdue'. 'Start fresh' dismisses it; reopening same-day does not re-show it.</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1386,7 +1386,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -1394,24 +1394,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -1426,7 +1426,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -1441,17 +1441,17 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1466,7 +1466,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -1481,17 +1481,17 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1506,12 +1506,12 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -1521,17 +1521,17 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1546,12 +1546,12 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -1561,17 +1561,17 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1586,32 +1586,32 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1626,7 +1626,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -1641,17 +1641,17 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1666,7 +1666,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1674,24 +1674,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1706,7 +1706,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1746,37 +1746,37 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr"/>
@@ -1786,7 +1786,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1801,22 +1801,22 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1841,17 +1841,17 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,7 +1866,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1874,24 +1874,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1921,22 +1921,22 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr"/>
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1961,22 +1961,22 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr"/>
@@ -1986,32 +1986,32 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2041,17 +2041,17 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2081,17 +2081,17 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2114,24 +2114,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2201,17 +2201,17 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,37 +2226,37 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr"/>
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2281,22 +2281,22 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr"/>
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2321,17 +2321,17 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2354,24 +2354,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C41" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,32 +2386,32 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2441,22 +2441,22 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr"/>
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2481,17 +2481,17 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2521,17 +2521,17 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,17 +2561,17 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2594,29 +2594,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C47" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr"/>
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,22 +2641,22 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr"/>
@@ -2666,37 +2666,37 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr"/>
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2714,24 +2714,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2761,17 +2761,17 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2801,17 +2801,17 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,12 +2826,12 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
@@ -2841,22 +2841,22 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2881,22 +2881,22 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2914,24 +2914,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C55" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,37 +2946,37 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr"/>
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -2994,24 +2994,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C57" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3041,17 +3041,17 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,32 +3066,32 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3114,24 +3114,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,37 +3146,37 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,12 +3186,12 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -3201,22 +3201,22 @@
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3241,22 +3241,22 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr"/>
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3274,29 +3274,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C64" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,37 +3306,37 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,22 +3361,22 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,17 +3401,17 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,22 +3481,22 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3514,24 +3514,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,22 +3561,22 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3594,29 +3594,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,17 +3681,17 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3714,24 +3714,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C75" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3743,9 +3743,49 @@
       <c r="I75" s="9" t="inlineStr"/>
       <c r="J75" s="7" t="inlineStr"/>
     </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr"/>
+      <c r="I76" s="9" t="inlineStr"/>
+      <c r="J76" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J75"/>
-  <conditionalFormatting sqref="H2:H75">
+  <autoFilter ref="A1:J76"/>
+  <conditionalFormatting sqref="H2:H76">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3757,7 +3797,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3793,7 +3833,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>75</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3844,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$75,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$76,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3815,7 +3855,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$75,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$76,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3826,7 +3866,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$75,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$76,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3837,7 +3877,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$75,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$76,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -3848,7 +3888,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>74-COUNTA('Test Suite'!$H$2:$H$75)</f>
+        <f>75-COUNTA('Test Suite'!$H$2:$H$76)</f>
         <v/>
       </c>
     </row>
@@ -3859,7 +3899,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$75,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$76,"P1")</f>
         <v/>
       </c>
     </row>
@@ -3870,7 +3910,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$75,"P1",'Test Suite'!$H$2:$H$75,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$76,"P1",'Test Suite'!$H$2:$H$76,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(today): "I also did that" logs off-list wins
This brain does loads that never made the list, and counting only ticked tasks feeds
the "I did nothing" lie. A quiet "+ I also did that" link in the day actions opens a
one-line input; what you type becomes a completed task stamped now, so it shows checked
on Today and lands in the Lookback like any finished thing. offplan.logged instrumented
so it also feeds the moat.

In-the-moment (not gated behind close-the-day) so the win is caught before it's
forgotten. A completed task in the normal store, no separate "done" list, reuses the
Lookback unchanged. 194 client tests green. E2E TOD-09 added. Verified in preview.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1386,32 +1386,32 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>TOD-09</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Log an off-list thing you did</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>Tap '+ I also did that' in the day actions, type something you did, then Add it.</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>It appears checked on Today and in the Lookback for today, counted as a completion, never as an unfinished task.</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -1426,7 +1426,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -1434,24 +1434,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1466,7 +1466,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -1481,17 +1481,17 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1506,7 +1506,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -1521,17 +1521,17 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1546,12 +1546,12 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -1561,17 +1561,17 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1586,12 +1586,12 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -1601,17 +1601,17 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1626,32 +1626,32 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1666,7 +1666,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1681,17 +1681,17 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1706,7 +1706,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1714,24 +1714,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1761,17 +1761,17 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1786,37 +1786,37 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1841,22 +1841,22 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr"/>
@@ -1866,7 +1866,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1881,17 +1881,17 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1914,24 +1914,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1961,22 +1961,22 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr"/>
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2001,22 +2001,22 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr"/>
@@ -2026,32 +2026,32 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2081,17 +2081,17 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2121,17 +2121,17 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2154,24 +2154,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2201,17 +2201,17 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,37 +2266,37 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr"/>
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2321,22 +2321,22 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr"/>
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2394,24 +2394,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C42" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,32 +2426,32 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2481,22 +2481,22 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr"/>
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2521,17 +2521,17 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,17 +2561,17 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,17 +2601,17 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2634,29 +2634,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C48" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr"/>
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,22 +2681,22 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr"/>
@@ -2706,37 +2706,37 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr"/>
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2754,24 +2754,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2801,17 +2801,17 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,17 +2841,17 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,12 +2866,12 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
@@ -2881,22 +2881,22 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,22 +2921,22 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2954,24 +2954,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C56" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,37 +2986,37 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3034,24 +3034,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C58" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3081,17 +3081,17 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,32 +3106,32 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3154,24 +3154,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C61" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,37 +3186,37 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,12 +3226,12 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
@@ -3241,22 +3241,22 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr"/>
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3281,22 +3281,22 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3314,29 +3314,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3346,37 +3346,37 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C66" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,22 +3401,22 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,17 +3441,17 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,22 +3481,22 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3521,22 +3521,22 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3554,24 +3554,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C71" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3601,22 +3601,22 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3634,29 +3634,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,17 +3681,17 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3721,17 +3721,17 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3754,24 +3754,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C76" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3783,9 +3783,49 @@
       <c r="I76" s="9" t="inlineStr"/>
       <c r="J76" s="7" t="inlineStr"/>
     </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E77" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F77" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr"/>
+      <c r="I77" s="9" t="inlineStr"/>
+      <c r="J77" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J76"/>
-  <conditionalFormatting sqref="H2:H76">
+  <autoFilter ref="A1:J77"/>
+  <conditionalFormatting sqref="H2:H77">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3797,7 +3837,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3833,7 +3873,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>76</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3884,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$76,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$77,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3855,7 +3895,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$76,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$77,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3866,7 +3906,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$76,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$77,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3877,7 +3917,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$76,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$77,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -3888,7 +3928,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>75-COUNTA('Test Suite'!$H$2:$H$76)</f>
+        <f>76-COUNTA('Test Suite'!$H$2:$H$77)</f>
         <v/>
       </c>
     </row>
@@ -3899,7 +3939,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$76,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$77,"P1")</f>
         <v/>
       </c>
     </row>
@@ -3910,7 +3950,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$76,"P1",'Test Suite'!$H$2:$H$76,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$77,"P1",'Test Suite'!$H$2:$H$77,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(today): "just this one" focus mode
Starting is the #1 ADHD blocker and a full list is paralysing. "Focus on one thing"
opens a full-screen single-task view, everything else gone: "JUST THIS ONE / <task>",
"Not this one" to skip, "Done" to complete (the next surfaces on its own), Exit. When
nothing is left: "That's everything for now."

A full-screen Modal in the Today screen (no new route, reuses the live list + commit),
first unfinished one-off not yet skipped. Recurring habits excluded (not the
wall-of-awful). focus.opened / focus.completed instrumented. Optional timer deferred to
a fast-follow. 194 client tests green. E2E TOD-10 added. Verified in preview (skip
advances, done completes + advances past skipped, empty state).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$78</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1426,32 +1426,32 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>TOD-10</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Focus mode: just this one</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>With a few tasks present, tap 'Focus on one thing'. Try 'Not this one' (skip), 'Done' (complete), and Exit.</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>Full-screen single task, everything else hidden. Skip advances, Done completes and advances, Exit returns. When none left: 'That's everything for now.'</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1466,7 +1466,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -1474,24 +1474,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1506,7 +1506,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -1521,17 +1521,17 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1546,7 +1546,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -1561,17 +1561,17 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1586,12 +1586,12 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -1601,17 +1601,17 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1626,12 +1626,12 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -1641,17 +1641,17 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1666,32 +1666,32 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1706,7 +1706,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1754,24 +1754,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1801,17 +1801,17 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -1826,37 +1826,37 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr"/>
@@ -1866,7 +1866,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1881,22 +1881,22 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr"/>
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1921,17 +1921,17 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1954,24 +1954,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2001,22 +2001,22 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr"/>
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2041,22 +2041,22 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr"/>
@@ -2066,32 +2066,32 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2121,17 +2121,17 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2194,24 +2194,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2281,17 +2281,17 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,37 +2306,37 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr"/>
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2361,22 +2361,22 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr"/>
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2401,17 +2401,17 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2434,24 +2434,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C43" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,32 +2466,32 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2521,22 +2521,22 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr"/>
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,17 +2561,17 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,17 +2601,17 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,17 +2641,17 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2674,29 +2674,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr"/>
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2721,22 +2721,22 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr"/>
@@ -2746,37 +2746,37 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr"/>
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2794,24 +2794,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C52" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,17 +2841,17 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2881,17 +2881,17 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,12 +2906,12 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -2921,22 +2921,22 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,22 +2961,22 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr"/>
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -2994,24 +2994,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C57" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,37 +3026,37 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr"/>
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3074,24 +3074,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C59" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3121,17 +3121,17 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,32 +3146,32 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3194,24 +3194,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3226,37 +3226,37 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr"/>
@@ -3266,12 +3266,12 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
@@ -3281,22 +3281,22 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3321,22 +3321,22 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3354,29 +3354,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C66" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr"/>
@@ -3386,37 +3386,37 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,17 +3481,17 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3521,22 +3521,22 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,22 +3561,22 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3594,24 +3594,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C72" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,22 +3641,22 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3674,29 +3674,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr"/>
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3721,17 +3721,17 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3761,17 +3761,17 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3794,24 +3794,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C77" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -3823,9 +3823,49 @@
       <c r="I77" s="9" t="inlineStr"/>
       <c r="J77" s="7" t="inlineStr"/>
     </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H78" s="7" t="inlineStr"/>
+      <c r="I78" s="9" t="inlineStr"/>
+      <c r="J78" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J77"/>
-  <conditionalFormatting sqref="H2:H77">
+  <autoFilter ref="A1:J78"/>
+  <conditionalFormatting sqref="H2:H78">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3837,7 +3877,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3873,7 +3913,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>77</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3924,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$77,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$78,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3895,7 +3935,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$77,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$78,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3906,7 +3946,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$77,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$78,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3917,7 +3957,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$77,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$78,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -3928,7 +3968,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>76-COUNTA('Test Suite'!$H$2:$H$77)</f>
+        <f>77-COUNTA('Test Suite'!$H$2:$H$78)</f>
         <v/>
       </c>
     </row>
@@ -3939,7 +3979,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$77,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$78,"P1")</f>
         <v/>
       </c>
     </row>
@@ -3950,7 +3990,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$77,"P1",'Test Suite'!$H$2:$H$77,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$78,"P1",'Test Suite'!$H$2:$H$78,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(today): honest "weight of today" load gauge
Time-blindness lets Today silently overfill. A slim gauge under the spine shows the
day's load honestly: a mauve fill (0..1) plus a plain label (clear / light / full /
heavy) from the count of unfinished one-offs (dayWeight, pure + tested, extends
lib/estimate). Complements the Strategise nudge with a glanceable read.

Count-based, not time-based (most tasks carry no estimate, so minutes would be
fabricated). No alarm colour at any level; hidden on a clear day. 196 client tests
green (+2). E2E TOD-11 added. Verified in preview (4 tasks = "A full day", ~67% bar).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J78"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1466,32 +1466,32 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>TOD-11</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Weight-of-today gauge</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>Add a few tasks and watch the slim gauge under 'Just today'.</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>A calm bar + label (clear / light / full / heavy) reflects the count of unfinished one-offs, honest, never alarming, hidden on a clear day.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1506,7 +1506,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -1514,24 +1514,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1546,7 +1546,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -1561,17 +1561,17 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1586,7 +1586,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1601,17 +1601,17 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1626,12 +1626,12 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -1641,17 +1641,17 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1666,12 +1666,12 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -1681,17 +1681,17 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1706,32 +1706,32 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1761,17 +1761,17 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1794,24 +1794,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -1826,7 +1826,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1841,17 +1841,17 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,37 +1866,37 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr"/>
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1921,22 +1921,22 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr"/>
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1961,17 +1961,17 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -1994,24 +1994,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2041,22 +2041,22 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr"/>
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2081,22 +2081,22 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr"/>
@@ -2106,32 +2106,32 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2201,17 +2201,17 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2234,24 +2234,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2281,17 +2281,17 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2321,17 +2321,17 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2346,37 +2346,37 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr"/>
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2401,22 +2401,22 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr"/>
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2441,17 +2441,17 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2474,24 +2474,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C44" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,32 +2506,32 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,22 +2561,22 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr"/>
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,17 +2601,17 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,17 +2641,17 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2714,29 +2714,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr"/>
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2761,22 +2761,22 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr"/>
@@ -2786,37 +2786,37 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr"/>
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2834,24 +2834,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C53" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2881,17 +2881,17 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,17 +2921,17 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,12 +2946,12 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -2961,22 +2961,22 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr"/>
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3001,22 +3001,22 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3034,24 +3034,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C58" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,37 +3066,37 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr"/>
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3114,24 +3114,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3161,17 +3161,17 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,32 +3186,32 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3234,24 +3234,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,37 +3266,37 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,12 +3306,12 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
@@ -3321,22 +3321,22 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,22 +3361,22 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3394,29 +3394,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C67" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,37 +3426,37 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C68" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,22 +3481,22 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3521,17 +3521,17 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,22 +3561,22 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3601,22 +3601,22 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3634,24 +3634,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C73" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,22 +3681,22 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr"/>
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3714,29 +3714,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr"/>
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3761,17 +3761,17 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3801,17 +3801,17 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3834,24 +3834,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C78" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -3863,9 +3863,49 @@
       <c r="I78" s="9" t="inlineStr"/>
       <c r="J78" s="7" t="inlineStr"/>
     </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F79" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr"/>
+      <c r="I79" s="9" t="inlineStr"/>
+      <c r="J79" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J78"/>
-  <conditionalFormatting sqref="H2:H78">
+  <autoFilter ref="A1:J79"/>
+  <conditionalFormatting sqref="H2:H79">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3877,7 +3917,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3913,7 +3953,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>78</t>
         </is>
       </c>
     </row>
@@ -3924,7 +3964,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$78,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$79,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3935,7 +3975,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$78,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$79,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3946,7 +3986,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$78,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$79,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3957,7 +3997,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$78,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$79,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -3968,7 +4008,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>77-COUNTA('Test Suite'!$H$2:$H$78)</f>
+        <f>78-COUNTA('Test Suite'!$H$2:$H$79)</f>
         <v/>
       </c>
     </row>
@@ -3979,7 +4019,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$78,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$79,"P1")</f>
         <v/>
       </c>
     </row>
@@ -3990,7 +4030,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$78,"P1",'Test Suite'!$H$2:$H$78,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$79,"P1",'Test Suite'!$H$2:$H$79,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(settings): export your data (your stuff is yours)
A "Your data" section in Settings (always visible, no account needed) exports tasks +
completions as doubledone-export-<date>.json: web downloads a Blob, native opens the
share sheet. buildExport is pure + tested; tombstones dropped, completion data kept, so
the file is the whole record. data.exported instrumented.

Tasks-only (not the huge base64 scrapbook images). Completes the privacy posture
alongside account deletion. 198 client tests green (+2). E2E SET-05 added. Verified in
preview (real Blob, correct filename + JSON incl. a completed task).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2986,12 +2986,12 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -3001,22 +3001,22 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3041,22 +3041,22 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr"/>
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3074,24 +3074,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C59" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,37 +3106,37 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr"/>
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3154,24 +3154,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C61" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3201,17 +3201,17 @@
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3226,32 +3226,32 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3274,24 +3274,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C64" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,37 +3306,37 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3346,12 +3346,12 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
@@ -3361,22 +3361,22 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,22 +3401,22 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3434,29 +3434,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C68" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,37 +3466,37 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3521,22 +3521,22 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,17 +3561,17 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3601,22 +3601,22 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,22 +3641,22 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3674,24 +3674,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C74" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3721,22 +3721,22 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr"/>
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3754,29 +3754,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr"/>
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3801,17 +3801,17 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3841,17 +3841,17 @@
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3874,24 +3874,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C79" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
@@ -3903,9 +3903,49 @@
       <c r="I79" s="9" t="inlineStr"/>
       <c r="J79" s="7" t="inlineStr"/>
     </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H80" s="7" t="inlineStr"/>
+      <c r="I80" s="9" t="inlineStr"/>
+      <c r="J80" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J79"/>
-  <conditionalFormatting sqref="H2:H79">
+  <autoFilter ref="A1:J80"/>
+  <conditionalFormatting sqref="H2:H80">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3917,7 +3957,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3953,7 +3993,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>79</t>
         </is>
       </c>
     </row>
@@ -3964,7 +4004,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$79,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$80,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3975,7 +4015,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$79,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$80,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3986,7 +4026,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$79,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$80,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3997,7 +4037,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$79,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$80,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -4008,7 +4048,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>78-COUNTA('Test Suite'!$H$2:$H$79)</f>
+        <f>79-COUNTA('Test Suite'!$H$2:$H$80)</f>
         <v/>
       </c>
     </row>
@@ -4019,7 +4059,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$79,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$80,"P1")</f>
         <v/>
       </c>
     </row>
@@ -4030,7 +4070,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$79,"P1",'Test Suite'!$H$2:$H$79,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$80,"P1",'Test Suite'!$H$2:$H$80,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(today): multi-select bulk actions (Done / Tomorrow / Remove)
Clearing several tasks meant repeating the long-press menu one at a time. A "Select
several" link now enters a select mode: every row becomes a checkbox, the day actions
+ capture give way to a calm bottom bar (Done / Tomorrow / Remove / Cancel), and the
action applies to all picked tasks at once. Long-press keeps its single-task menu, so
nothing is lost.

Bulk Done (same completion path), Tomorrow (one-offs; recurring skipped), Remove
(soft-delete, danger colour). Scoped to today's main list for v1. select.opened /
bulk.* instrumented. 198 client tests green. E2E TOD-12 added. Verified in preview:
pick two of three, Remove -> two soft-delete, third survives, mode exits.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J80"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1506,32 +1506,32 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>TOD-12</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Multi-select bulk actions</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>Tap 'Select several', tap a few tasks to select, then use the bar: Done / Tomorrow / Remove. Cancel exits.</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>Rows become checkboxes, the count updates, the bulk action applies to all selected at once and exits select mode. Long-press still gives a single task its own menu.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1546,7 +1546,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -1554,24 +1554,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1586,7 +1586,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1601,17 +1601,17 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1626,7 +1626,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -1641,17 +1641,17 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1666,12 +1666,12 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -1681,17 +1681,17 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1706,12 +1706,12 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1746,32 +1746,32 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1801,17 +1801,17 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -1826,7 +1826,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1834,24 +1834,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,7 +1866,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1881,17 +1881,17 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,37 +1906,37 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr"/>
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1961,22 +1961,22 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr"/>
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2001,17 +2001,17 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2034,24 +2034,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2081,22 +2081,22 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr"/>
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2121,22 +2121,22 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr"/>
@@ -2146,32 +2146,32 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2201,17 +2201,17 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2274,24 +2274,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2321,17 +2321,17 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,37 +2386,37 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr"/>
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2441,22 +2441,22 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr"/>
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2481,17 +2481,17 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2514,24 +2514,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C45" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,32 +2546,32 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,22 +2601,22 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr"/>
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,17 +2641,17 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2754,29 +2754,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr"/>
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2801,22 +2801,22 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr"/>
@@ -2826,37 +2826,37 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2874,24 +2874,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,17 +2921,17 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,17 +2961,17 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3001,17 +3001,17 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,12 +3026,12 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -3041,22 +3041,22 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr"/>
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3081,22 +3081,22 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr"/>
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3114,24 +3114,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,37 +3146,37 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3194,24 +3194,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3241,17 +3241,17 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,32 +3266,32 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3314,24 +3314,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,37 +3346,37 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C66" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr"/>
@@ -3386,12 +3386,12 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
@@ -3401,22 +3401,22 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3474,29 +3474,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C69" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,37 +3506,37 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C70" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,22 +3561,22 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3601,17 +3601,17 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,22 +3641,22 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,22 +3681,22 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr"/>
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3714,24 +3714,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C75" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3761,22 +3761,22 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr"/>
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3794,29 +3794,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C77" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3841,17 +3841,17 @@
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3881,17 +3881,17 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3914,24 +3914,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C80" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
@@ -3943,9 +3943,49 @@
       <c r="I80" s="9" t="inlineStr"/>
       <c r="J80" s="7" t="inlineStr"/>
     </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr"/>
+      <c r="I81" s="9" t="inlineStr"/>
+      <c r="J81" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J80"/>
-  <conditionalFormatting sqref="H2:H80">
+  <autoFilter ref="A1:J81"/>
+  <conditionalFormatting sqref="H2:H81">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3957,7 +3997,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3993,7 +4033,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>80</t>
         </is>
       </c>
     </row>
@@ -4004,7 +4044,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$80,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$81,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -4015,7 +4055,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$80,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$81,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -4026,7 +4066,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$80,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$81,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -4037,7 +4077,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$80,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$81,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -4048,7 +4088,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>79-COUNTA('Test Suite'!$H$2:$H$80)</f>
+        <f>80-COUNTA('Test Suite'!$H$2:$H$81)</f>
         <v/>
       </c>
     </row>
@@ -4059,7 +4099,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$80,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$81,"P1")</f>
         <v/>
       </c>
     </row>
@@ -4070,7 +4110,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$80,"P1",'Test Suite'!$H$2:$H$80,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$81,"P1",'Test Suite'!$H$2:$H$81,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
test(qa): refresh Today E2E cases for the redesign
The Today redesign changed several manual flows, so the suite is brought current
(the launch gate, per the E2E rule):
- TOD-04 close-day now includes the "Anything else you did?" prompt
- TOD-07 long-press menu -> tap-and-hold selection + adaptive bar
- TOD-09 "I also did that" now beneath the list
- TOD-10 Focus is pick-and-go ("Which one?")
- TOD-11 weight gauge carries the warm labels
- TOD-12 multi-select via tap-and-hold + Select all
- TOD-13 (new) Move selected tasks to a chosen day
Regenerated the .xlsx + .md (81 cases).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Close the day', read the wrap, then tap 'Goodnight'.</t>
+          <t>Tap 'Close the day', read the wrap, optionally type a final win in 'Anything else you did?', then tap 'Goodnight'.</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Wrap celebrates what you finished (zero guilt, unfinished never shamed). After Goodnight, Today becomes a calm 'You've closed today' rested screen with the task list + capture hidden. Survives reload.</t>
+          <t>Wrap celebrates what you finished (zero guilt, unfinished never shamed). Any text in 'Anything else you did?' is logged as a completed task. After Goodnight, Today becomes a calm 'You've closed today' rested screen with the task list + capture hidden. Survives reload.</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1321,17 +1321,17 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Long-press a task: the action menu</t>
+          <t>Tap-and-hold a task -&gt; selection</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Press and hold a task to open its menu: Tomorrow, Break down, Remove, Close.</t>
+          <t>Press and hold a task. It enters selection with that task already ticked and the action bar appears.</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Remove is the only 'danger' (brick) coloured action; Close (mauve, to the right of Remove) just dismisses with nothing lost. Tomorrow defers, Break down opens decompose.</t>
+          <t>With one selected the bar offers Done / Tomorrow / Move to... / Break down / Remove (Break down is single-task only); Remove is the brick 'danger' colour. There is no separate long-press menu any more.</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Tap '+ I also did that' in the day actions, type something you did, then Add it.</t>
+          <t>Tap '+ I also did that' (beneath the task list), type something you did, then Add it.</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -1441,17 +1441,17 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Focus mode: just this one</t>
+          <t>Focus mode: pick-and-go</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>With a few tasks present, tap 'Focus on one thing'. Try 'Not this one' (skip), 'Done' (complete), and Exit.</t>
+          <t>Tap 'Focus on one thing' (the prominent entry above the list). On 'Which one?' pick a task; try 'Done' (complete), 'Choose another' (back to the list), and Exit.</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Full-screen single task, everything else hidden. Skip advances, Done completes and advances, Exit returns. When none left: 'That's everything for now.'</t>
+          <t>Full-screen single task, everything else hidden. Done completes it and returns to 'Which one?'; Choose another returns without completing; Exit closes. When none left: 'That's everything for now.'</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>A calm bar + label (clear / light / full / heavy) reflects the count of unfinished one-offs, honest, never alarming, hidden on a clear day.</t>
+          <t>A calm bar + warm label ('A gentle day. Room to breathe.' up to ~4, then 'A full day, but doable.', then 'A lot on. Be gentle with yourself.') reflects the count of unfinished one-offs, honest, never alarming, hidden on a clear day.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Select several', tap a few tasks to select, then use the bar: Done / Tomorrow / Remove. Cancel exits.</t>
+          <t>Tap-and-hold a task to enter selection, tap more to add them (or 'Select all'), then use the bar: Done / Tomorrow / Move to... / Remove. Cancel exits.</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Rows become checkboxes, the count updates, the bulk action applies to all selected at once and exits select mode. Long-press still gives a single task its own menu.</t>
+          <t>Rows become checkboxes, the count updates, 'Break down' hides once more than one is selected, the bulk action applies to all at once and exits select mode.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1546,32 +1546,32 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>TOD-13</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Today</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Move selected tasks to a chosen day</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>Tap-and-hold to select one or more tasks, tap 'Move to...', then pick 'This weekend', 'Next week', or a calendar day.</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>Selected one-offs move to that date and wait in the Later list until then (recurring tasks are left alone); select mode exits.</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1586,7 +1586,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1594,24 +1594,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1626,7 +1626,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -1641,17 +1641,17 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1666,7 +1666,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1681,17 +1681,17 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1706,12 +1706,12 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1746,12 +1746,12 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
@@ -1761,17 +1761,17 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1786,32 +1786,32 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -1826,7 +1826,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1841,17 +1841,17 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,7 +1866,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1874,24 +1874,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1921,17 +1921,17 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,37 +1946,37 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr"/>
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2001,22 +2001,22 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr"/>
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2041,17 +2041,17 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2074,24 +2074,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2121,22 +2121,22 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr"/>
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2161,22 +2161,22 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr"/>
@@ -2186,32 +2186,32 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2281,17 +2281,17 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2314,24 +2314,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2401,17 +2401,17 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,37 +2426,37 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr"/>
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2481,22 +2481,22 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr"/>
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2521,17 +2521,17 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2554,24 +2554,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C46" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2586,32 +2586,32 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,22 +2641,22 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr"/>
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2761,17 +2761,17 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2794,29 +2794,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C52" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr"/>
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,22 +2841,22 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2866,37 +2866,37 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2914,24 +2914,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C55" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,17 +2961,17 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3001,17 +3001,17 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3041,17 +3041,17 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,12 +3066,12 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
@@ -3081,22 +3081,22 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr"/>
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3121,22 +3121,22 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr"/>
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3154,24 +3154,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C61" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,37 +3186,37 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3234,24 +3234,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3281,17 +3281,17 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,32 +3306,32 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3354,24 +3354,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C66" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,37 +3386,37 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,12 +3426,12 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,22 +3481,22 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3514,29 +3514,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,37 +3546,37 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C71" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3601,22 +3601,22 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,22 +3681,22 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr"/>
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3721,22 +3721,22 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr"/>
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3754,24 +3754,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C76" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3801,22 +3801,22 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3834,29 +3834,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr"/>
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3881,17 +3881,17 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3921,17 +3921,17 @@
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3954,24 +3954,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C81" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -3983,9 +3983,49 @@
       <c r="I81" s="9" t="inlineStr"/>
       <c r="J81" s="7" t="inlineStr"/>
     </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F82" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H82" s="7" t="inlineStr"/>
+      <c r="I82" s="9" t="inlineStr"/>
+      <c r="J82" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J81"/>
-  <conditionalFormatting sqref="H2:H81">
+  <autoFilter ref="A1:J82"/>
+  <conditionalFormatting sqref="H2:H82">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3997,7 +4037,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4033,7 +4073,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>81</t>
         </is>
       </c>
     </row>
@@ -4044,7 +4084,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$81,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$82,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -4055,7 +4095,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$81,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$82,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -4066,7 +4106,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$81,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$82,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -4077,7 +4117,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$81,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$82,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -4088,7 +4128,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>80-COUNTA('Test Suite'!$H$2:$H$81)</f>
+        <f>81-COUNTA('Test Suite'!$H$2:$H$82)</f>
         <v/>
       </c>
     </row>
@@ -4099,7 +4139,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$81,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$82,"P1")</f>
         <v/>
       </c>
     </row>
@@ -4110,7 +4150,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$81,"P1",'Test Suite'!$H$2:$H$81,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$82,"P1",'Test Suite'!$H$2:$H$82,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(welcome): replay from Settings, non-destructive (merges, never overwrites)
Melroy: the first-run is lovely but should be repeatable. Added "See the welcome
again" to Settings (not a "?" on Today, which was just decluttered; replay is an
occasional action, Settings' job). The link opens /welcome?replay=1; in replay mode
the flow is identical but confirm() MERGES the triaged tasks into the existing list
and leaves the onboarded flag alone, so re-running can never wipe a real list.

Verified in preview: seeded two tasks, replayed, dumped two more, confirmed -> four
tasks, both kept and both added. Added E2E case ONB-02.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1626,32 +1626,32 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>ONB-02</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Replay the welcome from Settings (non-destructive)</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1666,7 +1666,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1674,24 +1674,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1706,7 +1706,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1761,17 +1761,17 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1786,12 +1786,12 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
@@ -1801,17 +1801,17 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -1826,12 +1826,12 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -1841,17 +1841,17 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,32 +1866,32 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1921,17 +1921,17 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1954,24 +1954,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2001,17 +2001,17 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,37 +2026,37 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr"/>
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2081,22 +2081,22 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr"/>
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2121,17 +2121,17 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2154,24 +2154,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2201,22 +2201,22 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr"/>
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,22 +2241,22 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr"/>
@@ -2266,32 +2266,32 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2321,17 +2321,17 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2394,24 +2394,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2441,17 +2441,17 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2481,17 +2481,17 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,37 +2506,37 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr"/>
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,22 +2561,22 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr"/>
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,17 +2601,17 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2634,24 +2634,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,32 +2666,32 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2721,22 +2721,22 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr"/>
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2761,17 +2761,17 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2801,17 +2801,17 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,17 +2841,17 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2874,29 +2874,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,22 +2921,22 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2946,37 +2946,37 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr"/>
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -2994,24 +2994,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C57" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3041,17 +3041,17 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3081,17 +3081,17 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3121,17 +3121,17 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,12 +3146,12 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -3161,22 +3161,22 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3201,22 +3201,22 @@
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3234,24 +3234,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C63" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,37 +3266,37 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3314,24 +3314,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,17 +3361,17 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,32 +3386,32 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3434,24 +3434,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C68" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -3466,37 +3466,37 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,12 +3506,12 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
@@ -3521,22 +3521,22 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,22 +3561,22 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3594,29 +3594,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C72" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,37 +3626,37 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,22 +3681,22 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr"/>
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3721,17 +3721,17 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3761,22 +3761,22 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr"/>
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3801,22 +3801,22 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3834,24 +3834,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C78" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3881,22 +3881,22 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3914,29 +3914,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C80" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr"/>
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3961,17 +3961,17 @@
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -3986,7 +3986,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -4001,17 +4001,17 @@
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4034,24 +4034,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C83" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
@@ -4063,9 +4063,49 @@
       <c r="I83" s="9" t="inlineStr"/>
       <c r="J83" s="7" t="inlineStr"/>
     </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F84" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G84" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H84" s="7" t="inlineStr"/>
+      <c r="I84" s="9" t="inlineStr"/>
+      <c r="J84" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J83"/>
-  <conditionalFormatting sqref="H2:H83">
+  <autoFilter ref="A1:J84"/>
+  <conditionalFormatting sqref="H2:H84">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -4077,7 +4117,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4113,7 +4153,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>83</t>
         </is>
       </c>
     </row>
@@ -4124,7 +4164,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$83,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$84,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -4135,7 +4175,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$83,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$84,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -4146,7 +4186,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$83,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$84,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -4157,7 +4197,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$83,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$84,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -4168,7 +4208,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>82-COUNTA('Test Suite'!$H$2:$H$83)</f>
+        <f>83-COUNTA('Test Suite'!$H$2:$H$84)</f>
         <v/>
       </c>
     </row>
@@ -4179,7 +4219,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$83,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$84,"P1")</f>
         <v/>
       </c>
     </row>
@@ -4190,7 +4230,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$83,"P1",'Test Suite'!$H$2:$H$83,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$84,"P1",'Test Suite'!$H$2:$H$84,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(haptics): tactile cues on Android, gated on reduced motion
Earned-moment haptics for the native build via expo-haptics, behind a platform-split lib (haptics.ts native, haptics.web.ts no-op) so the web bundle never imports the native module. Cues: soft tap on completing a task, a fuller success when the day clears, a warm tap on the gentle close, a light tap when steps land, and a success flourish at the scrapbook reveal.

Each cue takes the resolved reduced-motion flag from useReducedMotion(), so the accessibility gate is type-enforced at every call site; a unit test locks the guarantee that reduced motion silences every cue. No new setting (the existing Motion control covers it), no buzz on errors (RSD-safe), and the scrapbook cue marks the reveal rather than a sustained generation rumble (see decision-log).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1586,37 +1586,37 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>ONB-01</t>
+          <t>HAP-01</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Haptics</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Guided welcome on first run</t>
+          <t>Earned-moment haptics fire (Android)</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
+          <t>On a physical Android device with a haptic motor: complete a single task; clear the whole day; close the day with Goodnight; break a dreaded task into steps; and (premium) reveal a scrapbook.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
+          <t>Soft tap on a single completion; a fuller success buzz when the day clears; a warm soft tap on Goodnight; a light tap when steps land; a success flourish when the scrapbook image appears. Nothing buzzes on plain taps, navigation, capture, or any error.</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr"/>
@@ -1626,12 +1626,12 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>ONB-02</t>
+          <t>HAP-02</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Haptics</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -1641,22 +1641,22 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Replay the welcome from Settings (non-destructive)</t>
+          <t>Reduced motion silences haptics</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
+          <t>Set Settings -&gt; Motion -&gt; Reduce (or enable the OS reduce-motion), then complete a task and close the day.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
+          <t>No haptic fires for any cue while motion is reduced (the accessibility guarantee). The Motion hint states Reduce also stops the buzz.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr"/>
@@ -1666,12 +1666,12 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>ONB-01</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -1681,17 +1681,17 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Guided welcome on first run</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1706,12 +1706,12 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>ONB-02</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Replay the welcome from Settings (non-destructive)</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1754,24 +1754,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1801,17 +1801,17 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -1826,12 +1826,12 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -1841,17 +1841,17 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,12 +1866,12 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -1881,17 +1881,17 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,32 +1906,32 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI triage</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,32 +1946,32 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -1994,24 +1994,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2034,24 +2034,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,37 +2066,37 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr"/>
@@ -2106,32 +2106,32 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2161,22 +2161,22 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr"/>
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2194,24 +2194,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2234,29 +2234,29 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr"/>
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2281,17 +2281,17 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,37 +2306,37 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr"/>
@@ -2346,32 +2346,32 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2401,17 +2401,17 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2434,24 +2434,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2474,24 +2474,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2521,17 +2521,17 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,37 +2546,37 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr"/>
@@ -2586,32 +2586,32 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,22 +2641,22 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr"/>
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2674,24 +2674,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C49" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,12 +2706,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
+          <t>Account deletion</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,37 +2746,37 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr"/>
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2801,22 +2801,22 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr"/>
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,17 +2841,17 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2881,17 +2881,17 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2914,29 +2914,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C55" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2954,24 +2954,24 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C56" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,37 +2986,37 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>
@@ -3026,12 +3026,12 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -3041,22 +3041,22 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr"/>
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3074,24 +3074,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C59" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3121,17 +3121,17 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3161,17 +3161,17 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,12 +3186,12 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
@@ -3201,22 +3201,22 @@
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,12 +3226,12 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
@@ -3241,17 +3241,17 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3274,29 +3274,29 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,37 +3306,37 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3346,37 +3346,37 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C66" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3394,24 +3394,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C67" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,32 +3426,32 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C68" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -3466,12 +3466,12 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
+          <t>Visual</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -3481,17 +3481,17 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -3506,12 +3506,12 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
+          <t>Reminders</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
@@ -3521,22 +3521,22 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,37 +3546,37 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C71" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,12 +3586,12 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
@@ -3601,22 +3601,22 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3634,29 +3634,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C73" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3666,12 +3666,12 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Deploy</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
@@ -3681,22 +3681,22 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr"/>
@@ -3706,32 +3706,32 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3761,22 +3761,22 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr"/>
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3801,22 +3801,22 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3841,17 +3841,17 @@
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3874,29 +3874,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C79" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3914,29 +3914,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C80" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr"/>
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3954,29 +3954,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C81" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr"/>
@@ -3986,7 +3986,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -3994,29 +3994,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C82" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr"/>
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4041,17 +4041,17 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
@@ -4066,7 +4066,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4074,24 +4074,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C84" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
@@ -4103,9 +4103,89 @@
       <c r="I84" s="9" t="inlineStr"/>
       <c r="J84" s="7" t="inlineStr"/>
     </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>PREM-09</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>Cancel reverts to free</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="inlineStr">
+        <is>
+          <t>In the portal, cancel immediately, then return to the app.</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="inlineStr">
+        <is>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H85" s="7" t="inlineStr"/>
+      <c r="I85" s="9" t="inlineStr"/>
+      <c r="J85" s="7" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D86" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E86" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F86" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G86" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H86" s="7" t="inlineStr"/>
+      <c r="I86" s="9" t="inlineStr"/>
+      <c r="J86" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J84"/>
-  <conditionalFormatting sqref="H2:H84">
+  <autoFilter ref="A1:J86"/>
+  <conditionalFormatting sqref="H2:H86">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -4117,7 +4197,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4153,7 +4233,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>85</t>
         </is>
       </c>
     </row>
@@ -4164,7 +4244,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$84,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$86,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -4175,7 +4255,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$84,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$86,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -4186,7 +4266,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$84,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$86,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -4197,7 +4277,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$84,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$86,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -4208,7 +4288,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>83-COUNTA('Test Suite'!$H$2:$H$84)</f>
+        <f>85-COUNTA('Test Suite'!$H$2:$H$86)</f>
         <v/>
       </c>
     </row>
@@ -4219,7 +4299,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$84,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$86,"P1")</f>
         <v/>
       </c>
     </row>
@@ -4230,7 +4310,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$84,"P1",'Test Suite'!$H$2:$H$84,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$86,"P1",'Test Suite'!$H$2:$H$86,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(android): launcher shortcuts + the inbound bridge
Long-press the icon for 'Brain dump' (open with the capture box focused) and 'Focus on one thing' (jump into Focus mode): one-tap capture/act for an ADHD brain. A small pure lib/inbound.ts bridge stashes a launch intent at the root; Today drains it once. BrainDump gains an imperative seed(text|null) via forwardRef (the React Compiler lint forbids setState in an effect, so a ref method plus a subscribe-only effect are the clean shape). Registered with expo-quick-actions setItems/initial/addListener; web gates it out.

The same bridge serves shared text next. The suite caught up with on-device cases for the native batch (keep-awake, system bars, shortcuts).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J86"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1666,37 +1666,37 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>ONB-01</t>
+          <t>AND-01</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Guided welcome on first run</t>
+          <t>Screen stays awake in Focus mode</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
+          <t>On an Android device, open Focus (Focus on one thing) and leave the screen untouched past the usual sleep timeout.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
+          <t>The screen stays on while Focus is open, and returns to normal sleep behaviour once Focus is closed.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr"/>
@@ -1706,37 +1706,37 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>ONB-02</t>
+          <t>AND-02</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Replay the welcome from Settings (non-destructive)</t>
+          <t>System bars match the theme</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
+          <t>On Android, switch the in-app theme (Settings) between light and dark, including a case where the app theme differs from the system theme. Watch the status bar and the bottom navigation bar.</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
+          <t>Status-bar and navigation-bar icons stay legible against the app background in both themes; no white flash on launch or overscroll.</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr"/>
@@ -1746,37 +1746,37 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>AND-03</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Launcher long-press shortcuts</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>On Android, long-press the DoubleDone home-screen icon. Tap 'Brain dump'; relaunch and tap 'Focus on one thing'. Try both from a cold start and with the app backgrounded.</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>'Brain dump' opens the app with the capture box focused and ready to type. 'Focus on one thing' opens directly in Focus mode.</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr"/>
@@ -1786,32 +1786,32 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>ONB-01</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Guided welcome on first run</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -1826,12 +1826,12 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>ONB-02</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -1841,17 +1841,17 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Replay the welcome from Settings (non-destructive)</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,7 +1866,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1874,24 +1874,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,12 +1906,12 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
@@ -1921,17 +1921,17 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,12 +1946,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
@@ -1961,17 +1961,17 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,32 +1986,32 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI decompose</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,32 +2026,32 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI triage</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,12 +2066,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
+          <t>AI strategise</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -2081,17 +2081,17 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2114,24 +2114,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,12 +2146,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
+          <t>Lookback</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
@@ -2161,22 +2161,22 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr"/>
@@ -2186,32 +2186,32 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,32 +2226,32 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2274,29 +2274,29 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr"/>
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2314,29 +2314,29 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr"/>
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2354,24 +2354,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C41" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,32 +2386,32 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,37 +2426,37 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr"/>
@@ -2466,32 +2466,32 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2514,24 +2514,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2554,24 +2554,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C46" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2594,24 +2594,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C47" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,37 +2626,37 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr"/>
@@ -2666,32 +2666,32 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,32 +2706,32 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2754,29 +2754,29 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C51" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr"/>
@@ -2786,12 +2786,12 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
+          <t>Account deletion</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
@@ -2801,17 +2801,17 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,12 +2826,12 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
+          <t>Account deletion</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
@@ -2841,22 +2841,22 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2866,37 +2866,37 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,22 +2921,22 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,17 +2961,17 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -2994,29 +2994,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C57" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3034,24 +3034,24 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C58" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,12 +3066,12 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
@@ -3081,22 +3081,22 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr"/>
@@ -3106,12 +3106,12 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
@@ -3121,22 +3121,22 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr"/>
@@ -3146,12 +3146,12 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -3161,22 +3161,22 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3194,24 +3194,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3241,17 +3241,17 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,12 +3266,12 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
@@ -3281,22 +3281,22 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,12 +3306,12 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
@@ -3321,17 +3321,17 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,32 +3346,32 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="C66" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="C66" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,32 +3386,32 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,12 +3426,12 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,37 +3466,37 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C69" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,12 +3506,12 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
+          <t>Visual</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
@@ -3521,17 +3521,17 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -3546,12 +3546,12 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
+          <t>Visual</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -3561,17 +3561,17 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,37 +3586,37 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,12 +3626,12 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Reminders</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
@@ -3641,22 +3641,22 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3666,32 +3666,32 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,32 +3706,32 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
-        </is>
-      </c>
-      <c r="C75" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Privacy</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,12 +3746,12 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Deploy</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
@@ -3761,22 +3761,22 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr"/>
@@ -3786,12 +3786,12 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Deploy</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
@@ -3801,22 +3801,22 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3826,32 +3826,32 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3881,22 +3881,22 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3921,17 +3921,17 @@
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3954,24 +3954,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C81" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -3986,7 +3986,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -3994,29 +3994,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C82" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr"/>
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4041,22 +4041,22 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr"/>
@@ -4066,7 +4066,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4074,29 +4074,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C84" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -4114,29 +4114,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C85" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr"/>
@@ -4146,7 +4146,7 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
@@ -4154,24 +4154,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C86" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
@@ -4183,9 +4183,129 @@
       <c r="I86" s="9" t="inlineStr"/>
       <c r="J86" s="7" t="inlineStr"/>
     </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>PREM-08</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="inlineStr">
+        <is>
+          <t>Manage subscription opens the billing portal</t>
+        </is>
+      </c>
+      <c r="E87" s="9" t="inlineStr">
+        <is>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="inlineStr">
+        <is>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H87" s="7" t="inlineStr"/>
+      <c r="I87" s="9" t="inlineStr"/>
+      <c r="J87" s="7" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>PREM-09</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="inlineStr">
+        <is>
+          <t>Cancel reverts to free</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="inlineStr">
+        <is>
+          <t>In the portal, cancel immediately, then return to the app.</t>
+        </is>
+      </c>
+      <c r="F88" s="9" t="inlineStr">
+        <is>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+        </is>
+      </c>
+      <c r="G88" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H88" s="7" t="inlineStr"/>
+      <c r="I88" s="9" t="inlineStr"/>
+      <c r="J88" s="7" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E89" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F89" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H89" s="7" t="inlineStr"/>
+      <c r="I89" s="9" t="inlineStr"/>
+      <c r="J89" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J86"/>
-  <conditionalFormatting sqref="H2:H86">
+  <autoFilter ref="A1:J89"/>
+  <conditionalFormatting sqref="H2:H89">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -4197,7 +4317,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4233,7 +4353,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>88</t>
         </is>
       </c>
     </row>
@@ -4244,7 +4364,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$86,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$89,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -4255,7 +4375,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$86,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$89,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -4266,7 +4386,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$86,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$89,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -4277,7 +4397,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$86,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$89,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -4288,7 +4408,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>85-COUNTA('Test Suite'!$H$2:$H$86)</f>
+        <f>88-COUNTA('Test Suite'!$H$2:$H$89)</f>
         <v/>
       </c>
     </row>
@@ -4299,7 +4419,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$86,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$89,"P1")</f>
         <v/>
       </c>
     </row>
@@ -4310,7 +4430,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$86,"P1",'Test Suite'!$H$2:$H$86,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$89,"P1",'Test Suite'!$H$2:$H$89,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(android): share text into DoubleDone (share-sheet target)
DoubleDone appears in the Android share sheet: share text or a URL from any app and it lands in the capture box on Today, ready to add. Reuses the inbound bridge (a capture intent seeds the box). Behind a platform split (share-intent.ts native / .web.ts no-op) so expo-share-intent never enters the web bundle. The plugin's default text/* SEND filter covers text and URLs, so no app.json config was needed.

Seed-then-add (not auto-add) keeps a shared URL or quote one edit from done. expo-share-intent 7.0.0 targets SDK 56; its npm-audit advisories are the pre-existing Expo build-toolchain chain, not shipped.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J89"/>
+  <dimension ref="A1:J90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1786,37 +1786,37 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>ONB-01</t>
+          <t>AND-04</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Guided welcome on first run</t>
+          <t>Share text into DoubleDone</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
+          <t>On Android, from another app (a browser, notes, a chat) use the system Share sheet and pick DoubleDone. Try sharing a line of text, and a URL.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
+          <t>DoubleDone opens with the shared text (or URL) already in the capture box on Today, focused and ready to add. Adding it makes a normal task; nothing is sent anywhere until you do.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>ONB-02</t>
+          <t>ONB-01</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1834,24 +1834,24 @@
           <t>Onboarding</t>
         </is>
       </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Replay the welcome from Settings (non-destructive)</t>
+          <t>Guided welcome on first run</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
+          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
+          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,32 +1866,32 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>ONB-02</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Replay the welcome from Settings (non-destructive)</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1914,24 +1914,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1961,17 +1961,17 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2001,17 +2001,17 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,12 +2026,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
@@ -2041,17 +2041,17 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,12 +2066,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -2081,17 +2081,17 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,32 +2106,32 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2194,24 +2194,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,37 +2266,37 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr"/>
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2321,22 +2321,22 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr"/>
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2394,24 +2394,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2441,22 +2441,22 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr"/>
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2481,22 +2481,22 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr"/>
@@ -2506,32 +2506,32 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,17 +2561,17 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,17 +2601,17 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2634,24 +2634,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C48" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,37 +2746,37 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr"/>
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2801,22 +2801,22 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr"/>
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,17 +2841,17 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2874,24 +2874,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C54" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,32 +2906,32 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,22 +2961,22 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr"/>
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3001,17 +3001,17 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3041,17 +3041,17 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3081,17 +3081,17 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3114,29 +3114,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr"/>
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3161,22 +3161,22 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,37 +3186,37 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3234,24 +3234,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3281,17 +3281,17 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3321,17 +3321,17 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,17 +3361,17 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,12 +3386,12 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -3401,22 +3401,22 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3474,24 +3474,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C69" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -3506,37 +3506,37 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3554,24 +3554,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C71" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3601,17 +3601,17 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3626,32 +3626,32 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3674,24 +3674,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C74" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,37 +3706,37 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr"/>
@@ -3746,12 +3746,12 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
@@ -3761,22 +3761,22 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr"/>
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3801,22 +3801,22 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3834,29 +3834,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C78" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr"/>
@@ -3866,37 +3866,37 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C79" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3921,22 +3921,22 @@
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr"/>
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3961,17 +3961,17 @@
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -3986,7 +3986,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -4001,22 +4001,22 @@
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr"/>
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4041,22 +4041,22 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr"/>
@@ -4066,7 +4066,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4074,24 +4074,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C84" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
@@ -4106,7 +4106,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -4121,22 +4121,22 @@
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr"/>
@@ -4146,7 +4146,7 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
@@ -4154,29 +4154,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C86" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr"/>
@@ -4186,7 +4186,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -4201,17 +4201,17 @@
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
@@ -4226,7 +4226,7 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -4241,17 +4241,17 @@
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
@@ -4266,7 +4266,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -4274,24 +4274,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C89" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
@@ -4303,9 +4303,49 @@
       <c r="I89" s="9" t="inlineStr"/>
       <c r="J89" s="7" t="inlineStr"/>
     </row>
+    <row r="90">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F90" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G90" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H90" s="7" t="inlineStr"/>
+      <c r="I90" s="9" t="inlineStr"/>
+      <c r="J90" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J89"/>
-  <conditionalFormatting sqref="H2:H89">
+  <autoFilter ref="A1:J90"/>
+  <conditionalFormatting sqref="H2:H90">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -4317,7 +4357,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4353,7 +4393,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>89</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4404,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$89,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$90,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -4375,7 +4415,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$89,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$90,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -4386,7 +4426,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$89,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$90,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -4397,7 +4437,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$89,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$90,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -4408,7 +4448,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>88-COUNTA('Test Suite'!$H$2:$H$89)</f>
+        <f>89-COUNTA('Test Suite'!$H$2:$H$90)</f>
         <v/>
       </c>
     </row>
@@ -4419,7 +4459,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$89,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$90,"P1")</f>
         <v/>
       </c>
     </row>
@@ -4430,7 +4470,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$89,"P1",'Test Suite'!$H$2:$H$89,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$90,"P1",'Test Suite'!$H$2:$H$90,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(android): home-screen Today widget
A native Android widget showing today: the top unfinished titles, or a calm rested line (all done / nothing yet / closed), Dusk light+dark, tap to open. Built on react-native-android-widget; the headless render task reads the same AsyncStorage the app writes and reuses the app's pure today-filter plus a new buildWidgetModel (one source of truth). The app pushes requestWidgetUpdate from commit; a 30-minute periodic update is the fallback.

Web-safe via platform splits (register/update .web no-ops) and a custom index.js entry that registers the headless task on native only. Verified the web app still boots from the new entry and the plugin generates a valid AppWidgetProvider (expo config introspect). 5 view-model tests.

The native build on RN 0.85 (library tested on 0.83) is the genuine test; see decision-log.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J90"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1826,37 +1826,37 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>ONB-01</t>
+          <t>AND-05</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Guided welcome on first run</t>
+          <t>Home-screen Today widget</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
+          <t>On Android, long-press the home screen and add the 'DoubleDone: Today' widget. Check it with tasks left, with all done, and after closing the day. Complete a task in the app and watch the widget. Tap the widget.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
+          <t>The widget shows today's top unfinished titles (or a calm 'All done for today.' / 'Nothing for today yet.'), in light or dark to match the device. It refreshes within a moment of a change in the app (and at least every 30 minutes). Tapping it opens DoubleDone.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr"/>
@@ -1866,7 +1866,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>ONB-02</t>
+          <t>ONB-01</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1874,24 +1874,24 @@
           <t>Onboarding</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Replay the welcome from Settings (non-destructive)</t>
+          <t>Guided welcome on first run</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
+          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
+          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,32 +1906,32 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>ONB-02</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Replay the welcome from Settings (non-destructive)</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1954,24 +1954,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2001,17 +2001,17 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2041,17 +2041,17 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,12 +2066,12 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -2081,17 +2081,17 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,12 +2106,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
@@ -2121,17 +2121,17 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,32 +2146,32 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2201,17 +2201,17 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2234,24 +2234,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2281,17 +2281,17 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,37 +2306,37 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr"/>
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2361,22 +2361,22 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr"/>
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2401,17 +2401,17 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2434,24 +2434,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2481,22 +2481,22 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr"/>
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2521,22 +2521,22 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr"/>
@@ -2546,32 +2546,32 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,17 +2601,17 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,17 +2641,17 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2674,24 +2674,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2761,17 +2761,17 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,37 +2786,37 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr"/>
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,22 +2841,22 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2881,17 +2881,17 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2914,24 +2914,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C55" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,32 +2946,32 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3001,22 +3001,22 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3041,17 +3041,17 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3081,17 +3081,17 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3121,17 +3121,17 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3154,29 +3154,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C61" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3201,22 +3201,22 @@
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,37 +3226,37 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr"/>
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3274,24 +3274,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C64" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3321,17 +3321,17 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,17 +3361,17 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,17 +3401,17 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,12 +3426,12 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,22 +3481,22 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3514,24 +3514,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C70" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C70" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -3546,37 +3546,37 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3594,24 +3594,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C72" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,32 +3666,32 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3714,24 +3714,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C75" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,37 +3746,37 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr"/>
@@ -3786,12 +3786,12 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
@@ -3801,22 +3801,22 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3841,22 +3841,22 @@
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr"/>
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3874,29 +3874,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C79" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3906,37 +3906,37 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C80" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr"/>
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3961,22 +3961,22 @@
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr"/>
@@ -3986,7 +3986,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -4001,17 +4001,17 @@
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4041,22 +4041,22 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr"/>
@@ -4066,7 +4066,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4081,22 +4081,22 @@
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -4114,24 +4114,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C85" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
@@ -4146,7 +4146,7 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
@@ -4161,22 +4161,22 @@
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr"/>
@@ -4186,7 +4186,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -4194,29 +4194,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr"/>
@@ -4226,7 +4226,7 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -4241,17 +4241,17 @@
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
@@ -4266,7 +4266,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -4281,17 +4281,17 @@
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
@@ -4306,7 +4306,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
@@ -4314,24 +4314,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C90" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
@@ -4343,9 +4343,49 @@
       <c r="I90" s="9" t="inlineStr"/>
       <c r="J90" s="7" t="inlineStr"/>
     </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D91" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F91" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G91" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H91" s="7" t="inlineStr"/>
+      <c r="I91" s="9" t="inlineStr"/>
+      <c r="J91" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J90"/>
-  <conditionalFormatting sqref="H2:H90">
+  <autoFilter ref="A1:J91"/>
+  <conditionalFormatting sqref="H2:H91">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -4357,7 +4397,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4393,7 +4433,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -4404,7 +4444,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$90,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$91,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -4415,7 +4455,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$90,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$91,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -4426,7 +4466,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$90,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$91,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -4437,7 +4477,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$90,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$91,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -4448,7 +4488,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>89-COUNTA('Test Suite'!$H$2:$H$90)</f>
+        <f>90-COUNTA('Test Suite'!$H$2:$H$91)</f>
         <v/>
       </c>
     </row>
@@ -4459,7 +4499,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$90,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$91,"P1")</f>
         <v/>
       </c>
     </row>
@@ -4470,7 +4510,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$90,"P1",'Test Suite'!$H$2:$H$90,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$91,"P1",'Test Suite'!$H$2:$H$91,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(android): per-task 'remind me in X hours' nudges (Phase 1)
A gentle, local per-task nudge for today tasks: tap-and-hold a task, 'Remind me', pick In 1 hour / In 3 hours / This evening. Fires a local notification (task as title, 'whenever you are ready'); the row shows a bell + time. A poke, never a deadline - relative deferral, the sibling of push-to-tomorrow one scale down.

Pure nudge.ts enforces a 9pm cutoff (no small-hours pokes; late presets hidden). One clearNudgeIfAny helper cancels the nudge when a task is done / removed / deferred, so you are never poked about a handled task. The daily reminder now cancels only itself (fixed id), so it and the nudges coexist on separate channels. Fully local - nothing leaves the phone. Native only; web no-ops and hides the action (web reminders are Phase 2). 8 unit tests.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1866,37 +1866,37 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>ONB-01</t>
+          <t>AND-06</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Guided welcome on first run</t>
+          <t>Remind me in X hours (per-task nudge)</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
+          <t>On Android, tap-and-hold a today task, tap 'Remind me', pick a preset (e.g. 'In 1 hour'). Check the row indicator. Then complete (or remove, or push to tomorrow) the task before the nudge fires. Separately, open 'Remind me' after 9pm.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
+          <t>A local notification fires at the chosen time (the task as the title, 'Whenever you are ready.' as the body); the row shows a small bell + time. Completing / removing / deferring the task cancels the pending nudge (no poke about a handled task). After 9pm the late presets are hidden. Web does not show 'Remind me'.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr"/>
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>ONB-02</t>
+          <t>ONB-01</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1914,24 +1914,24 @@
           <t>Onboarding</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Replay the welcome from Settings (non-destructive)</t>
+          <t>Guided welcome on first run</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
+          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
+          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,32 +1946,32 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>ONB-02</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Replay the welcome from Settings (non-destructive)</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -1994,24 +1994,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2041,17 +2041,17 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2081,17 +2081,17 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,12 +2106,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
@@ -2121,17 +2121,17 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,12 +2146,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,32 +2186,32 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2274,24 +2274,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2321,17 +2321,17 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2346,37 +2346,37 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr"/>
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2401,22 +2401,22 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr"/>
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2441,17 +2441,17 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2474,24 +2474,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2521,22 +2521,22 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr"/>
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,22 +2561,22 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr"/>
@@ -2586,32 +2586,32 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,17 +2641,17 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2714,24 +2714,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2761,17 +2761,17 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2801,17 +2801,17 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,37 +2826,37 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2881,22 +2881,22 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,17 +2921,17 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2954,24 +2954,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C56" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,32 +2986,32 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3041,22 +3041,22 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr"/>
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3081,17 +3081,17 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3121,17 +3121,17 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3161,17 +3161,17 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3194,29 +3194,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3241,22 +3241,22 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr"/>
@@ -3266,37 +3266,37 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3314,24 +3314,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,17 +3361,17 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,17 +3401,17 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,17 +3441,17 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -3466,12 +3466,12 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -3481,22 +3481,22 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3521,22 +3521,22 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3554,24 +3554,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C71" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C71" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,37 +3586,37 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3634,24 +3634,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C73" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,17 +3681,17 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,32 +3706,32 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3754,24 +3754,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C76" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3786,37 +3786,37 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C77" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3826,12 +3826,12 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
@@ -3841,22 +3841,22 @@
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr"/>
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3881,22 +3881,22 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3914,29 +3914,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C80" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr"/>
@@ -3946,37 +3946,37 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C81" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr"/>
@@ -3986,7 +3986,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -4001,22 +4001,22 @@
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr"/>
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4041,17 +4041,17 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
@@ -4066,7 +4066,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4081,22 +4081,22 @@
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -4121,22 +4121,22 @@
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr"/>
@@ -4146,7 +4146,7 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
@@ -4154,24 +4154,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C86" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
@@ -4186,7 +4186,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -4201,22 +4201,22 @@
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr"/>
@@ -4226,7 +4226,7 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -4234,29 +4234,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C88" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr"/>
@@ -4266,7 +4266,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -4281,17 +4281,17 @@
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
@@ -4306,7 +4306,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
@@ -4321,17 +4321,17 @@
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
@@ -4346,7 +4346,7 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
@@ -4354,24 +4354,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C91" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
@@ -4383,9 +4383,49 @@
       <c r="I91" s="9" t="inlineStr"/>
       <c r="J91" s="7" t="inlineStr"/>
     </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D92" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E92" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F92" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H92" s="7" t="inlineStr"/>
+      <c r="I92" s="9" t="inlineStr"/>
+      <c r="J92" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J91"/>
-  <conditionalFormatting sqref="H2:H91">
+  <autoFilter ref="A1:J92"/>
+  <conditionalFormatting sqref="H2:H92">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -4397,7 +4437,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4433,7 +4473,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>91</t>
         </is>
       </c>
     </row>
@@ -4444,7 +4484,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$91,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$92,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -4455,7 +4495,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$91,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$92,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -4466,7 +4506,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$91,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$92,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -4477,7 +4517,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$91,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$92,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -4488,7 +4528,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>90-COUNTA('Test Suite'!$H$2:$H$91)</f>
+        <f>91-COUNTA('Test Suite'!$H$2:$H$92)</f>
         <v/>
       </c>
     </row>
@@ -4499,7 +4539,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$91,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$92,"P1")</f>
         <v/>
       </c>
     </row>
@@ -4510,7 +4550,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$91,"P1",'Test Suite'!$H$2:$H$91,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$92,"P1",'Test Suite'!$H$2:$H$92,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(push): VAPID sender + daily cron (Phase 2, part 3)
The sender. webpush.ts signs a VAPID JWT (ES256) with Web Crypto and POSTs a payloadless push (no body) to the subscription endpoint - no payload encryption, the message lives in the service worker, so nothing about the user crosses the wire. The public key is derived from the private JWK (only VAPID_PRIVATE_KEY + VAPID_SUBJECT secrets needed). A sign-then-verify roundtrip test proves the signing.

An hourly Cloudflare Cron Trigger fires scheduled() -> sendDailyNudges: send to each sub whose local hour matches now, prune 404/410. Phase 2 is code-complete; gen-vapid.mjs + deploy config (keys, secrets, D1 migration, cron) are Melroy's. 12 push/webpush tests.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J92"/>
+  <dimension ref="A1:J93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1906,37 +1906,37 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>ONB-01</t>
+          <t>WEB-01</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Guided welcome on first run</t>
+          <t>Daily reminder via web push</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
+          <t>On the deployed web app (PC or Android Chrome) with VAPID configured, toggle 'Daily reminder' on and allow notifications. Check around your daily hour (the hourly cron can be run manually to verify without waiting).</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
+          <t>Toggling on registers a service worker and subscribes the browser; a calm 'Your today is here when you are ready.' notification arrives around the daily hour, and tapping it opens the app. Toggling off unsubscribes. The push carries no task content. The toggle is hidden when VAPID is unconfigured.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr"/>
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>ONB-02</t>
+          <t>ONB-01</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1954,24 +1954,24 @@
           <t>Onboarding</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Replay the welcome from Settings (non-destructive)</t>
+          <t>Guided welcome on first run</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
+          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
+          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,32 +1986,32 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>ONB-02</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Replay the welcome from Settings (non-destructive)</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2034,24 +2034,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2081,17 +2081,17 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2121,17 +2121,17 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,12 +2146,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,12 +2186,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
@@ -2201,17 +2201,17 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,32 +2226,32 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2281,17 +2281,17 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2314,24 +2314,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2346,7 +2346,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2361,17 +2361,17 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2386,37 +2386,37 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr"/>
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2441,22 +2441,22 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr"/>
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2481,17 +2481,17 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2514,24 +2514,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,22 +2561,22 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr"/>
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,22 +2601,22 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr"/>
@@ -2626,32 +2626,32 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,7 +2746,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2754,24 +2754,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2801,17 +2801,17 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,17 +2841,17 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,37 +2866,37 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,22 +2921,22 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,17 +2961,17 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -2994,24 +2994,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C57" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,32 +3026,32 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3081,22 +3081,22 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr"/>
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3121,17 +3121,17 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3161,17 +3161,17 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3201,17 +3201,17 @@
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3234,29 +3234,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr"/>
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3281,22 +3281,22 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr"/>
@@ -3306,37 +3306,37 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3354,24 +3354,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C66" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,17 +3401,17 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,17 +3441,17 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,17 +3481,17 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -3506,12 +3506,12 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -3521,22 +3521,22 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,22 +3561,22 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3594,24 +3594,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C72" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3626,37 +3626,37 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3674,24 +3674,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C74" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3721,17 +3721,17 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,32 +3746,32 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3794,24 +3794,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C77" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -3826,37 +3826,37 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr"/>
@@ -3866,12 +3866,12 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
@@ -3881,22 +3881,22 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3921,22 +3921,22 @@
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr"/>
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3954,29 +3954,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C81" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr"/>
@@ -3986,37 +3986,37 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C82" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr"/>
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4041,22 +4041,22 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr"/>
@@ -4066,7 +4066,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4081,17 +4081,17 @@
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
@@ -4106,7 +4106,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -4121,22 +4121,22 @@
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr"/>
@@ -4146,7 +4146,7 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
@@ -4161,22 +4161,22 @@
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr"/>
@@ -4186,7 +4186,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -4194,24 +4194,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C87" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
@@ -4226,7 +4226,7 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -4241,22 +4241,22 @@
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr"/>
@@ -4266,7 +4266,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -4274,29 +4274,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C89" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr"/>
@@ -4306,7 +4306,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
@@ -4321,17 +4321,17 @@
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
@@ -4346,7 +4346,7 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
@@ -4361,17 +4361,17 @@
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
@@ -4386,7 +4386,7 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
@@ -4394,24 +4394,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C92" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F92" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
@@ -4423,9 +4423,49 @@
       <c r="I92" s="9" t="inlineStr"/>
       <c r="J92" s="7" t="inlineStr"/>
     </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F93" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G93" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H93" s="7" t="inlineStr"/>
+      <c r="I93" s="9" t="inlineStr"/>
+      <c r="J93" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J92"/>
-  <conditionalFormatting sqref="H2:H92">
+  <autoFilter ref="A1:J93"/>
+  <conditionalFormatting sqref="H2:H93">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -4437,7 +4477,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4473,7 +4513,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>92</t>
         </is>
       </c>
     </row>
@@ -4484,7 +4524,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$92,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$93,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -4495,7 +4535,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$92,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$93,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -4506,7 +4546,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$92,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$93,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -4517,7 +4557,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$92,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$93,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -4528,7 +4568,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>91-COUNTA('Test Suite'!$H$2:$H$92)</f>
+        <f>92-COUNTA('Test Suite'!$H$2:$H$93)</f>
         <v/>
       </c>
     </row>
@@ -4539,7 +4579,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$92,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$93,"P1")</f>
         <v/>
       </c>
     </row>
@@ -4550,7 +4590,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$92,"P1",'Test Suite'!$H$2:$H$92,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$93,"P1",'Test Suite'!$H$2:$H$93,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(capture): relabel the AI split affordance to "Tidy this into tasks"
Voice capture usually yields one rambly sentence ("I feel like I want to do
something fun"), not several discrete things, so the old "More than one thing in
there? Split into tasks" prompt misread the commonest voice case, sitting there
asking "more than one thing?" under a single sentence. "Tidy this into tasks" is
honest whether the AI returns one cleaned task or several. Loading state is now
"Tidying...", the accessibility label matches. Mechanism unchanged (still the
/split route and capture.split.used), only the user-facing copy. Verified in the
preview, CAP-09 updated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -1121,17 +1121,17 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Split a run-on into separate tasks (AI)</t>
+          <t>Tidy a run-on or rambly line into tasks (AI)</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Type or speak a single run-on line of several things ('buy milk and walk the dog and email Sarah'), then tap 'More than one thing in there? Split into tasks'.</t>
+          <t>Type or speak a single long line, either several things ('buy milk and walk the dog and email Sarah') or one rambly thought ('I feel like I want to do something fun'), then tap 'Tidy this into tasks'.</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>The line is replaced by the separate tasks, one per line, in your own words (nothing invented or reordered), and 'Sort for me' then appears to sort them. On failure it degrades calmly ('Couldn't split that just now'), text kept. Works on web and Android. Needs the Worker deployed with /split.</t>
+          <t>The line is replaced by clean task(s) in your own words, nothing invented or reordered. A run-on becomes several lines (and 'Sort for me' appears); a single rambly thought becomes one tidy task ('do something fun'). On failure it degrades calmly ('Couldn't tidy that just now'), text kept. Works on web and Android. Needs the Worker deployed with /split.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat(redesign): the whole-task-finish bloom (slice 3)
The last sub-task of a broken-down task now raises a held celebration instead of a 3.5s text line (Melroy's 'too feeble' feedback). A warm radial bloom over a dimming scrim, an eyebrow, the task in Newsreader italic, and a warm context line, scaled by celebrationTier (quick/real/dreaded) and held for that duration or until tap. completeAncestors widened to return the finished parent objects so the bloom reads the real createdAt/complexity/step-count. finishContext (pure, tested) writes the warm line. Fixed warm-glow palette (same in light and dark). Reduced motion keeps the held title, drops the movement. Manual case AI-09 added.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J105"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2611,7 +2611,7 @@
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>The original task disappears from Today and Later (it becomes a silent parent, not clutter beside its steps). When the last step is done, the real task completes on its own with a bigger 'you finished the whole thing' line and lands in the Lookback as the finished real task. Multi-phase: finishing a milestone's steps cascades up to the root.</t>
+          <t>The original task disappears from Today and Later (it becomes a silent parent, not clutter beside its steps). When the last step is done, the real task completes on its own with the held 'you finished the whole thing' bloom (see AI-09) and lands in the Lookback as the finished real task. Multi-phase: finishing a milestone's steps cascades up to the root.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2666,12 +2666,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-09</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Whole-task finish raises the held bloom (scaled)</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Finish the LAST step of a broken-down task. Try it on a long-lingering or chunky task, and separately on a small same-day one. Then repeat with Reduce Motion on.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A warm radial bloom rises over a dimming scrim: 'You finished the whole thing', the task name in Newsreader italic, and a warm context line ('... since you first wrote it down. N small steps. All done.'). It holds longer and blooms larger for a long-dreaded or chunky task than for a quick same-day one. A tap dismisses it early, otherwise it auto-settles. Never confetti, points, or a number on screen. With Reduce Motion on, the held title and warm colour still show, only the movement is removed.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,12 +2706,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,32 +2746,32 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2801,17 +2801,17 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2834,24 +2834,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C53" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2881,17 +2881,17 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,37 +2906,37 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,22 +2961,22 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr"/>
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3001,17 +3001,17 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3034,24 +3034,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C58" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3081,22 +3081,22 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr"/>
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3121,22 +3121,22 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr"/>
@@ -3146,32 +3146,32 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3201,17 +3201,17 @@
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3241,17 +3241,17 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3274,24 +3274,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C64" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3321,17 +3321,17 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,17 +3361,17 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,37 +3386,37 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,17 +3481,17 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3514,24 +3514,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C70" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -3546,32 +3546,32 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3601,22 +3601,22 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,17 +3681,17 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3721,17 +3721,17 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3754,29 +3754,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C76" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr"/>
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3801,22 +3801,22 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3826,37 +3826,37 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr"/>
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3874,24 +3874,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C79" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3921,17 +3921,17 @@
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3961,17 +3961,17 @@
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -3986,7 +3986,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -4001,17 +4001,17 @@
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
@@ -4026,12 +4026,12 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
@@ -4041,22 +4041,22 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr"/>
@@ -4066,7 +4066,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4081,22 +4081,22 @@
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -4114,24 +4114,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C85" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
@@ -4146,37 +4146,37 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C86" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C86" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr"/>
@@ -4186,7 +4186,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -4194,24 +4194,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C87" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
@@ -4226,7 +4226,7 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -4241,17 +4241,17 @@
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
@@ -4266,32 +4266,32 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C89" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
@@ -4306,7 +4306,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
@@ -4314,24 +4314,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C90" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
@@ -4346,37 +4346,37 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C91" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr"/>
@@ -4386,12 +4386,12 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
@@ -4401,22 +4401,22 @@
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F92" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H92" s="7" t="inlineStr"/>
@@ -4426,7 +4426,7 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
@@ -4441,22 +4441,22 @@
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F93" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr"/>
@@ -4466,7 +4466,7 @@
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
@@ -4474,29 +4474,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C94" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F94" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G94" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr"/>
@@ -4506,37 +4506,37 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F95" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr"/>
@@ -4546,7 +4546,7 @@
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
@@ -4561,22 +4561,22 @@
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F96" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr"/>
@@ -4586,7 +4586,7 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
@@ -4601,17 +4601,17 @@
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F97" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
@@ -4626,7 +4626,7 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
@@ -4641,22 +4641,22 @@
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr"/>
@@ -4666,7 +4666,7 @@
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
@@ -4681,22 +4681,22 @@
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F99" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr"/>
@@ -4706,7 +4706,7 @@
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -4714,24 +4714,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C100" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F100" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G100" s="7" t="inlineStr">
@@ -4746,7 +4746,7 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
@@ -4761,22 +4761,22 @@
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr"/>
@@ -4786,7 +4786,7 @@
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
@@ -4794,29 +4794,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G102" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H102" s="7" t="inlineStr"/>
@@ -4826,7 +4826,7 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
@@ -4841,17 +4841,17 @@
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
@@ -4866,7 +4866,7 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
@@ -4881,17 +4881,17 @@
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
@@ -4906,7 +4906,7 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
@@ -4914,24 +4914,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C105" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
@@ -4943,9 +4943,49 @@
       <c r="I105" s="9" t="inlineStr"/>
       <c r="J105" s="7" t="inlineStr"/>
     </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C106" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E106" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F106" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G106" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H106" s="7" t="inlineStr"/>
+      <c r="I106" s="9" t="inlineStr"/>
+      <c r="J106" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J105"/>
-  <conditionalFormatting sqref="H2:H105">
+  <autoFilter ref="A1:J106"/>
+  <conditionalFormatting sqref="H2:H106">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -4957,7 +4997,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4993,7 +5033,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>105</t>
         </is>
       </c>
     </row>
@@ -5004,7 +5044,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$105,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$106,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -5015,7 +5055,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$105,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$106,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -5026,7 +5066,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$105,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$106,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -5037,7 +5077,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$105,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$106,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -5048,7 +5088,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>104-COUNTA('Test Suite'!$H$2:$H$105)</f>
+        <f>105-COUNTA('Test Suite'!$H$2:$H$106)</f>
         <v/>
       </c>
     </row>
@@ -5059,7 +5099,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$105,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$106,"P1")</f>
         <v/>
       </c>
     </row>
@@ -5070,7 +5110,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$105,"P1",'Test Suite'!$H$2:$H$105,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$106,"P1",'Test Suite'!$H$2:$H$106,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(redesign): Today reborn, Rooms pill + phase greeting + soft cards (slice 4)
The crowded four-link Today header (Repeating, Routines, Lookback, Settings), which wrapped the date on narrow phones, collapses into one translucent Rooms pill that opens a calm bottom sheet (RoomsSheet). The greeting under Today is now phase-aware (phaseGreeting): morning / afternoon / winding-down / late-night. Task rows gain a soft elevation shadow so they float above the living background. Avoided expo-glass-effect for the pill (iOS-only, no-ops on web and Android); a translucent fill over the gradient is the cross-platform call. Manual case TOD-16 added.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1786,7 +1786,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>OCD-01</t>
+          <t>TOD-16</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1801,17 +1801,17 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Done is done (completion affirmation)</t>
+          <t>Rooms pill, phase greeting, soft cards (Today reborn)</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Complete any task: tap a Today task, or select tasks and tap Done.</t>
+          <t>Look at the Today header and the line under 'Today'. Tap the 'Rooms' pill, then a room. Open the app at different times of day.</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>A brief, consistent calm line appears near the capture ('Done is done. Recorded.') and clears itself after a few seconds. It is the SAME line every time (never a rotating or variable reward), reduce-motion safe, and never shaming.</t>
+          <t>The header shows the date plus one 'Rooms' pill (three dots and a label), never the old four-link row that wrapped on narrow phones. Tapping Rooms opens a calm bottom sheet listing Repeating, Routines, Lookback, Settings (each with a one-line hint); tap one to go, tap the scrim to close. The greeting under 'Today' changes with the clock: 'Good morning/afternoon. Just today.', 'Winding down. Just today.' in the evening, a restful line late at night. Task rows sit on a soft shadow, floating a hair above the living background.</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -1826,7 +1826,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>OCD-02</t>
+          <t>OCD-01</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1841,17 +1841,17 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Good enough (release a stuck-perfected task)</t>
+          <t>Done is done (completion affirmation)</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>On Today, long-press a task to select it, then tap 'Good enough'. On a Later task, long-press it and tap 'Good enough' in the menu.</t>
+          <t>Complete any task: tap a Today task, or select tasks and tap Done.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>The task completes with a gentler line ('Good enough is done. Let it go.'). The action only appears for an incomplete one-off. It is permission to release, never a nag.</t>
+          <t>A brief, consistent calm line appears near the capture ('Done is done. Recorded.') and clears itself after a few seconds. It is the SAME line every time (never a rotating or variable reward), reduce-motion safe, and never shaming.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,12 +1866,12 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>RTN-01</t>
+          <t>OCD-02</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Routines</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -1881,17 +1881,17 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Create and run a routine</t>
+          <t>Good enough (release a stuck-perfected task)</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>From the Today header tap Routines, then + New routine. Name it (e.g. Morning), pick Morning / Evening / Anytime, type a few steps one per line, tap Add routine. Then tick some steps.</t>
+          <t>On Today, long-press a task to select it, then tap 'Good enough'. On a Later task, long-press it and tap 'Good enough' in the menu.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>The routine appears grouped under its time-of-day with an 'N of M' progress. Tapping a step marks it done for today (a sage tick and a strike-through) and updates the count. Calm, with no streak and no celebration pressure.</t>
+          <t>The task completes with a gentler line ('Good enough is done. Let it go.'). The action only appears for an incomplete one-off. It is permission to release, never a nag.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,7 +1906,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>RTN-02</t>
+          <t>RTN-01</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1921,17 +1921,17 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>A routine is fresh tomorrow (never a streak)</t>
+          <t>Create and run a routine</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>Tick some routine steps today, then advance the device clock to tomorrow and reopen Routines.</t>
+          <t>From the Today header tap Routines, then + New routine. Name it (e.g. Morning), pick Morning / Evening / Anytime, type a few steps one per line, tap Add routine. Then tick some steps.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Every step is un-ticked again and the progress is back to 0 of M. There is NO streak count, no 'you missed it', and no chain to break: yesterday simply falls away with no guilt (the never-shame spine).</t>
+          <t>The routine appears grouped under its time-of-day with an 'N of M' progress. Tapping a step marks it done for today (a sage tick and a strike-through) and updates the count. Calm, with no streak and no celebration pressure.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>RTN-03</t>
+          <t>RTN-02</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1954,24 +1954,24 @@
           <t>Routines</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Remove a routine (recoverable)</t>
+          <t>A routine is fresh tomorrow (never a streak)</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>On a routine card tap Remove, then optionally tap Undo.</t>
+          <t>Tick some routine steps today, then advance the device clock to tomorrow and reopen Routines.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>The routine is removed with a brief 'Routine removed. Undo' banner, not a confirmation dialog. Tapping Undo within a few seconds restores it, otherwise it stays gone. Recoverable, never a confirm gauntlet.</t>
+          <t>Every step is un-ticked again and the progress is back to 0 of M. There is NO streak count, no 'you missed it', and no chain to break: yesterday simply falls away with no guilt (the never-shame spine).</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,12 +1986,12 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>HAP-01</t>
+          <t>RTN-03</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Haptics</t>
+          <t>Routines</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -2001,22 +2001,22 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Earned-moment haptics fire (Android)</t>
+          <t>Remove a routine (recoverable)</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>On a physical Android device with a haptic motor: complete a single task; clear the whole day; close the day with Goodnight; break a dreaded task into steps; and (premium) reveal a scrapbook.</t>
+          <t>On a routine card tap Remove, then optionally tap Undo.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Soft tap on a single completion; a fuller success buzz when the day clears; a warm soft tap on Goodnight; a light tap when steps land; a success flourish when the scrapbook image appears. Nothing buzzes on plain taps, navigation, capture, or any error.</t>
+          <t>The routine is removed with a brief 'Routine removed. Undo' banner, not a confirmation dialog. Tapping Undo within a few seconds restores it, otherwise it stays gone. Recoverable, never a confirm gauntlet.</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr"/>
@@ -2026,7 +2026,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>HAP-02</t>
+          <t>HAP-01</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2034,24 +2034,24 @@
           <t>Haptics</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Reduced motion silences haptics</t>
+          <t>Earned-moment haptics fire (Android)</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Set Settings -&gt; Motion -&gt; Reduce (or enable the OS reduce-motion), then complete a task and close the day.</t>
+          <t>On a physical Android device with a haptic motor: complete a single task; clear the whole day; close the day with Goodnight; break a dreaded task into steps; and (premium) reveal a scrapbook.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>No haptic fires for any cue while motion is reduced (the accessibility guarantee). The Motion hint states Reduce also stops the buzz.</t>
+          <t>Soft tap on a single completion; a fuller success buzz when the day clears; a warm soft tap on Goodnight; a light tap when steps land; a success flourish when the scrapbook image appears. Nothing buzzes on plain taps, navigation, capture, or any error.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2066,32 +2066,32 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>AND-01</t>
+          <t>HAP-02</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Haptics</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Screen stays awake in Focus mode</t>
+          <t>Reduced motion silences haptics</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>On an Android device, open Focus (Focus on one thing) and leave the screen untouched past the usual sleep timeout.</t>
+          <t>Set Settings -&gt; Motion -&gt; Reduce (or enable the OS reduce-motion), then complete a task and close the day.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>The screen stays on while Focus is open, and returns to normal sleep behaviour once Focus is closed.</t>
+          <t>No haptic fires for any cue while motion is reduced (the accessibility guarantee). The Motion hint states Reduce also stops the buzz.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AND-02</t>
+          <t>AND-01</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2121,17 +2121,17 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>System bars match the theme</t>
+          <t>Screen stays awake in Focus mode</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>On Android, switch the in-app theme (Settings) between light and dark, including a case where the app theme differs from the system theme. Watch the status bar and the bottom navigation bar.</t>
+          <t>On an Android device, open Focus (Focus on one thing) and leave the screen untouched past the usual sleep timeout.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>Status-bar and navigation-bar icons stay legible against the app background in both themes; no white flash on launch or overscroll.</t>
+          <t>The screen stays on while Focus is open, and returns to normal sleep behaviour once Focus is closed.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AND-03</t>
+          <t>AND-02</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2154,24 +2154,24 @@
           <t>Android</t>
         </is>
       </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Launcher long-press shortcuts</t>
+          <t>System bars match the theme</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>On Android, long-press the DoubleDone home-screen icon. Tap 'Brain dump'; relaunch and tap 'Focus on one thing'. Try both from a cold start and with the app backgrounded.</t>
+          <t>On Android, switch the in-app theme (Settings) between light and dark, including a case where the app theme differs from the system theme. Watch the status bar and the bottom navigation bar.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>'Brain dump' opens the app with the capture box focused and ready to type. 'Focus on one thing' opens directly in Focus mode.</t>
+          <t>Status-bar and navigation-bar icons stay legible against the app background in both themes; no white flash on launch or overscroll.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>AND-04</t>
+          <t>AND-03</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2201,17 +2201,17 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Share text into DoubleDone</t>
+          <t>Launcher long-press shortcuts</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>On Android, from another app (a browser, notes, a chat) use the system Share sheet and pick DoubleDone. Try sharing a line of text, and a URL.</t>
+          <t>On Android, long-press the DoubleDone home-screen icon. Tap 'Brain dump'; relaunch and tap 'Focus on one thing'. Try both from a cold start and with the app backgrounded.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>DoubleDone opens with the shared text (or URL) already in the capture box on Today, focused and ready to add. Adding it makes a normal task; nothing is sent anywhere until you do.</t>
+          <t>'Brain dump' opens the app with the capture box focused and ready to type. 'Focus on one thing' opens directly in Focus mode.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>AND-05</t>
+          <t>AND-04</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Home-screen Today widget</t>
+          <t>Share text into DoubleDone</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>On Android, long-press the home screen and add the 'DoubleDone: Today' widget. Check it with tasks left, with all done, and after closing the day. Complete a task in the app and watch the widget. Tap the widget.</t>
+          <t>On Android, from another app (a browser, notes, a chat) use the system Share sheet and pick DoubleDone. Try sharing a line of text, and a URL.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>The widget shows today's top unfinished titles (or a calm 'All done for today.' / 'Nothing for today yet.'), in light or dark to match the device. It refreshes within a moment of a change in the app (and at least every 30 minutes). Tapping it opens DoubleDone.</t>
+          <t>DoubleDone opens with the shared text (or URL) already in the capture box on Today, focused and ready to add. Adding it makes a normal task; nothing is sent anywhere until you do.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>AND-06</t>
+          <t>AND-05</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2281,17 +2281,17 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Remind me in X hours (per-task nudge)</t>
+          <t>Home-screen Today widget</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>On Android, tap-and-hold a today task, tap 'Remind me', pick a preset (e.g. 'In 1 hour'). Check the row indicator. Then complete (or remove, or push to tomorrow) the task before the nudge fires. Separately, open 'Remind me' after 9pm.</t>
+          <t>On Android, long-press the home screen and add the 'DoubleDone: Today' widget. Check it with tasks left, with all done, and after closing the day. Complete a task in the app and watch the widget. Tap the widget.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>A local notification fires at the chosen time (the task as the title, 'Whenever you are ready.' as the body); the row shows a small bell + time. Completing / removing / deferring the task cancels the pending nudge (no poke about a handled task). After 9pm the late presets are hidden. Web does not show 'Remind me'.</t>
+          <t>The widget shows today's top unfinished titles (or a calm 'All done for today.' / 'Nothing for today yet.'), in light or dark to match the device. It refreshes within a moment of a change in the app (and at least every 30 minutes). Tapping it opens DoubleDone.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,12 +2306,12 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>WEB-01</t>
+          <t>AND-06</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
@@ -2321,22 +2321,22 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder via web push</t>
+          <t>Remind me in X hours (per-task nudge)</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>On the deployed web app (PC or Android Chrome) with VAPID configured, toggle 'Daily reminder' on and allow notifications. Check around your daily hour (the hourly cron can be run manually to verify without waiting).</t>
+          <t>On Android, tap-and-hold a today task, tap 'Remind me', pick a preset (e.g. 'In 1 hour'). Check the row indicator. Then complete (or remove, or push to tomorrow) the task before the nudge fires. Separately, open 'Remind me' after 9pm.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Toggling on registers a service worker and subscribes the browser; a calm 'Your today is here when you are ready.' notification arrives around the daily hour, and tapping it opens the app. Toggling off unsubscribes. The push carries no task content. The toggle is hidden when VAPID is unconfigured.</t>
+          <t>A local notification fires at the chosen time (the task as the title, 'Whenever you are ready.' as the body); the row shows a small bell + time. Completing / removing / deferring the task cancels the pending nudge (no poke about a handled task). After 9pm the late presets are hidden. Web does not show 'Remind me'.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr"/>
@@ -2346,37 +2346,37 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>ONB-01</t>
+          <t>WEB-01</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Guided welcome on first run</t>
+          <t>Daily reminder via web push</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
+          <t>On the deployed web app (PC or Android Chrome) with VAPID configured, toggle 'Daily reminder' on and allow notifications. Check around your daily hour (the hourly cron can be run manually to verify without waiting).</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
+          <t>Toggling on registers a service worker and subscribes the browser; a calm 'Your today is here when you are ready.' notification arrives around the daily hour, and tapping it opens the app. Toggling off unsubscribes. The push carries no task content. The toggle is hidden when VAPID is unconfigured.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr"/>
@@ -2386,7 +2386,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>ONB-02</t>
+          <t>ONB-01</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2394,24 +2394,24 @@
           <t>Onboarding</t>
         </is>
       </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Replay the welcome from Settings (non-destructive)</t>
+          <t>Guided welcome on first run</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
+          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
+          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2426,32 +2426,32 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>ONB-02</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Replay the welcome from Settings (non-destructive)</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,7 +2466,7 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2474,24 +2474,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2521,17 +2521,17 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,17 +2561,17 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>AI-07</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,17 +2601,17 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Breakdown keeps the real task as a silent parent (chain)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Break down a task (e.g. 'Plan the party'), then complete all of its steps, in any order.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>The original task disappears from Today and Later (it becomes a silent parent, not clutter beside its steps). When the last step is done, the real task completes on its own with the held 'you finished the whole thing' bloom (see AI-09) and lands in the Lookback as the finished real task. Multi-phase: finishing a milestone's steps cascades up to the root.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>AI-08</t>
+          <t>AI-07</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,17 +2641,17 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Make it tiny keeps the real task (open parent), no pile-up</t>
+          <t>Breakdown keeps the real task as a silent parent (chain)</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>On a dreaded task choose 'Make it tiny' and do the 2-minute version. Then shrink the same task again to confirm pebbles do not accumulate.</t>
+          <t>Break down a task (e.g. 'Plan the party'), then complete all of its steps, in any order.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>The dreaded task disappears and a 2-minute starter takes its place on Today. Completing the starter does NOT mark the big task done: the spent starter is retired (no clutter) and the real task reappears with a calm progress line ('A step done. You're chipping away at X.'). Shrinking the same task repeatedly never piles up duplicate pebbles, only one is open at a time. Make it tiny again for the next step, or just complete the task.</t>
+          <t>The original task disappears from Today and Later (it becomes a silent parent, not clutter beside its steps). When the last step is done, the real task completes on its own with the held 'you finished the whole thing' bloom (see AI-09) and lands in the Lookback as the finished real task. Multi-phase: finishing a milestone's steps cascades up to the root.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>AI-09</t>
+          <t>AI-08</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Whole-task finish raises the held bloom (scaled)</t>
+          <t>Make it tiny keeps the real task (open parent), no pile-up</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Finish the LAST step of a broken-down task. Try it on a long-lingering or chunky task, and separately on a small same-day one. Then repeat with Reduce Motion on.</t>
+          <t>On a dreaded task choose 'Make it tiny' and do the 2-minute version. Then shrink the same task again to confirm pebbles do not accumulate.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>A warm radial bloom rises over a dimming scrim: 'You finished the whole thing', the task name in Newsreader italic, and a warm context line ('... since you first wrote it down. N small steps. All done.'). It holds longer and blooms larger for a long-dreaded or chunky task than for a quick same-day one. A tap dismisses it early, otherwise it auto-settles. Never confetti, points, or a number on screen. With Reduce Motion on, the held title and warm colour still show, only the movement is removed.</t>
+          <t>The dreaded task disappears and a 2-minute starter takes its place on Today. Completing the starter does NOT mark the big task done: the spent starter is retired (no clutter) and the real task reappears with a calm progress line ('A step done. You're chipping away at X.'). Shrinking the same task repeatedly never piles up duplicate pebbles, only one is open at a time. Make it tiny again for the next step, or just complete the task.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,12 +2706,12 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-09</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Whole-task finish raises the held bloom (scaled)</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Finish the LAST step of a broken-down task. Try it on a long-lingering or chunky task, and separately on a small same-day one. Then repeat with Reduce Motion on.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A warm radial bloom rises over a dimming scrim: 'You finished the whole thing', the task name in Newsreader italic, and a warm context line ('... since you first wrote it down. N small steps. All done.'). It holds longer and blooms larger for a long-dreaded or chunky task than for a quick same-day one. A tap dismisses it early, otherwise it auto-settles. Never confetti, points, or a number on screen. With Reduce Motion on, the held title and warm colour still show, only the movement is removed.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,12 +2746,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
@@ -2761,17 +2761,17 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,32 +2786,32 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,17 +2841,17 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2874,24 +2874,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,17 +2921,17 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,37 +2946,37 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr"/>
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3001,22 +3001,22 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3041,17 +3041,17 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3074,24 +3074,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C59" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3121,22 +3121,22 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr"/>
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3161,22 +3161,22 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,32 +3186,32 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3241,17 +3241,17 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3281,17 +3281,17 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3314,24 +3314,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,17 +3361,17 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,17 +3401,17 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,37 +3426,37 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C68" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C68" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,22 +3481,22 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3521,17 +3521,17 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3554,24 +3554,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C71" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,32 +3586,32 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,22 +3641,22 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr"/>
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,17 +3681,17 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3721,17 +3721,17 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3761,17 +3761,17 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3794,29 +3794,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C77" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr"/>
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3841,22 +3841,22 @@
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr"/>
@@ -3866,37 +3866,37 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C79" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3914,24 +3914,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C80" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3961,17 +3961,17 @@
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -3986,7 +3986,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -4001,17 +4001,17 @@
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4041,17 +4041,17 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
@@ -4066,12 +4066,12 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
@@ -4081,22 +4081,22 @@
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -4121,22 +4121,22 @@
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr"/>
@@ -4146,7 +4146,7 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
@@ -4154,24 +4154,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C86" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
@@ -4186,37 +4186,37 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr"/>
@@ -4226,7 +4226,7 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -4234,24 +4234,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C88" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
@@ -4266,7 +4266,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -4281,17 +4281,17 @@
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
@@ -4306,32 +4306,32 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C90" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
@@ -4346,7 +4346,7 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
@@ -4354,24 +4354,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C91" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
@@ -4386,37 +4386,37 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F92" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H92" s="7" t="inlineStr"/>
@@ -4426,12 +4426,12 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
@@ -4441,22 +4441,22 @@
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F93" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr"/>
@@ -4466,7 +4466,7 @@
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
@@ -4481,22 +4481,22 @@
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F94" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G94" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr"/>
@@ -4506,7 +4506,7 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
@@ -4514,29 +4514,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C95" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F95" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr"/>
@@ -4546,37 +4546,37 @@
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C96" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F96" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr"/>
@@ -4586,7 +4586,7 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
@@ -4601,22 +4601,22 @@
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F97" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr"/>
@@ -4626,7 +4626,7 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
@@ -4641,17 +4641,17 @@
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">
@@ -4666,7 +4666,7 @@
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
@@ -4681,22 +4681,22 @@
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F99" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr"/>
@@ -4706,7 +4706,7 @@
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -4721,22 +4721,22 @@
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F100" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G100" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H100" s="7" t="inlineStr"/>
@@ -4746,7 +4746,7 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
@@ -4754,24 +4754,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C101" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
@@ -4786,7 +4786,7 @@
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
@@ -4801,22 +4801,22 @@
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G102" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H102" s="7" t="inlineStr"/>
@@ -4826,7 +4826,7 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
@@ -4834,29 +4834,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C103" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H103" s="7" t="inlineStr"/>
@@ -4866,7 +4866,7 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
@@ -4881,17 +4881,17 @@
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
@@ -4906,7 +4906,7 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
@@ -4921,17 +4921,17 @@
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
@@ -4946,7 +4946,7 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
@@ -4954,24 +4954,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C106" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D106" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F106" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G106" s="7" t="inlineStr">
@@ -4983,9 +4983,49 @@
       <c r="I106" s="9" t="inlineStr"/>
       <c r="J106" s="7" t="inlineStr"/>
     </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C107" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E107" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F107" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G107" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H107" s="7" t="inlineStr"/>
+      <c r="I107" s="9" t="inlineStr"/>
+      <c r="J107" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J106"/>
-  <conditionalFormatting sqref="H2:H106">
+  <autoFilter ref="A1:J107"/>
+  <conditionalFormatting sqref="H2:H107">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -4997,7 +5037,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5033,7 +5073,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>106</t>
         </is>
       </c>
     </row>
@@ -5044,7 +5084,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$106,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$107,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -5055,7 +5095,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$106,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$107,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -5066,7 +5106,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$106,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$107,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -5077,7 +5117,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$106,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$107,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -5088,7 +5128,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>105-COUNTA('Test Suite'!$H$2:$H$106)</f>
+        <f>106-COUNTA('Test Suite'!$H$2:$H$107)</f>
         <v/>
       </c>
     </row>
@@ -5099,7 +5139,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$106,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$107,"P1")</f>
         <v/>
       </c>
     </row>
@@ -5110,7 +5150,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$106,"P1",'Test Suite'!$H$2:$H$106,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$107,"P1",'Test Suite'!$H$2:$H$107,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(redesign): inheriting surfaces, the living background app-wide (slice 6)
Lookback, Settings, Routines, Premium, Sign-in, Privacy, and the first-run welcome now use a transparent screen root, so the single LivingBackground in the root layout breathes through the whole app, not just Today. The Routines card moves to surfaceCard with Today's soft elevation. Legibility holds: the gradient shows only in the margins, text stays on near-opaque cards. This completes the six-slice 'Dusk, evolved' redesign (foundation, living background, whole-task-finish bloom, Today reborn, Make-it-tiny polish, inheriting surfaces). Manual case VIS-01 added.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1826,12 +1826,12 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>OCD-01</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>Visual</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -1841,17 +1841,17 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Done is done (completion affirmation)</t>
+          <t>The living background (app-wide, calm, reduced-motion aware)</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Complete any task: tap a Today task, or select tasks and tap Done.</t>
+          <t>Open the app at different times of day, on light and dark. Move between Today, Routines, Lookback, Settings. Turn on Reduce Motion (in Settings or the OS) and watch the background.</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>A brief, consistent calm line appears near the capture ('Done is done. Recorded.') and clears itself after a few seconds. It is the SAME line every time (never a rotating or variable reward), reduce-motion safe, and never shaming.</t>
+          <t>A soft time-of-day gradient (dawn / day / dusk / night) with two slowly drifting light pools sits behind every screen, not just Today. It only ever shows in the margins: cards and rows stay on near-opaque surfaces, so text is always full-contrast, never washed out over the gradient. With Reduce Motion on, the colour still resolves to the time of day but the drift stops. Navigating between screens never flashes a hard background edge.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1866,7 +1866,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>OCD-02</t>
+          <t>OCD-01</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1881,17 +1881,17 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Good enough (release a stuck-perfected task)</t>
+          <t>Done is done (completion affirmation)</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>On Today, long-press a task to select it, then tap 'Good enough'. On a Later task, long-press it and tap 'Good enough' in the menu.</t>
+          <t>Complete any task: tap a Today task, or select tasks and tap Done.</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>The task completes with a gentler line ('Good enough is done. Let it go.'). The action only appears for an incomplete one-off. It is permission to release, never a nag.</t>
+          <t>A brief, consistent calm line appears near the capture ('Done is done. Recorded.') and clears itself after a few seconds. It is the SAME line every time (never a rotating or variable reward), reduce-motion safe, and never shaming.</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -1906,12 +1906,12 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>RTN-01</t>
+          <t>OCD-02</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Routines</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
@@ -1921,17 +1921,17 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Create and run a routine</t>
+          <t>Good enough (release a stuck-perfected task)</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>From the Today header tap Routines, then + New routine. Name it (e.g. Morning), pick Morning / Evening / Anytime, type a few steps one per line, tap Add routine. Then tick some steps.</t>
+          <t>On Today, long-press a task to select it, then tap 'Good enough'. On a Later task, long-press it and tap 'Good enough' in the menu.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>The routine appears grouped under its time-of-day with an 'N of M' progress. Tapping a step marks it done for today (a sage tick and a strike-through) and updates the count. Calm, with no streak and no celebration pressure.</t>
+          <t>The task completes with a gentler line ('Good enough is done. Let it go.'). The action only appears for an incomplete one-off. It is permission to release, never a nag.</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1946,7 +1946,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>RTN-02</t>
+          <t>RTN-01</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1961,17 +1961,17 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>A routine is fresh tomorrow (never a streak)</t>
+          <t>Create and run a routine</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>Tick some routine steps today, then advance the device clock to tomorrow and reopen Routines.</t>
+          <t>From the Today header tap Routines, then + New routine. Name it (e.g. Morning), pick Morning / Evening / Anytime, type a few steps one per line, tap Add routine. Then tick some steps.</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Every step is un-ticked again and the progress is back to 0 of M. There is NO streak count, no 'you missed it', and no chain to break: yesterday simply falls away with no guilt (the never-shame spine).</t>
+          <t>The routine appears grouped under its time-of-day with an 'N of M' progress. Tapping a step marks it done for today (a sage tick and a strike-through) and updates the count. Calm, with no streak and no celebration pressure.</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>RTN-03</t>
+          <t>RTN-02</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -1994,24 +1994,24 @@
           <t>Routines</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Remove a routine (recoverable)</t>
+          <t>A routine is fresh tomorrow (never a streak)</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>On a routine card tap Remove, then optionally tap Undo.</t>
+          <t>Tick some routine steps today, then advance the device clock to tomorrow and reopen Routines.</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>The routine is removed with a brief 'Routine removed. Undo' banner, not a confirmation dialog. Tapping Undo within a few seconds restores it, otherwise it stays gone. Recoverable, never a confirm gauntlet.</t>
+          <t>Every step is un-ticked again and the progress is back to 0 of M. There is NO streak count, no 'you missed it', and no chain to break: yesterday simply falls away with no guilt (the never-shame spine).</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2026,12 +2026,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>HAP-01</t>
+          <t>RTN-03</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Haptics</t>
+          <t>Routines</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
@@ -2041,22 +2041,22 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Earned-moment haptics fire (Android)</t>
+          <t>Remove a routine (recoverable)</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>On a physical Android device with a haptic motor: complete a single task; clear the whole day; close the day with Goodnight; break a dreaded task into steps; and (premium) reveal a scrapbook.</t>
+          <t>On a routine card tap Remove, then optionally tap Undo.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Soft tap on a single completion; a fuller success buzz when the day clears; a warm soft tap on Goodnight; a light tap when steps land; a success flourish when the scrapbook image appears. Nothing buzzes on plain taps, navigation, capture, or any error.</t>
+          <t>The routine is removed with a brief 'Routine removed. Undo' banner, not a confirmation dialog. Tapping Undo within a few seconds restores it, otherwise it stays gone. Recoverable, never a confirm gauntlet.</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr"/>
@@ -2066,7 +2066,7 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>HAP-02</t>
+          <t>HAP-01</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2074,24 +2074,24 @@
           <t>Haptics</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Reduced motion silences haptics</t>
+          <t>Earned-moment haptics fire (Android)</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Set Settings -&gt; Motion -&gt; Reduce (or enable the OS reduce-motion), then complete a task and close the day.</t>
+          <t>On a physical Android device with a haptic motor: complete a single task; clear the whole day; close the day with Goodnight; break a dreaded task into steps; and (premium) reveal a scrapbook.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>No haptic fires for any cue while motion is reduced (the accessibility guarantee). The Motion hint states Reduce also stops the buzz.</t>
+          <t>Soft tap on a single completion; a fuller success buzz when the day clears; a warm soft tap on Goodnight; a light tap when steps land; a success flourish when the scrapbook image appears. Nothing buzzes on plain taps, navigation, capture, or any error.</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2106,32 +2106,32 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>AND-01</t>
+          <t>HAP-02</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
-        </is>
-      </c>
-      <c r="C35" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Haptics</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Screen stays awake in Focus mode</t>
+          <t>Reduced motion silences haptics</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>On an Android device, open Focus (Focus on one thing) and leave the screen untouched past the usual sleep timeout.</t>
+          <t>Set Settings -&gt; Motion -&gt; Reduce (or enable the OS reduce-motion), then complete a task and close the day.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>The screen stays on while Focus is open, and returns to normal sleep behaviour once Focus is closed.</t>
+          <t>No haptic fires for any cue while motion is reduced (the accessibility guarantee). The Motion hint states Reduce also stops the buzz.</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AND-02</t>
+          <t>AND-01</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2161,17 +2161,17 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>System bars match the theme</t>
+          <t>Screen stays awake in Focus mode</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>On Android, switch the in-app theme (Settings) between light and dark, including a case where the app theme differs from the system theme. Watch the status bar and the bottom navigation bar.</t>
+          <t>On an Android device, open Focus (Focus on one thing) and leave the screen untouched past the usual sleep timeout.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Status-bar and navigation-bar icons stay legible against the app background in both themes; no white flash on launch or overscroll.</t>
+          <t>The screen stays on while Focus is open, and returns to normal sleep behaviour once Focus is closed.</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2186,7 +2186,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>AND-03</t>
+          <t>AND-02</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2194,24 +2194,24 @@
           <t>Android</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Launcher long-press shortcuts</t>
+          <t>System bars match the theme</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>On Android, long-press the DoubleDone home-screen icon. Tap 'Brain dump'; relaunch and tap 'Focus on one thing'. Try both from a cold start and with the app backgrounded.</t>
+          <t>On Android, switch the in-app theme (Settings) between light and dark, including a case where the app theme differs from the system theme. Watch the status bar and the bottom navigation bar.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>'Brain dump' opens the app with the capture box focused and ready to type. 'Focus on one thing' opens directly in Focus mode.</t>
+          <t>Status-bar and navigation-bar icons stay legible against the app background in both themes; no white flash on launch or overscroll.</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>AND-04</t>
+          <t>AND-03</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Share text into DoubleDone</t>
+          <t>Launcher long-press shortcuts</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>On Android, from another app (a browser, notes, a chat) use the system Share sheet and pick DoubleDone. Try sharing a line of text, and a URL.</t>
+          <t>On Android, long-press the DoubleDone home-screen icon. Tap 'Brain dump'; relaunch and tap 'Focus on one thing'. Try both from a cold start and with the app backgrounded.</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>DoubleDone opens with the shared text (or URL) already in the capture box on Today, focused and ready to add. Adding it makes a normal task; nothing is sent anywhere until you do.</t>
+          <t>'Brain dump' opens the app with the capture box focused and ready to type. 'Focus on one thing' opens directly in Focus mode.</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2266,7 +2266,7 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>AND-05</t>
+          <t>AND-04</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2281,17 +2281,17 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Home-screen Today widget</t>
+          <t>Share text into DoubleDone</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>On Android, long-press the home screen and add the 'DoubleDone: Today' widget. Check it with tasks left, with all done, and after closing the day. Complete a task in the app and watch the widget. Tap the widget.</t>
+          <t>On Android, from another app (a browser, notes, a chat) use the system Share sheet and pick DoubleDone. Try sharing a line of text, and a URL.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>The widget shows today's top unfinished titles (or a calm 'All done for today.' / 'Nothing for today yet.'), in light or dark to match the device. It refreshes within a moment of a change in the app (and at least every 30 minutes). Tapping it opens DoubleDone.</t>
+          <t>DoubleDone opens with the shared text (or URL) already in the capture box on Today, focused and ready to add. Adding it makes a normal task; nothing is sent anywhere until you do.</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2306,7 +2306,7 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>AND-06</t>
+          <t>AND-05</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2321,17 +2321,17 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Remind me in X hours (per-task nudge)</t>
+          <t>Home-screen Today widget</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>On Android, tap-and-hold a today task, tap 'Remind me', pick a preset (e.g. 'In 1 hour'). Check the row indicator. Then complete (or remove, or push to tomorrow) the task before the nudge fires. Separately, open 'Remind me' after 9pm.</t>
+          <t>On Android, long-press the home screen and add the 'DoubleDone: Today' widget. Check it with tasks left, with all done, and after closing the day. Complete a task in the app and watch the widget. Tap the widget.</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>A local notification fires at the chosen time (the task as the title, 'Whenever you are ready.' as the body); the row shows a small bell + time. Completing / removing / deferring the task cancels the pending nudge (no poke about a handled task). After 9pm the late presets are hidden. Web does not show 'Remind me'.</t>
+          <t>The widget shows today's top unfinished titles (or a calm 'All done for today.' / 'Nothing for today yet.'), in light or dark to match the device. It refreshes within a moment of a change in the app (and at least every 30 minutes). Tapping it opens DoubleDone.</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2346,12 +2346,12 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>WEB-01</t>
+          <t>AND-06</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
@@ -2361,22 +2361,22 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder via web push</t>
+          <t>Remind me in X hours (per-task nudge)</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>On the deployed web app (PC or Android Chrome) with VAPID configured, toggle 'Daily reminder' on and allow notifications. Check around your daily hour (the hourly cron can be run manually to verify without waiting).</t>
+          <t>On Android, tap-and-hold a today task, tap 'Remind me', pick a preset (e.g. 'In 1 hour'). Check the row indicator. Then complete (or remove, or push to tomorrow) the task before the nudge fires. Separately, open 'Remind me' after 9pm.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Toggling on registers a service worker and subscribes the browser; a calm 'Your today is here when you are ready.' notification arrives around the daily hour, and tapping it opens the app. Toggling off unsubscribes. The push carries no task content. The toggle is hidden when VAPID is unconfigured.</t>
+          <t>A local notification fires at the chosen time (the task as the title, 'Whenever you are ready.' as the body); the row shows a small bell + time. Completing / removing / deferring the task cancels the pending nudge (no poke about a handled task). After 9pm the late presets are hidden. Web does not show 'Remind me'.</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr"/>
@@ -2386,37 +2386,37 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>ONB-01</t>
+          <t>WEB-01</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Guided welcome on first run</t>
+          <t>Daily reminder via web push</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
+          <t>On the deployed web app (PC or Android Chrome) with VAPID configured, toggle 'Daily reminder' on and allow notifications. Check around your daily hour (the hourly cron can be run manually to verify without waiting).</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
+          <t>Toggling on registers a service worker and subscribes the browser; a calm 'Your today is here when you are ready.' notification arrives around the daily hour, and tapping it opens the app. Toggling off unsubscribes. The push carries no task content. The toggle is hidden when VAPID is unconfigured.</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr"/>
@@ -2426,7 +2426,7 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>ONB-02</t>
+          <t>ONB-01</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2434,24 +2434,24 @@
           <t>Onboarding</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Replay the welcome from Settings (non-destructive)</t>
+          <t>Guided welcome on first run</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
+          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Make my day -&gt; This looks right -&gt; Open Today. Separately, try Skip for now.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
+          <t>Today redirects to the welcome exactly once. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); confirming saves the tasks and opens Today. Skip (or an empty Make my day) goes straight to Today. It never reappears once done; if the AI is offline, everything lands on Today, nothing lost.</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2466,32 +2466,32 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>ONB-02</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Replay the welcome from Settings (non-destructive)</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Make my day -&gt; This looks right.</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>The welcome replays identically, but the new tasks MERGE into the existing list (nothing is overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2506,7 +2506,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2514,24 +2514,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2561,17 +2561,17 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2586,7 +2586,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2601,17 +2601,17 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>AI-07</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2641,17 +2641,17 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Breakdown keeps the real task as a silent parent (chain)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>Break down a task (e.g. 'Plan the party'), then complete all of its steps, in any order.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>The original task disappears from Today and Later (it becomes a silent parent, not clutter beside its steps). When the last step is done, the real task completes on its own with the held 'you finished the whole thing' bloom (see AI-09) and lands in the Lookback as the finished real task. Multi-phase: finishing a milestone's steps cascades up to the root.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2666,7 +2666,7 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>AI-08</t>
+          <t>AI-07</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Make it tiny keeps the real task (open parent), no pile-up</t>
+          <t>Breakdown keeps the real task as a silent parent (chain)</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>On a dreaded task choose 'Make it tiny' and do the 2-minute version. Then shrink the same task again to confirm pebbles do not accumulate.</t>
+          <t>Break down a task (e.g. 'Plan the party'), then complete all of its steps, in any order.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>The dreaded task disappears and a 2-minute starter takes its place on Today, carrying an 'A tiny step toward X' eyebrow so the real task stays visible. Completing the starter does NOT mark the big task done: the spent starter is retired (no clutter) and the real task reappears with a warm nudge ('You started, that's the hard part. X is back when you're ready.'). Shrinking the same task repeatedly never piles up duplicate pebbles, only one is open at a time. Make it tiny again for the next step, or just complete the task.</t>
+          <t>The original task disappears from Today and Later (it becomes a silent parent, not clutter beside its steps). When the last step is done, the real task completes on its own with the held 'you finished the whole thing' bloom (see AI-09) and lands in the Lookback as the finished real task. Multi-phase: finishing a milestone's steps cascades up to the root.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>AI-09</t>
+          <t>AI-08</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2721,17 +2721,17 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Whole-task finish raises the held bloom (scaled)</t>
+          <t>Make it tiny keeps the real task (open parent), no pile-up</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Finish the LAST step of a broken-down task. Try it on a long-lingering or chunky task, and separately on a small same-day one. Then repeat with Reduce Motion on.</t>
+          <t>On a dreaded task choose 'Make it tiny' and do the 2-minute version. Then shrink the same task again to confirm pebbles do not accumulate.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>A warm radial bloom rises over a dimming scrim: 'You finished the whole thing', the task name in Newsreader italic, and a warm context line ('... since you first wrote it down. N small steps. All done.'). It holds longer and blooms larger for a long-dreaded or chunky task than for a quick same-day one. A tap dismisses it early, otherwise it auto-settles. Never confetti, points, or a number on screen. With Reduce Motion on, the held title and warm colour still show, only the movement is removed.</t>
+          <t>The dreaded task disappears and a 2-minute starter takes its place on Today, carrying an 'A tiny step toward X' eyebrow so the real task stays visible. Completing the starter does NOT mark the big task done: the spent starter is retired (no clutter) and the real task reappears with a warm nudge ('You started, that's the hard part. X is back when you're ready.'). Shrinking the same task repeatedly never piles up duplicate pebbles, only one is open at a time. Make it tiny again for the next step, or just complete the task.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,12 +2746,12 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-09</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
@@ -2761,17 +2761,17 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Whole-task finish raises the held bloom (scaled)</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Finish the LAST step of a broken-down task. Try it on a long-lingering or chunky task, and separately on a small same-day one. Then repeat with Reduce Motion on.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A warm radial bloom rises over a dimming scrim: 'You finished the whole thing', the task name in Newsreader italic, and a warm context line ('... since you first wrote it down. N small steps. All done.'). It holds longer and blooms larger for a long-dreaded or chunky task than for a quick same-day one. A tap dismisses it early, otherwise it auto-settles. Never confetti, points, or a number on screen. With Reduce Motion on, the held title and warm colour still show, only the movement is removed.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,12 +2786,12 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>AI strategise</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
@@ -2801,17 +2801,17 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Strategise (chart a course)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>When the list feels heavy, run Strategise.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,32 +2826,32 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI strategise</t>
+        </is>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Strategise (chart a course)</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When the list feels heavy, run Strategise.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>Returns a weighted, ordered plan of action. No overwhelm.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2881,17 +2881,17 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2914,24 +2914,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C55" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,17 +2961,17 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,37 +2986,37 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr"/>
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3041,22 +3041,22 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr"/>
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3081,17 +3081,17 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,7 +3106,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3114,24 +3114,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3161,22 +3161,22 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr"/>
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3201,22 +3201,22 @@
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr"/>
@@ -3226,32 +3226,32 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3281,17 +3281,17 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3321,17 +3321,17 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3354,24 +3354,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C66" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,17 +3401,17 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,17 +3441,17 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -3466,37 +3466,37 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3521,22 +3521,22 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,17 +3561,17 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3594,24 +3594,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C72" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today and the Lookback.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3626,32 +3626,32 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,22 +3681,22 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr"/>
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3721,17 +3721,17 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3761,17 +3761,17 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3801,17 +3801,17 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3834,29 +3834,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C78" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr"/>
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3881,22 +3881,22 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3906,37 +3906,37 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C80" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr"/>
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3954,24 +3954,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C81" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -3986,7 +3986,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -4001,17 +4001,17 @@
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4041,17 +4041,17 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
@@ -4066,7 +4066,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4081,17 +4081,17 @@
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
@@ -4106,12 +4106,12 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
@@ -4121,22 +4121,22 @@
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr"/>
@@ -4146,7 +4146,7 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
@@ -4161,22 +4161,22 @@
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr"/>
@@ -4186,7 +4186,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -4194,24 +4194,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C87" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
@@ -4226,37 +4226,37 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C88" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C88" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr"/>
@@ -4266,7 +4266,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -4274,24 +4274,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C89" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
@@ -4306,7 +4306,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
@@ -4321,17 +4321,17 @@
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
@@ -4346,32 +4346,32 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C91" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
@@ -4386,7 +4386,7 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
@@ -4394,24 +4394,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C92" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F92" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
@@ -4426,37 +4426,37 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C93" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F93" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr"/>
@@ -4466,12 +4466,12 @@
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
@@ -4481,22 +4481,22 @@
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F94" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G94" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr"/>
@@ -4506,7 +4506,7 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
@@ -4521,22 +4521,22 @@
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F95" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr"/>
@@ -4546,7 +4546,7 @@
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
@@ -4554,29 +4554,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C96" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F96" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr"/>
@@ -4586,37 +4586,37 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C97" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F97" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr"/>
@@ -4626,7 +4626,7 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
@@ -4641,22 +4641,22 @@
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr"/>
@@ -4666,7 +4666,7 @@
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
@@ -4681,17 +4681,17 @@
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F99" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
@@ -4706,7 +4706,7 @@
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -4721,22 +4721,22 @@
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F100" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G100" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H100" s="7" t="inlineStr"/>
@@ -4746,7 +4746,7 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
@@ -4761,22 +4761,22 @@
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr"/>
@@ -4786,7 +4786,7 @@
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
@@ -4794,24 +4794,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C102" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G102" s="7" t="inlineStr">
@@ -4826,7 +4826,7 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
@@ -4841,22 +4841,22 @@
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H103" s="7" t="inlineStr"/>
@@ -4866,7 +4866,7 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
@@ -4874,29 +4874,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C104" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr"/>
@@ -4906,7 +4906,7 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
@@ -4921,17 +4921,17 @@
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
@@ -4946,7 +4946,7 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
@@ -4961,17 +4961,17 @@
       </c>
       <c r="D106" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F106" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G106" s="7" t="inlineStr">
@@ -4986,7 +4986,7 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -4994,24 +4994,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C107" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F107" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
@@ -5023,9 +5023,49 @@
       <c r="I107" s="9" t="inlineStr"/>
       <c r="J107" s="7" t="inlineStr"/>
     </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C108" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E108" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F108" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G108" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H108" s="7" t="inlineStr"/>
+      <c r="I108" s="9" t="inlineStr"/>
+      <c r="J108" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J107"/>
-  <conditionalFormatting sqref="H2:H107">
+  <autoFilter ref="A1:J108"/>
+  <conditionalFormatting sqref="H2:H108">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -5037,7 +5077,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5073,7 +5113,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>107</t>
         </is>
       </c>
     </row>
@@ -5084,7 +5124,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$107,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$108,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -5095,7 +5135,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$107,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$108,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -5106,7 +5146,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$107,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$108,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -5117,7 +5157,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$107,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$108,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -5128,7 +5168,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>106-COUNTA('Test Suite'!$H$2:$H$107)</f>
+        <f>107-COUNTA('Test Suite'!$H$2:$H$108)</f>
         <v/>
       </c>
     </row>
@@ -5139,7 +5179,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$107,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$108,"P1")</f>
         <v/>
       </c>
     </row>
@@ -5150,7 +5190,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$107,"P1",'Test Suite'!$H$2:$H$107,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$108,"P1",'Test Suite'!$H$2:$H$108,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(feedback): in-app send box that emails the support inbox
The Send-feedback link was a mailto: (no mail client on web, kicks you out on mobile).
Now it opens an inline textarea + Send that POSTs to a new POST /feedback on the AI
Worker, which emails the note to the support inbox via Cloudflare Email Routing's
send_email binding. Calm sending / sent / error states, no leaving the app.

- server: /feedback route + send_email binding + FEEDBACK_TO secret; pure validation
  and the RFC 5322 MIME builder in feedback.ts (unit-tested); cloudflare:email is a
  runtime dynamic import so the node test never resolves it. Origin-gated + rate-limited.
- client: settings.tsx reveal-form replacing the mailto; posts { text, context }.
- QA: SET-06 added + suite regenerated. decision-log records the send_email choice.

Ships behind two ops (Melroy): wrangler secret put FEEDBACK_TO + the Worker deploy.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4146,12 +4146,12 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-06</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -4161,22 +4161,22 @@
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Send feedback in-app</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings, tap 'Send feedback', type a note, tap Send.</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>An inline box opens (no mail client, no leaving the app). Send shows 'Sending...' then a calm 'Thank you. It is on its way.', and the note arrives at the support inbox. On failure it shows a calm retry with the typed text kept. Needs the Worker deployed with /feedback + the FEEDBACK_TO secret set.</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr"/>
@@ -4186,7 +4186,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -4201,22 +4201,22 @@
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr"/>
@@ -4226,7 +4226,7 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -4234,24 +4234,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C88" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
@@ -4266,37 +4266,37 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C89" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C89" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr"/>
@@ -4306,7 +4306,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
@@ -4314,24 +4314,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C90" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
@@ -4346,7 +4346,7 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
@@ -4361,17 +4361,17 @@
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
@@ -4386,32 +4386,32 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F92" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
@@ -4426,7 +4426,7 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
@@ -4434,24 +4434,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C93" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
         </is>
       </c>
       <c r="F93" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm notification arrives at the right time.</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
@@ -4466,37 +4466,37 @@
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C94" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C94" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F94" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G94" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr"/>
@@ -4506,12 +4506,12 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
@@ -4521,22 +4521,22 @@
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F95" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr"/>
@@ -4546,7 +4546,7 @@
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
@@ -4561,22 +4561,22 @@
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F96" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr"/>
@@ -4586,7 +4586,7 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
@@ -4594,29 +4594,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C97" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F97" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr"/>
@@ -4626,37 +4626,37 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C98" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C98" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr"/>
@@ -4666,7 +4666,7 @@
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
@@ -4681,22 +4681,22 @@
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F99" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr"/>
@@ -4706,7 +4706,7 @@
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -4721,17 +4721,17 @@
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F100" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G100" s="7" t="inlineStr">
@@ -4746,7 +4746,7 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
@@ -4761,22 +4761,22 @@
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr"/>
@@ -4786,7 +4786,7 @@
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
@@ -4801,22 +4801,22 @@
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G102" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H102" s="7" t="inlineStr"/>
@@ -4826,7 +4826,7 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
@@ -4834,24 +4834,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C103" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
@@ -4866,7 +4866,7 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
@@ -4881,22 +4881,22 @@
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr"/>
@@ -4906,7 +4906,7 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
@@ -4914,29 +4914,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C105" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C105" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H105" s="7" t="inlineStr"/>
@@ -4946,7 +4946,7 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
@@ -4961,17 +4961,17 @@
       </c>
       <c r="D106" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F106" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G106" s="7" t="inlineStr">
@@ -4986,7 +4986,7 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -5001,17 +5001,17 @@
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F107" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
@@ -5026,7 +5026,7 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
@@ -5034,24 +5034,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C108" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F108" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G108" s="7" t="inlineStr">
@@ -5063,9 +5063,49 @@
       <c r="I108" s="9" t="inlineStr"/>
       <c r="J108" s="7" t="inlineStr"/>
     </row>
+    <row r="109">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>PREM-10</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C109" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="inlineStr">
+        <is>
+          <t>Premium screen shows the renew / cancel date</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+        </is>
+      </c>
+      <c r="F109" s="9" t="inlineStr">
+        <is>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+        </is>
+      </c>
+      <c r="G109" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H109" s="7" t="inlineStr"/>
+      <c r="I109" s="9" t="inlineStr"/>
+      <c r="J109" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J108"/>
-  <conditionalFormatting sqref="H2:H108">
+  <autoFilter ref="A1:J109"/>
+  <conditionalFormatting sqref="H2:H109">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -5077,7 +5117,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5113,7 +5153,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>108</t>
         </is>
       </c>
     </row>
@@ -5124,7 +5164,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$108,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$109,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -5135,7 +5175,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$108,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$109,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -5146,7 +5186,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$108,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$109,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -5157,7 +5197,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$108,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$109,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -5168,7 +5208,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>107-COUNTA('Test Suite'!$H$2:$H$108)</f>
+        <f>108-COUNTA('Test Suite'!$H$2:$H$109)</f>
         <v/>
       </c>
     </row>
@@ -5179,7 +5219,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$108,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$109,"P1")</f>
         <v/>
       </c>
     </row>
@@ -5190,7 +5230,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$108,"P1",'Test Suite'!$H$2:$H$108,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$109,"P1",'Test Suite'!$H$2:$H$109,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(privacy): account deletion now wipes the scrapbook and all local content
Deleting an account left the local scrapbook (and routines, and per-day state) behind:
both deletion paths cleared only tasks, on a "local-only data was never part of the
account" assumption that does not hold for a keepsake made from your finished tasks. Add
one wipeLocalData() in storage.ts, called by the in-app delete and the detected
remote-deletion path, clearing all user content and history while keeping device display
prefs. Regression-tested; QA case DEL-02 now checks the scrapbook explicitly.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -3606,12 +3606,12 @@
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today and the Lookback.</t>
+          <t>On the device you deleted from, look at Today, the Lookback calendar, the scrapbook, and any routines.</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally.</t>
+          <t>Nothing of the account remains locally: no tasks, an empty Lookback, no scrapbook, no routines. Only display prefs (theme, text size) persist.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat: daily-reminder test button, and disable the non-functional Android widget
- Disable the Android home-screen widget: it never rendered (react-native-android-widget 0.20.3
  predates RN 0.85's new-arch headless-task support). Removed the app.json plugin and the index.js
  registration and made updateWidget() a no-op. The widget/ source is kept for a one-line re-enable
  when the library catches up. adb would not run for a logcat and the widget is not needed, so we cut it.
- Add a Settings "Send a test reminder (~90s)" button (native only) so the daily reminder's delivery
  can be checked on device without waiting for the scheduled hour. Fires a one-off on the daily channel.
- /combine Worker deployed (78a5a0aa) and confirmed live, so Combine's AI title works on the deployed app.

QA: AND-05 now checks the widget is absent, REM-01 uses the test button. Gate green (309 client + 146 server).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -2514,24 +2514,24 @@
           <t>Android</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Home-screen Today widget</t>
+          <t>Home-screen widget is disabled (absent from the picker)</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>On Android, long-press the home screen and add the 'DoubleDone: Today' widget. Check it with tasks left, with all done, and after closing the day. Complete a task in the app and watch the widget. Tap the widget.</t>
+          <t>On Android, long-press the home screen and open the widget picker.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>The widget shows today's top unfinished titles (or a calm 'All done for today.' / 'Nothing for today yet.'), in light or dark to match the device. It refreshes within a moment of a change in the app (and at least every 30 minutes). Tapping it opens DoubleDone.</t>
+          <t>DoubleDone offers NO widget. It was removed (decision-log 2026-06-24) because react-native-android-widget 0.20.3 does not support RN 0.85's new architecture, so the widget only ever rendered blank. Nothing transparent or broken appears in the picker.</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -4646,12 +4646,12 @@
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Set up the daily reminder; wait for its time (or trigger the channel).</t>
+          <t>Turn the daily reminder on (Settings &gt; Daily reminder, or the Today footer) and grant permission. Then tap Settings &gt; 'Send a test reminder (~90s)' to fire one on the daily channel without waiting for the scheduled hour. For the real schedule, also leave it on until the daily time.</t>
         </is>
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>A calm notification arrives at the right time.</t>
+          <t>The test reminder appears in the tray within about 90 seconds (the inline status line confirms it was scheduled), proving the daily channel delivers on this device. The status line warns if notification permission is off. The real daily reminder then arrives at its scheduled hour.</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">

</xml_diff>

<commit_message>
chore(release): cut v1.0.0, remove the daily-reminder debug button
DoubleDone goes gold: Combine, the daily reminder firing, and the (now removed) Android widget are all
verified on device. Bumped to 1.0.0 (versionCode is EAS-managed, appVersionSource remote, and the
production profile builds an AAB with autoIncrement). Removed the Settings test-reminder button and
scheduleReminderTest now that reminders are confirmed working. QA REM-01 reverted to the scheduled-hour check.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -4646,12 +4646,12 @@
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Turn the daily reminder on (Settings &gt; Daily reminder, or the Today footer) and grant permission. Then tap Settings &gt; 'Send a test reminder (~90s)' to fire one on the daily channel without waiting for the scheduled hour. For the real schedule, also leave it on until the daily time.</t>
+          <t>Turn the daily reminder on (Settings &gt; Daily reminder, or the Today footer), grant permission, and leave it on until the daily hour.</t>
         </is>
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>The test reminder appears in the tray within about 90 seconds (the inline status line confirms it was scheduled), proving the daily channel delivers on this device. The status line warns if notification permission is off. The real daily reminder then arrives at its scheduled hour.</t>
+          <t>A calm 'Your today is here when you are ready.' notification arrives at the scheduled hour (verified firing on a real Samsung device). Toggling it off cancels it.</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat(premium): comp allowlist so an email is always premium (owner test path)
A small server-side email allowlist (server/src/comp.ts: isCompEmail + COMP_EMAILS)
grants premium with no Stripe subscription. Two callers honour it: requirePremium reads
the email from the cryptographically VERIFIED token and short-circuits to ok before the
D1 read (a forged comp-email token is still rejected 401, tested), and handleEntitlement
returns a comp premium view for the CLIENT flag (decode-only, matching that endpoint's
existing posture, and the costed gate stays verified). Keyed by email, in code, so it
works the instant the owner signs in and no Stripe event can flip it.

11 server tests (179 total), QA case PREM-11. The Worker deploy that makes it live is
gated on Melroy's per-instance OK.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J126"/>
+  <dimension ref="A1:J127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5306,32 +5306,32 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>PIN-01</t>
+          <t>PREM-11</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
         <is>
-          <t>Pin</t>
-        </is>
-      </c>
-      <c r="C115" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C115" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D115" s="9" t="inlineStr">
         <is>
-          <t>Premium: pin a task as the day's one thing</t>
+          <t>Comp allowlist: the owner email is always premium</t>
         </is>
       </c>
       <c r="E115" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), tap-and-hold a one-off task to select it, then tap 'Pin' in the select bar.</t>
+          <t>Sign in with the comp email (the owner account listed in server/src/comp.ts), without ever paying.</t>
         </is>
       </c>
       <c r="F115" s="9" t="inlineStr">
         <is>
-          <t>The task gets a calm mauve star and border and floats to the top of Today. 'Focus on one thing' then opens straight to it.</t>
+          <t>Premium is active immediately: Settings and the Lookback show the scrapbook unlocked and Scan works, with no Stripe charge. A non-allowlisted free account stays free. The allowlist is checked against a cryptographically verified token on the costed gate, so a forged token cannot claim premium compute.</t>
         </is>
       </c>
       <c r="G115" s="7" t="inlineStr">
@@ -5346,7 +5346,7 @@
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>PIN-02</t>
+          <t>PIN-01</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
@@ -5361,17 +5361,17 @@
       </c>
       <c r="D116" s="9" t="inlineStr">
         <is>
-          <t>Free: Pin routes to the upsell, never pins</t>
+          <t>Premium: pin a task as the day's one thing</t>
         </is>
       </c>
       <c r="E116" s="9" t="inlineStr">
         <is>
-          <t>As a free user, select a single one-off task and tap the dimmed 'Pin' action.</t>
+          <t>As premium (or with the dev Premium override on), tap-and-hold a one-off task to select it, then tap 'Pin' in the select bar.</t>
         </is>
       </c>
       <c r="F116" s="9" t="inlineStr">
         <is>
-          <t>No task is pinned, and the Premium screen opens calmly (never a shaming wall). A 'premium.gate_hit' with reason 'pin' is logged.</t>
+          <t>The task gets a calm mauve star and border and floats to the top of Today. 'Focus on one thing' then opens straight to it.</t>
         </is>
       </c>
       <c r="G116" s="7" t="inlineStr">
@@ -5386,7 +5386,7 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>PIN-03</t>
+          <t>PIN-02</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
@@ -5394,24 +5394,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C117" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D117" s="9" t="inlineStr">
         <is>
-          <t>Only one task is pinned at a time</t>
+          <t>Free: Pin routes to the upsell, never pins</t>
         </is>
       </c>
       <c r="E117" s="9" t="inlineStr">
         <is>
-          <t>As premium, pin task A, then select task B and pin it.</t>
+          <t>As a free user, select a single one-off task and tap the dimmed 'Pin' action.</t>
         </is>
       </c>
       <c r="F117" s="9" t="inlineStr">
         <is>
-          <t>Task B is now pinned (starred, floated to the top), and task A is no longer pinned. At most one pin ever exists.</t>
+          <t>No task is pinned, and the Premium screen opens calmly (never a shaming wall). A 'premium.gate_hit' with reason 'pin' is logged.</t>
         </is>
       </c>
       <c r="G117" s="7" t="inlineStr">
@@ -5426,7 +5426,7 @@
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>PIN-04</t>
+          <t>PIN-03</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
@@ -5441,17 +5441,17 @@
       </c>
       <c r="D118" s="9" t="inlineStr">
         <is>
-          <t>A pin syncs across devices</t>
+          <t>Only one task is pinned at a time</t>
         </is>
       </c>
       <c r="E118" s="9" t="inlineStr">
         <is>
-          <t>As premium and signed in, pin a task, then sign out and back in (or open a second device).</t>
+          <t>As premium, pin task A, then select task B and pin it.</t>
         </is>
       </c>
       <c r="F118" s="9" t="inlineStr">
         <is>
-          <t>The task is still pinned after the sync round-trip (the star and float persist). Needs the pinned_at column applied in Supabase.</t>
+          <t>Task B is now pinned (starred, floated to the top), and task A is no longer pinned. At most one pin ever exists.</t>
         </is>
       </c>
       <c r="G118" s="7" t="inlineStr">
@@ -5466,7 +5466,7 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>PIN-05</t>
+          <t>PIN-04</t>
         </is>
       </c>
       <c r="B119" s="7" t="inlineStr">
@@ -5474,24 +5474,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C119" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D119" s="9" t="inlineStr">
         <is>
-          <t>Pin is offered only on one-off Today rows</t>
+          <t>A pin syncs across devices</t>
         </is>
       </c>
       <c r="E119" s="9" t="inlineStr">
         <is>
-          <t>Select a recurring task, then separately look at a task in the 'Later' list.</t>
+          <t>As premium and signed in, pin a task, then sign out and back in (or open a second device).</t>
         </is>
       </c>
       <c r="F119" s="9" t="inlineStr">
         <is>
-          <t>No 'Pin' action appears for a recurring task, and Later rows carry no pin affordance (pinning is Today-only and one-offs only).</t>
+          <t>The task is still pinned after the sync round-trip (the star and float persist). Needs the pinned_at column applied in Supabase.</t>
         </is>
       </c>
       <c r="G119" s="7" t="inlineStr">
@@ -5506,32 +5506,32 @@
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>OCR-01</t>
+          <t>PIN-05</t>
         </is>
       </c>
       <c r="B120" s="7" t="inlineStr">
         <is>
-          <t>Scan</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="C120" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D120" s="9" t="inlineStr">
         <is>
-          <t>Premium: the Scan button opens the camera</t>
+          <t>Pin is offered only on one-off Today rows</t>
         </is>
       </c>
       <c r="E120" s="9" t="inlineStr">
         <is>
-          <t>As premium, open the add panel and tap the Scan (camera) pill beside Speak.</t>
+          <t>Select a recurring task, then separately look at a task in the 'Later' list.</t>
         </is>
       </c>
       <c r="F120" s="9" t="inlineStr">
         <is>
-          <t>The camera screen opens: a live viewfinder with a shutter and a Photos shortcut on a device, or a 'Choose a photo' prompt on web. No paywall.</t>
+          <t>No 'Pin' action appears for a recurring task, and Later rows carry no pin affordance (pinning is Today-only and one-offs only).</t>
         </is>
       </c>
       <c r="G120" s="7" t="inlineStr">
@@ -5546,7 +5546,7 @@
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>OCR-02</t>
+          <t>OCR-01</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
@@ -5561,17 +5561,17 @@
       </c>
       <c r="D121" s="9" t="inlineStr">
         <is>
-          <t>Free: Scan routes to the upsell, never opens the camera</t>
+          <t>Premium: the Scan button opens the camera</t>
         </is>
       </c>
       <c r="E121" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open the add panel and tap the Scan pill.</t>
+          <t>As premium, open the add panel and tap the Scan (camera) pill beside Speak.</t>
         </is>
       </c>
       <c r="F121" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium screen calmly (never a wall). A 'premium.gate_hit' with reason 'ocr' is logged. No camera opens.</t>
+          <t>The camera screen opens: a live viewfinder with a shutter and a Photos shortcut on a device, or a 'Choose a photo' prompt on web. No paywall.</t>
         </is>
       </c>
       <c r="G121" s="7" t="inlineStr">
@@ -5586,7 +5586,7 @@
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>OCR-03</t>
+          <t>OCR-02</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
@@ -5601,22 +5601,22 @@
       </c>
       <c r="D122" s="9" t="inlineStr">
         <is>
-          <t>Photograph a list and the tasks land in the box</t>
+          <t>Free: Scan routes to the upsell, never opens the camera</t>
         </is>
       </c>
       <c r="E122" s="9" t="inlineStr">
         <is>
-          <t>As premium on a device, tap Scan, photograph a short printed or handwritten list (fill the frame), wait for 'Reading your list...'.</t>
+          <t>As a free user, open the add panel and tap the Scan pill.</t>
         </is>
       </c>
       <c r="F122" s="9" t="inlineStr">
         <is>
-          <t>The tasks it reads appear in the brain-dump box, one per line, editable. Nothing is auto-added to Today, and tapping Add commits them. An 'ocr.captured' event is logged.</t>
+          <t>Routed to the Premium screen calmly (never a wall). A 'premium.gate_hit' with reason 'ocr' is logged. No camera opens.</t>
         </is>
       </c>
       <c r="G122" s="7" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H122" s="7" t="inlineStr"/>
@@ -5626,7 +5626,7 @@
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>OCR-04</t>
+          <t>OCR-03</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
@@ -5634,29 +5634,29 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C123" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C123" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D123" s="9" t="inlineStr">
         <is>
-          <t>Gallery fallback reads an existing photo</t>
+          <t>Photograph a list and the tasks land in the box</t>
         </is>
       </c>
       <c r="E123" s="9" t="inlineStr">
         <is>
-          <t>Tap Scan, then 'Photos' (device) or 'Choose a photo' (web), and pick a photo of a list, a note, or a whiteboard.</t>
+          <t>As premium on a device, tap Scan, photograph a short printed or handwritten list (fill the frame), wait for 'Reading your list...'.</t>
         </is>
       </c>
       <c r="F123" s="9" t="inlineStr">
         <is>
-          <t>Same result: the read tasks land in the box for review. Covers a screenshot of a texted list, or a photo taken earlier.</t>
+          <t>The tasks it reads appear in the brain-dump box, one per line, editable. Nothing is auto-added to Today, and tapping Add commits them. An 'ocr.captured' event is logged.</t>
         </is>
       </c>
       <c r="G123" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="H123" s="7" t="inlineStr"/>
@@ -5666,7 +5666,7 @@
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>OCR-05</t>
+          <t>OCR-04</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
@@ -5681,17 +5681,17 @@
       </c>
       <c r="D124" s="9" t="inlineStr">
         <is>
-          <t>An unreadable photo fails calmly</t>
+          <t>Gallery fallback reads an existing photo</t>
         </is>
       </c>
       <c r="E124" s="9" t="inlineStr">
         <is>
-          <t>Scan a blank, blurry, or list-free image.</t>
+          <t>Tap Scan, then 'Photos' (device) or 'Choose a photo' (web), and pick a photo of a list, a note, or a whiteboard.</t>
         </is>
       </c>
       <c r="F124" s="9" t="inlineStr">
         <is>
-          <t>A calm line ('I couldn't read any tasks from that. Try again...'), the camera stays open, never a crash and never a shaming message.</t>
+          <t>Same result: the read tasks land in the box for review. Covers a screenshot of a texted list, or a photo taken earlier.</t>
         </is>
       </c>
       <c r="G124" s="7" t="inlineStr">
@@ -5706,7 +5706,7 @@
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>OCR-06</t>
+          <t>OCR-05</t>
         </is>
       </c>
       <c r="B125" s="7" t="inlineStr">
@@ -5721,22 +5721,22 @@
       </c>
       <c r="D125" s="9" t="inlineStr">
         <is>
-          <t>Camera denial is never a dead end</t>
+          <t>An unreadable photo fails calmly</t>
         </is>
       </c>
       <c r="E125" s="9" t="inlineStr">
         <is>
-          <t>On a device, deny the camera permission when prompted.</t>
+          <t>Scan a blank, blurry, or list-free image.</t>
         </is>
       </c>
       <c r="F125" s="9" t="inlineStr">
         <is>
-          <t>A calm screen offers 'Allow camera' and 'Choose from photos instead', and the gallery path still reads a list.</t>
+          <t>A calm line ('I couldn't read any tasks from that. Try again...'), the camera stays open, never a crash and never a shaming message.</t>
         </is>
       </c>
       <c r="G125" s="7" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H125" s="7" t="inlineStr"/>
@@ -5746,7 +5746,7 @@
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>OCR-07</t>
+          <t>OCR-06</t>
         </is>
       </c>
       <c r="B126" s="7" t="inlineStr">
@@ -5754,38 +5754,78 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C126" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C126" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D126" s="9" t="inlineStr">
         <is>
-          <t>AI egress is disclosed at the point of use</t>
+          <t>Camera denial is never a dead end</t>
         </is>
       </c>
       <c r="E126" s="9" t="inlineStr">
         <is>
-          <t>Open the Scan screen (device or web).</t>
+          <t>On a device, deny the camera permission when prompted.</t>
         </is>
       </c>
       <c r="F126" s="9" t="inlineStr">
         <is>
-          <t>The note 'Your photo is sent to the AI to read your list, then discarded. It is never stored.' is visible. The D1 'ocr' telemetry row holds only the image size and task count, never the image or the titles.</t>
+          <t>A calm screen offers 'Allow camera' and 'Choose from photos instead', and the gallery path still reads a list.</t>
         </is>
       </c>
       <c r="G126" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="H126" s="7" t="inlineStr"/>
       <c r="I126" s="9" t="inlineStr"/>
       <c r="J126" s="7" t="inlineStr"/>
     </row>
+    <row r="127">
+      <c r="A127" s="6" t="inlineStr">
+        <is>
+          <t>OCR-07</t>
+        </is>
+      </c>
+      <c r="B127" s="7" t="inlineStr">
+        <is>
+          <t>Scan</t>
+        </is>
+      </c>
+      <c r="C127" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>AI egress is disclosed at the point of use</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="inlineStr">
+        <is>
+          <t>Open the Scan screen (device or web).</t>
+        </is>
+      </c>
+      <c r="F127" s="9" t="inlineStr">
+        <is>
+          <t>The note 'Your photo is sent to the AI to read your list, then discarded. It is never stored.' is visible. The D1 'ocr' telemetry row holds only the image size and task count, never the image or the titles.</t>
+        </is>
+      </c>
+      <c r="G127" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H127" s="7" t="inlineStr"/>
+      <c r="I127" s="9" t="inlineStr"/>
+      <c r="J127" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J126"/>
-  <conditionalFormatting sqref="H2:H126">
+  <autoFilter ref="A1:J127"/>
+  <conditionalFormatting sqref="H2:H127">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -5797,7 +5837,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5833,7 +5873,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>126</t>
         </is>
       </c>
     </row>
@@ -5844,7 +5884,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$126,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$127,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -5855,7 +5895,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$126,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$127,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -5866,7 +5906,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$126,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$127,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -5877,7 +5917,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$126,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$127,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -5888,7 +5928,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>125-COUNTA('Test Suite'!$H$2:$H$126)</f>
+        <f>126-COUNTA('Test Suite'!$H$2:$H$127)</f>
         <v/>
       </c>
     </row>
@@ -5899,7 +5939,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$126,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$127,"P1")</f>
         <v/>
       </c>
     </row>
@@ -5910,7 +5950,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$126,"P1",'Test Suite'!$H$2:$H$126,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$127,"P1",'Test Suite'!$H$2:$H$127,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(premium): Tier 2 Chart a course, goal -> flat tasks into Today
Tier 2 feature 2: name a goal, get a calm ordered list of the next 3-7 concrete steps
toward it (a new Sonnet /chart route behind requirePremium like /ocr), review and accept.
Accepted steps are minted as FLAT one-off tasks into the single Today/backlog (first on
Today, the rest spread gently forward via spreadDueDates), never a project or workspace.
The premium gate sits at the moment of asking for a plan (tapping Suggest steps), never on
opening the screen, and free users route calmly to /premium. Entry is a quiet "Chart a
course" room in the Rooms sheet.

Propose-then-accept: nothing is added until accepted, only the ticked steps. v1 has no
target-date picker (a deadline-paced spread is a fast-follow). Prompt wording is Melroy's
to tune.

Gate green: client 332, server 190, lint + typecheck clean. QA CHART-01..04.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J129"/>
+  <dimension ref="A1:J133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5903,9 +5903,169 @@
       <c r="I129" s="9" t="inlineStr"/>
       <c r="J129" s="7" t="inlineStr"/>
     </row>
+    <row r="130">
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>CHART-01</t>
+        </is>
+      </c>
+      <c r="B130" s="7" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>Premium: chart a course toward a goal</t>
+        </is>
+      </c>
+      <c r="E130" s="9" t="inlineStr">
+        <is>
+          <t>As premium (or dev Premium override on), open Rooms, tap 'Chart a course', type a goal like 'get fit for a 10k', tap 'Suggest steps'.</t>
+        </is>
+      </c>
+      <c r="F130" s="9" t="inlineStr">
+        <is>
+          <t>A calm one-line heading plus 3-7 ticked next steps appear, and nothing is added yet. Tapping 'Add N tasks' lands them on Today (the first undated, later ones spread forward), each an ordinary task, and returns to Today. The 'chart.requested' then 'chart.added' events are logged.</t>
+        </is>
+      </c>
+      <c r="G130" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H130" s="7" t="inlineStr"/>
+      <c r="I130" s="9" t="inlineStr"/>
+      <c r="J130" s="7" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>CHART-02</t>
+        </is>
+      </c>
+      <c r="B131" s="7" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C131" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>Free: charting routes to the upsell, never plans</t>
+        </is>
+      </c>
+      <c r="E131" s="9" t="inlineStr">
+        <is>
+          <t>As a free user, open Rooms, tap 'Chart a course', type a goal, tap 'Suggest steps'.</t>
+        </is>
+      </c>
+      <c r="F131" s="9" t="inlineStr">
+        <is>
+          <t>Routed to the Premium screen calmly (never a wall), and a 'premium.gate_hit' with reason 'chart' is logged. No plan is generated and nothing is added.</t>
+        </is>
+      </c>
+      <c r="G131" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H131" s="7" t="inlineStr"/>
+      <c r="I131" s="9" t="inlineStr"/>
+      <c r="J131" s="7" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="6" t="inlineStr">
+        <is>
+          <t>CHART-03</t>
+        </is>
+      </c>
+      <c r="B132" s="7" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C132" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D132" s="9" t="inlineStr">
+        <is>
+          <t>Propose-then-accept: nothing auto-adds</t>
+        </is>
+      </c>
+      <c r="E132" s="9" t="inlineStr">
+        <is>
+          <t>As premium, generate a plan, untick two steps, then tap 'Add'. Separately, generate a plan and back out with 'Not these, start over' or Back.</t>
+        </is>
+      </c>
+      <c r="F132" s="9" t="inlineStr">
+        <is>
+          <t>Only the ticked steps are added as plain tasks, and backing out adds nothing. Today was unchanged before accepting.</t>
+        </is>
+      </c>
+      <c r="G132" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H132" s="7" t="inlineStr"/>
+      <c r="I132" s="9" t="inlineStr"/>
+      <c r="J132" s="7" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="6" t="inlineStr">
+        <is>
+          <t>CHART-04</t>
+        </is>
+      </c>
+      <c r="B133" s="7" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C133" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>A goal that cannot be mapped fails calmly</t>
+        </is>
+      </c>
+      <c r="E133" s="9" t="inlineStr">
+        <is>
+          <t>Enter an empty goal (the button is disabled), then a nonsensical goal and submit.</t>
+        </is>
+      </c>
+      <c r="F133" s="9" t="inlineStr">
+        <is>
+          <t>The empty case cannot submit. A nonsensical goal shows one calm line ('I couldn't map that out just now'), the goal stays editable, never a crash or a shaming message.</t>
+        </is>
+      </c>
+      <c r="G133" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H133" s="7" t="inlineStr"/>
+      <c r="I133" s="9" t="inlineStr"/>
+      <c r="J133" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J129"/>
-  <conditionalFormatting sqref="H2:H129">
+  <autoFilter ref="A1:J133"/>
+  <conditionalFormatting sqref="H2:H133">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -5917,7 +6077,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H133" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5953,7 +6113,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>132</t>
         </is>
       </c>
     </row>
@@ -5964,7 +6124,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$129,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$133,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -5975,7 +6135,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$129,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$133,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -5986,7 +6146,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$129,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$133,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -5997,7 +6157,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$129,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$133,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -6008,7 +6168,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>128-COUNTA('Test Suite'!$H$2:$H$129)</f>
+        <f>132-COUNTA('Test Suite'!$H$2:$H$133)</f>
         <v/>
       </c>
     </row>
@@ -6019,7 +6179,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$129,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$133,"P1")</f>
         <v/>
       </c>
     </row>
@@ -6030,7 +6190,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$129,"P1",'Test Suite'!$H$2:$H$129,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$133,"P1",'Test Suite'!$H$2:$H$133,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(premium): Chart a course asks "by when" and spreads steps to that date
From Melroy's live feedback: a "2 months" goal crammed its 6 steps into 5 days because v1
had no deadline. Added a "By when?" question (relative chips: No deadline / In 2 weeks /
In a month / In 2 months / In 3 months). The chosen date paces the AI's steps (via the
existing context.dueDate in buildChartRequest) and spreads the accepted tasks from Today
out to the date via spreadDueDates, instead of one-per-day. The /chart route parses an
optional ISO context.dueDate (parseChartContext), and the client seam sends it.

Gate green: client 338, server 196, lint + typecheck clean. QA CHART-05. Chips verified
in preview.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$140</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:J140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6106,32 +6106,32 @@
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>SEQ-01</t>
+          <t>CHART-05</t>
         </is>
       </c>
       <c r="B135" s="7" t="inlineStr">
         <is>
-          <t>Sequence</t>
-        </is>
-      </c>
-      <c r="C135" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C135" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D135" s="9" t="inlineStr">
         <is>
-          <t>Premium: Plan my order suggests a calm sequence</t>
+          <t>A deadline spreads the steps across the timeframe</t>
         </is>
       </c>
       <c r="E135" s="9" t="inlineStr">
         <is>
-          <t>As premium with 3+ open one-off tasks on Today, tap 'Plan my order'.</t>
+          <t>As premium, type a goal, tap a 'By when?' chip (e.g. 'In 2 months'), then Suggest steps and Add.</t>
         </is>
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>A proposal card lists today's tasks in a suggested order, each with a short calm reason. Nothing reorders until 'Use this order' is tapped, then the list re-sequences in place (no dates change, no task moves to another day). A 'sequence.accepted' event is logged.</t>
+          <t>The steps are paced for that timeframe, and the accepted tasks spread from Today out to the chosen date (not crammed into the next few days). 'No deadline' keeps the gentle one-per-day default.</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
@@ -6146,7 +6146,7 @@
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>SEQ-02</t>
+          <t>SEQ-01</t>
         </is>
       </c>
       <c r="B136" s="7" t="inlineStr">
@@ -6161,17 +6161,17 @@
       </c>
       <c r="D136" s="9" t="inlineStr">
         <is>
-          <t>Free: Plan my order routes to the upsell, never reorders</t>
+          <t>Premium: Plan my order suggests a calm sequence</t>
         </is>
       </c>
       <c r="E136" s="9" t="inlineStr">
         <is>
-          <t>As a free user with 2+ tasks on Today, tap 'Plan my order'.</t>
+          <t>As premium with 3+ open one-off tasks on Today, tap 'Plan my order'.</t>
         </is>
       </c>
       <c r="F136" s="9" t="inlineStr">
         <is>
-          <t>The Premium screen opens calmly (never a wall), a 'premium.gate_hit' with reason 'sequence' is logged, and the day's order is unchanged.</t>
+          <t>A proposal card lists today's tasks in a suggested order, each with a short calm reason. Nothing reorders until 'Use this order' is tapped, then the list re-sequences in place (no dates change, no task moves to another day). A 'sequence.accepted' event is logged.</t>
         </is>
       </c>
       <c r="G136" s="7" t="inlineStr">
@@ -6186,7 +6186,7 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>SEQ-03</t>
+          <t>SEQ-02</t>
         </is>
       </c>
       <c r="B137" s="7" t="inlineStr">
@@ -6194,24 +6194,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C137" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D137" s="9" t="inlineStr">
         <is>
-          <t>'Not now' leaves the day untouched</t>
+          <t>Free: Plan my order routes to the upsell, never reorders</t>
         </is>
       </c>
       <c r="E137" s="9" t="inlineStr">
         <is>
-          <t>As premium, open the proposal, then tap 'Not now' or the backdrop.</t>
+          <t>As a free user with 2+ tasks on Today, tap 'Plan my order'.</t>
         </is>
       </c>
       <c r="F137" s="9" t="inlineStr">
         <is>
-          <t>The order is exactly as before, nothing reordered, and no manualOrder is written.</t>
+          <t>The Premium screen opens calmly (never a wall), a 'premium.gate_hit' with reason 'sequence' is logged, and the day's order is unchanged.</t>
         </is>
       </c>
       <c r="G137" s="7" t="inlineStr">
@@ -6226,7 +6226,7 @@
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>SEQ-04</t>
+          <t>SEQ-03</t>
         </is>
       </c>
       <c r="B138" s="7" t="inlineStr">
@@ -6241,17 +6241,17 @@
       </c>
       <c r="D138" s="9" t="inlineStr">
         <is>
-          <t>An accepted order survives a reload (local-first)</t>
+          <t>'Not now' leaves the day untouched</t>
         </is>
       </c>
       <c r="E138" s="9" t="inlineStr">
         <is>
-          <t>As premium, accept an order, then fully reload the app.</t>
+          <t>As premium, open the proposal, then tap 'Not now' or the backdrop.</t>
         </is>
       </c>
       <c r="F138" s="9" t="inlineStr">
         <is>
-          <t>Today still shows the accepted order after reload (manualOrder persists on-device). Note: the order does not yet sync across devices, which is a documented follow-up.</t>
+          <t>The order is exactly as before, nothing reordered, and no manualOrder is written.</t>
         </is>
       </c>
       <c r="G138" s="7" t="inlineStr">
@@ -6266,7 +6266,7 @@
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>SEQ-05</t>
+          <t>SEQ-04</t>
         </is>
       </c>
       <c r="B139" s="7" t="inlineStr">
@@ -6274,24 +6274,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C139" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C139" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D139" s="9" t="inlineStr">
         <is>
-          <t>A pinned task still wins the very top</t>
+          <t>An accepted order survives a reload (local-first)</t>
         </is>
       </c>
       <c r="E139" s="9" t="inlineStr">
         <is>
-          <t>As premium, pin a task, then accept a 'Plan my order' sequence that puts a different task first.</t>
+          <t>As premium, accept an order, then fully reload the app.</t>
         </is>
       </c>
       <c r="F139" s="9" t="inlineStr">
         <is>
-          <t>The pinned task stays at the very top, and the accepted order applies to everything below it.</t>
+          <t>Today still shows the accepted order after reload (manualOrder persists on-device). Note: the order does not yet sync across devices, which is a documented follow-up.</t>
         </is>
       </c>
       <c r="G139" s="7" t="inlineStr">
@@ -6303,9 +6303,49 @@
       <c r="I139" s="9" t="inlineStr"/>
       <c r="J139" s="7" t="inlineStr"/>
     </row>
+    <row r="140">
+      <c r="A140" s="6" t="inlineStr">
+        <is>
+          <t>SEQ-05</t>
+        </is>
+      </c>
+      <c r="B140" s="7" t="inlineStr">
+        <is>
+          <t>Sequence</t>
+        </is>
+      </c>
+      <c r="C140" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D140" s="9" t="inlineStr">
+        <is>
+          <t>A pinned task still wins the very top</t>
+        </is>
+      </c>
+      <c r="E140" s="9" t="inlineStr">
+        <is>
+          <t>As premium, pin a task, then accept a 'Plan my order' sequence that puts a different task first.</t>
+        </is>
+      </c>
+      <c r="F140" s="9" t="inlineStr">
+        <is>
+          <t>The pinned task stays at the very top, and the accepted order applies to everything below it.</t>
+        </is>
+      </c>
+      <c r="G140" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H140" s="7" t="inlineStr"/>
+      <c r="I140" s="9" t="inlineStr"/>
+      <c r="J140" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J139"/>
-  <conditionalFormatting sqref="H2:H139">
+  <autoFilter ref="A1:J140"/>
+  <conditionalFormatting sqref="H2:H140">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -6317,7 +6357,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6353,7 +6393,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>139</t>
         </is>
       </c>
     </row>
@@ -6364,7 +6404,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$139,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$140,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -6375,7 +6415,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$139,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$140,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -6386,7 +6426,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$139,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$140,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -6397,7 +6437,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$139,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$140,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -6408,7 +6448,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>138-COUNTA('Test Suite'!$H$2:$H$139)</f>
+        <f>139-COUNTA('Test Suite'!$H$2:$H$140)</f>
         <v/>
       </c>
     </row>
@@ -6419,7 +6459,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$139,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$140,"P1")</f>
         <v/>
       </c>
     </row>
@@ -6430,7 +6470,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$139,"P1",'Test Suite'!$H$2:$H$139,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$140,"P1",'Test Suite'!$H$2:$H$140,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(web): a real landing page at the front door (audit Tier 1)
The audit's last Tier-1 gap: doubledone.app/ was the app shell booting into
onboarding, no marketing front door. Approach A1: a Landing route at /, the app
moved to /today. The SPA stays at root, so checkout (returns to /premium), the
service worker, and deep links are untouched, no server change, no redeploy.

app/index.tsx (Today) -> app/today.tsx; the new app/index.tsx is the Landing (spine,
audience, never-shame promise, three-step loop, payoff, Begin CTAs, in the app's own
theme). Web first-touch only: native + returning onboarded users redirect to /today,
so only a fresh visitor or a crawler sees it. The four go-home navs and the
screenshot harness now target /today. Added E2E LP-01.

Verified in-preview: / = Landing for a fresh visitor, /today = Today, onboarded / ->
Today. Decision-logged.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$152</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2666,12 +2666,12 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>ONB-01</t>
+          <t>LP-01</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Landing</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Guided welcome on first run (7-screen)</t>
+          <t>The web landing is the front door</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Sort it for me -&gt; This looks right -&gt; Got it -&gt; Almost there -&gt; a Premium teaser -&gt; Open Today. Try Back to a previous screen, and separately try Skip.</t>
+          <t>On the web in a fresh browser (or after clearing 'doubledone.onboarded.v1'), open doubledone.app/. Read the page, then tap Begin. Separately, as a returning (onboarded) user, open doubledone.app/. On Android, just open the app.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Today redirects to the welcome exactly once: a 7-screen sequence with a quiet 7-dot progress, Skip on every screen but the last, and Back (top-left) from screen 2 on with the typed text intact. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); the safety-net and 'what you keep' screens follow as calm info; the penultimate screen is a calm one-screen teaser of what Premium adds (never a hard gate, fully skippable); Open Today saves the tasks and opens Today. Skip, or an empty Sort, leaves immediately, saving whatever was revealed. Never reappears once done. If the AI is slow or offline, everything lands on Today, nothing lost.</t>
+          <t>A calm marketing page renders at the root: the wordmark, 'Today is finite and achievable.', the never-shame promise, the audience line (ADHD / autism / OCD), the three-step loop, the Lookback payoff, and a Begin CTA. Begin opens the app at /today (a first-timer continues into the welcome). A returning, onboarded visitor is redirected straight to /today and never sees the landing. On native the app opens to Today, never the landing. Checkout still returns to /premium and deep links still resolve.</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>ONB-02</t>
+          <t>ONB-01</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2714,24 +2714,24 @@
           <t>Onboarding</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Replay the welcome from Settings (non-destructive)</t>
+          <t>Guided welcome on first run (7-screen)</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Sort it for me -&gt; This looks right -&gt; through to Open Today.</t>
+          <t>On a fresh install (or after clearing 'doubledone.onboarded.v1'), open the app. Walk Begin -&gt; type a few lines -&gt; Sort it for me -&gt; This looks right -&gt; Got it -&gt; Almost there -&gt; a Premium teaser -&gt; Open Today. Try Back to a previous screen, and separately try Skip.</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>The welcome replays identically (all 7 screens), but the new tasks MERGE into the existing list (nothing overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
+          <t>Today redirects to the welcome exactly once: a 7-screen sequence with a quiet 7-dot progress, Skip on every screen but the last, and Back (top-left) from screen 2 on with the typed text intact. The dump is triaged into a doable Today (some pushed to later, any big one flagged 'Looks big, break it down?'); the safety-net and 'what you keep' screens follow as calm info; the penultimate screen is a calm one-screen teaser of what Premium adds (never a hard gate, fully skippable); Open Today saves the tasks and opens Today. Skip, or an empty Sort, leaves immediately, saving whatever was revealed. Never reappears once done. If the AI is slow or offline, everything lands on Today, nothing lost.</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2746,32 +2746,32 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>ONB-02</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Onboarding</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Replay the welcome from Settings (non-destructive)</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>With tasks already on Today, open Settings -&gt; 'See the welcome again'. Walk Begin -&gt; dump a couple of lines -&gt; Sort it for me -&gt; This looks right -&gt; through to Open Today.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>The welcome replays identically (all 7 screens), but the new tasks MERGE into the existing list (nothing overwritten) and the onboarded flag is untouched. Skipping returns to Today with no change.</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2794,24 +2794,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C52" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -2826,7 +2826,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2841,17 +2841,17 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2881,17 +2881,17 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>AI-07</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,17 +2921,17 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Breakdown keeps the real task as a silent parent (chain)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Break down a task (e.g. 'Plan the party'), then complete all of its steps, in any order.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>The original task disappears from Today and Later (it becomes a silent parent, not clutter beside its steps). When the last step is done, the real task completes on its own with the held 'you finished the whole thing' bloom (see AI-09) and lands in the Lookback as the finished real task. Multi-phase: finishing a milestone's steps cascades up to the root.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>AI-08</t>
+          <t>AI-07</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,17 +2961,17 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Make it tiny keeps the real task (open parent), no pile-up</t>
+          <t>Breakdown keeps the real task as a silent parent (chain)</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>On a dreaded task choose 'Make it tiny' and do the 2-minute version. Then shrink the same task again to confirm pebbles do not accumulate.</t>
+          <t>Break down a task (e.g. 'Plan the party'), then complete all of its steps, in any order.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>The dreaded task disappears and a 2-minute starter takes its place on Today, carrying an 'A tiny step toward X' eyebrow so the real task stays visible. Completing the starter does NOT mark the big task done: the spent starter is retired (no clutter) and the real task reappears with a warm nudge ('You started, that's the hard part. X is back when you're ready.'). Shrinking the same task repeatedly never piles up duplicate pebbles, only one is open at a time. Make it tiny again for the next step, or just complete the task.</t>
+          <t>The original task disappears from Today and Later (it becomes a silent parent, not clutter beside its steps). When the last step is done, the real task completes on its own with the held 'you finished the whole thing' bloom (see AI-09) and lands in the Lookback as the finished real task. Multi-phase: finishing a milestone's steps cascades up to the root.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>AI-09</t>
+          <t>AI-08</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3001,17 +3001,17 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Whole-task finish raises the held bloom (scaled)</t>
+          <t>Make it tiny keeps the real task (open parent), no pile-up</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Finish the LAST step of a broken-down task. Try it on a long-lingering or chunky task, and separately on a small same-day one. Then repeat with Reduce Motion on.</t>
+          <t>On a dreaded task choose 'Make it tiny' and do the 2-minute version. Then shrink the same task again to confirm pebbles do not accumulate.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>A warm radial bloom rises over a dimming scrim: 'You finished the whole thing', the task name in Newsreader italic, and a warm context line ('... since you first wrote it down. N small steps. All done.'). It holds longer and blooms larger for a long-dreaded or chunky task than for a quick same-day one. A tap dismisses it early, otherwise it auto-settles. Never confetti, points, or a number on screen. On Android the dimmed scrim is clean, with NO vertical pillar or banding behind it (the SVG background pools are disabled on Android, where they mis-render at large size). With Reduce Motion on, the held title and warm colour still show, only the movement is removed.</t>
+          <t>The dreaded task disappears and a 2-minute starter takes its place on Today, carrying an 'A tiny step toward X' eyebrow so the real task stays visible. Completing the starter does NOT mark the big task done: the spent starter is retired (no clutter) and the real task reappears with a warm nudge ('You started, that's the hard part. X is back when you're ready.'). Shrinking the same task repeatedly never piles up duplicate pebbles, only one is open at a time. Make it tiny again for the next step, or just complete the task.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,12 +3026,12 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-09</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -3041,17 +3041,17 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Whole-task finish raises the held bloom (scaled)</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Finish the LAST step of a broken-down task. Try it on a long-lingering or chunky task, and separately on a small same-day one. Then repeat with Reduce Motion on.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A warm radial bloom rises over a dimming scrim: 'You finished the whole thing', the task name in Newsreader italic, and a warm context line ('... since you first wrote it down. N small steps. All done.'). It holds longer and blooms larger for a long-dreaded or chunky task than for a quick same-day one. A tap dismisses it early, otherwise it auto-settles. Never confetti, points, or a number on screen. On Android the dimmed scrim is clean, with NO vertical pillar or banding behind it (the SVG background pools are disabled on Android, where they mis-render at large size). With Reduce Motion on, the held title and warm colour still show, only the movement is removed.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,12 +3066,12 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>AI lighten</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
@@ -3081,17 +3081,17 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Lighten today (re-spread a full day)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>When today is heavy (6+ tasks, or 4+ on a low day), tap 'Lighten today'.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>The button only appears on a heavy day. It proposes re-spreading a few tasks to later days so today becomes doable, propose-then-accept. Free and ungated for everyone, never scolding.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,32 +3106,32 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI lighten</t>
+        </is>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Lighten today (re-spread a full day)</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When today is heavy (6+ tasks, or 4+ on a low day), tap 'Lighten today'.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>The button only appears on a heavy day. It proposes re-spreading a few tasks to later days so today becomes doable, propose-then-accept. Free and ungated for everyone, never scolding.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,7 +3146,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -3161,17 +3161,17 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,7 +3186,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3194,24 +3194,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3241,17 +3241,17 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>LB-05</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3281,17 +3281,17 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>First-ever open is warm, not empty</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>On a brand-new install with nothing ever completed, open the Lookback.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>The month reads 'This is where everything you finish will gather. Nothing yet, and that's a fine place to start.' (a welcome, never 'you did nothing'). No day shows a 'Nothing logged' line on this first run. Once anything is completed, the normal calendar behaviour returns.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,37 +3306,37 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-05</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>First-ever open is warm, not empty</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>On a brand-new install with nothing ever completed, open the Lookback.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The month reads 'This is where everything you finish will gather. Nothing yet, and that's a fine place to start.' (a welcome, never 'you did nothing'). No day shows a 'Nothing logged' line on this first run. Once anything is completed, the normal calendar behaviour returns.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr"/>
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,22 +3361,22 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr"/>
@@ -3386,7 +3386,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3401,17 +3401,17 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3434,24 +3434,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C68" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,22 +3481,22 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr"/>
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3521,22 +3521,22 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr"/>
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>SB-07</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,17 +3561,17 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>A missing keepsake image degrades gracefully</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Open a week whose scrapbook image is gone (e.g. the R2 object was purged on an account delete while the local entry survived, or the stored image is corrupt).</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>No blank polaroid. The week falls back to the calm 'That keepsake's picture isn't available anymore. Make a new one?' invite, and remaking overwrites it with a fresh image. Never a broken frame.</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3586,32 +3586,32 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-07</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>A missing keepsake image degrades gracefully</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Open a week whose scrapbook image is gone (e.g. the R2 object was purged on an account delete while the local entry survived, or the stored image is corrupt).</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>No blank polaroid. The week falls back to the calm 'That keepsake's picture isn't available anymore. Make a new one?' invite, and remaking overwrites it with a fresh image. Never a broken frame.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,7 +3666,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3681,17 +3681,17 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3714,24 +3714,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C75" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3761,17 +3761,17 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3801,17 +3801,17 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -3826,37 +3826,37 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr"/>
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3881,22 +3881,22 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr"/>
@@ -3906,7 +3906,7 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -3921,17 +3921,17 @@
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today, the Lookback calendar, the scrapbook, and any routines.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally: no tasks, an empty Lookback, no scrapbook, no routines. Only display prefs (theme, text size) persist.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3954,24 +3954,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C81" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today, the Lookback calendar, the scrapbook, and any routines.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally: no tasks, an empty Lookback, no scrapbook, no routines. Only display prefs (theme, text size) persist.</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -3986,32 +3986,32 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C82" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C82" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4041,22 +4041,22 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr"/>
@@ -4066,7 +4066,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4081,17 +4081,17 @@
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
@@ -4106,7 +4106,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -4121,17 +4121,17 @@
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
@@ -4146,7 +4146,7 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
@@ -4161,17 +4161,17 @@
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
@@ -4186,7 +4186,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -4194,29 +4194,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C87" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr"/>
@@ -4226,7 +4226,7 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -4241,22 +4241,22 @@
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr"/>
@@ -4266,37 +4266,37 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C89" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr"/>
@@ -4306,7 +4306,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
@@ -4314,24 +4314,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C90" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
@@ -4346,7 +4346,7 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
@@ -4361,17 +4361,17 @@
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
@@ -4386,7 +4386,7 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
@@ -4401,17 +4401,17 @@
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F92" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
@@ -4426,7 +4426,7 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
@@ -4441,17 +4441,17 @@
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F93" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
@@ -4466,7 +4466,7 @@
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>SET-06</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
@@ -4481,17 +4481,17 @@
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Send feedback in-app</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>In Settings, tap 'Send feedback', type a note, tap Send.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F94" s="9" t="inlineStr">
         <is>
-          <t>An inline box opens (no mail client, no leaving the app). Send shows 'Sending...' then a calm 'Thank you. It is on its way.', and the note arrives at the support inbox. On failure it shows a calm retry with the typed text kept. Needs the Worker deployed with /feedback + the FEEDBACK_TO secret set.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G94" s="7" t="inlineStr">
@@ -4506,7 +4506,7 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>SET-07</t>
+          <t>SET-06</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
@@ -4521,17 +4521,17 @@
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder explains why it can't turn on</t>
+          <t>Send feedback in-app</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>In Settings, set 'Daily reminder' to On in a context where it can't be granted: deny the browser notification prompt on web, or have notifications blocked.</t>
+          <t>In Settings, tap 'Send feedback', type a note, tap Send.</t>
         </is>
       </c>
       <c r="F95" s="9" t="inlineStr">
         <is>
-          <t>The toggle returns to Off and a calm one-line reason appears under it (e.g. 'Notifications are off for DoubleDone. Turn them on in your settings, then try again.'), never a silent failure and never a raw error. Granting permission and retrying turns it On.</t>
+          <t>An inline box opens (no mail client, no leaving the app). Send shows 'Sending...' then a calm 'Thank you. It is on its way.', and the note arrives at the support inbox. On failure it shows a calm retry with the typed text kept. Needs the Worker deployed with /feedback + the FEEDBACK_TO secret set.</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
@@ -4546,12 +4546,12 @@
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-07</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
@@ -4561,22 +4561,22 @@
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Daily reminder explains why it can't turn on</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>In Settings, set 'Daily reminder' to On in a context where it can't be granted: deny the browser notification prompt on web, or have notifications blocked.</t>
         </is>
       </c>
       <c r="F96" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>The toggle returns to Off and a calm one-line reason appears under it (e.g. 'Notifications are off for DoubleDone. Turn them on in your settings, then try again.'), never a silent failure and never a raw error. Granting permission and retrying turns it On.</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr"/>
@@ -4586,7 +4586,7 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
@@ -4601,22 +4601,22 @@
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F97" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr"/>
@@ -4626,7 +4626,7 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
@@ -4634,24 +4634,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C98" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C98" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">
@@ -4666,37 +4666,37 @@
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C99" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C99" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F99" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr"/>
@@ -4706,7 +4706,7 @@
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -4714,24 +4714,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C100" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F100" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G100" s="7" t="inlineStr">
@@ -4746,7 +4746,7 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
@@ -4761,17 +4761,17 @@
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
@@ -4786,32 +4786,32 @@
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>Turn the daily reminder on (Settings &gt; Daily reminder, or the Today footer), grant permission, and leave it on until the daily hour.</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
-          <t>A calm 'Your today is here when you are ready.' notification arrives at the scheduled hour (verified firing on a real Samsung device). Toggling it off cancels it.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G102" s="7" t="inlineStr">
@@ -4826,7 +4826,7 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
@@ -4834,24 +4834,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C103" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Turn the daily reminder on (Settings &gt; Daily reminder, or the Today footer), grant permission, and leave it on until the daily hour.</t>
         </is>
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm 'Your today is here when you are ready.' notification arrives at the scheduled hour (verified firing on a real Samsung device). Toggling it off cancels it.</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
@@ -4866,37 +4866,37 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C104" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr"/>
@@ -4906,12 +4906,12 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
@@ -4921,22 +4921,22 @@
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H105" s="7" t="inlineStr"/>
@@ -4946,7 +4946,7 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
@@ -4961,22 +4961,22 @@
       </c>
       <c r="D106" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F106" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G106" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H106" s="7" t="inlineStr"/>
@@ -4986,7 +4986,7 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -4994,29 +4994,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C107" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F107" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H107" s="7" t="inlineStr"/>
@@ -5026,37 +5026,37 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C108" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F108" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G108" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H108" s="7" t="inlineStr"/>
@@ -5066,7 +5066,7 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
@@ -5081,22 +5081,22 @@
       </c>
       <c r="D109" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E109" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F109" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H109" s="7" t="inlineStr"/>
@@ -5106,7 +5106,7 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
@@ -5121,17 +5121,17 @@
       </c>
       <c r="D110" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E110" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F110" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G110" s="7" t="inlineStr">
@@ -5146,7 +5146,7 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
@@ -5161,22 +5161,22 @@
       </c>
       <c r="D111" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F111" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G111" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H111" s="7" t="inlineStr"/>
@@ -5186,7 +5186,7 @@
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
@@ -5201,22 +5201,22 @@
       </c>
       <c r="D112" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F112" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G112" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H112" s="7" t="inlineStr"/>
@@ -5226,7 +5226,7 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
@@ -5234,24 +5234,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C113" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D113" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E113" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F113" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G113" s="7" t="inlineStr">
@@ -5266,7 +5266,7 @@
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
@@ -5281,22 +5281,22 @@
       </c>
       <c r="D114" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E114" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F114" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G114" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H114" s="7" t="inlineStr"/>
@@ -5306,7 +5306,7 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
@@ -5314,29 +5314,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C115" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C115" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D115" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E115" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F115" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G115" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H115" s="7" t="inlineStr"/>
@@ -5346,7 +5346,7 @@
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
@@ -5361,17 +5361,17 @@
       </c>
       <c r="D116" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E116" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F116" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G116" s="7" t="inlineStr">
@@ -5386,7 +5386,7 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
@@ -5401,17 +5401,17 @@
       </c>
       <c r="D117" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E117" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F117" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G117" s="7" t="inlineStr">
@@ -5426,7 +5426,7 @@
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
@@ -5434,24 +5434,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C118" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D118" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E118" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F118" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G118" s="7" t="inlineStr">
@@ -5466,7 +5466,7 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>PREM-11</t>
+          <t>PREM-10</t>
         </is>
       </c>
       <c r="B119" s="7" t="inlineStr">
@@ -5474,29 +5474,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C119" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D119" s="9" t="inlineStr">
         <is>
-          <t>Comp allowlist: the owner email is always premium</t>
+          <t>Premium screen shows the renew / cancel date</t>
         </is>
       </c>
       <c r="E119" s="9" t="inlineStr">
         <is>
-          <t>Sign in with the comp email (the owner account listed in server/src/comp.ts), without ever paying.</t>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
         </is>
       </c>
       <c r="F119" s="9" t="inlineStr">
         <is>
-          <t>Premium is active immediately: Settings and the Lookback show the scrapbook unlocked and Scan works, with no Stripe charge. A non-allowlisted free account stays free. The allowlist is checked against a cryptographically verified token on the costed gate, so a forged token cannot claim premium compute.</t>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
         </is>
       </c>
       <c r="G119" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H119" s="7" t="inlineStr"/>
@@ -5506,7 +5506,7 @@
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>PREM-12</t>
+          <t>PREM-11</t>
         </is>
       </c>
       <c r="B120" s="7" t="inlineStr">
@@ -5514,24 +5514,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C120" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D120" s="9" t="inlineStr">
         <is>
-          <t>Lookback insights: the premium 'Your patterns' card</t>
+          <t>Comp allowlist: the owner email is always premium</t>
         </is>
       </c>
       <c r="E120" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), finish a few tasks across a couple of days this week including one big/dreaded one, then open the Lookback and scroll below the Scrapbook. Tap 'Reflect on this week'.</t>
+          <t>Sign in with the comp email (the owner account listed in server/src/comp.ts), without ever paying.</t>
         </is>
       </c>
       <c r="F120" s="9" t="inlineStr">
         <is>
-          <t>A calm 'Your patterns' card shows warm counts (finished this week, 'on N days', reclaimed old tasks named) with NO streak, score, percent, or 'missed' wording. 'Reflect on this week' returns one warm paragraph that only celebrates what was done (never a performance review) and changes nothing about your tasks. A 'lookback.summary.made' event is logged.</t>
+          <t>Premium is active immediately: Settings and the Lookback show the scrapbook unlocked and Scan works, with no Stripe charge. A non-allowlisted free account stays free. The allowlist is checked against a cryptographically verified token on the costed gate, so a forged token cannot claim premium compute.</t>
         </is>
       </c>
       <c r="G120" s="7" t="inlineStr">
@@ -5546,7 +5546,7 @@
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>PREM-13</t>
+          <t>PREM-12</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
@@ -5561,17 +5561,17 @@
       </c>
       <c r="D121" s="9" t="inlineStr">
         <is>
-          <t>Lookback insights: free sees a calm upsell, not a wall</t>
+          <t>Lookback insights: the premium 'Your patterns' card</t>
         </is>
       </c>
       <c r="E121" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open the Lookback and scroll below the Scrapbook, then tap the 'Your patterns' card.</t>
+          <t>As premium (or with the dev Premium override on), finish a few tasks across a couple of days this week including one big/dreaded one, then open the Lookback and scroll below the Scrapbook. Tap 'Reflect on this week'.</t>
         </is>
       </c>
       <c r="F121" s="9" t="inlineStr">
         <is>
-          <t>A calm one-line invite ('See what your weeks and months add up to'), never a teased count and never a wall. Tapping routes to /premium and logs 'premium.gate_hit' with reason 'insights'. The free user's calendar and their one monthly scrapbook are completely untouched.</t>
+          <t>A calm 'Your patterns' card shows warm counts (finished this week, 'on N days', reclaimed old tasks named) with NO streak, score, percent, or 'missed' wording. 'Reflect on this week' returns one warm paragraph that only celebrates what was done (never a performance review) and changes nothing about your tasks. A 'lookback.summary.made' event is logged.</t>
         </is>
       </c>
       <c r="G121" s="7" t="inlineStr">
@@ -5586,7 +5586,7 @@
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>PREM-14</t>
+          <t>PREM-13</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
@@ -5594,24 +5594,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C122" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D122" s="9" t="inlineStr">
         <is>
-          <t>Premium: custom accent colour</t>
+          <t>Lookback insights: free sees a calm upsell, not a wall</t>
         </is>
       </c>
       <c r="E122" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), open Settings -&gt; Comfort -&gt; 'Accent colour' and tap each of Mauve / Teal / Rose / Gold, reloading after choosing one. Then as a FREE user, tap a swatch.</t>
+          <t>As a free user, open the Lookback and scroll below the Scrapbook, then tap the 'Your patterns' card.</t>
         </is>
       </c>
       <c r="F122" s="9" t="inlineStr">
         <is>
-          <t>Premium: tapping a swatch repaints the whole app in that accent (buttons, highlights, the brand) and the choice survives reload; the chosen swatch is ringed; mauve is the default. Dark mode shows the lifted dark variant of each. Free: the block shows a 'Premium' tag and tapping any swatch routes to the paywall with no change applied. A lapsed subscriber keeps the accent they chose.</t>
+          <t>A calm one-line invite ('See what your weeks and months add up to'), never a teased count and never a wall. Tapping routes to /premium and logs 'premium.gate_hit' with reason 'insights'. The free user's calendar and their one monthly scrapbook are completely untouched.</t>
         </is>
       </c>
       <c r="G122" s="7" t="inlineStr">
@@ -5626,7 +5626,7 @@
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>PREM-15</t>
+          <t>PREM-14</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
@@ -5641,17 +5641,17 @@
       </c>
       <c r="D123" s="9" t="inlineStr">
         <is>
-          <t>Post-payment 'taking a while' recovery</t>
+          <t>Premium: custom accent colour</t>
         </is>
       </c>
       <c r="E123" s="9" t="inlineStr">
         <is>
-          <t>Complete a test checkout, then on the return /premium success screen simulate the entitlement being slow (e.g. the webhook delayed) so polling does not flip within ~10 tries.</t>
+          <t>As premium (or with the dev Premium override on), open Settings -&gt; Comfort -&gt; 'Accent colour' and tap each of Mauve / Teal / Rose / Gold, reloading after choosing one. Then as a FREE user, tap a swatch.</t>
         </is>
       </c>
       <c r="F123" s="9" t="inlineStr">
         <is>
-          <t>Instead of spinning forever it shows a calm message ('This is taking longer than usual. Your payment went through, give it a minute, then tap Refresh.') with a Refresh button and a pointer to send a note from Settings if it persists. Tapping Refresh re-checks and flips to premium once the entitlement lands. It never says the payment failed.</t>
+          <t>Premium: tapping a swatch repaints the whole app in that accent (buttons, highlights, the brand) and the choice survives reload; the chosen swatch is ringed; mauve is the default. Dark mode shows the lifted dark variant of each. Free: the block shows a 'Premium' tag and tapping any swatch routes to the paywall with no change applied. A lapsed subscriber keeps the accent they chose.</t>
         </is>
       </c>
       <c r="G123" s="7" t="inlineStr">
@@ -5666,32 +5666,32 @@
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>PIN-01</t>
+          <t>PREM-15</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
         <is>
-          <t>Pin</t>
-        </is>
-      </c>
-      <c r="C124" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D124" s="9" t="inlineStr">
         <is>
-          <t>Premium: pin a task as the day's one thing</t>
+          <t>Post-payment 'taking a while' recovery</t>
         </is>
       </c>
       <c r="E124" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), tap-and-hold a one-off task to select it, then tap 'Pin' in the select bar.</t>
+          <t>Complete a test checkout, then on the return /premium success screen simulate the entitlement being slow (e.g. the webhook delayed) so polling does not flip within ~10 tries.</t>
         </is>
       </c>
       <c r="F124" s="9" t="inlineStr">
         <is>
-          <t>The task gets a calm mauve star and border and floats to the top of Today. 'Focus on one thing' then opens straight to it.</t>
+          <t>Instead of spinning forever it shows a calm message ('This is taking longer than usual. Your payment went through, give it a minute, then tap Refresh.') with a Refresh button and a pointer to send a note from Settings if it persists. Tapping Refresh re-checks and flips to premium once the entitlement lands. It never says the payment failed.</t>
         </is>
       </c>
       <c r="G124" s="7" t="inlineStr">
@@ -5706,7 +5706,7 @@
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>PIN-02</t>
+          <t>PIN-01</t>
         </is>
       </c>
       <c r="B125" s="7" t="inlineStr">
@@ -5721,17 +5721,17 @@
       </c>
       <c r="D125" s="9" t="inlineStr">
         <is>
-          <t>Free: Pin routes to the upsell, never pins</t>
+          <t>Premium: pin a task as the day's one thing</t>
         </is>
       </c>
       <c r="E125" s="9" t="inlineStr">
         <is>
-          <t>As a free user, select a single one-off task and tap the dimmed 'Pin' action.</t>
+          <t>As premium (or with the dev Premium override on), tap-and-hold a one-off task to select it, then tap 'Pin' in the select bar.</t>
         </is>
       </c>
       <c r="F125" s="9" t="inlineStr">
         <is>
-          <t>No task is pinned, and the Premium screen opens calmly (never a shaming wall). A 'premium.gate_hit' with reason 'pin' is logged.</t>
+          <t>The task gets a calm mauve star and border and floats to the top of Today. 'Focus on one thing' then opens straight to it.</t>
         </is>
       </c>
       <c r="G125" s="7" t="inlineStr">
@@ -5746,7 +5746,7 @@
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>PIN-03</t>
+          <t>PIN-02</t>
         </is>
       </c>
       <c r="B126" s="7" t="inlineStr">
@@ -5754,24 +5754,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C126" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C126" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D126" s="9" t="inlineStr">
         <is>
-          <t>Only one task is pinned at a time</t>
+          <t>Free: Pin routes to the upsell, never pins</t>
         </is>
       </c>
       <c r="E126" s="9" t="inlineStr">
         <is>
-          <t>As premium, pin task A, then select task B and pin it.</t>
+          <t>As a free user, select a single one-off task and tap the dimmed 'Pin' action.</t>
         </is>
       </c>
       <c r="F126" s="9" t="inlineStr">
         <is>
-          <t>Task B is now pinned (starred, floated to the top), and task A is no longer pinned. At most one pin ever exists.</t>
+          <t>No task is pinned, and the Premium screen opens calmly (never a shaming wall). A 'premium.gate_hit' with reason 'pin' is logged.</t>
         </is>
       </c>
       <c r="G126" s="7" t="inlineStr">
@@ -5786,7 +5786,7 @@
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>PIN-04</t>
+          <t>PIN-03</t>
         </is>
       </c>
       <c r="B127" s="7" t="inlineStr">
@@ -5801,17 +5801,17 @@
       </c>
       <c r="D127" s="9" t="inlineStr">
         <is>
-          <t>A pin syncs across devices</t>
+          <t>Only one task is pinned at a time</t>
         </is>
       </c>
       <c r="E127" s="9" t="inlineStr">
         <is>
-          <t>As premium and signed in, pin a task, then sign out and back in (or open a second device).</t>
+          <t>As premium, pin task A, then select task B and pin it.</t>
         </is>
       </c>
       <c r="F127" s="9" t="inlineStr">
         <is>
-          <t>The task is still pinned after the sync round-trip (the star and float persist). Needs the pinned_at column applied in Supabase.</t>
+          <t>Task B is now pinned (starred, floated to the top), and task A is no longer pinned. At most one pin ever exists.</t>
         </is>
       </c>
       <c r="G127" s="7" t="inlineStr">
@@ -5826,7 +5826,7 @@
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>PIN-05</t>
+          <t>PIN-04</t>
         </is>
       </c>
       <c r="B128" s="7" t="inlineStr">
@@ -5834,24 +5834,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C128" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D128" s="9" t="inlineStr">
         <is>
-          <t>Pin is offered only on one-off Today rows</t>
+          <t>A pin syncs across devices</t>
         </is>
       </c>
       <c r="E128" s="9" t="inlineStr">
         <is>
-          <t>Select a recurring task, then separately look at a task in the 'Later' list.</t>
+          <t>As premium and signed in, pin a task, then sign out and back in (or open a second device).</t>
         </is>
       </c>
       <c r="F128" s="9" t="inlineStr">
         <is>
-          <t>No 'Pin' action appears for a recurring task, and Later rows carry no pin affordance (pinning is Today-only and one-offs only).</t>
+          <t>The task is still pinned after the sync round-trip (the star and float persist). Needs the pinned_at column applied in Supabase.</t>
         </is>
       </c>
       <c r="G128" s="7" t="inlineStr">
@@ -5866,32 +5866,32 @@
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>OCR-01</t>
+          <t>PIN-05</t>
         </is>
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>Scan</t>
-        </is>
-      </c>
-      <c r="C129" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="C129" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D129" s="9" t="inlineStr">
         <is>
-          <t>Premium: the Scan button opens the camera</t>
+          <t>Pin is offered only on one-off Today rows</t>
         </is>
       </c>
       <c r="E129" s="9" t="inlineStr">
         <is>
-          <t>As premium, open the add panel and tap the Scan (camera) pill beside Speak.</t>
+          <t>Select a recurring task, then separately look at a task in the 'Later' list.</t>
         </is>
       </c>
       <c r="F129" s="9" t="inlineStr">
         <is>
-          <t>The camera screen opens: a live viewfinder with a shutter and a Photos shortcut on a device, or a 'Choose a photo' prompt on web. No paywall.</t>
+          <t>No 'Pin' action appears for a recurring task, and Later rows carry no pin affordance (pinning is Today-only and one-offs only).</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr">
@@ -5906,7 +5906,7 @@
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>OCR-02</t>
+          <t>OCR-01</t>
         </is>
       </c>
       <c r="B130" s="7" t="inlineStr">
@@ -5921,17 +5921,17 @@
       </c>
       <c r="D130" s="9" t="inlineStr">
         <is>
-          <t>Free: Scan routes to the upsell, never opens the camera</t>
+          <t>Premium: the Scan button opens the camera</t>
         </is>
       </c>
       <c r="E130" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open the add panel and tap the Scan pill.</t>
+          <t>As premium, open the add panel and tap the Scan (camera) pill beside Speak.</t>
         </is>
       </c>
       <c r="F130" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium screen calmly (never a wall). A 'premium.gate_hit' with reason 'ocr' is logged. No camera opens.</t>
+          <t>The camera screen opens: a live viewfinder with a shutter and a Photos shortcut on a device, or a 'Choose a photo' prompt on web. No paywall.</t>
         </is>
       </c>
       <c r="G130" s="7" t="inlineStr">
@@ -5946,7 +5946,7 @@
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>OCR-03</t>
+          <t>OCR-02</t>
         </is>
       </c>
       <c r="B131" s="7" t="inlineStr">
@@ -5961,22 +5961,22 @@
       </c>
       <c r="D131" s="9" t="inlineStr">
         <is>
-          <t>Photograph a list and the tasks land in the box</t>
+          <t>Free: Scan routes to the upsell, never opens the camera</t>
         </is>
       </c>
       <c r="E131" s="9" t="inlineStr">
         <is>
-          <t>As premium on a device, tap Scan, photograph a short printed or handwritten list (fill the frame), wait for 'Reading your list...'.</t>
+          <t>As a free user, open the add panel and tap the Scan pill.</t>
         </is>
       </c>
       <c r="F131" s="9" t="inlineStr">
         <is>
-          <t>The tasks it reads appear in the brain-dump box, one per line, editable. Nothing is auto-added to Today, and tapping Add commits them. An 'ocr.captured' event is logged.</t>
+          <t>Routed to the Premium screen calmly (never a wall). A 'premium.gate_hit' with reason 'ocr' is logged. No camera opens.</t>
         </is>
       </c>
       <c r="G131" s="7" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H131" s="7" t="inlineStr"/>
@@ -5986,7 +5986,7 @@
     <row r="132">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>OCR-04</t>
+          <t>OCR-03</t>
         </is>
       </c>
       <c r="B132" s="7" t="inlineStr">
@@ -5994,29 +5994,29 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C132" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C132" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D132" s="9" t="inlineStr">
         <is>
-          <t>Gallery fallback reads an existing photo</t>
+          <t>Photograph a list and the tasks land in the box</t>
         </is>
       </c>
       <c r="E132" s="9" t="inlineStr">
         <is>
-          <t>Tap Scan, then 'Photos' (device) or 'Choose a photo' (web), and pick a photo of a list, a note, or a whiteboard.</t>
+          <t>As premium on a device, tap Scan, photograph a short printed or handwritten list (fill the frame), wait for 'Reading your list...'.</t>
         </is>
       </c>
       <c r="F132" s="9" t="inlineStr">
         <is>
-          <t>Same result: the read tasks land in the box for review. Covers a screenshot of a texted list, or a photo taken earlier.</t>
+          <t>The tasks it reads appear in the brain-dump box, one per line, editable. Nothing is auto-added to Today, and tapping Add commits them. An 'ocr.captured' event is logged.</t>
         </is>
       </c>
       <c r="G132" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="H132" s="7" t="inlineStr"/>
@@ -6026,7 +6026,7 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>OCR-05</t>
+          <t>OCR-04</t>
         </is>
       </c>
       <c r="B133" s="7" t="inlineStr">
@@ -6041,17 +6041,17 @@
       </c>
       <c r="D133" s="9" t="inlineStr">
         <is>
-          <t>An unreadable photo fails calmly</t>
+          <t>Gallery fallback reads an existing photo</t>
         </is>
       </c>
       <c r="E133" s="9" t="inlineStr">
         <is>
-          <t>Scan a blank, blurry, or list-free image.</t>
+          <t>Tap Scan, then 'Photos' (device) or 'Choose a photo' (web), and pick a photo of a list, a note, or a whiteboard.</t>
         </is>
       </c>
       <c r="F133" s="9" t="inlineStr">
         <is>
-          <t>A calm line ('I couldn't read any tasks from that. Try again...'), the camera stays open, never a crash and never a shaming message.</t>
+          <t>Same result: the read tasks land in the box for review. Covers a screenshot of a texted list, or a photo taken earlier.</t>
         </is>
       </c>
       <c r="G133" s="7" t="inlineStr">
@@ -6066,7 +6066,7 @@
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>OCR-06</t>
+          <t>OCR-05</t>
         </is>
       </c>
       <c r="B134" s="7" t="inlineStr">
@@ -6081,22 +6081,22 @@
       </c>
       <c r="D134" s="9" t="inlineStr">
         <is>
-          <t>Camera denial is never a dead end</t>
+          <t>An unreadable photo fails calmly</t>
         </is>
       </c>
       <c r="E134" s="9" t="inlineStr">
         <is>
-          <t>On a device, deny the camera permission when prompted.</t>
+          <t>Scan a blank, blurry, or list-free image.</t>
         </is>
       </c>
       <c r="F134" s="9" t="inlineStr">
         <is>
-          <t>A calm screen offers 'Allow camera' and 'Choose from photos instead', and the gallery path still reads a list.</t>
+          <t>A calm line ('I couldn't read any tasks from that. Try again...'), the camera stays open, never a crash and never a shaming message.</t>
         </is>
       </c>
       <c r="G134" s="7" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr"/>
@@ -6106,7 +6106,7 @@
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>OCR-07</t>
+          <t>OCR-06</t>
         </is>
       </c>
       <c r="B135" s="7" t="inlineStr">
@@ -6114,29 +6114,29 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C135" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C135" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D135" s="9" t="inlineStr">
         <is>
-          <t>AI egress is disclosed at the point of use</t>
+          <t>Camera denial is never a dead end</t>
         </is>
       </c>
       <c r="E135" s="9" t="inlineStr">
         <is>
-          <t>Open the Scan screen (device or web).</t>
+          <t>On a device, deny the camera permission when prompted.</t>
         </is>
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>The note 'Your photo is sent to the AI to read your list, then discarded. It is never stored.' is visible. The D1 'ocr' telemetry row holds only the image size and task count, never the image or the titles.</t>
+          <t>A calm screen offers 'Allow camera' and 'Choose from photos instead', and the gallery path still reads a list.</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="H135" s="7" t="inlineStr"/>
@@ -6146,32 +6146,32 @@
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>CHART-01</t>
+          <t>OCR-07</t>
         </is>
       </c>
       <c r="B136" s="7" t="inlineStr">
         <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C136" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scan</t>
+        </is>
+      </c>
+      <c r="C136" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D136" s="9" t="inlineStr">
         <is>
-          <t>Premium: chart a course toward a goal</t>
+          <t>AI egress is disclosed at the point of use</t>
         </is>
       </c>
       <c r="E136" s="9" t="inlineStr">
         <is>
-          <t>As premium (or dev Premium override on), open Rooms, tap 'Chart a course', type a goal like 'get fit for a 10k', tap 'Suggest steps'.</t>
+          <t>Open the Scan screen (device or web).</t>
         </is>
       </c>
       <c r="F136" s="9" t="inlineStr">
         <is>
-          <t>A calm one-line heading plus 3-7 ticked next steps appear, and nothing is added yet. Tapping 'Add N tasks' lands them on Today (the first undated, later ones spread forward), each an ordinary task, and returns to Today. The 'chart.requested' then 'chart.added' events are logged.</t>
+          <t>The note 'Your photo is sent to the AI to read your list, then discarded. It is never stored.' is visible. The D1 'ocr' telemetry row holds only the image size and task count, never the image or the titles.</t>
         </is>
       </c>
       <c r="G136" s="7" t="inlineStr">
@@ -6186,7 +6186,7 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>CHART-02</t>
+          <t>CHART-01</t>
         </is>
       </c>
       <c r="B137" s="7" t="inlineStr">
@@ -6201,17 +6201,17 @@
       </c>
       <c r="D137" s="9" t="inlineStr">
         <is>
-          <t>Free: charting routes to the upsell, never plans</t>
+          <t>Premium: chart a course toward a goal</t>
         </is>
       </c>
       <c r="E137" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open Rooms, tap 'Chart a course', type a goal, tap 'Suggest steps'.</t>
+          <t>As premium (or dev Premium override on), open Rooms, tap 'Chart a course', type a goal like 'get fit for a 10k', tap 'Suggest steps'.</t>
         </is>
       </c>
       <c r="F137" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium screen calmly (never a wall), and a 'premium.gate_hit' with reason 'chart' is logged. No plan is generated and nothing is added.</t>
+          <t>A calm one-line heading plus 3-7 ticked next steps appear, and nothing is added yet. Tapping 'Add N tasks' lands them on Today (the first undated, later ones spread forward), each an ordinary task, and returns to Today. The 'chart.requested' then 'chart.added' events are logged.</t>
         </is>
       </c>
       <c r="G137" s="7" t="inlineStr">
@@ -6226,7 +6226,7 @@
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>CHART-03</t>
+          <t>CHART-02</t>
         </is>
       </c>
       <c r="B138" s="7" t="inlineStr">
@@ -6234,24 +6234,24 @@
           <t>Chart</t>
         </is>
       </c>
-      <c r="C138" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D138" s="9" t="inlineStr">
         <is>
-          <t>Propose-then-accept: nothing auto-adds</t>
+          <t>Free: charting routes to the upsell, never plans</t>
         </is>
       </c>
       <c r="E138" s="9" t="inlineStr">
         <is>
-          <t>As premium, generate a plan, untick two steps, then tap 'Add'. Separately, generate a plan and back out with 'Not these, start over' or Back.</t>
+          <t>As a free user, open Rooms, tap 'Chart a course', type a goal, tap 'Suggest steps'.</t>
         </is>
       </c>
       <c r="F138" s="9" t="inlineStr">
         <is>
-          <t>Only the ticked steps are added as plain tasks, and backing out adds nothing. Today was unchanged before accepting.</t>
+          <t>Routed to the Premium screen calmly (never a wall), and a 'premium.gate_hit' with reason 'chart' is logged. No plan is generated and nothing is added.</t>
         </is>
       </c>
       <c r="G138" s="7" t="inlineStr">
@@ -6266,7 +6266,7 @@
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>CHART-04</t>
+          <t>CHART-03</t>
         </is>
       </c>
       <c r="B139" s="7" t="inlineStr">
@@ -6281,17 +6281,17 @@
       </c>
       <c r="D139" s="9" t="inlineStr">
         <is>
-          <t>A goal that cannot be mapped fails calmly</t>
+          <t>Propose-then-accept: nothing auto-adds</t>
         </is>
       </c>
       <c r="E139" s="9" t="inlineStr">
         <is>
-          <t>Enter an empty goal (the button is disabled), then a nonsensical goal and submit.</t>
+          <t>As premium, generate a plan, untick two steps, then tap 'Add'. Separately, generate a plan and back out with 'Not these, start over' or Back.</t>
         </is>
       </c>
       <c r="F139" s="9" t="inlineStr">
         <is>
-          <t>The empty case cannot submit. A nonsensical goal shows one calm line ('I couldn't map that out just now'), the goal stays editable, never a crash or a shaming message.</t>
+          <t>Only the ticked steps are added as plain tasks, and backing out adds nothing. Today was unchanged before accepting.</t>
         </is>
       </c>
       <c r="G139" s="7" t="inlineStr">
@@ -6306,7 +6306,7 @@
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>CHART-05</t>
+          <t>CHART-04</t>
         </is>
       </c>
       <c r="B140" s="7" t="inlineStr">
@@ -6321,17 +6321,17 @@
       </c>
       <c r="D140" s="9" t="inlineStr">
         <is>
-          <t>A deadline spreads the steps across the timeframe</t>
+          <t>A goal that cannot be mapped fails calmly</t>
         </is>
       </c>
       <c r="E140" s="9" t="inlineStr">
         <is>
-          <t>As premium, type a goal, tap a 'By when?' chip (e.g. 'In 2 months'), then Suggest steps and Add.</t>
+          <t>Enter an empty goal (the button is disabled), then a nonsensical goal and submit.</t>
         </is>
       </c>
       <c r="F140" s="9" t="inlineStr">
         <is>
-          <t>The steps are paced for that timeframe, and the accepted tasks spread from Today out to the chosen date (not crammed into the next few days). 'No deadline' keeps the gentle one-per-day default.</t>
+          <t>The empty case cannot submit. A nonsensical goal shows one calm line ('I couldn't map that out just now'), the goal stays editable, never a crash or a shaming message.</t>
         </is>
       </c>
       <c r="G140" s="7" t="inlineStr">
@@ -6346,32 +6346,32 @@
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>SEQ-01</t>
+          <t>CHART-05</t>
         </is>
       </c>
       <c r="B141" s="7" t="inlineStr">
         <is>
-          <t>Sequence</t>
-        </is>
-      </c>
-      <c r="C141" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C141" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D141" s="9" t="inlineStr">
         <is>
-          <t>Premium: Plan my day suggests a calm sequence</t>
+          <t>A deadline spreads the steps across the timeframe</t>
         </is>
       </c>
       <c r="E141" s="9" t="inlineStr">
         <is>
-          <t>As premium with 3+ open one-off tasks on Today, tap 'Plan my day'.</t>
+          <t>As premium, type a goal, tap a 'By when?' chip (e.g. 'In 2 months'), then Suggest steps and Add.</t>
         </is>
       </c>
       <c r="F141" s="9" t="inlineStr">
         <is>
-          <t>A proposal card lists today's tasks in a suggested order, each with a short calm reason. Nothing reorders until 'Use this order' is tapped, then the list re-sequences in place (no dates change, no task moves to another day). A 'sequence.accepted' event is logged.</t>
+          <t>The steps are paced for that timeframe, and the accepted tasks spread from Today out to the chosen date (not crammed into the next few days). 'No deadline' keeps the gentle one-per-day default.</t>
         </is>
       </c>
       <c r="G141" s="7" t="inlineStr">
@@ -6386,7 +6386,7 @@
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>SEQ-02</t>
+          <t>SEQ-01</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
@@ -6401,17 +6401,17 @@
       </c>
       <c r="D142" s="9" t="inlineStr">
         <is>
-          <t>Free: Plan my day routes to the upsell, never reorders</t>
+          <t>Premium: Plan my day suggests a calm sequence</t>
         </is>
       </c>
       <c r="E142" s="9" t="inlineStr">
         <is>
-          <t>As a free user with 2+ tasks on Today, tap 'Plan my day'.</t>
+          <t>As premium with 3+ open one-off tasks on Today, tap 'Plan my day'.</t>
         </is>
       </c>
       <c r="F142" s="9" t="inlineStr">
         <is>
-          <t>The Premium screen opens calmly (never a wall), a 'premium.gate_hit' with reason 'sequence' is logged, and the day's order is unchanged.</t>
+          <t>A proposal card lists today's tasks in a suggested order, each with a short calm reason. Nothing reorders until 'Use this order' is tapped, then the list re-sequences in place (no dates change, no task moves to another day). A 'sequence.accepted' event is logged.</t>
         </is>
       </c>
       <c r="G142" s="7" t="inlineStr">
@@ -6426,7 +6426,7 @@
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>SEQ-03</t>
+          <t>SEQ-02</t>
         </is>
       </c>
       <c r="B143" s="7" t="inlineStr">
@@ -6434,24 +6434,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C143" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C143" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D143" s="9" t="inlineStr">
         <is>
-          <t>'Not now' leaves the day untouched</t>
+          <t>Free: Plan my day routes to the upsell, never reorders</t>
         </is>
       </c>
       <c r="E143" s="9" t="inlineStr">
         <is>
-          <t>As premium, open the proposal, then tap 'Not now' or the backdrop.</t>
+          <t>As a free user with 2+ tasks on Today, tap 'Plan my day'.</t>
         </is>
       </c>
       <c r="F143" s="9" t="inlineStr">
         <is>
-          <t>The order is exactly as before, nothing reordered, and no manualOrder is written.</t>
+          <t>The Premium screen opens calmly (never a wall), a 'premium.gate_hit' with reason 'sequence' is logged, and the day's order is unchanged.</t>
         </is>
       </c>
       <c r="G143" s="7" t="inlineStr">
@@ -6466,7 +6466,7 @@
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>SEQ-04</t>
+          <t>SEQ-03</t>
         </is>
       </c>
       <c r="B144" s="7" t="inlineStr">
@@ -6481,17 +6481,17 @@
       </c>
       <c r="D144" s="9" t="inlineStr">
         <is>
-          <t>An accepted order survives a reload (local-first)</t>
+          <t>'Not now' leaves the day untouched</t>
         </is>
       </c>
       <c r="E144" s="9" t="inlineStr">
         <is>
-          <t>As premium, accept an order, then fully reload the app.</t>
+          <t>As premium, open the proposal, then tap 'Not now' or the backdrop.</t>
         </is>
       </c>
       <c r="F144" s="9" t="inlineStr">
         <is>
-          <t>Today still shows the accepted order after reload (manualOrder persists on-device). Note: the order does not yet sync across devices, which is a documented follow-up.</t>
+          <t>The order is exactly as before, nothing reordered, and no manualOrder is written.</t>
         </is>
       </c>
       <c r="G144" s="7" t="inlineStr">
@@ -6506,7 +6506,7 @@
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>SEQ-05</t>
+          <t>SEQ-04</t>
         </is>
       </c>
       <c r="B145" s="7" t="inlineStr">
@@ -6514,24 +6514,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C145" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C145" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D145" s="9" t="inlineStr">
         <is>
-          <t>A pinned task still wins the very top</t>
+          <t>An accepted order survives a reload (local-first)</t>
         </is>
       </c>
       <c r="E145" s="9" t="inlineStr">
         <is>
-          <t>As premium, pin a task, then accept a 'Plan my day' sequence that puts a different task first.</t>
+          <t>As premium, accept an order, then fully reload the app.</t>
         </is>
       </c>
       <c r="F145" s="9" t="inlineStr">
         <is>
-          <t>The pinned task stays at the very top, and the accepted order applies to everything below it.</t>
+          <t>Today still shows the accepted order after reload (manualOrder persists on-device). Note: the order does not yet sync across devices, which is a documented follow-up.</t>
         </is>
       </c>
       <c r="G145" s="7" t="inlineStr">
@@ -6546,7 +6546,7 @@
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
         <is>
-          <t>SEQ-06</t>
+          <t>SEQ-05</t>
         </is>
       </c>
       <c r="B146" s="7" t="inlineStr">
@@ -6554,24 +6554,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C146" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C146" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D146" s="9" t="inlineStr">
         <is>
-          <t>Plan my day offers to lighten a heavy day</t>
+          <t>A pinned task still wins the very top</t>
         </is>
       </c>
       <c r="E146" s="9" t="inlineStr">
         <is>
-          <t>As premium on a heavy day (6+ tasks), tap 'Plan my day', accept the order.</t>
+          <t>As premium, pin a task, then accept a 'Plan my day' sequence that puts a different task first.</t>
         </is>
       </c>
       <c r="F146" s="9" t="inlineStr">
         <is>
-          <t>After the order applies, a 'Still a full day?' card offers to push a few tasks out to later days. Yes runs the re-spread (propose-then-accept), No leaves it ordered. On a calm day the offer never appears.</t>
+          <t>The pinned task stays at the very top, and the accepted order applies to everything below it.</t>
         </is>
       </c>
       <c r="G146" s="7" t="inlineStr">
@@ -6586,32 +6586,32 @@
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>BIG-01</t>
+          <t>SEQ-06</t>
         </is>
       </c>
       <c r="B147" s="7" t="inlineStr">
         <is>
-          <t>Big task</t>
-        </is>
-      </c>
-      <c r="C147" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Sequence</t>
+        </is>
+      </c>
+      <c r="C147" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D147" s="9" t="inlineStr">
         <is>
-          <t>Mark a task big: the tag, and the weight it adds</t>
+          <t>Plan my day offers to lighten a heavy day</t>
         </is>
       </c>
       <c r="E147" s="9" t="inlineStr">
         <is>
-          <t>On Today with a few one-off tasks, tap and hold one to enter select mode, then tap 'Big' in the action bar.</t>
+          <t>As premium on a heavy day (6+ tasks), tap 'Plan my day', accept the order.</t>
         </is>
       </c>
       <c r="F147" s="9" t="inlineStr">
         <is>
-          <t>Selection clears and the task shows a calm accent 'Big' tag beside its title (never red, never a warning), with a brief validating note ('Marked as a lot...'). The weight gauge fills further and reads heavier (one big task floors the bar to at least 'A full day, but doable.'). Free for everyone, no upsell.</t>
+          <t>After the order applies, a 'Still a full day?' card offers to push a few tasks out to later days. Yes runs the re-spread (propose-then-accept), No leaves it ordered. On a calm day the offer never appears.</t>
         </is>
       </c>
       <c r="G147" s="7" t="inlineStr">
@@ -6626,7 +6626,7 @@
     <row r="148">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t>BIG-02</t>
+          <t>BIG-01</t>
         </is>
       </c>
       <c r="B148" s="7" t="inlineStr">
@@ -6634,24 +6634,24 @@
           <t>Big task</t>
         </is>
       </c>
-      <c r="C148" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C148" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D148" s="9" t="inlineStr">
         <is>
-          <t>Big is a multi-select toggle</t>
+          <t>Mark a task big: the tag, and the weight it adds</t>
         </is>
       </c>
       <c r="E148" s="9" t="inlineStr">
         <is>
-          <t>Select two or more tasks and tap 'Big'; then re-select tasks that are all big and tap the action again (it now reads 'Not big').</t>
+          <t>On Today with a few one-off tasks, tap and hold one to enter select mode, then tap 'Big' in the action bar.</t>
         </is>
       </c>
       <c r="F148" s="9" t="inlineStr">
         <is>
-          <t>The first tap marks every selected task big at once. When all selected tasks are already big the action reads 'Not big' and clears the mark off all of them. A mixed selection marks all big (the additive default).</t>
+          <t>Selection clears and the task shows a calm accent 'Big' tag beside its title (never red, never a warning), with a brief validating note ('Marked as a lot...'). The weight gauge fills further and reads heavier (one big task floors the bar to at least 'A full day, but doable.'). Free for everyone, no upsell.</t>
         </is>
       </c>
       <c r="G148" s="7" t="inlineStr">
@@ -6666,7 +6666,7 @@
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>BIG-03</t>
+          <t>BIG-02</t>
         </is>
       </c>
       <c r="B149" s="7" t="inlineStr">
@@ -6681,17 +6681,17 @@
       </c>
       <c r="D149" s="9" t="inlineStr">
         <is>
-          <t>A lone big task lifts the bar but is not a re-spread problem</t>
+          <t>Big is a multi-select toggle</t>
         </is>
       </c>
       <c r="E149" s="9" t="inlineStr">
         <is>
-          <t>Have just one or two tasks on Today, one marked big.</t>
+          <t>Select two or more tasks and tap 'Big'; then re-select tasks that are all big and tap the action again (it now reads 'Not big').</t>
         </is>
       </c>
       <c r="F149" s="9" t="inlineStr">
         <is>
-          <t>The weight gauge reads at least 'A full day, but doable.' (the big task is felt), but 'Today's looking full' and 'Lighten today' do NOT appear for a lone big task (re-spreading cannot dissolve one big rock; Break it down is the tool). A big task plus a real pile (weighted load 6+) does surface Lighten today.</t>
+          <t>The first tap marks every selected task big at once. When all selected tasks are already big the action reads 'Not big' and clears the mark off all of them. A mixed selection marks all big (the additive default).</t>
         </is>
       </c>
       <c r="G149" s="7" t="inlineStr">
@@ -6706,7 +6706,7 @@
     <row r="150">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t>BIG-04</t>
+          <t>BIG-03</t>
         </is>
       </c>
       <c r="B150" s="7" t="inlineStr">
@@ -6721,17 +6721,17 @@
       </c>
       <c r="D150" s="9" t="inlineStr">
         <is>
-          <t>Finishing a big task is a big-win in the Lookback</t>
+          <t>A lone big task lifts the bar but is not a re-spread problem</t>
         </is>
       </c>
       <c r="E150" s="9" t="inlineStr">
         <is>
-          <t>Mark a task big, complete it, then open the Lookback to its day.</t>
+          <t>Have just one or two tasks on Today, one marked big.</t>
         </is>
       </c>
       <c r="F150" s="9" t="inlineStr">
         <is>
-          <t>The completed task carries the warmer 'a big one' treatment on its day, the same payoff a long-dreaded or chunky task earns. The big flag never adds disappointment if the task is left unfinished.</t>
+          <t>The weight gauge reads at least 'A full day, but doable.' (the big task is felt), but 'Today's looking full' and 'Lighten today' do NOT appear for a lone big task (re-spreading cannot dissolve one big rock; Break it down is the tool). A big task plus a real pile (weighted load 6+) does surface Lighten today.</t>
         </is>
       </c>
       <c r="G150" s="7" t="inlineStr">
@@ -6746,46 +6746,86 @@
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>NAV-01</t>
+          <t>BIG-04</t>
         </is>
       </c>
       <c r="B151" s="7" t="inlineStr">
         <is>
-          <t>Rooms</t>
-        </is>
-      </c>
-      <c r="C151" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Big task</t>
+        </is>
+      </c>
+      <c r="C151" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D151" s="9" t="inlineStr">
         <is>
-          <t>Rooms sheet caps its width on wide web</t>
+          <t>Finishing a big task is a big-win in the Lookback</t>
         </is>
       </c>
       <c r="E151" s="9" t="inlineStr">
         <is>
-          <t>On a wide desktop browser, open Rooms (the header pill).</t>
+          <t>Mark a task big, complete it, then open the Lookback to its day.</t>
         </is>
       </c>
       <c r="F151" s="9" t="inlineStr">
         <is>
-          <t>The sheet is a centred column (about 560px, matching the page content), not full-bleed, so the 'Premium' gradient pill on 'Chart a course' sits beside its label rather than at the far screen edge. On a phone the sheet stays full-width with the pill at the row's edge.</t>
+          <t>The completed task carries the warmer 'a big one' treatment on its day, the same payoff a long-dreaded or chunky task earns. The big flag never adds disappointment if the task is left unfinished.</t>
         </is>
       </c>
       <c r="G151" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H151" s="7" t="inlineStr"/>
       <c r="I151" s="9" t="inlineStr"/>
       <c r="J151" s="7" t="inlineStr"/>
     </row>
+    <row r="152">
+      <c r="A152" s="6" t="inlineStr">
+        <is>
+          <t>NAV-01</t>
+        </is>
+      </c>
+      <c r="B152" s="7" t="inlineStr">
+        <is>
+          <t>Rooms</t>
+        </is>
+      </c>
+      <c r="C152" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D152" s="9" t="inlineStr">
+        <is>
+          <t>Rooms sheet caps its width on wide web</t>
+        </is>
+      </c>
+      <c r="E152" s="9" t="inlineStr">
+        <is>
+          <t>On a wide desktop browser, open Rooms (the header pill).</t>
+        </is>
+      </c>
+      <c r="F152" s="9" t="inlineStr">
+        <is>
+          <t>The sheet is a centred column (about 560px, matching the page content), not full-bleed, so the 'Premium' gradient pill on 'Chart a course' sits beside its label rather than at the far screen edge. On a phone the sheet stays full-width with the pill at the row's edge.</t>
+        </is>
+      </c>
+      <c r="G152" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H152" s="7" t="inlineStr"/>
+      <c r="I152" s="9" t="inlineStr"/>
+      <c r="J152" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J151"/>
-  <conditionalFormatting sqref="H2:H151">
+  <autoFilter ref="A1:J152"/>
+  <conditionalFormatting sqref="H2:H152">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -6797,7 +6837,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H152" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6833,7 +6873,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>151</t>
         </is>
       </c>
     </row>
@@ -6844,7 +6884,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$151,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$152,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -6855,7 +6895,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$151,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$152,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -6866,7 +6906,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$151,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$152,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -6877,7 +6917,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$151,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$152,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -6888,7 +6928,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>150-COUNTA('Test Suite'!$H$2:$H$151)</f>
+        <f>151-COUNTA('Test Suite'!$H$2:$H$152)</f>
         <v/>
       </c>
     </row>
@@ -6899,7 +6939,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$151,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$152,"P1")</f>
         <v/>
       </c>
     </row>
@@ -6910,7 +6950,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$151,"P1",'Test Suite'!$H$2:$H$151,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$152,"P1",'Test Suite'!$H$2:$H$152,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(copy): scrapbook singular + one name for Scan; add trial/annual E2E cases
From the pre-merge review's copy lens (the deferred adversarial copy audit):
- The premium scrapbook-cap line read "That's this week's scrapb. (the
  allowance starts at one a week, and an OCD-leaning reader fixates on the
  broken plural at a paywall moment).
- The OCR feature had four names across one flow (Snap your list / Photograph
  your list / Read a list from a photo / Scan). Unified on "Scan": the modal
  header is "Scan a list", both prompts "Scan a photo of your list", matching
  the entry chip and the premium list.

Plus the two highest-stakes new surfaces shipped without an E2E case, against
the "a feature without a case is not done" rule: added PREM-16 (card-free
trial: grant, one-per-account never-shame, auto-revert) and PREM-17 (annual
vs monthly checkout + the already-subscribed 409 guard). Suite at 155 cases.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$154</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J154"/>
+  <dimension ref="A1:J156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5786,32 +5786,32 @@
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>PIN-01</t>
+          <t>PREM-16</t>
         </is>
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t>Pin</t>
-        </is>
-      </c>
-      <c r="C127" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C127" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D127" s="9" t="inlineStr">
         <is>
-          <t>Premium: pin a task as the day's one thing</t>
+          <t>Card-free 'Try Premium' one-month trial</t>
         </is>
       </c>
       <c r="E127" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), tap-and-hold a one-off task to select it, then tap 'Pin' in the select bar.</t>
+          <t>Signed in, on /premium tap 'Try Premium free for a month'. Confirm Premium unlocks. Tap it again on the SAME account. Advance the clock past 30 days (or inspect the trials row) and re-check entitlement. Also open the trial link signed OUT.</t>
         </is>
       </c>
       <c r="F127" s="9" t="inlineStr">
         <is>
-          <t>The task gets a calm mauve star and border and floats to the top of Today. 'Focus on one thing' then opens straight to it.</t>
+          <t>First tap: a calm confirm, Premium turns on with NO card and NO Stripe (status 'trial'); the page shows 'Your free month', 'Free until &lt;date&gt;', and 'Go Premium to keep it' (not 'Manage'). Second tap, same account: a gentle 'You've already had your free month' (never shame), no second trial granted. After expiry it reverts to free on its own, no charge ever. Signed out: an account is required (one trial per account), so the link routes to sign-in rather than granting.</t>
         </is>
       </c>
       <c r="G127" s="7" t="inlineStr">
@@ -5826,32 +5826,32 @@
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>PIN-02</t>
+          <t>PREM-17</t>
         </is>
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t>Pin</t>
-        </is>
-      </c>
-      <c r="C128" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D128" s="9" t="inlineStr">
         <is>
-          <t>Free: Pin routes to the upsell, never pins</t>
+          <t>Annual vs monthly plan checkout</t>
         </is>
       </c>
       <c r="E128" s="9" t="inlineStr">
         <is>
-          <t>As a free user, select a single one-off task and tap the dimmed 'Pin' action.</t>
+          <t>On /premium use the Monthly / Annual toggle, then Subscribe. Confirm the Stripe Checkout reflects the chosen plan. Complete a test annual checkout. Then, as an already-subscribed user, hit Subscribe again.</t>
         </is>
       </c>
       <c r="F128" s="9" t="inlineStr">
         <is>
-          <t>No task is pinned, and the Premium screen opens calmly (never a shaming wall). A 'premium.gate_hit' with reason 'pin' is logged.</t>
+          <t>The toggle shows 'A$50/year, about two months free' for annual; Checkout opens the YEARLY price for Annual and the monthly price for Monthly, and the success path grants Premium either way. An already-subscribed user is refused a second Checkout (the server 409s and the app says 'You're already on Premium', never a double charge). Prerequisite: the Worker deployed with STRIPE_PRICE_ID_ANNUAL and that price live in Stripe.</t>
         </is>
       </c>
       <c r="G128" s="7" t="inlineStr">
@@ -5866,7 +5866,7 @@
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>PIN-03</t>
+          <t>PIN-01</t>
         </is>
       </c>
       <c r="B129" s="7" t="inlineStr">
@@ -5874,24 +5874,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C129" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D129" s="9" t="inlineStr">
         <is>
-          <t>Only one task is pinned at a time</t>
+          <t>Premium: pin a task as the day's one thing</t>
         </is>
       </c>
       <c r="E129" s="9" t="inlineStr">
         <is>
-          <t>As premium, pin task A, then select task B and pin it.</t>
+          <t>As premium (or with the dev Premium override on), tap-and-hold a one-off task to select it, then tap 'Pin' in the select bar.</t>
         </is>
       </c>
       <c r="F129" s="9" t="inlineStr">
         <is>
-          <t>Task B is now pinned (starred, floated to the top), and task A is no longer pinned. At most one pin ever exists.</t>
+          <t>The task gets a calm mauve star and border and floats to the top of Today. 'Focus on one thing' then opens straight to it.</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr">
@@ -5906,7 +5906,7 @@
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>PIN-04</t>
+          <t>PIN-02</t>
         </is>
       </c>
       <c r="B130" s="7" t="inlineStr">
@@ -5914,24 +5914,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C130" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C130" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D130" s="9" t="inlineStr">
         <is>
-          <t>A pin syncs across devices</t>
+          <t>Free: Pin routes to the upsell, never pins</t>
         </is>
       </c>
       <c r="E130" s="9" t="inlineStr">
         <is>
-          <t>As premium and signed in, pin a task, then sign out and back in (or open a second device).</t>
+          <t>As a free user, select a single one-off task and tap the dimmed 'Pin' action.</t>
         </is>
       </c>
       <c r="F130" s="9" t="inlineStr">
         <is>
-          <t>The task is still pinned after the sync round-trip (the star and float persist). Needs the pinned_at column applied in Supabase.</t>
+          <t>No task is pinned, and the Premium screen opens calmly (never a shaming wall). A 'premium.gate_hit' with reason 'pin' is logged.</t>
         </is>
       </c>
       <c r="G130" s="7" t="inlineStr">
@@ -5946,7 +5946,7 @@
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>PIN-05</t>
+          <t>PIN-03</t>
         </is>
       </c>
       <c r="B131" s="7" t="inlineStr">
@@ -5954,24 +5954,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C131" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C131" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D131" s="9" t="inlineStr">
         <is>
-          <t>Pin is offered only on one-off Today rows</t>
+          <t>Only one task is pinned at a time</t>
         </is>
       </c>
       <c r="E131" s="9" t="inlineStr">
         <is>
-          <t>Select a recurring task, then separately look at a task in the 'Later' list.</t>
+          <t>As premium, pin task A, then select task B and pin it.</t>
         </is>
       </c>
       <c r="F131" s="9" t="inlineStr">
         <is>
-          <t>No 'Pin' action appears for a recurring task, and Later rows carry no pin affordance (pinning is Today-only and one-offs only).</t>
+          <t>Task B is now pinned (starred, floated to the top), and task A is no longer pinned. At most one pin ever exists.</t>
         </is>
       </c>
       <c r="G131" s="7" t="inlineStr">
@@ -5986,32 +5986,32 @@
     <row r="132">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>OCR-01</t>
+          <t>PIN-04</t>
         </is>
       </c>
       <c r="B132" s="7" t="inlineStr">
         <is>
-          <t>Scan</t>
-        </is>
-      </c>
-      <c r="C132" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="C132" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D132" s="9" t="inlineStr">
         <is>
-          <t>Premium: the Scan button opens the camera</t>
+          <t>A pin syncs across devices</t>
         </is>
       </c>
       <c r="E132" s="9" t="inlineStr">
         <is>
-          <t>As premium, open the add panel and tap the Scan (camera) pill beside Speak.</t>
+          <t>As premium and signed in, pin a task, then sign out and back in (or open a second device).</t>
         </is>
       </c>
       <c r="F132" s="9" t="inlineStr">
         <is>
-          <t>The camera screen opens: a live viewfinder with a shutter and a Photos shortcut on a device, or a 'Choose a photo' prompt on web. No paywall.</t>
+          <t>The task is still pinned after the sync round-trip (the star and float persist). Needs the pinned_at column applied in Supabase.</t>
         </is>
       </c>
       <c r="G132" s="7" t="inlineStr">
@@ -6026,32 +6026,32 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>OCR-02</t>
+          <t>PIN-05</t>
         </is>
       </c>
       <c r="B133" s="7" t="inlineStr">
         <is>
-          <t>Scan</t>
-        </is>
-      </c>
-      <c r="C133" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="C133" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D133" s="9" t="inlineStr">
         <is>
-          <t>Free: Scan routes to the upsell, never opens the camera</t>
+          <t>Pin is offered only on one-off Today rows</t>
         </is>
       </c>
       <c r="E133" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open the add panel and tap the Scan pill.</t>
+          <t>Select a recurring task, then separately look at a task in the 'Later' list.</t>
         </is>
       </c>
       <c r="F133" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium screen calmly (never a wall). A 'premium.gate_hit' with reason 'ocr' is logged. No camera opens.</t>
+          <t>No 'Pin' action appears for a recurring task, and Later rows carry no pin affordance (pinning is Today-only and one-offs only).</t>
         </is>
       </c>
       <c r="G133" s="7" t="inlineStr">
@@ -6066,7 +6066,7 @@
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>OCR-03</t>
+          <t>OCR-01</t>
         </is>
       </c>
       <c r="B134" s="7" t="inlineStr">
@@ -6081,22 +6081,22 @@
       </c>
       <c r="D134" s="9" t="inlineStr">
         <is>
-          <t>Photograph a list and the tasks land in the box</t>
+          <t>Premium: the Scan button opens the camera</t>
         </is>
       </c>
       <c r="E134" s="9" t="inlineStr">
         <is>
-          <t>As premium on a device, tap Scan, photograph a short printed or handwritten list (fill the frame), wait for 'Reading your list...'.</t>
+          <t>As premium, open the add panel and tap the Scan (camera) pill beside Speak.</t>
         </is>
       </c>
       <c r="F134" s="9" t="inlineStr">
         <is>
-          <t>The tasks it reads appear in the brain-dump box, one per line, editable. Nothing is auto-added to Today, and tapping Add commits them. An 'ocr.captured' event is logged.</t>
+          <t>The camera screen opens: a live viewfinder with a shutter and a Photos shortcut on a device, or a 'Choose a photo' prompt on web. No paywall.</t>
         </is>
       </c>
       <c r="G134" s="7" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr"/>
@@ -6106,7 +6106,7 @@
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>OCR-04</t>
+          <t>OCR-02</t>
         </is>
       </c>
       <c r="B135" s="7" t="inlineStr">
@@ -6114,24 +6114,24 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C135" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C135" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D135" s="9" t="inlineStr">
         <is>
-          <t>Gallery fallback reads an existing photo</t>
+          <t>Free: Scan routes to the upsell, never opens the camera</t>
         </is>
       </c>
       <c r="E135" s="9" t="inlineStr">
         <is>
-          <t>Tap Scan, then 'Photos' (device) or 'Choose a photo' (web), and pick a photo of a list, a note, or a whiteboard.</t>
+          <t>As a free user, open the add panel and tap the Scan pill.</t>
         </is>
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>Same result: the read tasks land in the box for review. Covers a screenshot of a texted list, or a photo taken earlier.</t>
+          <t>Routed to the Premium screen calmly (never a wall). A 'premium.gate_hit' with reason 'ocr' is logged. No camera opens.</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
@@ -6146,7 +6146,7 @@
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>OCR-05</t>
+          <t>OCR-03</t>
         </is>
       </c>
       <c r="B136" s="7" t="inlineStr">
@@ -6154,29 +6154,29 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C136" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C136" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D136" s="9" t="inlineStr">
         <is>
-          <t>An unreadable photo fails calmly</t>
+          <t>Photograph a list and the tasks land in the box</t>
         </is>
       </c>
       <c r="E136" s="9" t="inlineStr">
         <is>
-          <t>Scan a blank, blurry, or list-free image.</t>
+          <t>As premium on a device, tap Scan, photograph a short printed or handwritten list (fill the frame), wait for 'Reading your list...'.</t>
         </is>
       </c>
       <c r="F136" s="9" t="inlineStr">
         <is>
-          <t>A calm line ('I couldn't read any tasks from that. Try again...'), the camera stays open, never a crash and never a shaming message.</t>
+          <t>The tasks it reads appear in the brain-dump box, one per line, editable. Nothing is auto-added to Today, and tapping Add commits them. An 'ocr.captured' event is logged.</t>
         </is>
       </c>
       <c r="G136" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr"/>
@@ -6186,7 +6186,7 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>OCR-06</t>
+          <t>OCR-04</t>
         </is>
       </c>
       <c r="B137" s="7" t="inlineStr">
@@ -6201,22 +6201,22 @@
       </c>
       <c r="D137" s="9" t="inlineStr">
         <is>
-          <t>Camera denial is never a dead end</t>
+          <t>Gallery fallback reads an existing photo</t>
         </is>
       </c>
       <c r="E137" s="9" t="inlineStr">
         <is>
-          <t>On a device, deny the camera permission when prompted.</t>
+          <t>Tap Scan, then 'Photos' (device) or 'Choose a photo' (web), and pick a photo of a list, a note, or a whiteboard.</t>
         </is>
       </c>
       <c r="F137" s="9" t="inlineStr">
         <is>
-          <t>A calm screen offers 'Allow camera' and 'Choose from photos instead', and the gallery path still reads a list.</t>
+          <t>Same result: the read tasks land in the box for review. Covers a screenshot of a texted list, or a photo taken earlier.</t>
         </is>
       </c>
       <c r="G137" s="7" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr"/>
@@ -6226,7 +6226,7 @@
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>OCR-07</t>
+          <t>OCR-05</t>
         </is>
       </c>
       <c r="B138" s="7" t="inlineStr">
@@ -6234,24 +6234,24 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C138" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C138" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D138" s="9" t="inlineStr">
         <is>
-          <t>AI egress is disclosed at the point of use</t>
+          <t>An unreadable photo fails calmly</t>
         </is>
       </c>
       <c r="E138" s="9" t="inlineStr">
         <is>
-          <t>Open the Scan screen (device or web).</t>
+          <t>Scan a blank, blurry, or list-free image.</t>
         </is>
       </c>
       <c r="F138" s="9" t="inlineStr">
         <is>
-          <t>The note 'Your photo is sent to the AI to read your list, then discarded. It is never stored.' is visible. The D1 'ocr' telemetry row holds only the image size and task count, never the image or the titles.</t>
+          <t>A calm line ('I couldn't read any tasks from that. Try again...'), the camera stays open, never a crash and never a shaming message.</t>
         </is>
       </c>
       <c r="G138" s="7" t="inlineStr">
@@ -6266,37 +6266,37 @@
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>CHART-01</t>
+          <t>OCR-06</t>
         </is>
       </c>
       <c r="B139" s="7" t="inlineStr">
         <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C139" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scan</t>
+        </is>
+      </c>
+      <c r="C139" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D139" s="9" t="inlineStr">
         <is>
-          <t>Premium: chart a course toward a goal</t>
+          <t>Camera denial is never a dead end</t>
         </is>
       </c>
       <c r="E139" s="9" t="inlineStr">
         <is>
-          <t>As premium (or dev Premium override on), open Rooms, tap 'Chart a course', type a goal like 'get fit for a 10k', tap 'Suggest steps'.</t>
+          <t>On a device, deny the camera permission when prompted.</t>
         </is>
       </c>
       <c r="F139" s="9" t="inlineStr">
         <is>
-          <t>A calm one-line heading plus 3-7 ticked next steps appear, and nothing is added yet. Tapping 'Add N tasks' lands them on Today (the first undated, later ones spread forward), each an ordinary task, and returns to Today. The 'chart.requested' then 'chart.added' events are logged.</t>
+          <t>A calm screen offers 'Allow camera' and 'Choose from photos instead', and the gallery path still reads a list.</t>
         </is>
       </c>
       <c r="G139" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr"/>
@@ -6306,32 +6306,32 @@
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>CHART-02</t>
+          <t>OCR-07</t>
         </is>
       </c>
       <c r="B140" s="7" t="inlineStr">
         <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C140" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scan</t>
+        </is>
+      </c>
+      <c r="C140" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D140" s="9" t="inlineStr">
         <is>
-          <t>Free: charting routes to the upsell, never plans</t>
+          <t>AI egress is disclosed at the point of use</t>
         </is>
       </c>
       <c r="E140" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open Rooms, tap 'Chart a course', type a goal, tap 'Suggest steps'.</t>
+          <t>Open the Scan screen (device or web).</t>
         </is>
       </c>
       <c r="F140" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium screen calmly (never a wall), and a 'premium.gate_hit' with reason 'chart' is logged. No plan is generated and nothing is added.</t>
+          <t>The note 'Your photo is sent to the AI to read your list, then discarded. It is never stored.' is visible. The D1 'ocr' telemetry row holds only the image size and task count, never the image or the titles.</t>
         </is>
       </c>
       <c r="G140" s="7" t="inlineStr">
@@ -6346,7 +6346,7 @@
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>CHART-03</t>
+          <t>CHART-01</t>
         </is>
       </c>
       <c r="B141" s="7" t="inlineStr">
@@ -6354,24 +6354,24 @@
           <t>Chart</t>
         </is>
       </c>
-      <c r="C141" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C141" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D141" s="9" t="inlineStr">
         <is>
-          <t>Propose-then-accept: nothing auto-adds</t>
+          <t>Premium: chart a course toward a goal</t>
         </is>
       </c>
       <c r="E141" s="9" t="inlineStr">
         <is>
-          <t>As premium, generate a plan, untick two steps, then tap 'Add'. Separately, generate a plan and back out with 'Not these, start over' or Back.</t>
+          <t>As premium (or dev Premium override on), open Rooms, tap 'Chart a course', type a goal like 'get fit for a 10k', tap 'Suggest steps'.</t>
         </is>
       </c>
       <c r="F141" s="9" t="inlineStr">
         <is>
-          <t>Only the ticked steps are added as plain tasks, and backing out adds nothing. Today was unchanged before accepting.</t>
+          <t>A calm one-line heading plus 3-7 ticked next steps appear, and nothing is added yet. Tapping 'Add N tasks' lands them on Today (the first undated, later ones spread forward), each an ordinary task, and returns to Today. The 'chart.requested' then 'chart.added' events are logged.</t>
         </is>
       </c>
       <c r="G141" s="7" t="inlineStr">
@@ -6386,7 +6386,7 @@
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>CHART-04</t>
+          <t>CHART-02</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
@@ -6394,24 +6394,24 @@
           <t>Chart</t>
         </is>
       </c>
-      <c r="C142" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C142" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D142" s="9" t="inlineStr">
         <is>
-          <t>A goal that cannot be mapped fails calmly</t>
+          <t>Free: charting routes to the upsell, never plans</t>
         </is>
       </c>
       <c r="E142" s="9" t="inlineStr">
         <is>
-          <t>Enter an empty goal (the button is disabled), then a nonsensical goal and submit.</t>
+          <t>As a free user, open Rooms, tap 'Chart a course', type a goal, tap 'Suggest steps'.</t>
         </is>
       </c>
       <c r="F142" s="9" t="inlineStr">
         <is>
-          <t>The empty case cannot submit. A nonsensical goal shows one calm line ('I couldn't map that out just now'), the goal stays editable, never a crash or a shaming message.</t>
+          <t>Routed to the Premium screen calmly (never a wall), and a 'premium.gate_hit' with reason 'chart' is logged. No plan is generated and nothing is added.</t>
         </is>
       </c>
       <c r="G142" s="7" t="inlineStr">
@@ -6426,7 +6426,7 @@
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>CHART-05</t>
+          <t>CHART-03</t>
         </is>
       </c>
       <c r="B143" s="7" t="inlineStr">
@@ -6441,17 +6441,17 @@
       </c>
       <c r="D143" s="9" t="inlineStr">
         <is>
-          <t>A deadline spreads the steps across the timeframe</t>
+          <t>Propose-then-accept: nothing auto-adds</t>
         </is>
       </c>
       <c r="E143" s="9" t="inlineStr">
         <is>
-          <t>As premium, type a goal, tap a 'By when?' chip (e.g. 'In 2 months'), then Suggest steps and Add.</t>
+          <t>As premium, generate a plan, untick two steps, then tap 'Add'. Separately, generate a plan and back out with 'Not these, start over' or Back.</t>
         </is>
       </c>
       <c r="F143" s="9" t="inlineStr">
         <is>
-          <t>The steps are paced for that timeframe, and the accepted tasks spread from Today out to the chosen date (not crammed into the next few days). 'No deadline' keeps the gentle one-per-day default.</t>
+          <t>Only the ticked steps are added as plain tasks, and backing out adds nothing. Today was unchanged before accepting.</t>
         </is>
       </c>
       <c r="G143" s="7" t="inlineStr">
@@ -6466,32 +6466,32 @@
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>SEQ-01</t>
+          <t>CHART-04</t>
         </is>
       </c>
       <c r="B144" s="7" t="inlineStr">
         <is>
-          <t>Sequence</t>
-        </is>
-      </c>
-      <c r="C144" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C144" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D144" s="9" t="inlineStr">
         <is>
-          <t>Premium: Plan my day suggests a calm sequence</t>
+          <t>A goal that cannot be mapped fails calmly</t>
         </is>
       </c>
       <c r="E144" s="9" t="inlineStr">
         <is>
-          <t>As premium with 3+ open one-off tasks on Today, tap 'Plan my day'.</t>
+          <t>Enter an empty goal (the button is disabled), then a nonsensical goal and submit.</t>
         </is>
       </c>
       <c r="F144" s="9" t="inlineStr">
         <is>
-          <t>A proposal card lists today's tasks in a suggested order, each with a short calm reason. Nothing reorders until 'Use this order' is tapped, then the list re-sequences in place (no dates change, no task moves to another day). A 'sequence.accepted' event is logged.</t>
+          <t>The empty case cannot submit. A nonsensical goal shows one calm line ('I couldn't map that out just now'), the goal stays editable, never a crash or a shaming message.</t>
         </is>
       </c>
       <c r="G144" s="7" t="inlineStr">
@@ -6506,32 +6506,32 @@
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>SEQ-02</t>
+          <t>CHART-05</t>
         </is>
       </c>
       <c r="B145" s="7" t="inlineStr">
         <is>
-          <t>Sequence</t>
-        </is>
-      </c>
-      <c r="C145" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C145" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D145" s="9" t="inlineStr">
         <is>
-          <t>Free: Plan my day routes to the upsell, never reorders</t>
+          <t>A deadline spreads the steps across the timeframe</t>
         </is>
       </c>
       <c r="E145" s="9" t="inlineStr">
         <is>
-          <t>As a free user with 2+ tasks on Today, tap 'Plan my day'.</t>
+          <t>As premium, type a goal, tap a 'By when?' chip (e.g. 'In 2 months'), then Suggest steps and Add.</t>
         </is>
       </c>
       <c r="F145" s="9" t="inlineStr">
         <is>
-          <t>The Premium screen opens calmly (never a wall), a 'premium.gate_hit' with reason 'sequence' is logged, and the day's order is unchanged.</t>
+          <t>The steps are paced for that timeframe, and the accepted tasks spread from Today out to the chosen date (not crammed into the next few days). 'No deadline' keeps the gentle one-per-day default.</t>
         </is>
       </c>
       <c r="G145" s="7" t="inlineStr">
@@ -6546,7 +6546,7 @@
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
         <is>
-          <t>SEQ-03</t>
+          <t>SEQ-01</t>
         </is>
       </c>
       <c r="B146" s="7" t="inlineStr">
@@ -6554,24 +6554,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C146" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C146" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D146" s="9" t="inlineStr">
         <is>
-          <t>'Not now' leaves the day untouched</t>
+          <t>Premium: Plan my day suggests a calm sequence</t>
         </is>
       </c>
       <c r="E146" s="9" t="inlineStr">
         <is>
-          <t>As premium, open the proposal, then tap 'Not now' or the backdrop.</t>
+          <t>As premium with 3+ open one-off tasks on Today, tap 'Plan my day'.</t>
         </is>
       </c>
       <c r="F146" s="9" t="inlineStr">
         <is>
-          <t>The order is exactly as before, nothing reordered, and no manualOrder is written.</t>
+          <t>A proposal card lists today's tasks in a suggested order, each with a short calm reason. Nothing reorders until 'Use this order' is tapped, then the list re-sequences in place (no dates change, no task moves to another day). A 'sequence.accepted' event is logged.</t>
         </is>
       </c>
       <c r="G146" s="7" t="inlineStr">
@@ -6586,7 +6586,7 @@
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>SEQ-04</t>
+          <t>SEQ-02</t>
         </is>
       </c>
       <c r="B147" s="7" t="inlineStr">
@@ -6594,24 +6594,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C147" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C147" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D147" s="9" t="inlineStr">
         <is>
-          <t>An accepted order survives a reload (local-first)</t>
+          <t>Free: Plan my day routes to the upsell, never reorders</t>
         </is>
       </c>
       <c r="E147" s="9" t="inlineStr">
         <is>
-          <t>As premium, accept an order, then fully reload the app.</t>
+          <t>As a free user with 2+ tasks on Today, tap 'Plan my day'.</t>
         </is>
       </c>
       <c r="F147" s="9" t="inlineStr">
         <is>
-          <t>Today still shows the accepted order after reload (manualOrder persists on-device). Note: the order does not yet sync across devices, which is a documented follow-up.</t>
+          <t>The Premium screen opens calmly (never a wall), a 'premium.gate_hit' with reason 'sequence' is logged, and the day's order is unchanged.</t>
         </is>
       </c>
       <c r="G147" s="7" t="inlineStr">
@@ -6626,7 +6626,7 @@
     <row r="148">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t>SEQ-05</t>
+          <t>SEQ-03</t>
         </is>
       </c>
       <c r="B148" s="7" t="inlineStr">
@@ -6634,24 +6634,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C148" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C148" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D148" s="9" t="inlineStr">
         <is>
-          <t>A pinned task still wins the very top</t>
+          <t>'Not now' leaves the day untouched</t>
         </is>
       </c>
       <c r="E148" s="9" t="inlineStr">
         <is>
-          <t>As premium, pin a task, then accept a 'Plan my day' sequence that puts a different task first.</t>
+          <t>As premium, open the proposal, then tap 'Not now' or the backdrop.</t>
         </is>
       </c>
       <c r="F148" s="9" t="inlineStr">
         <is>
-          <t>The pinned task stays at the very top, and the accepted order applies to everything below it.</t>
+          <t>The order is exactly as before, nothing reordered, and no manualOrder is written.</t>
         </is>
       </c>
       <c r="G148" s="7" t="inlineStr">
@@ -6666,7 +6666,7 @@
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>SEQ-06</t>
+          <t>SEQ-04</t>
         </is>
       </c>
       <c r="B149" s="7" t="inlineStr">
@@ -6681,17 +6681,17 @@
       </c>
       <c r="D149" s="9" t="inlineStr">
         <is>
-          <t>Plan my day offers to lighten a heavy day</t>
+          <t>An accepted order survives a reload (local-first)</t>
         </is>
       </c>
       <c r="E149" s="9" t="inlineStr">
         <is>
-          <t>As premium on a heavy day (6+ tasks), tap 'Plan my day', accept the order.</t>
+          <t>As premium, accept an order, then fully reload the app.</t>
         </is>
       </c>
       <c r="F149" s="9" t="inlineStr">
         <is>
-          <t>After the order applies, a 'Still a full day?' card offers to push a few tasks out to later days. Yes runs the re-spread (propose-then-accept), No leaves it ordered. On a calm day the offer never appears.</t>
+          <t>Today still shows the accepted order after reload (manualOrder persists on-device). Note: the order does not yet sync across devices, which is a documented follow-up.</t>
         </is>
       </c>
       <c r="G149" s="7" t="inlineStr">
@@ -6706,32 +6706,32 @@
     <row r="150">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t>BIG-01</t>
+          <t>SEQ-05</t>
         </is>
       </c>
       <c r="B150" s="7" t="inlineStr">
         <is>
-          <t>Big task</t>
-        </is>
-      </c>
-      <c r="C150" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Sequence</t>
+        </is>
+      </c>
+      <c r="C150" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D150" s="9" t="inlineStr">
         <is>
-          <t>Mark a task big: the tag, and the weight it adds</t>
+          <t>A pinned task still wins the very top</t>
         </is>
       </c>
       <c r="E150" s="9" t="inlineStr">
         <is>
-          <t>On Today with a few one-off tasks, tap and hold one to enter select mode, then tap 'Big' in the action bar.</t>
+          <t>As premium, pin a task, then accept a 'Plan my day' sequence that puts a different task first.</t>
         </is>
       </c>
       <c r="F150" s="9" t="inlineStr">
         <is>
-          <t>Selection clears and the task shows a calm accent 'Big' tag beside its title (never red, never a warning), with a brief validating note ('Marked as a lot...'). The weight gauge fills further and reads heavier (one big task floors the bar to at least 'A full day, but doable.'). Free for everyone, no upsell.</t>
+          <t>The pinned task stays at the very top, and the accepted order applies to everything below it.</t>
         </is>
       </c>
       <c r="G150" s="7" t="inlineStr">
@@ -6746,12 +6746,12 @@
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>BIG-02</t>
+          <t>SEQ-06</t>
         </is>
       </c>
       <c r="B151" s="7" t="inlineStr">
         <is>
-          <t>Big task</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="C151" s="10" t="inlineStr">
@@ -6761,17 +6761,17 @@
       </c>
       <c r="D151" s="9" t="inlineStr">
         <is>
-          <t>Big is a multi-select toggle</t>
+          <t>Plan my day offers to lighten a heavy day</t>
         </is>
       </c>
       <c r="E151" s="9" t="inlineStr">
         <is>
-          <t>Select two or more tasks and tap 'Big'; then re-select tasks that are all big and tap the action again (it now reads 'Not big').</t>
+          <t>As premium on a heavy day (6+ tasks), tap 'Plan my day', accept the order.</t>
         </is>
       </c>
       <c r="F151" s="9" t="inlineStr">
         <is>
-          <t>The first tap marks every selected task big at once. When all selected tasks are already big the action reads 'Not big' and clears the mark off all of them. A mixed selection marks all big (the additive default).</t>
+          <t>After the order applies, a 'Still a full day?' card offers to push a few tasks out to later days. Yes runs the re-spread (propose-then-accept), No leaves it ordered. On a calm day the offer never appears.</t>
         </is>
       </c>
       <c r="G151" s="7" t="inlineStr">
@@ -6786,7 +6786,7 @@
     <row r="152">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t>BIG-03</t>
+          <t>BIG-01</t>
         </is>
       </c>
       <c r="B152" s="7" t="inlineStr">
@@ -6794,24 +6794,24 @@
           <t>Big task</t>
         </is>
       </c>
-      <c r="C152" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D152" s="9" t="inlineStr">
         <is>
-          <t>A lone big task lifts the bar but is not a re-spread problem</t>
+          <t>Mark a task big: the tag, and the weight it adds</t>
         </is>
       </c>
       <c r="E152" s="9" t="inlineStr">
         <is>
-          <t>Have just one or two tasks on Today, one marked big.</t>
+          <t>On Today with a few one-off tasks, tap and hold one to enter select mode, then tap 'Big' in the action bar.</t>
         </is>
       </c>
       <c r="F152" s="9" t="inlineStr">
         <is>
-          <t>The weight gauge reads at least 'A full day, but doable.' (the big task is felt), but 'Today's looking full' and 'Lighten today' do NOT appear for a lone big task (re-spreading cannot dissolve one big rock; Break it down is the tool). A big task plus a real pile (weighted load 6+) does surface Lighten today.</t>
+          <t>Selection clears and the task shows a calm accent 'Big' tag beside its title (never red, never a warning), with a brief validating note ('Marked as a lot...'). The weight gauge fills further and reads heavier (one big task floors the bar to at least 'A full day, but doable.'). Free for everyone, no upsell.</t>
         </is>
       </c>
       <c r="G152" s="7" t="inlineStr">
@@ -6826,7 +6826,7 @@
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>BIG-04</t>
+          <t>BIG-02</t>
         </is>
       </c>
       <c r="B153" s="7" t="inlineStr">
@@ -6841,17 +6841,17 @@
       </c>
       <c r="D153" s="9" t="inlineStr">
         <is>
-          <t>Finishing a big task is a big-win in the Lookback</t>
+          <t>Big is a multi-select toggle</t>
         </is>
       </c>
       <c r="E153" s="9" t="inlineStr">
         <is>
-          <t>Mark a task big, complete it, then open the Lookback to its day.</t>
+          <t>Select two or more tasks and tap 'Big'; then re-select tasks that are all big and tap the action again (it now reads 'Not big').</t>
         </is>
       </c>
       <c r="F153" s="9" t="inlineStr">
         <is>
-          <t>The completed task carries the warmer 'a big one' treatment on its day, the same payoff a long-dreaded or chunky task earns. The big flag never adds disappointment if the task is left unfinished.</t>
+          <t>The first tap marks every selected task big at once. When all selected tasks are already big the action reads 'Not big' and clears the mark off all of them. A mixed selection marks all big (the additive default).</t>
         </is>
       </c>
       <c r="G153" s="7" t="inlineStr">
@@ -6866,46 +6866,126 @@
     <row r="154">
       <c r="A154" s="6" t="inlineStr">
         <is>
-          <t>NAV-01</t>
+          <t>BIG-03</t>
         </is>
       </c>
       <c r="B154" s="7" t="inlineStr">
         <is>
-          <t>Rooms</t>
-        </is>
-      </c>
-      <c r="C154" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Big task</t>
+        </is>
+      </c>
+      <c r="C154" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D154" s="9" t="inlineStr">
         <is>
-          <t>Rooms sheet caps its width on wide web</t>
+          <t>A lone big task lifts the bar but is not a re-spread problem</t>
         </is>
       </c>
       <c r="E154" s="9" t="inlineStr">
         <is>
-          <t>On a wide desktop browser, open Rooms (the header pill).</t>
+          <t>Have just one or two tasks on Today, one marked big.</t>
         </is>
       </c>
       <c r="F154" s="9" t="inlineStr">
         <is>
-          <t>The sheet is a centred column (about 560px, matching the page content), not full-bleed, so the 'Premium' gradient pill on 'Chart a course' sits beside its label rather than at the far screen edge. On a phone the sheet stays full-width with the pill at the row's edge.</t>
+          <t>The weight gauge reads at least 'A full day, but doable.' (the big task is felt), but 'Today's looking full' and 'Lighten today' do NOT appear for a lone big task (re-spreading cannot dissolve one big rock; Break it down is the tool). A big task plus a real pile (weighted load 6+) does surface Lighten today.</t>
         </is>
       </c>
       <c r="G154" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H154" s="7" t="inlineStr"/>
       <c r="I154" s="9" t="inlineStr"/>
       <c r="J154" s="7" t="inlineStr"/>
     </row>
+    <row r="155">
+      <c r="A155" s="6" t="inlineStr">
+        <is>
+          <t>BIG-04</t>
+        </is>
+      </c>
+      <c r="B155" s="7" t="inlineStr">
+        <is>
+          <t>Big task</t>
+        </is>
+      </c>
+      <c r="C155" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D155" s="9" t="inlineStr">
+        <is>
+          <t>Finishing a big task is a big-win in the Lookback</t>
+        </is>
+      </c>
+      <c r="E155" s="9" t="inlineStr">
+        <is>
+          <t>Mark a task big, complete it, then open the Lookback to its day.</t>
+        </is>
+      </c>
+      <c r="F155" s="9" t="inlineStr">
+        <is>
+          <t>The completed task carries the warmer 'a big one' treatment on its day, the same payoff a long-dreaded or chunky task earns. The big flag never adds disappointment if the task is left unfinished.</t>
+        </is>
+      </c>
+      <c r="G155" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H155" s="7" t="inlineStr"/>
+      <c r="I155" s="9" t="inlineStr"/>
+      <c r="J155" s="7" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="6" t="inlineStr">
+        <is>
+          <t>NAV-01</t>
+        </is>
+      </c>
+      <c r="B156" s="7" t="inlineStr">
+        <is>
+          <t>Rooms</t>
+        </is>
+      </c>
+      <c r="C156" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D156" s="9" t="inlineStr">
+        <is>
+          <t>Rooms sheet caps its width on wide web</t>
+        </is>
+      </c>
+      <c r="E156" s="9" t="inlineStr">
+        <is>
+          <t>On a wide desktop browser, open Rooms (the header pill).</t>
+        </is>
+      </c>
+      <c r="F156" s="9" t="inlineStr">
+        <is>
+          <t>The sheet is a centred column (about 560px, matching the page content), not full-bleed, so the 'Premium' gradient pill on 'Chart a course' sits beside its label rather than at the far screen edge. On a phone the sheet stays full-width with the pill at the row's edge.</t>
+        </is>
+      </c>
+      <c r="G156" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H156" s="7" t="inlineStr"/>
+      <c r="I156" s="9" t="inlineStr"/>
+      <c r="J156" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J154"/>
-  <conditionalFormatting sqref="H2:H154">
+  <autoFilter ref="A1:J156"/>
+  <conditionalFormatting sqref="H2:H156">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -6917,7 +6997,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H154" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6953,7 +7033,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>155</t>
         </is>
       </c>
     </row>
@@ -6964,7 +7044,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$154,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$156,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -6975,7 +7055,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$154,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$156,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -6986,7 +7066,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$154,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$156,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -6997,7 +7077,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$154,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$156,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -7008,7 +7088,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>153-COUNTA('Test Suite'!$H$2:$H$154)</f>
+        <f>155-COUNTA('Test Suite'!$H$2:$H$156)</f>
         <v/>
       </c>
     </row>
@@ -7019,7 +7099,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$154,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$156,"P1")</f>
         <v/>
       </c>
     </row>
@@ -7030,7 +7110,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$154,"P1",'Test Suite'!$H$2:$H$154,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$156,"P1",'Test Suite'!$H$2:$H$156,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(welcome): let the introduction choose AI-free before any AI runs
The capture screen gains a quiet "I'll sort it myself" link beside "Sort for me" that persists
aiEnabled:false and sorts the first dump fully on-device, so an AI-objector reaches Today having made
zero AI calls. The default stays AI-on; the choice is a sibling action, not a forced fork. makeDay now
takes the chosen value as a parameter (stale-closure fix), the capture primary label is computed from
aiEnabled ("Sort for me" / "Put them on today"), and turning AI back on routes to the Settings consent
card (asymmetry preserved). Honesty fix: the handoff "nothing leaves your device" line is conditional
(true when off, honest about egress when on), plus one always-on capture line naming what each button
sends. Designed via a 4-design / 3-judge / 1-synthesis workflow. Verified in preview: the opt-out path
makes zero AI network calls and persists the choice. QA: ONB-03 + SET-09/SET-10.
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$159</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J156"/>
+  <dimension ref="A1:J159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2826,12 +2826,12 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>AI-01</t>
+          <t>ONB-03</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>AI decompose</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
@@ -2841,17 +2841,17 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Break down a dreaded task</t>
+          <t>Choose AI-free in the introduction (zero egress)</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
+          <t>On a fresh run, Begin, then on the capture screen type a couple of lines. Read the line under the box, then tap 'I'll sort it myself' instead of 'Sort for me'. Walk through to Open Today. To prove zero egress, watch the network: nothing should reach the AI backend.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Returns small atomic steps and drops them into Today.</t>
+          <t>The capture screen always shows one neutral line naming what each button does ('Sort for me sends these lines to Claude to order your day. I'll sort it myself keeps everything on this device'). Tapping 'I'll sort it myself' sets AI off, puts every line on today with NO call to the AI backend, and the reveal adds 'Sorted on your device, all on today for now.' The final screen reads 'Private by default, nothing leaves your device' (now literally true). AI stays off afterwards (Settings shows Off). Tapping 'Sort for me' instead gives the normal AI triage. Replaying the welcome while AI is off shows the primary as 'Put them on today' and the link as 'Change in Settings'.</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>AI-02</t>
+          <t>AI-01</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2874,24 +2874,24 @@
           <t>AI decompose</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Time estimate shows</t>
+          <t>Break down a dreaded task</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>On the breakdown review, look for the pace/time estimate.</t>
+          <t>Capture 'Do my taxes', tap Break it down, answer any clarifying questions.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
+          <t>Returns small atomic steps and drops them into Today.</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>AI-03</t>
+          <t>AI-02</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2921,17 +2921,17 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>AI egress disclosure at point of use</t>
+          <t>Time estimate shows</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Open the Break-it-down questions modal.</t>
+          <t>On the breakdown review, look for the pace/time estimate.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
+          <t>A sensible total estimate is shown (the crowd/pace estimate).</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -2946,7 +2946,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>AI-04</t>
+          <t>AI-03</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2961,17 +2961,17 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Friendly error state</t>
+          <t>AI egress disclosure at point of use</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
+          <t>Open the Break-it-down questions modal.</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
+          <t>A calm one-liner discloses the text is sent to an AI and kept anonymously.</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>AI-07</t>
+          <t>AI-04</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -3001,17 +3001,17 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Breakdown keeps the real task as a silent parent (chain)</t>
+          <t>Friendly error state</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Break down a task (e.g. 'Plan the party'), then complete all of its steps, in any order.</t>
+          <t>Turn off wifi (or block the AI URL), then Break it down.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>The original task disappears from Today and Later (it becomes a silent parent, not clutter beside its steps). When the last step is done, the real task completes on its own with the held 'you finished the whole thing' bloom (see AI-09) and lands in the Lookback as the finished real task. Multi-phase: finishing a milestone's steps cascades up to the root.</t>
+          <t>A calm friendly error. No raw HTTP/stack. App stays usable.</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>AI-08</t>
+          <t>AI-07</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3041,17 +3041,17 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Make it tiny keeps the real task (open parent), no pile-up</t>
+          <t>Breakdown keeps the real task as a silent parent (chain)</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>On a dreaded task choose 'Make it tiny' and do the 2-minute version. Then shrink the same task again to confirm pebbles do not accumulate.</t>
+          <t>Break down a task (e.g. 'Plan the party'), then complete all of its steps, in any order.</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>The dreaded task disappears and a 2-minute starter takes its place on Today, carrying an 'A tiny step toward X' eyebrow so the real task stays visible. Completing the starter does NOT mark the big task done: the spent starter is retired (no clutter) and the real task reappears with a warm nudge ('You started, that's the hard part. X is back when you're ready.'). Shrinking the same task repeatedly never piles up duplicate pebbles, only one is open at a time. Make it tiny again for the next step, or just complete the task.</t>
+          <t>The original task disappears from Today and Later (it becomes a silent parent, not clutter beside its steps). When the last step is done, the real task completes on its own with the held 'you finished the whole thing' bloom (see AI-09) and lands in the Lookback as the finished real task. Multi-phase: finishing a milestone's steps cascades up to the root.</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
@@ -3066,7 +3066,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>AI-09</t>
+          <t>AI-08</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -3081,17 +3081,17 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Whole-task finish raises the held bloom (scaled)</t>
+          <t>Make it tiny keeps the real task (open parent), no pile-up</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Finish the LAST step of a broken-down task. Try it on a long-lingering or chunky task, and separately on a small same-day one. Then repeat with Reduce Motion on.</t>
+          <t>On a dreaded task choose 'Make it tiny' and do the 2-minute version. Then shrink the same task again to confirm pebbles do not accumulate.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>A warm radial bloom rises over a dimming scrim: 'You finished the whole thing', the task name in Newsreader italic, and a warm context line ('... since you first wrote it down. N small steps. All done.'). It holds longer and blooms larger for a long-dreaded or chunky task than for a quick same-day one. A tap dismisses it early, otherwise it auto-settles. Never confetti, points, or a number on screen. On Android the dimmed scrim is clean, with NO vertical pillar or banding behind it (the SVG background pools are disabled on Android, where they mis-render at large size). With Reduce Motion on, the held title and warm colour still show, only the movement is removed.</t>
+          <t>The dreaded task disappears and a 2-minute starter takes its place on Today, carrying an 'A tiny step toward X' eyebrow so the real task stays visible. Completing the starter does NOT mark the big task done: the spent starter is retired (no clutter) and the real task reappears with a warm nudge ('You started, that's the hard part. X is back when you're ready.'). Shrinking the same task repeatedly never piles up duplicate pebbles, only one is open at a time. Make it tiny again for the next step, or just complete the task.</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3106,12 +3106,12 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>AI-05</t>
+          <t>AI-09</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>AI triage</t>
+          <t>AI decompose</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
@@ -3121,17 +3121,17 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Sort-for-me (triage + feedback)</t>
+          <t>Whole-task finish raises the held bloom (scaled)</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
+          <t>Finish the LAST step of a broken-down task. Try it on a long-lingering or chunky task, and separately on a small same-day one. Then repeat with Reduce Motion on.</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
+          <t>A warm radial bloom rises over a dimming scrim: 'You finished the whole thing', the task name in Newsreader italic, and a warm context line ('... since you first wrote it down. N small steps. All done.'). It holds longer and blooms larger for a long-dreaded or chunky task than for a quick same-day one. A tap dismisses it early, otherwise it auto-settles. Never confetti, points, or a number on screen. On Android the dimmed scrim is clean, with NO vertical pillar or banding behind it (the SVG background pools are disabled on Android, where they mis-render at large size). With Reduce Motion on, the held title and warm colour still show, only the movement is removed.</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
@@ -3146,12 +3146,12 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>AI-06</t>
+          <t>AI-05</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>AI lighten</t>
+          <t>AI triage</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -3161,17 +3161,17 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Lighten today (re-spread a full day)</t>
+          <t>Sort-for-me (triage + feedback)</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>When today is heavy (6+ tasks, or 4+ on a low day), tap 'Lighten today'.</t>
+          <t>In the brain-dump type a MIXED pile, one per line (a couple of quick things, one that can wait, one big/vague). At one line a hint nudges 'one per line'; at two, 'Break it down' becomes 'Sort for me'. Run it.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>The button only appears on a heavy day. It proposes re-spreading a few tasks to later days so today becomes doable, propose-then-accept. Free and ungated for everyone, never scolding.</t>
+          <t>Shows a summary line ('Sorted: N for today, M for tomorrow, K to break down.'). Quick items stay on Today, can-waits move to tomorrow, big ones get an inline 'Looks big, break it down?' prompt. Calm, never scolding.</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -3186,32 +3186,32 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>LB-01</t>
+          <t>AI-06</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Lookback</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>AI lighten</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Open the calendar</t>
+          <t>Lighten today (re-spread a full day)</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Open the Lookback. Browse to different days/months.</t>
+          <t>When today is heavy (6+ tasks, or 4+ on a low day), tap 'Lighten today'.</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>A real Gregorian calendar. Navigation works, no crash.</t>
+          <t>The button only appears on a heavy day. It proposes re-spreading a few tasks to later days so today becomes doable, propose-then-accept. Free and ungated for everyone, never scolding.</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3226,7 +3226,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>LB-02</t>
+          <t>LB-01</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -3241,17 +3241,17 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Completed tasks show on their day</t>
+          <t>Open the calendar</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Complete a task today, open the Lookback on today.</t>
+          <t>Open the Lookback. Browse to different days/months.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>The completed task is listed under today.</t>
+          <t>A real Gregorian calendar. Navigation works, no crash.</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3266,7 +3266,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>LB-03</t>
+          <t>LB-02</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3274,24 +3274,24 @@
           <t>Lookback</t>
         </is>
       </c>
-      <c r="C64" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Old dreaded task is celebrated</t>
+          <t>Completed tasks show on their day</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
+          <t>Complete a task today, open the Lookback on today.</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
+          <t>The completed task is listed under today.</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3306,7 +3306,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>LB-04</t>
+          <t>LB-03</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3321,17 +3321,17 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Scheduled tasks show on the calendar</t>
+          <t>Old dreaded task is celebrated</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
+          <t>Complete a task that is old or high-complexity; view it in the Lookback.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
+          <t>Marked 'a big one' / weighted celebration. Never shamed for being old.</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -3346,7 +3346,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>LB-05</t>
+          <t>LB-04</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3361,17 +3361,17 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>First-ever open is warm, not empty</t>
+          <t>Scheduled tasks show on the calendar</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>On a brand-new install with nothing ever completed, open the Lookback.</t>
+          <t>Defer a task to tomorrow (or use 'Date...'), then open the Lookback and tap that future day.</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>The month reads 'This is where everything you finish will gather. Nothing yet, and that's a fine place to start.' (a welcome, never 'you did nothing'). No day shows a 'Nothing logged' line on this first run. Once anything is completed, the normal calendar behaviour returns.</t>
+          <t>The future day shows an outline marker; tapping it lists the task under 'Scheduled'.</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3386,37 +3386,37 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>SB-01</t>
+          <t>LB-05</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Scrapbook</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Lookback</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook</t>
+          <t>First-ever open is warm, not empty</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>In a week with completions, tap 'Make a scrapbook'.</t>
+          <t>On a brand-new install with nothing ever completed, open the Lookback.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
+          <t>The month reads 'This is where everything you finish will gather. Nothing yet, and that's a fine place to start.' (a welcome, never 'you did nothing'). No day shows a 'Nothing logged' line on this first run. Once anything is completed, the normal calendar behaviour returns.</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr"/>
@@ -3426,7 +3426,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>SB-02</t>
+          <t>SB-01</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3441,22 +3441,22 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Image surfaces the tasks</t>
+          <t>Make a scrapbook</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Look at the generated image/caption for a known week.</t>
+          <t>In a week with completions, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
+          <t>Loading shimmer, then a still-life image + caption in the polaroid.</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr"/>
@@ -3466,7 +3466,7 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>SB-03</t>
+          <t>SB-02</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3481,17 +3481,17 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Finished list + 'a big one'</t>
+          <t>Image surfaces the tasks</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Below the polaroid, read the 'This week you finished' list.</t>
+          <t>Look at the generated image/caption for a known week.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
+          <t>Objects evoke the actual tasks (e.g. laundry -&gt; folded linen). No text in image.</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -3506,7 +3506,7 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>SB-04</t>
+          <t>SB-03</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3514,24 +3514,24 @@
           <t>Scrapbook</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Invite state</t>
+          <t>Finished list + 'a big one'</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Open a week that has completions but no scrapbook yet.</t>
+          <t>Below the polaroid, read the 'This week you finished' list.</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
+          <t>All week's completed titles listed; big wins marked 'a big one'.</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -3546,7 +3546,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>SB-05</t>
+          <t>SB-04</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3561,22 +3561,22 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Free-tier limit is graceful</t>
+          <t>Invite state</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
+          <t>Open a week that has completions but no scrapbook yet.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
+          <t>Dashed frame + mauve '+', 'Turn this week into a keepsake', and the finished list still shows.</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr"/>
@@ -3586,7 +3586,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>SB-06</t>
+          <t>SB-05</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3601,22 +3601,22 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Scrapbook persists</t>
+          <t>Free-tier limit is graceful</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Make a scrapbook, restart the app.</t>
+          <t>Generate a few scrapbooks in one day (free tier ~1-2/day).</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>It is still there (device-local).</t>
+          <t>When exhausted, a calm wait/error. No crash, the holder stays intact.</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr"/>
@@ -3626,7 +3626,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>SB-07</t>
+          <t>SB-06</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3641,17 +3641,17 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>A missing keepsake image degrades gracefully</t>
+          <t>Scrapbook persists</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Open a week whose scrapbook image is gone (e.g. the R2 object was purged on an account delete while the local entry survived, or the stored image is corrupt).</t>
+          <t>Make a scrapbook, restart the app.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>No blank polaroid. The week falls back to the calm 'That keepsake's picture isn't available anymore. Make a new one?' invite, and remaking overwrites it with a fresh image. Never a broken frame.</t>
+          <t>It is still there (device-local).</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3666,32 +3666,32 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>AUTH-01</t>
+          <t>SB-07</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>Auth &amp; sync</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scrapbook</t>
+        </is>
+      </c>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Email sign-in (OTP)</t>
+          <t>A missing keepsake image degrades gracefully</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
+          <t>Open a week whose scrapbook image is gone (e.g. the R2 object was purged on an account delete while the local entry survived, or the stored image is corrupt).</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
+          <t>No blank polaroid. The week falls back to the calm 'That keepsake's picture isn't available anymore. Make a new one?' invite, and remaking overwrites it with a fresh image. Never a broken frame.</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3706,7 +3706,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>AUTH-02</t>
+          <t>AUTH-01</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3721,17 +3721,17 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Local tasks migrate on first sign-in</t>
+          <t>Email sign-in (OTP)</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Have some local tasks, then sign in for the first time.</t>
+          <t>Sign in, enter your email, get the 6-digit code from your inbox, verify.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Local tasks sync into the account. None lost or duplicated.</t>
+          <t>Signed in. Settings shows 'Synced to &lt;your email&gt;'. (This emails your inbox.)</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>AUTH-03</t>
+          <t>AUTH-02</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3761,17 +3761,17 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Sync across two devices</t>
+          <t>Local tasks migrate on first sign-in</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Sign in on web and the Android build. Add a task on one.</t>
+          <t>Have some local tasks, then sign in for the first time.</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>It appears on the other after sync.</t>
+          <t>Local tasks sync into the account. None lost or duplicated.</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>AUTH-04</t>
+          <t>AUTH-03</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3794,24 +3794,24 @@
           <t>Auth &amp; sync</t>
         </is>
       </c>
-      <c r="C77" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Last-write-wins, no dupes</t>
+          <t>Sync across two devices</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Complete / edit the same task on both devices close together.</t>
+          <t>Sign in on web and the Android build. Add a task on one.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>State converges. No duplicate rows, no flip-flop.</t>
+          <t>It appears on the other after sync.</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -3826,7 +3826,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>AUTH-05</t>
+          <t>AUTH-04</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -3841,17 +3841,17 @@
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Sign out</t>
+          <t>Last-write-wins, no dupes</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>Sign out from Settings.</t>
+          <t>Complete / edit the same task on both devices close together.</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Returns to local/anonymous. No account data left visible.</t>
+          <t>State converges. No duplicate rows, no flip-flop.</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>AUTH-06</t>
+          <t>AUTH-05</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
@@ -3881,17 +3881,17 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Offline then online</t>
+          <t>Sign out</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Go offline, add/complete tasks, then reconnect.</t>
+          <t>Sign out from Settings.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Changes sync up on reconnect. Nothing lost.</t>
+          <t>Returns to local/anonymous. No account data left visible.</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
@@ -3906,37 +3906,37 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>DEL-00</t>
+          <t>AUTH-06</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>Account deletion</t>
-        </is>
-      </c>
-      <c r="C80" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Auth &amp; sync</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: create the delete function</t>
+          <t>Offline then online</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
+          <t>Go offline, add/complete tasks, then reconnect.</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Function created. (One-time setup; cannot be rolled back.)</t>
+          <t>Changes sync up on reconnect. Nothing lost.</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr"/>
@@ -3946,7 +3946,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>DEL-01</t>
+          <t>DEL-00</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -3961,22 +3961,22 @@
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Delete account + data</t>
+          <t>PREREQ: create the delete function</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
+          <t>Run the delete_account() function from supabase/schema.sql once in the Supabase SQL editor.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
+          <t>Function created. (One-time setup; cannot be rolled back.)</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr"/>
@@ -3986,7 +3986,7 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>DEL-02</t>
+          <t>DEL-01</t>
         </is>
       </c>
       <c r="B82" s="7" t="inlineStr">
@@ -4001,17 +4001,17 @@
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Originating device is wiped</t>
+          <t>Delete account + data</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>On the device you deleted from, look at Today, the Lookback calendar, the scrapbook, and any routines.</t>
+          <t>Settings -&gt; Delete account and data -&gt; confirm. (Use a throwaway account first.)</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>Nothing of the account remains locally: no tasks, an empty Lookback, no scrapbook, no routines. Only display prefs (theme, text size) persist.</t>
+          <t>Account and synced data are gone. Returns to a clean, signed-out Today.</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
@@ -4026,7 +4026,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>DEL-03</t>
+          <t>DEL-02</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4034,24 +4034,24 @@
           <t>Account deletion</t>
         </is>
       </c>
-      <c r="C83" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Known limit: second device</t>
+          <t>Originating device is wiped</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>On a second signed-in device after deletion, observe behaviour.</t>
+          <t>On the device you deleted from, look at Today, the Lookback calendar, the scrapbook, and any routines.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
+          <t>Nothing of the account remains locally: no tasks, an empty Lookback, no scrapbook, no routines. Only display prefs (theme, text size) persist.</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
@@ -4066,32 +4066,32 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>MCP-00</t>
+          <t>DEL-03</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C84" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Account deletion</t>
+        </is>
+      </c>
+      <c r="C84" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: copy your token</t>
+          <t>Known limit: second device</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
+          <t>On a second signed-in device after deletion, observe behaviour.</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>Token copied (web) / shown selectable. Server URL visible.</t>
+          <t>It keeps local data until its next sync fails auth (documented limitation).</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
@@ -4106,7 +4106,7 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>MCP-01</t>
+          <t>MCP-00</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -4121,22 +4121,22 @@
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Connect a client</t>
+          <t>PREREQ: copy your token</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
+          <t>Sign in, Settings -&gt; AI agent access (MCP) -&gt; Copy my token.</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
+          <t>Token copied (web) / shown selectable. Server URL visible.</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr"/>
@@ -4146,7 +4146,7 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>MCP-02</t>
+          <t>MCP-01</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
@@ -4161,17 +4161,17 @@
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>add_task round-trip</t>
+          <t>Connect a client</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
+          <t>Add the /mcp server to Claude Desktop via mcp-remote + your token (see docs/mcp.md).</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>Task appears in your Today (web/app) after sync.</t>
+          <t>Client connects. Lists 3 tools: add_task, list_today, complete_task.</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
@@ -4186,7 +4186,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>MCP-03</t>
+          <t>MCP-02</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -4201,17 +4201,17 @@
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>list_today</t>
+          <t>add_task round-trip</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent: what's on my DoubleDone today?</t>
+          <t>Ask the agent: add 'book the dentist' to my DoubleDone.</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>Returns your open tasks, each with an id.</t>
+          <t>Task appears in your Today (web/app) after sync.</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
@@ -4226,7 +4226,7 @@
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>MCP-04</t>
+          <t>MCP-03</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -4241,17 +4241,17 @@
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>complete_task</t>
+          <t>list_today</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>Ask the agent to complete one of the listed tasks by id.</t>
+          <t>Ask the agent: what's on my DoubleDone today?</t>
         </is>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>Marked done; reflects in the app after sync.</t>
+          <t>Returns your open tasks, each with an id.</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
@@ -4266,7 +4266,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>MCP-05</t>
+          <t>MCP-04</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -4274,29 +4274,29 @@
           <t>MCP</t>
         </is>
       </c>
-      <c r="C89" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>No-token gate</t>
+          <t>complete_task</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
+          <t>Ask the agent to complete one of the listed tasks by id.</t>
         </is>
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
+          <t>Marked done; reflects in the app after sync.</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>Inspector</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr"/>
@@ -4306,7 +4306,7 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>MCP-06</t>
+          <t>MCP-05</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
@@ -4321,22 +4321,22 @@
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Expired token re-copy</t>
+          <t>No-token gate</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
+          <t>In the MCP Inspector, call a tool WITHOUT the Authorization header.</t>
         </is>
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
+          <t>Calm 'Not connected' result (isError). Nothing in your account changes.</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
         <is>
-          <t>Desktop</t>
+          <t>Inspector</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr"/>
@@ -4346,37 +4346,37 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>SET-01</t>
+          <t>MCP-06</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C91" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>Theme light / dark / system</t>
+          <t>Expired token re-copy</t>
         </is>
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>Switch theme between Light, Dark, and System.</t>
+          <t>Use a token older than ~1 hour, then re-copy a fresh one.</t>
         </is>
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
+          <t>Stale token fails cleanly; fresh token works. No data exposed.</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Desktop</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr"/>
@@ -4386,7 +4386,7 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>SET-02</t>
+          <t>SET-01</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
@@ -4394,24 +4394,24 @@
           <t>Settings</t>
         </is>
       </c>
-      <c r="C92" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Text size small / default / large</t>
+          <t>Theme light / dark / system</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>Change text size across all three.</t>
+          <t>Switch theme between Light, Dark, and System.</t>
         </is>
       </c>
       <c r="F92" s="9" t="inlineStr">
         <is>
-          <t>App scales. No clipping or broken layout at large.</t>
+          <t>Applies immediately. Dusk palette correct in both; System follows the OS.</t>
         </is>
       </c>
       <c r="G92" s="7" t="inlineStr">
@@ -4426,7 +4426,7 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>SET-03</t>
+          <t>SET-02</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
@@ -4441,17 +4441,17 @@
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>Motion -&gt; Reduce</t>
+          <t>Text size small / default / large</t>
         </is>
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>Set Motion to Reduce.</t>
+          <t>Change text size across all three.</t>
         </is>
       </c>
       <c r="F93" s="9" t="inlineStr">
         <is>
-          <t>Gentle fades and scrolling titles stop.</t>
+          <t>App scales. No clipping or broken layout at large.</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
@@ -4466,7 +4466,7 @@
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>SET-04</t>
+          <t>SET-03</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
@@ -4481,17 +4481,17 @@
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Privacy &amp; data link</t>
+          <t>Motion -&gt; Reduce</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>Tap 'Privacy &amp; data' in Settings.</t>
+          <t>Set Motion to Reduce.</t>
         </is>
       </c>
       <c r="F94" s="9" t="inlineStr">
         <is>
-          <t>Opens the privacy screen.</t>
+          <t>Gentle fades and scrolling titles stop.</t>
         </is>
       </c>
       <c r="G94" s="7" t="inlineStr">
@@ -4506,7 +4506,7 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>SET-05</t>
+          <t>SET-04</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
@@ -4521,17 +4521,17 @@
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>Export your data</t>
+          <t>Privacy &amp; data link</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
+          <t>Tap 'Privacy &amp; data' in Settings.</t>
         </is>
       </c>
       <c r="F95" s="9" t="inlineStr">
         <is>
-          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
+          <t>Opens the privacy screen.</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
@@ -4546,7 +4546,7 @@
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>SET-06</t>
+          <t>SET-05</t>
         </is>
       </c>
       <c r="B96" s="7" t="inlineStr">
@@ -4561,17 +4561,17 @@
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>Send feedback in-app</t>
+          <t>Export your data</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>In Settings, tap 'Send feedback', type a note, tap Send.</t>
+          <t>In Settings -&gt; Your data, tap 'Export your data' (works with no account).</t>
         </is>
       </c>
       <c r="F96" s="9" t="inlineStr">
         <is>
-          <t>An inline box opens (no mail client, no leaving the app). Send shows 'Sending...' then a calm 'Thank you. It is on its way.', and the note arrives at the support inbox. On failure it shows a calm retry with the typed text kept. Needs the Worker deployed with /feedback + the FEEDBACK_TO secret set.</t>
+          <t>Web downloads a doubledone-export-&lt;date&gt;.json with your tasks + completions; native opens the share sheet. Tombstones excluded, completion data kept.</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
@@ -4586,7 +4586,7 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>SET-07</t>
+          <t>SET-06</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
@@ -4601,17 +4601,17 @@
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder explains why it can't turn on</t>
+          <t>Send feedback in-app</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>In Settings, set 'Daily reminder' to On in a context where it can't be granted: deny the browser notification prompt on web, or have notifications blocked.</t>
+          <t>In Settings, tap 'Send feedback', type a note, tap Send.</t>
         </is>
       </c>
       <c r="F97" s="9" t="inlineStr">
         <is>
-          <t>The toggle returns to Off and a calm one-line reason appears under it (e.g. 'Notifications are off for DoubleDone. Turn them on in your settings, then try again.'), never a silent failure and never a raw error. Granting permission and retrying turns it On.</t>
+          <t>An inline box opens (no mail client, no leaving the app). Send shows 'Sending...' then a calm 'Thank you. It is on its way.', and the note arrives at the support inbox. On failure it shows a calm retry with the typed text kept. Needs the Worker deployed with /feedback + the FEEDBACK_TO secret set.</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
@@ -4626,7 +4626,7 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>SET-08</t>
+          <t>SET-07</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
@@ -4641,17 +4641,17 @@
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder time picker</t>
+          <t>Daily reminder explains why it can't turn on</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Turn 'Daily reminder' On, then use the - / + stepper that appears under it to change the time. Step down toward 12:00 AM and up toward 11:00 PM (the ends disable). Reload and re-open Settings; also turn the reminder on from the Today footer and confirm it uses the chosen time.</t>
+          <t>In Settings, set 'Daily reminder' to On in a context where it can't be granted: deny the browser notification prompt on web, or have notifications blocked.</t>
         </is>
       </c>
       <c r="F98" s="9" t="inlineStr">
         <is>
-          <t>A '- TIME +' stepper shows ONLY while the reminder is On, with a calm 12-hour label (e.g. '9:00 AM'). Each tap moves the hour by one and the label updates instantly; the minus disables at 12:00 AM, the plus at 11:00 PM. The chosen time survives reload and the daily nudge fires at that hour (not a fixed 9am), consistently wherever the reminder is switched on. Free for everyone, no upsell.</t>
+          <t>The toggle returns to Off and a calm one-line reason appears under it (e.g. 'Notifications are off for DoubleDone. Turn them on in your settings, then try again.'), never a silent failure and never a raw error. Granting permission and retrying turns it On.</t>
         </is>
       </c>
       <c r="G98" s="7" t="inlineStr">
@@ -4666,12 +4666,12 @@
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>SET-08</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
@@ -4681,22 +4681,22 @@
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>Daily reminder time picker</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Turn 'Daily reminder' On, then use the - / + stepper that appears under it to change the time. Step down toward 12:00 AM and up toward 11:00 PM (the ends disable). Reload and re-open Settings; also turn the reminder on from the Today footer and confirm it uses the chosen time.</t>
         </is>
       </c>
       <c r="F99" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>A '- TIME +' stepper shows ONLY while the reminder is On, with a calm 12-hour label (e.g. '9:00 AM'). Each tap moves the hour by one and the label updates instantly; the minus disables at 12:00 AM, the plus at 11:00 PM. The chosen time survives reload and the daily nudge fires at that hour (not a fixed 9am), consistently wherever the reminder is switched on. Free for everyone, no upsell.</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr"/>
@@ -4706,32 +4706,32 @@
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>SET-09</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="C100" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Turn AI off, the app whole without it</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>In Settings under 'AI', tap 'Turn AI off'. Then move through the app: capture, Today (long-press a task), the Menu, Lookback.</t>
         </is>
       </c>
       <c r="F100" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Turning off is instant with a warm line ('AI is off. Everything stays on your device.'). Every AI affordance then disappears: Sort for me / Tidy this / Scan in capture; Break it down / Make it tiny / Combine / Plan my day on Today, including the per-task Break-down and Make-tiny; the 'Chart a course' menu entry (and the screen redirects away); and Lookback's scrapbook + weekly reflection. On-device Speak stays. Nothing calls the AI backend and the calm to-do loop still works fully.</t>
         </is>
       </c>
       <c r="G100" s="7" t="inlineStr">
@@ -4746,32 +4746,32 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>SET-10</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="C101" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="C101" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Turn AI back on (informed consent)</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>With AI off, in Settings tap 'Turn AI on', read the card, and tap 'Turn on AI' (also try 'Not now').</t>
         </is>
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Turning ON asks first: a card naming exactly what is sent and to whom ('sends the text you choose... to Anthropic's Claude... Nothing else ever leaves your device.'). 'Not now' cancels with no change. 'Turn on AI' restores every AI affordance across the app. The asymmetry is deliberate: off is one instant tap, on is a clear informed tap.</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
@@ -4786,32 +4786,32 @@
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G102" s="7" t="inlineStr">
@@ -4826,12 +4826,12 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
@@ -4841,22 +4841,22 @@
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H103" s="7" t="inlineStr"/>
@@ -4866,37 +4866,37 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C104" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C104" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D104" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr"/>
@@ -4906,12 +4906,12 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
+          <t>Visual</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
@@ -4921,17 +4921,17 @@
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>Turn the daily reminder on (Settings &gt; Daily reminder, or the Today footer), grant permission, and leave it on until the daily hour.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>A calm 'Your today is here when you are ready.' notification arrives at the scheduled hour (verified firing on a real Samsung device). Toggling it off cancels it.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
@@ -4946,12 +4946,12 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
+          <t>Visual</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
@@ -4961,17 +4961,17 @@
       </c>
       <c r="D106" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F106" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G106" s="7" t="inlineStr">
@@ -4986,37 +4986,37 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C107" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C107" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F107" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H107" s="7" t="inlineStr"/>
@@ -5026,12 +5026,12 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Reminders</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
@@ -5041,22 +5041,22 @@
       </c>
       <c r="D108" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Turn the daily reminder on (Settings &gt; Daily reminder, or the Today footer), grant permission, and leave it on until the daily hour.</t>
         </is>
       </c>
       <c r="F108" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>A calm 'Your today is here when you are ready.' notification arrives at the scheduled hour (verified firing on a real Samsung device). Toggling it off cancels it.</t>
         </is>
       </c>
       <c r="G108" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H108" s="7" t="inlineStr"/>
@@ -5066,32 +5066,32 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
-        </is>
-      </c>
-      <c r="C109" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C109" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D109" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E109" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F109" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
@@ -5106,32 +5106,32 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
-        </is>
-      </c>
-      <c r="C110" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Privacy</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D110" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E110" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F110" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G110" s="7" t="inlineStr">
@@ -5146,12 +5146,12 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Deploy</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
@@ -5161,22 +5161,22 @@
       </c>
       <c r="D111" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F111" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G111" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H111" s="7" t="inlineStr"/>
@@ -5186,12 +5186,12 @@
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Deploy</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
@@ -5201,22 +5201,22 @@
       </c>
       <c r="D112" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F112" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G112" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H112" s="7" t="inlineStr"/>
@@ -5226,32 +5226,32 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C113" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C113" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D113" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E113" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F113" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G113" s="7" t="inlineStr">
@@ -5266,7 +5266,7 @@
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
@@ -5281,22 +5281,22 @@
       </c>
       <c r="D114" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E114" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F114" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G114" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H114" s="7" t="inlineStr"/>
@@ -5306,7 +5306,7 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
@@ -5321,17 +5321,17 @@
       </c>
       <c r="D115" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E115" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F115" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G115" s="7" t="inlineStr">
@@ -5346,7 +5346,7 @@
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
@@ -5354,24 +5354,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C116" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D116" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E116" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F116" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G116" s="7" t="inlineStr">
@@ -5386,7 +5386,7 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
@@ -5394,29 +5394,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C117" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D117" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E117" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F117" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G117" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H117" s="7" t="inlineStr"/>
@@ -5426,7 +5426,7 @@
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
@@ -5441,22 +5441,22 @@
       </c>
       <c r="D118" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E118" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F118" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G118" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H118" s="7" t="inlineStr"/>
@@ -5466,7 +5466,7 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B119" s="7" t="inlineStr">
@@ -5474,29 +5474,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D119" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E119" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F119" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G119" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H119" s="7" t="inlineStr"/>
@@ -5506,7 +5506,7 @@
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B120" s="7" t="inlineStr">
@@ -5514,29 +5514,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C120" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D120" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E120" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F120" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G120" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H120" s="7" t="inlineStr"/>
@@ -5546,7 +5546,7 @@
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
@@ -5554,24 +5554,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C121" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D121" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E121" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F121" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G121" s="7" t="inlineStr">
@@ -5586,7 +5586,7 @@
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>PREM-11</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
@@ -5594,29 +5594,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C122" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D122" s="9" t="inlineStr">
         <is>
-          <t>Comp allowlist: the owner email is always premium</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E122" s="9" t="inlineStr">
         <is>
-          <t>Sign in with the comp email (the owner account listed in server/src/comp.ts), without ever paying.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F122" s="9" t="inlineStr">
         <is>
-          <t>Premium is active immediately: Settings and the Lookback show the scrapbook unlocked and Scan works, with no Stripe charge. A non-allowlisted free account stays free. The allowlist is checked against a cryptographically verified token on the costed gate, so a forged token cannot claim premium compute.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G122" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H122" s="7" t="inlineStr"/>
@@ -5626,7 +5626,7 @@
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>PREM-12</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
@@ -5641,22 +5641,22 @@
       </c>
       <c r="D123" s="9" t="inlineStr">
         <is>
-          <t>Lookback insights: the premium 'Your patterns' card</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E123" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), finish a few tasks across a couple of days this week including one big/dreaded one, then open the Lookback and scroll below the Scrapbook. Tap 'Reflect on this week'.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F123" s="9" t="inlineStr">
         <is>
-          <t>A calm 'Your patterns' card shows warm counts (finished this week, 'on N days', reclaimed old tasks named) with NO streak, score, percent, or 'missed' wording. 'Reflect on this week' returns one warm paragraph that only celebrates what was done (never a performance review) and changes nothing about your tasks. A 'lookback.summary.made' event is logged.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G123" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H123" s="7" t="inlineStr"/>
@@ -5666,7 +5666,7 @@
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>PREM-13</t>
+          <t>PREM-10</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
@@ -5674,29 +5674,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C124" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D124" s="9" t="inlineStr">
         <is>
-          <t>Lookback insights: free sees a calm upsell, not a wall</t>
+          <t>Premium screen shows the renew / cancel date</t>
         </is>
       </c>
       <c r="E124" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open the Lookback and scroll below the Scrapbook, then tap the 'Your patterns' card.</t>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
         </is>
       </c>
       <c r="F124" s="9" t="inlineStr">
         <is>
-          <t>A calm one-line invite ('See what your weeks and months add up to'), never a teased count and never a wall. Tapping routes to /premium and logs 'premium.gate_hit' with reason 'insights'. The free user's calendar and their one monthly scrapbook are completely untouched.</t>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
         </is>
       </c>
       <c r="G124" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H124" s="7" t="inlineStr"/>
@@ -5706,7 +5706,7 @@
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>PREM-14</t>
+          <t>PREM-11</t>
         </is>
       </c>
       <c r="B125" s="7" t="inlineStr">
@@ -5714,24 +5714,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C125" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C125" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D125" s="9" t="inlineStr">
         <is>
-          <t>Premium: custom colour theme</t>
+          <t>Comp allowlist: the owner email is always premium</t>
         </is>
       </c>
       <c r="E125" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), open Settings -&gt; Comfort -&gt; 'Colour theme' and tap each of Dusk / Sage / Slate / Heather / Fog / Honey / Rose, reloading after choosing one, in BOTH light and dark mode. Then as a FREE user, tap a preset.</t>
+          <t>Sign in with the comp email (the owner account listed in server/src/comp.ts), without ever paying.</t>
         </is>
       </c>
       <c r="F125" s="9" t="inlineStr">
         <is>
-          <t>Premium: tapping a preset repaints the WHOLE app in that palette (background, cards, accent, the brand) and the choice survives reload; the chosen preset is ringed; Dusk is the default and looks identical to the pre-themes app. Each preset has a tuned light and dark variant. Honey's buttons keep DARK labels (a calm gold can't carry white text). Free: the block shows a 'Premium' tag and tapping any preset routes to the paywall with no change applied. A lapsed subscriber keeps the preset they chose.</t>
+          <t>Premium is active immediately: Settings and the Lookback show the scrapbook unlocked and Scan works, with no Stripe charge. A non-allowlisted free account stays free. The allowlist is checked against a cryptographically verified token on the costed gate, so a forged token cannot claim premium compute.</t>
         </is>
       </c>
       <c r="G125" s="7" t="inlineStr">
@@ -5746,7 +5746,7 @@
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>PREM-15</t>
+          <t>PREM-12</t>
         </is>
       </c>
       <c r="B126" s="7" t="inlineStr">
@@ -5754,24 +5754,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C126" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C126" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D126" s="9" t="inlineStr">
         <is>
-          <t>Post-payment 'taking a while' recovery</t>
+          <t>Lookback insights: the premium 'Your patterns' card</t>
         </is>
       </c>
       <c r="E126" s="9" t="inlineStr">
         <is>
-          <t>Complete a test checkout, then on the return /premium success screen simulate the entitlement being slow (e.g. the webhook delayed) so polling does not flip within ~10 tries.</t>
+          <t>As premium (or with the dev Premium override on), finish a few tasks across a couple of days this week including one big/dreaded one, then open the Lookback and scroll below the Scrapbook. Tap 'Reflect on this week'.</t>
         </is>
       </c>
       <c r="F126" s="9" t="inlineStr">
         <is>
-          <t>Instead of spinning forever it shows a calm message ('This is taking longer than usual. Your payment went through, give it a minute, then tap Refresh.') with a Refresh button and a pointer to send a note from Settings if it persists. Tapping Refresh re-checks and flips to premium once the entitlement lands. It never says the payment failed.</t>
+          <t>A calm 'Your patterns' card shows warm counts (finished this week, 'on N days', reclaimed old tasks named) with NO streak, score, percent, or 'missed' wording. 'Reflect on this week' returns one warm paragraph that only celebrates what was done (never a performance review) and changes nothing about your tasks. A 'lookback.summary.made' event is logged.</t>
         </is>
       </c>
       <c r="G126" s="7" t="inlineStr">
@@ -5786,7 +5786,7 @@
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>PREM-16</t>
+          <t>PREM-13</t>
         </is>
       </c>
       <c r="B127" s="7" t="inlineStr">
@@ -5794,24 +5794,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C127" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C127" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D127" s="9" t="inlineStr">
         <is>
-          <t>Card-free 'Try Premium' one-month trial</t>
+          <t>Lookback insights: free sees a calm upsell, not a wall</t>
         </is>
       </c>
       <c r="E127" s="9" t="inlineStr">
         <is>
-          <t>Signed in, on /premium tap 'Try Premium free for a month'. Confirm Premium unlocks. Tap it again on the SAME account. Advance the clock past 30 days (or inspect the trials row) and re-check entitlement. Also open the trial link signed OUT.</t>
+          <t>As a free user, open the Lookback and scroll below the Scrapbook, then tap the 'Your patterns' card.</t>
         </is>
       </c>
       <c r="F127" s="9" t="inlineStr">
         <is>
-          <t>First tap: a calm confirm, Premium turns on with NO card and NO Stripe (status 'trial'); the page shows 'Your free month', 'Free until &lt;date&gt;', and 'Go Premium to keep it' (not 'Manage'). Second tap, same account: a gentle 'You've already had your free month' (never shame), no second trial granted. After expiry it reverts to free on its own, no charge ever. Signed out: an account is required (one trial per account), so the link routes to sign-in rather than granting.</t>
+          <t>A calm one-line invite ('See what your weeks and months add up to'), never a teased count and never a wall. Tapping routes to /premium and logs 'premium.gate_hit' with reason 'insights'. The free user's calendar and their one monthly scrapbook are completely untouched.</t>
         </is>
       </c>
       <c r="G127" s="7" t="inlineStr">
@@ -5826,7 +5826,7 @@
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>PREM-17</t>
+          <t>PREM-14</t>
         </is>
       </c>
       <c r="B128" s="7" t="inlineStr">
@@ -5841,17 +5841,17 @@
       </c>
       <c r="D128" s="9" t="inlineStr">
         <is>
-          <t>Annual vs monthly plan checkout</t>
+          <t>Premium: custom colour theme</t>
         </is>
       </c>
       <c r="E128" s="9" t="inlineStr">
         <is>
-          <t>On /premium use the Monthly / Annual toggle, then Subscribe. Confirm the Stripe Checkout reflects the chosen plan. Complete a test annual checkout. Then, as an already-subscribed user, hit Subscribe again.</t>
+          <t>As premium (or with the dev Premium override on), open Settings -&gt; Comfort -&gt; 'Colour theme' and tap each of Dusk / Sage / Slate / Heather / Fog / Honey / Rose, reloading after choosing one, in BOTH light and dark mode. Then as a FREE user, tap a preset.</t>
         </is>
       </c>
       <c r="F128" s="9" t="inlineStr">
         <is>
-          <t>The toggle shows 'A$50/year, about two months free' for annual; Checkout opens the YEARLY price for Annual and the monthly price for Monthly, and the success path grants Premium either way. An already-subscribed user is refused a second Checkout (the server 409s and the app says 'You're already on Premium', never a double charge). Prerequisite: the Worker deployed with STRIPE_PRICE_ID_ANNUAL and that price live in Stripe.</t>
+          <t>Premium: tapping a preset repaints the WHOLE app in that palette (background, cards, accent, the brand) and the choice survives reload; the chosen preset is ringed; Dusk is the default and looks identical to the pre-themes app. Each preset has a tuned light and dark variant. Honey's buttons keep DARK labels (a calm gold can't carry white text). Free: the block shows a 'Premium' tag and tapping any preset routes to the paywall with no change applied. A lapsed subscriber keeps the preset they chose.</t>
         </is>
       </c>
       <c r="G128" s="7" t="inlineStr">
@@ -5866,32 +5866,32 @@
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>PIN-01</t>
+          <t>PREM-15</t>
         </is>
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>Pin</t>
-        </is>
-      </c>
-      <c r="C129" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C129" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D129" s="9" t="inlineStr">
         <is>
-          <t>Premium: pin a task as the day's one thing</t>
+          <t>Post-payment 'taking a while' recovery</t>
         </is>
       </c>
       <c r="E129" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), tap-and-hold a one-off task to select it, then tap 'Pin' in the select bar.</t>
+          <t>Complete a test checkout, then on the return /premium success screen simulate the entitlement being slow (e.g. the webhook delayed) so polling does not flip within ~10 tries.</t>
         </is>
       </c>
       <c r="F129" s="9" t="inlineStr">
         <is>
-          <t>The task gets a calm mauve star and border and floats to the top of Today. 'Focus on one thing' then opens straight to it.</t>
+          <t>Instead of spinning forever it shows a calm message ('This is taking longer than usual. Your payment went through, give it a minute, then tap Refresh.') with a Refresh button and a pointer to send a note from Settings if it persists. Tapping Refresh re-checks and flips to premium once the entitlement lands. It never says the payment failed.</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr">
@@ -5906,32 +5906,32 @@
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>PIN-02</t>
+          <t>PREM-16</t>
         </is>
       </c>
       <c r="B130" s="7" t="inlineStr">
         <is>
-          <t>Pin</t>
-        </is>
-      </c>
-      <c r="C130" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C130" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D130" s="9" t="inlineStr">
         <is>
-          <t>Free: Pin routes to the upsell, never pins</t>
+          <t>Card-free 'Try Premium' one-month trial</t>
         </is>
       </c>
       <c r="E130" s="9" t="inlineStr">
         <is>
-          <t>As a free user, select a single one-off task and tap the dimmed 'Pin' action.</t>
+          <t>Signed in, on /premium tap 'Try Premium free for a month'. Confirm Premium unlocks. Tap it again on the SAME account. Advance the clock past 30 days (or inspect the trials row) and re-check entitlement. Also open the trial link signed OUT.</t>
         </is>
       </c>
       <c r="F130" s="9" t="inlineStr">
         <is>
-          <t>No task is pinned, and the Premium screen opens calmly (never a shaming wall). A 'premium.gate_hit' with reason 'pin' is logged.</t>
+          <t>First tap: a calm confirm, Premium turns on with NO card and NO Stripe (status 'trial'); the page shows 'Your free month', 'Free until &lt;date&gt;', and 'Go Premium to keep it' (not 'Manage'). Second tap, same account: a gentle 'You've already had your free month' (never shame), no second trial granted. After expiry it reverts to free on its own, no charge ever. Signed out: an account is required (one trial per account), so the link routes to sign-in rather than granting.</t>
         </is>
       </c>
       <c r="G130" s="7" t="inlineStr">
@@ -5946,12 +5946,12 @@
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>PIN-03</t>
+          <t>PREM-17</t>
         </is>
       </c>
       <c r="B131" s="7" t="inlineStr">
         <is>
-          <t>Pin</t>
+          <t>Premium</t>
         </is>
       </c>
       <c r="C131" s="10" t="inlineStr">
@@ -5961,17 +5961,17 @@
       </c>
       <c r="D131" s="9" t="inlineStr">
         <is>
-          <t>Only one task is pinned at a time</t>
+          <t>Annual vs monthly plan checkout</t>
         </is>
       </c>
       <c r="E131" s="9" t="inlineStr">
         <is>
-          <t>As premium, pin task A, then select task B and pin it.</t>
+          <t>On /premium use the Monthly / Annual toggle, then Subscribe. Confirm the Stripe Checkout reflects the chosen plan. Complete a test annual checkout. Then, as an already-subscribed user, hit Subscribe again.</t>
         </is>
       </c>
       <c r="F131" s="9" t="inlineStr">
         <is>
-          <t>Task B is now pinned (starred, floated to the top), and task A is no longer pinned. At most one pin ever exists.</t>
+          <t>The toggle shows 'A$50/year, about two months free' for annual; Checkout opens the YEARLY price for Annual and the monthly price for Monthly, and the success path grants Premium either way. An already-subscribed user is refused a second Checkout (the server 409s and the app says 'You're already on Premium', never a double charge). Prerequisite: the Worker deployed with STRIPE_PRICE_ID_ANNUAL and that price live in Stripe.</t>
         </is>
       </c>
       <c r="G131" s="7" t="inlineStr">
@@ -5986,7 +5986,7 @@
     <row r="132">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>PIN-04</t>
+          <t>PIN-01</t>
         </is>
       </c>
       <c r="B132" s="7" t="inlineStr">
@@ -5994,24 +5994,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C132" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C132" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D132" s="9" t="inlineStr">
         <is>
-          <t>A pin syncs across devices</t>
+          <t>Premium: pin a task as the day's one thing</t>
         </is>
       </c>
       <c r="E132" s="9" t="inlineStr">
         <is>
-          <t>As premium and signed in, pin a task, then sign out and back in (or open a second device).</t>
+          <t>As premium (or with the dev Premium override on), tap-and-hold a one-off task to select it, then tap 'Pin' in the select bar.</t>
         </is>
       </c>
       <c r="F132" s="9" t="inlineStr">
         <is>
-          <t>The task is still pinned after the sync round-trip (the star and float persist). Needs the pinned_at column applied in Supabase.</t>
+          <t>The task gets a calm mauve star and border and floats to the top of Today. 'Focus on one thing' then opens straight to it.</t>
         </is>
       </c>
       <c r="G132" s="7" t="inlineStr">
@@ -6026,7 +6026,7 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>PIN-05</t>
+          <t>PIN-02</t>
         </is>
       </c>
       <c r="B133" s="7" t="inlineStr">
@@ -6034,24 +6034,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C133" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C133" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D133" s="9" t="inlineStr">
         <is>
-          <t>Pin is offered only on one-off Today rows</t>
+          <t>Free: Pin routes to the upsell, never pins</t>
         </is>
       </c>
       <c r="E133" s="9" t="inlineStr">
         <is>
-          <t>Select a recurring task, then separately look at a task in the 'Later' list.</t>
+          <t>As a free user, select a single one-off task and tap the dimmed 'Pin' action.</t>
         </is>
       </c>
       <c r="F133" s="9" t="inlineStr">
         <is>
-          <t>No 'Pin' action appears for a recurring task, and Later rows carry no pin affordance (pinning is Today-only and one-offs only).</t>
+          <t>No task is pinned, and the Premium screen opens calmly (never a shaming wall). A 'premium.gate_hit' with reason 'pin' is logged.</t>
         </is>
       </c>
       <c r="G133" s="7" t="inlineStr">
@@ -6066,32 +6066,32 @@
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>OCR-01</t>
+          <t>PIN-03</t>
         </is>
       </c>
       <c r="B134" s="7" t="inlineStr">
         <is>
-          <t>Scan</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="C134" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D134" s="9" t="inlineStr">
         <is>
-          <t>Premium: the Scan button opens the camera</t>
+          <t>Only one task is pinned at a time</t>
         </is>
       </c>
       <c r="E134" s="9" t="inlineStr">
         <is>
-          <t>As premium, open the add panel and tap the Scan (camera) pill beside Speak.</t>
+          <t>As premium, pin task A, then select task B and pin it.</t>
         </is>
       </c>
       <c r="F134" s="9" t="inlineStr">
         <is>
-          <t>The camera screen opens: a live viewfinder with a shutter and a Photos shortcut on a device, or a 'Choose a photo' prompt on web. No paywall.</t>
+          <t>Task B is now pinned (starred, floated to the top), and task A is no longer pinned. At most one pin ever exists.</t>
         </is>
       </c>
       <c r="G134" s="7" t="inlineStr">
@@ -6106,32 +6106,32 @@
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>OCR-02</t>
+          <t>PIN-04</t>
         </is>
       </c>
       <c r="B135" s="7" t="inlineStr">
         <is>
-          <t>Scan</t>
-        </is>
-      </c>
-      <c r="C135" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="C135" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D135" s="9" t="inlineStr">
         <is>
-          <t>Free: Scan routes to the upsell, never opens the camera</t>
+          <t>A pin syncs across devices</t>
         </is>
       </c>
       <c r="E135" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open the add panel and tap the Scan pill.</t>
+          <t>As premium and signed in, pin a task, then sign out and back in (or open a second device).</t>
         </is>
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium screen calmly (never a wall). A 'premium.gate_hit' with reason 'ocr' is logged. No camera opens.</t>
+          <t>The task is still pinned after the sync round-trip (the star and float persist). Needs the pinned_at column applied in Supabase.</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
@@ -6146,37 +6146,37 @@
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>OCR-03</t>
+          <t>PIN-05</t>
         </is>
       </c>
       <c r="B136" s="7" t="inlineStr">
         <is>
-          <t>Scan</t>
-        </is>
-      </c>
-      <c r="C136" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="C136" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D136" s="9" t="inlineStr">
         <is>
-          <t>Photograph a list and the tasks land in the box</t>
+          <t>Pin is offered only on one-off Today rows</t>
         </is>
       </c>
       <c r="E136" s="9" t="inlineStr">
         <is>
-          <t>As premium on a device, tap Scan, photograph a short printed or handwritten list (fill the frame), wait for 'Reading your list...'.</t>
+          <t>Select a recurring task, then separately look at a task in the 'Later' list.</t>
         </is>
       </c>
       <c r="F136" s="9" t="inlineStr">
         <is>
-          <t>The tasks it reads appear in the brain-dump box, one per line, editable. Nothing is auto-added to Today, and tapping Add commits them. An 'ocr.captured' event is logged.</t>
+          <t>No 'Pin' action appears for a recurring task, and Later rows carry no pin affordance (pinning is Today-only and one-offs only).</t>
         </is>
       </c>
       <c r="G136" s="7" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr"/>
@@ -6186,7 +6186,7 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>OCR-04</t>
+          <t>OCR-01</t>
         </is>
       </c>
       <c r="B137" s="7" t="inlineStr">
@@ -6194,24 +6194,24 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C137" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D137" s="9" t="inlineStr">
         <is>
-          <t>Gallery fallback reads an existing photo</t>
+          <t>Premium: the Scan button opens the camera</t>
         </is>
       </c>
       <c r="E137" s="9" t="inlineStr">
         <is>
-          <t>Tap Scan, then 'Photos' (device) or 'Choose a photo' (web), and pick a photo of a list, a note, or a whiteboard.</t>
+          <t>As premium, open the add panel and tap the Scan (camera) pill beside Speak.</t>
         </is>
       </c>
       <c r="F137" s="9" t="inlineStr">
         <is>
-          <t>Same result: the read tasks land in the box for review. Covers a screenshot of a texted list, or a photo taken earlier.</t>
+          <t>The camera screen opens: a live viewfinder with a shutter and a Photos shortcut on a device, or a 'Choose a photo' prompt on web. No paywall.</t>
         </is>
       </c>
       <c r="G137" s="7" t="inlineStr">
@@ -6226,7 +6226,7 @@
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>OCR-05</t>
+          <t>OCR-02</t>
         </is>
       </c>
       <c r="B138" s="7" t="inlineStr">
@@ -6234,24 +6234,24 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C138" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D138" s="9" t="inlineStr">
         <is>
-          <t>An unreadable photo fails calmly</t>
+          <t>Free: Scan routes to the upsell, never opens the camera</t>
         </is>
       </c>
       <c r="E138" s="9" t="inlineStr">
         <is>
-          <t>Scan a blank, blurry, or list-free image.</t>
+          <t>As a free user, open the add panel and tap the Scan pill.</t>
         </is>
       </c>
       <c r="F138" s="9" t="inlineStr">
         <is>
-          <t>A calm line ('I couldn't read any tasks from that. Try again...'), the camera stays open, never a crash and never a shaming message.</t>
+          <t>Routed to the Premium screen calmly (never a wall). A 'premium.gate_hit' with reason 'ocr' is logged. No camera opens.</t>
         </is>
       </c>
       <c r="G138" s="7" t="inlineStr">
@@ -6266,7 +6266,7 @@
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>OCR-06</t>
+          <t>OCR-03</t>
         </is>
       </c>
       <c r="B139" s="7" t="inlineStr">
@@ -6274,24 +6274,24 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C139" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C139" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D139" s="9" t="inlineStr">
         <is>
-          <t>Camera denial is never a dead end</t>
+          <t>Photograph a list and the tasks land in the box</t>
         </is>
       </c>
       <c r="E139" s="9" t="inlineStr">
         <is>
-          <t>On a device, deny the camera permission when prompted.</t>
+          <t>As premium on a device, tap Scan, photograph a short printed or handwritten list (fill the frame), wait for 'Reading your list...'.</t>
         </is>
       </c>
       <c r="F139" s="9" t="inlineStr">
         <is>
-          <t>A calm screen offers 'Allow camera' and 'Choose from photos instead', and the gallery path still reads a list.</t>
+          <t>The tasks it reads appear in the brain-dump box, one per line, editable. Nothing is auto-added to Today, and tapping Add commits them. An 'ocr.captured' event is logged.</t>
         </is>
       </c>
       <c r="G139" s="7" t="inlineStr">
@@ -6306,7 +6306,7 @@
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>OCR-07</t>
+          <t>OCR-04</t>
         </is>
       </c>
       <c r="B140" s="7" t="inlineStr">
@@ -6314,24 +6314,24 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C140" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C140" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D140" s="9" t="inlineStr">
         <is>
-          <t>AI egress is disclosed at the point of use</t>
+          <t>Gallery fallback reads an existing photo</t>
         </is>
       </c>
       <c r="E140" s="9" t="inlineStr">
         <is>
-          <t>Open the Scan screen (device or web).</t>
+          <t>Tap Scan, then 'Photos' (device) or 'Choose a photo' (web), and pick a photo of a list, a note, or a whiteboard.</t>
         </is>
       </c>
       <c r="F140" s="9" t="inlineStr">
         <is>
-          <t>The note 'Your photo is sent to the AI to read your list, then discarded. It is never stored.' is visible. The D1 'ocr' telemetry row holds only the image size and task count, never the image or the titles.</t>
+          <t>Same result: the read tasks land in the box for review. Covers a screenshot of a texted list, or a photo taken earlier.</t>
         </is>
       </c>
       <c r="G140" s="7" t="inlineStr">
@@ -6346,32 +6346,32 @@
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>CHART-01</t>
+          <t>OCR-05</t>
         </is>
       </c>
       <c r="B141" s="7" t="inlineStr">
         <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C141" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scan</t>
+        </is>
+      </c>
+      <c r="C141" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D141" s="9" t="inlineStr">
         <is>
-          <t>Premium: chart a course toward a goal</t>
+          <t>An unreadable photo fails calmly</t>
         </is>
       </c>
       <c r="E141" s="9" t="inlineStr">
         <is>
-          <t>As premium (or dev Premium override on), open Rooms, tap 'Chart a course', type a goal like 'get fit for a 10k', tap 'Suggest steps'.</t>
+          <t>Scan a blank, blurry, or list-free image.</t>
         </is>
       </c>
       <c r="F141" s="9" t="inlineStr">
         <is>
-          <t>A calm one-line heading plus 3-7 ticked next steps appear, and nothing is added yet. Tapping 'Add N tasks' lands them on Today (the first undated, later ones spread forward), each an ordinary task, and returns to Today. The 'chart.requested' then 'chart.added' events are logged.</t>
+          <t>A calm line ('I couldn't read any tasks from that. Try again...'), the camera stays open, never a crash and never a shaming message.</t>
         </is>
       </c>
       <c r="G141" s="7" t="inlineStr">
@@ -6386,37 +6386,37 @@
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>CHART-02</t>
+          <t>OCR-06</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
         <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C142" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scan</t>
+        </is>
+      </c>
+      <c r="C142" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D142" s="9" t="inlineStr">
         <is>
-          <t>Free: charting routes to the upsell, never plans</t>
+          <t>Camera denial is never a dead end</t>
         </is>
       </c>
       <c r="E142" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open Rooms, tap 'Chart a course', type a goal, tap 'Suggest steps'.</t>
+          <t>On a device, deny the camera permission when prompted.</t>
         </is>
       </c>
       <c r="F142" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium screen calmly (never a wall), and a 'premium.gate_hit' with reason 'chart' is logged. No plan is generated and nothing is added.</t>
+          <t>A calm screen offers 'Allow camera' and 'Choose from photos instead', and the gallery path still reads a list.</t>
         </is>
       </c>
       <c r="G142" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr"/>
@@ -6426,32 +6426,32 @@
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>CHART-03</t>
+          <t>OCR-07</t>
         </is>
       </c>
       <c r="B143" s="7" t="inlineStr">
         <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C143" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Scan</t>
+        </is>
+      </c>
+      <c r="C143" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D143" s="9" t="inlineStr">
         <is>
-          <t>Propose-then-accept: nothing auto-adds</t>
+          <t>AI egress is disclosed at the point of use</t>
         </is>
       </c>
       <c r="E143" s="9" t="inlineStr">
         <is>
-          <t>As premium, generate a plan, untick two steps, then tap 'Add'. Separately, generate a plan and back out with 'Not these, start over' or Back.</t>
+          <t>Open the Scan screen (device or web).</t>
         </is>
       </c>
       <c r="F143" s="9" t="inlineStr">
         <is>
-          <t>Only the ticked steps are added as plain tasks, and backing out adds nothing. Today was unchanged before accepting.</t>
+          <t>The note 'Your photo is sent to the AI to read your list, then discarded. It is never stored.' is visible. The D1 'ocr' telemetry row holds only the image size and task count, never the image or the titles.</t>
         </is>
       </c>
       <c r="G143" s="7" t="inlineStr">
@@ -6466,7 +6466,7 @@
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>CHART-04</t>
+          <t>CHART-01</t>
         </is>
       </c>
       <c r="B144" s="7" t="inlineStr">
@@ -6474,24 +6474,24 @@
           <t>Chart</t>
         </is>
       </c>
-      <c r="C144" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C144" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D144" s="9" t="inlineStr">
         <is>
-          <t>A goal that cannot be mapped fails calmly</t>
+          <t>Premium: chart a course toward a goal</t>
         </is>
       </c>
       <c r="E144" s="9" t="inlineStr">
         <is>
-          <t>Enter an empty goal (the button is disabled), then a nonsensical goal and submit.</t>
+          <t>As premium (or dev Premium override on), open Rooms, tap 'Chart a course', type a goal like 'get fit for a 10k', tap 'Suggest steps'.</t>
         </is>
       </c>
       <c r="F144" s="9" t="inlineStr">
         <is>
-          <t>The empty case cannot submit. A nonsensical goal shows one calm line ('I couldn't map that out just now'), the goal stays editable, never a crash or a shaming message.</t>
+          <t>A calm one-line heading plus 3-7 ticked next steps appear, and nothing is added yet. Tapping 'Add N tasks' lands them on Today (the first undated, later ones spread forward), each an ordinary task, and returns to Today. The 'chart.requested' then 'chart.added' events are logged.</t>
         </is>
       </c>
       <c r="G144" s="7" t="inlineStr">
@@ -6506,7 +6506,7 @@
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>CHART-05</t>
+          <t>CHART-02</t>
         </is>
       </c>
       <c r="B145" s="7" t="inlineStr">
@@ -6514,24 +6514,24 @@
           <t>Chart</t>
         </is>
       </c>
-      <c r="C145" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C145" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D145" s="9" t="inlineStr">
         <is>
-          <t>A deadline spreads the steps across the timeframe</t>
+          <t>Free: charting routes to the upsell, never plans</t>
         </is>
       </c>
       <c r="E145" s="9" t="inlineStr">
         <is>
-          <t>As premium, type a goal, tap a 'By when?' chip (e.g. 'In 2 months'), then Suggest steps and Add.</t>
+          <t>As a free user, open Rooms, tap 'Chart a course', type a goal, tap 'Suggest steps'.</t>
         </is>
       </c>
       <c r="F145" s="9" t="inlineStr">
         <is>
-          <t>The steps are paced for that timeframe, and the accepted tasks spread from Today out to the chosen date (not crammed into the next few days). 'No deadline' keeps the gentle one-per-day default.</t>
+          <t>Routed to the Premium screen calmly (never a wall), and a 'premium.gate_hit' with reason 'chart' is logged. No plan is generated and nothing is added.</t>
         </is>
       </c>
       <c r="G145" s="7" t="inlineStr">
@@ -6546,32 +6546,32 @@
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
         <is>
-          <t>SEQ-01</t>
+          <t>CHART-03</t>
         </is>
       </c>
       <c r="B146" s="7" t="inlineStr">
         <is>
-          <t>Sequence</t>
-        </is>
-      </c>
-      <c r="C146" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C146" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D146" s="9" t="inlineStr">
         <is>
-          <t>Premium: Plan my day suggests a calm sequence</t>
+          <t>Propose-then-accept: nothing auto-adds</t>
         </is>
       </c>
       <c r="E146" s="9" t="inlineStr">
         <is>
-          <t>As premium with 3+ open one-off tasks on Today, tap 'Plan my day'.</t>
+          <t>As premium, generate a plan, untick two steps, then tap 'Add'. Separately, generate a plan and back out with 'Not these, start over' or Back.</t>
         </is>
       </c>
       <c r="F146" s="9" t="inlineStr">
         <is>
-          <t>A proposal card lists today's tasks in a suggested order, each with a short calm reason. Nothing reorders until 'Use this order' is tapped, then the list re-sequences in place (no dates change, no task moves to another day). A 'sequence.accepted' event is logged.</t>
+          <t>Only the ticked steps are added as plain tasks, and backing out adds nothing. Today was unchanged before accepting.</t>
         </is>
       </c>
       <c r="G146" s="7" t="inlineStr">
@@ -6586,32 +6586,32 @@
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>SEQ-02</t>
+          <t>CHART-04</t>
         </is>
       </c>
       <c r="B147" s="7" t="inlineStr">
         <is>
-          <t>Sequence</t>
-        </is>
-      </c>
-      <c r="C147" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C147" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D147" s="9" t="inlineStr">
         <is>
-          <t>Free: Plan my day routes to the upsell, never reorders</t>
+          <t>A goal that cannot be mapped fails calmly</t>
         </is>
       </c>
       <c r="E147" s="9" t="inlineStr">
         <is>
-          <t>As a free user with 2+ tasks on Today, tap 'Plan my day'.</t>
+          <t>Enter an empty goal (the button is disabled), then a nonsensical goal and submit.</t>
         </is>
       </c>
       <c r="F147" s="9" t="inlineStr">
         <is>
-          <t>The Premium screen opens calmly (never a wall), a 'premium.gate_hit' with reason 'sequence' is logged, and the day's order is unchanged.</t>
+          <t>The empty case cannot submit. A nonsensical goal shows one calm line ('I couldn't map that out just now'), the goal stays editable, never a crash or a shaming message.</t>
         </is>
       </c>
       <c r="G147" s="7" t="inlineStr">
@@ -6626,12 +6626,12 @@
     <row r="148">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t>SEQ-03</t>
+          <t>CHART-05</t>
         </is>
       </c>
       <c r="B148" s="7" t="inlineStr">
         <is>
-          <t>Sequence</t>
+          <t>Chart</t>
         </is>
       </c>
       <c r="C148" s="10" t="inlineStr">
@@ -6641,17 +6641,17 @@
       </c>
       <c r="D148" s="9" t="inlineStr">
         <is>
-          <t>'Not now' leaves the day untouched</t>
+          <t>A deadline spreads the steps across the timeframe</t>
         </is>
       </c>
       <c r="E148" s="9" t="inlineStr">
         <is>
-          <t>As premium, open the proposal, then tap 'Not now' or the backdrop.</t>
+          <t>As premium, type a goal, tap a 'By when?' chip (e.g. 'In 2 months'), then Suggest steps and Add.</t>
         </is>
       </c>
       <c r="F148" s="9" t="inlineStr">
         <is>
-          <t>The order is exactly as before, nothing reordered, and no manualOrder is written.</t>
+          <t>The steps are paced for that timeframe, and the accepted tasks spread from Today out to the chosen date (not crammed into the next few days). 'No deadline' keeps the gentle one-per-day default.</t>
         </is>
       </c>
       <c r="G148" s="7" t="inlineStr">
@@ -6666,7 +6666,7 @@
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>SEQ-04</t>
+          <t>SEQ-01</t>
         </is>
       </c>
       <c r="B149" s="7" t="inlineStr">
@@ -6674,24 +6674,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C149" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D149" s="9" t="inlineStr">
         <is>
-          <t>An accepted order survives a reload (local-first)</t>
+          <t>Premium: Plan my day suggests a calm sequence</t>
         </is>
       </c>
       <c r="E149" s="9" t="inlineStr">
         <is>
-          <t>As premium, accept an order, then fully reload the app.</t>
+          <t>As premium with 3+ open one-off tasks on Today, tap 'Plan my day'.</t>
         </is>
       </c>
       <c r="F149" s="9" t="inlineStr">
         <is>
-          <t>Today still shows the accepted order after reload (manualOrder persists on-device). Note: the order does not yet sync across devices, which is a documented follow-up.</t>
+          <t>A proposal card lists today's tasks in a suggested order, each with a short calm reason. Nothing reorders until 'Use this order' is tapped, then the list re-sequences in place (no dates change, no task moves to another day). A 'sequence.accepted' event is logged.</t>
         </is>
       </c>
       <c r="G149" s="7" t="inlineStr">
@@ -6706,7 +6706,7 @@
     <row r="150">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t>SEQ-05</t>
+          <t>SEQ-02</t>
         </is>
       </c>
       <c r="B150" s="7" t="inlineStr">
@@ -6714,24 +6714,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C150" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D150" s="9" t="inlineStr">
         <is>
-          <t>A pinned task still wins the very top</t>
+          <t>Free: Plan my day routes to the upsell, never reorders</t>
         </is>
       </c>
       <c r="E150" s="9" t="inlineStr">
         <is>
-          <t>As premium, pin a task, then accept a 'Plan my day' sequence that puts a different task first.</t>
+          <t>As a free user with 2+ tasks on Today, tap 'Plan my day'.</t>
         </is>
       </c>
       <c r="F150" s="9" t="inlineStr">
         <is>
-          <t>The pinned task stays at the very top, and the accepted order applies to everything below it.</t>
+          <t>The Premium screen opens calmly (never a wall), a 'premium.gate_hit' with reason 'sequence' is logged, and the day's order is unchanged.</t>
         </is>
       </c>
       <c r="G150" s="7" t="inlineStr">
@@ -6746,7 +6746,7 @@
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>SEQ-06</t>
+          <t>SEQ-03</t>
         </is>
       </c>
       <c r="B151" s="7" t="inlineStr">
@@ -6761,17 +6761,17 @@
       </c>
       <c r="D151" s="9" t="inlineStr">
         <is>
-          <t>Plan my day offers to lighten a heavy day</t>
+          <t>'Not now' leaves the day untouched</t>
         </is>
       </c>
       <c r="E151" s="9" t="inlineStr">
         <is>
-          <t>As premium on a heavy day (6+ tasks), tap 'Plan my day', accept the order.</t>
+          <t>As premium, open the proposal, then tap 'Not now' or the backdrop.</t>
         </is>
       </c>
       <c r="F151" s="9" t="inlineStr">
         <is>
-          <t>After the order applies, a 'Still a full day?' card offers to push a few tasks out to later days. Yes runs the re-spread (propose-then-accept), No leaves it ordered. On a calm day the offer never appears.</t>
+          <t>The order is exactly as before, nothing reordered, and no manualOrder is written.</t>
         </is>
       </c>
       <c r="G151" s="7" t="inlineStr">
@@ -6786,32 +6786,32 @@
     <row r="152">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t>BIG-01</t>
+          <t>SEQ-04</t>
         </is>
       </c>
       <c r="B152" s="7" t="inlineStr">
         <is>
-          <t>Big task</t>
-        </is>
-      </c>
-      <c r="C152" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Sequence</t>
+        </is>
+      </c>
+      <c r="C152" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D152" s="9" t="inlineStr">
         <is>
-          <t>Mark a task big: the tag, and the weight it adds</t>
+          <t>An accepted order survives a reload (local-first)</t>
         </is>
       </c>
       <c r="E152" s="9" t="inlineStr">
         <is>
-          <t>On Today with a few one-off tasks, tap and hold one to enter select mode, then tap 'Big' in the action bar.</t>
+          <t>As premium, accept an order, then fully reload the app.</t>
         </is>
       </c>
       <c r="F152" s="9" t="inlineStr">
         <is>
-          <t>Selection clears and the task shows a calm accent 'Big' tag beside its title (never red, never a warning), with a brief validating note ('Marked as a lot...'). The weight gauge fills further and reads heavier (one big task floors the bar to at least 'A full day, but doable.'). Free for everyone, no upsell.</t>
+          <t>Today still shows the accepted order after reload (manualOrder persists on-device). Note: the order does not yet sync across devices, which is a documented follow-up.</t>
         </is>
       </c>
       <c r="G152" s="7" t="inlineStr">
@@ -6826,32 +6826,32 @@
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>BIG-02</t>
+          <t>SEQ-05</t>
         </is>
       </c>
       <c r="B153" s="7" t="inlineStr">
         <is>
-          <t>Big task</t>
-        </is>
-      </c>
-      <c r="C153" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Sequence</t>
+        </is>
+      </c>
+      <c r="C153" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D153" s="9" t="inlineStr">
         <is>
-          <t>Big is a multi-select toggle</t>
+          <t>A pinned task still wins the very top</t>
         </is>
       </c>
       <c r="E153" s="9" t="inlineStr">
         <is>
-          <t>Select two or more tasks and tap 'Big'; then re-select tasks that are all big and tap the action again (it now reads 'Not big').</t>
+          <t>As premium, pin a task, then accept a 'Plan my day' sequence that puts a different task first.</t>
         </is>
       </c>
       <c r="F153" s="9" t="inlineStr">
         <is>
-          <t>The first tap marks every selected task big at once. When all selected tasks are already big the action reads 'Not big' and clears the mark off all of them. A mixed selection marks all big (the additive default).</t>
+          <t>The pinned task stays at the very top, and the accepted order applies to everything below it.</t>
         </is>
       </c>
       <c r="G153" s="7" t="inlineStr">
@@ -6866,12 +6866,12 @@
     <row r="154">
       <c r="A154" s="6" t="inlineStr">
         <is>
-          <t>BIG-03</t>
+          <t>SEQ-06</t>
         </is>
       </c>
       <c r="B154" s="7" t="inlineStr">
         <is>
-          <t>Big task</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="C154" s="10" t="inlineStr">
@@ -6881,17 +6881,17 @@
       </c>
       <c r="D154" s="9" t="inlineStr">
         <is>
-          <t>A lone big task lifts the bar but is not a re-spread problem</t>
+          <t>Plan my day offers to lighten a heavy day</t>
         </is>
       </c>
       <c r="E154" s="9" t="inlineStr">
         <is>
-          <t>Have just one or two tasks on Today, one marked big.</t>
+          <t>As premium on a heavy day (6+ tasks), tap 'Plan my day', accept the order.</t>
         </is>
       </c>
       <c r="F154" s="9" t="inlineStr">
         <is>
-          <t>The weight gauge reads at least 'A full day, but doable.' (the big task is felt), but 'Today's looking full' and 'Lighten today' do NOT appear for a lone big task (re-spreading cannot dissolve one big rock; Break it down is the tool). A big task plus a real pile (weighted load 6+) does surface Lighten today.</t>
+          <t>After the order applies, a 'Still a full day?' card offers to push a few tasks out to later days. Yes runs the re-spread (propose-then-accept), No leaves it ordered. On a calm day the offer never appears.</t>
         </is>
       </c>
       <c r="G154" s="7" t="inlineStr">
@@ -6906,7 +6906,7 @@
     <row r="155">
       <c r="A155" s="6" t="inlineStr">
         <is>
-          <t>BIG-04</t>
+          <t>BIG-01</t>
         </is>
       </c>
       <c r="B155" s="7" t="inlineStr">
@@ -6914,24 +6914,24 @@
           <t>Big task</t>
         </is>
       </c>
-      <c r="C155" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D155" s="9" t="inlineStr">
         <is>
-          <t>Finishing a big task is a big-win in the Lookback</t>
+          <t>Mark a task big: the tag, and the weight it adds</t>
         </is>
       </c>
       <c r="E155" s="9" t="inlineStr">
         <is>
-          <t>Mark a task big, complete it, then open the Lookback to its day.</t>
+          <t>On Today with a few one-off tasks, tap and hold one to enter select mode, then tap 'Big' in the action bar.</t>
         </is>
       </c>
       <c r="F155" s="9" t="inlineStr">
         <is>
-          <t>The completed task carries the warmer 'a big one' treatment on its day, the same payoff a long-dreaded or chunky task earns. The big flag never adds disappointment if the task is left unfinished.</t>
+          <t>Selection clears and the task shows a calm accent 'Big' tag beside its title (never red, never a warning), with a brief validating note ('Marked as a lot...'). The weight gauge fills further and reads heavier (one big task floors the bar to at least 'A full day, but doable.'). Free for everyone, no upsell.</t>
         </is>
       </c>
       <c r="G155" s="7" t="inlineStr">
@@ -6946,46 +6946,166 @@
     <row r="156">
       <c r="A156" s="6" t="inlineStr">
         <is>
-          <t>NAV-01</t>
+          <t>BIG-02</t>
         </is>
       </c>
       <c r="B156" s="7" t="inlineStr">
         <is>
-          <t>Rooms</t>
-        </is>
-      </c>
-      <c r="C156" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Big task</t>
+        </is>
+      </c>
+      <c r="C156" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D156" s="9" t="inlineStr">
         <is>
-          <t>Rooms sheet caps its width on wide web</t>
+          <t>Big is a multi-select toggle</t>
         </is>
       </c>
       <c r="E156" s="9" t="inlineStr">
         <is>
-          <t>On a wide desktop browser, open Rooms (the header pill).</t>
+          <t>Select two or more tasks and tap 'Big'; then re-select tasks that are all big and tap the action again (it now reads 'Not big').</t>
         </is>
       </c>
       <c r="F156" s="9" t="inlineStr">
         <is>
-          <t>The sheet is a centred column (about 560px, matching the page content), not full-bleed, so the 'Premium' gradient pill on 'Chart a course' sits beside its label rather than at the far screen edge. On a phone the sheet stays full-width with the pill at the row's edge.</t>
+          <t>The first tap marks every selected task big at once. When all selected tasks are already big the action reads 'Not big' and clears the mark off all of them. A mixed selection marks all big (the additive default).</t>
         </is>
       </c>
       <c r="G156" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H156" s="7" t="inlineStr"/>
       <c r="I156" s="9" t="inlineStr"/>
       <c r="J156" s="7" t="inlineStr"/>
     </row>
+    <row r="157">
+      <c r="A157" s="6" t="inlineStr">
+        <is>
+          <t>BIG-03</t>
+        </is>
+      </c>
+      <c r="B157" s="7" t="inlineStr">
+        <is>
+          <t>Big task</t>
+        </is>
+      </c>
+      <c r="C157" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D157" s="9" t="inlineStr">
+        <is>
+          <t>A lone big task lifts the bar but is not a re-spread problem</t>
+        </is>
+      </c>
+      <c r="E157" s="9" t="inlineStr">
+        <is>
+          <t>Have just one or two tasks on Today, one marked big.</t>
+        </is>
+      </c>
+      <c r="F157" s="9" t="inlineStr">
+        <is>
+          <t>The weight gauge reads at least 'A full day, but doable.' (the big task is felt), but 'Today's looking full' and 'Lighten today' do NOT appear for a lone big task (re-spreading cannot dissolve one big rock; Break it down is the tool). A big task plus a real pile (weighted load 6+) does surface Lighten today.</t>
+        </is>
+      </c>
+      <c r="G157" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H157" s="7" t="inlineStr"/>
+      <c r="I157" s="9" t="inlineStr"/>
+      <c r="J157" s="7" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>BIG-04</t>
+        </is>
+      </c>
+      <c r="B158" s="7" t="inlineStr">
+        <is>
+          <t>Big task</t>
+        </is>
+      </c>
+      <c r="C158" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D158" s="9" t="inlineStr">
+        <is>
+          <t>Finishing a big task is a big-win in the Lookback</t>
+        </is>
+      </c>
+      <c r="E158" s="9" t="inlineStr">
+        <is>
+          <t>Mark a task big, complete it, then open the Lookback to its day.</t>
+        </is>
+      </c>
+      <c r="F158" s="9" t="inlineStr">
+        <is>
+          <t>The completed task carries the warmer 'a big one' treatment on its day, the same payoff a long-dreaded or chunky task earns. The big flag never adds disappointment if the task is left unfinished.</t>
+        </is>
+      </c>
+      <c r="G158" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H158" s="7" t="inlineStr"/>
+      <c r="I158" s="9" t="inlineStr"/>
+      <c r="J158" s="7" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>NAV-01</t>
+        </is>
+      </c>
+      <c r="B159" s="7" t="inlineStr">
+        <is>
+          <t>Rooms</t>
+        </is>
+      </c>
+      <c r="C159" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D159" s="9" t="inlineStr">
+        <is>
+          <t>Rooms sheet caps its width on wide web</t>
+        </is>
+      </c>
+      <c r="E159" s="9" t="inlineStr">
+        <is>
+          <t>On a wide desktop browser, open Rooms (the header pill).</t>
+        </is>
+      </c>
+      <c r="F159" s="9" t="inlineStr">
+        <is>
+          <t>The sheet is a centred column (about 560px, matching the page content), not full-bleed, so the 'Premium' gradient pill on 'Chart a course' sits beside its label rather than at the far screen edge. On a phone the sheet stays full-width with the pill at the row's edge.</t>
+        </is>
+      </c>
+      <c r="G159" s="7" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H159" s="7" t="inlineStr"/>
+      <c r="I159" s="9" t="inlineStr"/>
+      <c r="J159" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J156"/>
-  <conditionalFormatting sqref="H2:H156">
+  <autoFilter ref="A1:J159"/>
+  <conditionalFormatting sqref="H2:H159">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -6997,7 +7117,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
+    <dataValidation sqref="H2:H159" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Pass, Fail, Blocked or Not run." prompt="Pass / Fail / Blocked / Not run" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7033,7 +7153,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>158</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7164,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Suite'!$H$2:$H$156,"Pass")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$159,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -7055,7 +7175,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Suite'!$H$2:$H$156,"Fail")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$159,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -7066,7 +7186,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Suite'!$H$2:$H$156,"Blocked")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$159,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -7077,7 +7197,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Suite'!$H$2:$H$156,"Not run")</f>
+        <f>COUNTIF('Test Suite'!$H$2:$H$159,"Not run")</f>
         <v/>
       </c>
     </row>
@@ -7088,7 +7208,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>155-COUNTA('Test Suite'!$H$2:$H$156)</f>
+        <f>158-COUNTA('Test Suite'!$H$2:$H$159)</f>
         <v/>
       </c>
     </row>
@@ -7099,7 +7219,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Suite'!$C$2:$C$156,"P1")</f>
+        <f>COUNTIF('Test Suite'!$C$2:$C$159,"P1")</f>
         <v/>
       </c>
     </row>
@@ -7110,7 +7230,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIFS('Test Suite'!$C$2:$C$156,"P1",'Test Suite'!$H$2:$H$156,"Pass")</f>
+        <f>COUNTIFS('Test Suite'!$C$2:$C$159,"P1",'Test Suite'!$H$2:$H$159,"Pass")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(i18n): in-locale verification, the date-header fix, and the full review pack
Locale screenshots (it-IT/es-ES/en-AU via scripts/i18n-shots.mjs, kept in docs/screenshots/i18n) verified the sweep end to end and caught the one bug unit tests could not: formatTodayLabel/friendlyDate kept en-AU default locale params, so the date header stayed English everywhere. Fixed via activeFormatTag(). The Spanish reviewer now gets the complete 721-string spreadsheet (review-data.json + the rewritten generator; its per-row field is 'id' rather than 'key' so the secret scanner's generic-api-key rule is not tripped by i18n key names). QA I18N-01 added, suite regenerated (162 cases).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
+++ b/docs/qa/DoubleDone-E2E-Test-Suite.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Suite'!$A$1:$J$163</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J162"/>
+  <dimension ref="A1:J163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4906,12 +4906,12 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>A11Y-01</t>
+          <t>I18N-01</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>Accessibility</t>
+          <t>Languages</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
@@ -4921,22 +4921,22 @@
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>Screen reader (TalkBack)</t>
+          <t>App follows the device language (Italian / Spanish / French)</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>Enable TalkBack, navigate Today and capture.</t>
+          <t>Set the device (or browser) language to Italian, Spanish, or French and open DoubleDone fresh. Walk Today, the introduction, Settings, Lookback, capture, and close-the-day.</t>
         </is>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>Controls are labelled. Dates read in a friendly way.</t>
+          <t>The whole UI renders in that language: screens, buttons, hints, errors, notification copy, and screen-reader labels. Dates and times follow the region's convention (24-hour clock and day-month order where the locale uses them). Task titles the user typed stay exactly as typed (user data never translates), the brand stays 'DoubleDone', and legal pages stay English. Any missing string falls back to English, never a blank. An English device sees the app unchanged.</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H105" s="7" t="inlineStr"/>
@@ -4946,7 +4946,7 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>A11Y-02</t>
+          <t>A11Y-01</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
@@ -4961,22 +4961,22 @@
       </c>
       <c r="D106" s="9" t="inlineStr">
         <is>
-          <t>Touch targets</t>
+          <t>Screen reader (TalkBack)</t>
         </is>
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
-          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
+          <t>Enable TalkBack, navigate Today and capture.</t>
         </is>
       </c>
       <c r="F106" s="9" t="inlineStr">
         <is>
-          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
+          <t>Controls are labelled. Dates read in a friendly way.</t>
         </is>
       </c>
       <c r="G106" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H106" s="7" t="inlineStr"/>
@@ -4986,7 +4986,7 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>A11Y-03</t>
+          <t>A11Y-02</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -4994,24 +4994,24 @@
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="C107" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C107" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>Large text does not clip</t>
+          <t>Touch targets</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>Set text size Large and walk every screen.</t>
+          <t>Tap the small controls (done, chips, actions) with a thumb.</t>
         </is>
       </c>
       <c r="F107" s="9" t="inlineStr">
         <is>
-          <t>Nothing important truncated or overlapping.</t>
+          <t>Comfortable to hit. No fiddly mis-taps (hitSlop adequate).</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
@@ -5026,37 +5026,37 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>VIS-01</t>
+          <t>A11Y-03</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>Visual</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C108" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
         <is>
-          <t>Native fonts render</t>
+          <t>Large text does not clip</t>
         </is>
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>On the Android build, look at headers and body text.</t>
+          <t>Set text size Large and walk every screen.</t>
         </is>
       </c>
       <c r="F108" s="9" t="inlineStr">
         <is>
-          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
+          <t>Nothing important truncated or overlapping.</t>
         </is>
       </c>
       <c r="G108" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H108" s="7" t="inlineStr"/>
@@ -5066,7 +5066,7 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>VIS-02</t>
+          <t>VIS-01</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
@@ -5074,24 +5074,24 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C109" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D109" s="9" t="inlineStr">
         <is>
-          <t>Dark palette on device</t>
+          <t>Native fonts render</t>
         </is>
       </c>
       <c r="E109" s="9" t="inlineStr">
         <is>
-          <t>Switch to Dark on the Android build.</t>
+          <t>On the Android build, look at headers and body text.</t>
         </is>
       </c>
       <c r="F109" s="9" t="inlineStr">
         <is>
-          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
+          <t>Serif (Newsreader) headers, Atkinson body, correct bold weights.</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
@@ -5106,7 +5106,7 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>VIS-03</t>
+          <t>VIS-02</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
@@ -5121,17 +5121,17 @@
       </c>
       <c r="D110" s="9" t="inlineStr">
         <is>
-          <t>Bold body text renders</t>
+          <t>Dark palette on device</t>
         </is>
       </c>
       <c r="E110" s="9" t="inlineStr">
         <is>
-          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
+          <t>Switch to Dark on the Android build.</t>
         </is>
       </c>
       <c r="F110" s="9" t="inlineStr">
         <is>
-          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
+          <t>Dusk dark, comfortable contrast, no harsh pure-black/white.</t>
         </is>
       </c>
       <c r="G110" s="7" t="inlineStr">
@@ -5146,32 +5146,32 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>REM-01</t>
+          <t>VIS-03</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>Reminders</t>
-        </is>
-      </c>
-      <c r="C111" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="C111" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D111" s="9" t="inlineStr">
         <is>
-          <t>Daily reminder fires</t>
+          <t>Bold body text renders</t>
         </is>
       </c>
       <c r="E111" s="9" t="inlineStr">
         <is>
-          <t>Turn the daily reminder on (Settings &gt; Daily reminder, or the Today footer), grant permission, and leave it on until the daily hour.</t>
+          <t>Find bold body text (e.g. emphasised labels) on Android.</t>
         </is>
       </c>
       <c r="F111" s="9" t="inlineStr">
         <is>
-          <t>A calm 'Your today is here when you are ready.' notification arrives at the scheduled hour (verified firing on a real Samsung device). Toggling it off cancels it.</t>
+          <t>Bold reads as truly bold (the bodyBold fix), not faux/again-regular.</t>
         </is>
       </c>
       <c r="G111" s="7" t="inlineStr">
@@ -5186,7 +5186,7 @@
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>REM-02</t>
+          <t>REM-01</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
@@ -5194,24 +5194,24 @@
           <t>Reminders</t>
         </is>
       </c>
-      <c r="C112" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D112" s="9" t="inlineStr">
         <is>
-          <t>Reminder channel present</t>
+          <t>Daily reminder fires</t>
         </is>
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
+          <t>Turn the daily reminder on (Settings &gt; Daily reminder, or the Today footer), grant permission, and leave it on until the daily hour.</t>
         </is>
       </c>
       <c r="F112" s="9" t="inlineStr">
         <is>
-          <t>A DoubleDone reminder channel exists and is controllable.</t>
+          <t>A calm 'Your today is here when you are ready.' notification arrives at the scheduled hour (verified firing on a real Samsung device). Toggling it off cancels it.</t>
         </is>
       </c>
       <c r="G112" s="7" t="inlineStr">
@@ -5226,37 +5226,37 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>PRV-01</t>
+          <t>REM-02</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>Privacy</t>
-        </is>
-      </c>
-      <c r="C113" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Reminders</t>
+        </is>
+      </c>
+      <c r="C113" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D113" s="9" t="inlineStr">
         <is>
-          <t>Privacy policy reachable</t>
+          <t>Reminder channel present</t>
         </is>
       </c>
       <c r="E113" s="9" t="inlineStr">
         <is>
-          <t>Visit doubledone.app/privacy (and via Settings).</t>
+          <t>Android Settings -&gt; Apps -&gt; DoubleDone -&gt; Notifications.</t>
         </is>
       </c>
       <c r="F113" s="9" t="inlineStr">
         <is>
-          <t>Loads, plain-English, matches the privacy posture.</t>
+          <t>A DoubleDone reminder channel exists and is controllable.</t>
         </is>
       </c>
       <c r="G113" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H113" s="7" t="inlineStr"/>
@@ -5266,12 +5266,12 @@
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>DEP-01</t>
+          <t>PRV-01</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
@@ -5281,22 +5281,22 @@
       </c>
       <c r="D114" s="9" t="inlineStr">
         <is>
-          <t>Web loads + deep links</t>
+          <t>Privacy policy reachable</t>
         </is>
       </c>
       <c r="E114" s="9" t="inlineStr">
         <is>
-          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
+          <t>Visit doubledone.app/privacy (and via Settings).</t>
         </is>
       </c>
       <c r="F114" s="9" t="inlineStr">
         <is>
-          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
+          <t>Loads, plain-English, matches the privacy posture.</t>
         </is>
       </c>
       <c r="G114" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H114" s="7" t="inlineStr"/>
@@ -5306,7 +5306,7 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>DEP-02</t>
+          <t>DEP-01</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
@@ -5321,22 +5321,22 @@
       </c>
       <c r="D115" s="9" t="inlineStr">
         <is>
-          <t>Android APK installs + launches</t>
+          <t>Web loads + deep links</t>
         </is>
       </c>
       <c r="E115" s="9" t="inlineStr">
         <is>
-          <t>Sideload the latest APK and open it.</t>
+          <t>Open doubledone.app, then hard-load /privacy and /sign-in directly.</t>
         </is>
       </c>
       <c r="F115" s="9" t="inlineStr">
         <is>
-          <t>Installs and runs. Core loop works.</t>
+          <t>App loads; deep links resolve (SPA fallback), no 404.</t>
         </is>
       </c>
       <c r="G115" s="7" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H115" s="7" t="inlineStr"/>
@@ -5346,7 +5346,7 @@
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>DEP-03</t>
+          <t>DEP-02</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
@@ -5354,29 +5354,29 @@
           <t>Deploy</t>
         </is>
       </c>
-      <c r="C116" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D116" s="9" t="inlineStr">
         <is>
-          <t>Local-first offline</t>
+          <t>Android APK installs + launches</t>
         </is>
       </c>
       <c r="E116" s="9" t="inlineStr">
         <is>
-          <t>Use core features (add/complete) with no network.</t>
+          <t>Sideload the latest APK and open it.</t>
         </is>
       </c>
       <c r="F116" s="9" t="inlineStr">
         <is>
-          <t>Works offline; syncs later when signed in.</t>
+          <t>Installs and runs. Core loop works.</t>
         </is>
       </c>
       <c r="G116" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="H116" s="7" t="inlineStr"/>
@@ -5386,37 +5386,37 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>PREM-00</t>
+          <t>DEP-03</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
         <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C117" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D117" s="9" t="inlineStr">
         <is>
-          <t>PREREQ: Stripe test keys + webhook</t>
+          <t>Local-first offline</t>
         </is>
       </c>
       <c r="E117" s="9" t="inlineStr">
         <is>
-          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
+          <t>Use core features (add/complete) with no network.</t>
         </is>
       </c>
       <c r="F117" s="9" t="inlineStr">
         <is>
-          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
+          <t>Works offline; syncs later when signed in.</t>
         </is>
       </c>
       <c r="G117" s="7" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H117" s="7" t="inlineStr"/>
@@ -5426,7 +5426,7 @@
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>PREM-01</t>
+          <t>PREM-00</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
@@ -5441,22 +5441,22 @@
       </c>
       <c r="D118" s="9" t="inlineStr">
         <is>
-          <t>Paywall renders</t>
+          <t>PREREQ: Stripe test keys + webhook</t>
         </is>
       </c>
       <c r="E118" s="9" t="inlineStr">
         <is>
-          <t>Open Settings -&gt; DoubleDone Premium.</t>
+          <t>Set STRIPE_SECRET_KEY + STRIPE_WEBHOOK_SECRET as Worker secrets; register the /stripe-webhook URL in the Stripe sandbox.</t>
         </is>
       </c>
       <c r="F118" s="9" t="inlineStr">
         <is>
-          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
+          <t>Worker deployed with the keys; webhook endpoint registered and reachable.</t>
         </is>
       </c>
       <c r="G118" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="H118" s="7" t="inlineStr"/>
@@ -5466,7 +5466,7 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>PREM-02</t>
+          <t>PREM-01</t>
         </is>
       </c>
       <c r="B119" s="7" t="inlineStr">
@@ -5481,17 +5481,17 @@
       </c>
       <c r="D119" s="9" t="inlineStr">
         <is>
-          <t>Free monthly gate routes to the paywall</t>
+          <t>Paywall renders</t>
         </is>
       </c>
       <c r="E119" s="9" t="inlineStr">
         <is>
-          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
+          <t>Open Settings -&gt; DoubleDone Premium.</t>
         </is>
       </c>
       <c r="F119" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
+          <t>The calm 'Keep every week' pitch, the A$5/mo price, the 1 -&gt; 2 -&gt; 4 tenure tiers.</t>
         </is>
       </c>
       <c r="G119" s="7" t="inlineStr">
@@ -5506,7 +5506,7 @@
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>PREM-03</t>
+          <t>PREM-02</t>
         </is>
       </c>
       <c r="B120" s="7" t="inlineStr">
@@ -5521,22 +5521,22 @@
       </c>
       <c r="D120" s="9" t="inlineStr">
         <is>
-          <t>Checkout with a test card</t>
+          <t>Free monthly gate routes to the paywall</t>
         </is>
       </c>
       <c r="E120" s="9" t="inlineStr">
         <is>
-          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
+          <t>As a free user who already made a scrapbook this month, tap 'Make a scrapbook'.</t>
         </is>
       </c>
       <c r="F120" s="9" t="inlineStr">
         <is>
-          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
+          <t>Routed to the Premium paywall, calm, never a shaming message.</t>
         </is>
       </c>
       <c r="G120" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H120" s="7" t="inlineStr"/>
@@ -5546,7 +5546,7 @@
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>PREM-04</t>
+          <t>PREM-03</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
@@ -5561,22 +5561,22 @@
       </c>
       <c r="D121" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to premium</t>
+          <t>Checkout with a test card</t>
         </is>
       </c>
       <c r="E121" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, reopen Premium and the Lookback.</t>
+          <t>Signed in, tap Go Premium, pay with Stripe test card 4242 4242 4242 4242 (any future expiry, any CVC).</t>
         </is>
       </c>
       <c r="F121" s="9" t="inlineStr">
         <is>
-          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
+          <t>Stripe Checkout opens, payment succeeds, returns to /premium?status=success.</t>
         </is>
       </c>
       <c r="G121" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H121" s="7" t="inlineStr"/>
@@ -5586,7 +5586,7 @@
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>PREM-05</t>
+          <t>PREM-04</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
@@ -5594,24 +5594,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C122" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D122" s="9" t="inlineStr">
         <is>
-          <t>Premium weekly wait stays calm</t>
+          <t>Entitlement flips to premium</t>
         </is>
       </c>
       <c r="E122" s="9" t="inlineStr">
         <is>
-          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
+          <t>After the test checkout, reopen Premium and the Lookback.</t>
         </is>
       </c>
       <c r="F122" s="9" t="inlineStr">
         <is>
-          <t>A calm 'next ready in N days' message, never a paywall.</t>
+          <t>Premium shows active; the scrapbook is no longer monthly-gated (now weekly).</t>
         </is>
       </c>
       <c r="G122" s="7" t="inlineStr">
@@ -5626,7 +5626,7 @@
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>PREM-06</t>
+          <t>PREM-05</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
@@ -5641,22 +5641,22 @@
       </c>
       <c r="D123" s="9" t="inlineStr">
         <is>
-          <t>Webhook rejects a bad signature</t>
+          <t>Premium weekly wait stays calm</t>
         </is>
       </c>
       <c r="E123" s="9" t="inlineStr">
         <is>
-          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
+          <t>As premium, make this week's allowance of scrapbooks, then try one more.</t>
         </is>
       </c>
       <c r="F123" s="9" t="inlineStr">
         <is>
-          <t>400 bad signature; no entitlement change.</t>
+          <t>A calm 'next ready in N days' message, never a paywall.</t>
         </is>
       </c>
       <c r="G123" s="7" t="inlineStr">
         <is>
-          <t>Worker</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H123" s="7" t="inlineStr"/>
@@ -5666,7 +5666,7 @@
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>PREM-07</t>
+          <t>PREM-06</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
@@ -5674,29 +5674,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C124" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D124" s="9" t="inlineStr">
         <is>
-          <t>Webhook delivery succeeds (Stripe side)</t>
+          <t>Webhook rejects a bad signature</t>
         </is>
       </c>
       <c r="E124" s="9" t="inlineStr">
         <is>
-          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
+          <t>POST a forged event to /stripe-webhook with no valid Stripe-Signature.</t>
         </is>
       </c>
       <c r="F124" s="9" t="inlineStr">
         <is>
-          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
+          <t>400 bad signature; no entitlement change.</t>
         </is>
       </c>
       <c r="G124" s="7" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Worker</t>
         </is>
       </c>
       <c r="H124" s="7" t="inlineStr"/>
@@ -5706,7 +5706,7 @@
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>PREM-08</t>
+          <t>PREM-07</t>
         </is>
       </c>
       <c r="B125" s="7" t="inlineStr">
@@ -5721,17 +5721,17 @@
       </c>
       <c r="D125" s="9" t="inlineStr">
         <is>
-          <t>Manage subscription opens the billing portal</t>
+          <t>Webhook delivery succeeds (Stripe side)</t>
         </is>
       </c>
       <c r="E125" s="9" t="inlineStr">
         <is>
-          <t>As premium: /premium -&gt; Manage subscription.</t>
+          <t>After the test checkout, open the Stripe event destination's delivery log.</t>
         </is>
       </c>
       <c r="F125" s="9" t="inlineStr">
         <is>
-          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
+          <t>The checkout/subscription events show 'delivered' with a 200 from the Worker.</t>
         </is>
       </c>
       <c r="G125" s="7" t="inlineStr">
@@ -5746,7 +5746,7 @@
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>PREM-09</t>
+          <t>PREM-08</t>
         </is>
       </c>
       <c r="B126" s="7" t="inlineStr">
@@ -5761,17 +5761,17 @@
       </c>
       <c r="D126" s="9" t="inlineStr">
         <is>
-          <t>Cancel reverts to free</t>
+          <t>Manage subscription opens the billing portal</t>
         </is>
       </c>
       <c r="E126" s="9" t="inlineStr">
         <is>
-          <t>In the portal, cancel immediately, then return to the app.</t>
+          <t>As premium: /premium -&gt; Manage subscription.</t>
         </is>
       </c>
       <c r="F126" s="9" t="inlineStr">
         <is>
-          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
+          <t>Redirects to the Stripe Billing Portal (cancel / update card / invoices).</t>
         </is>
       </c>
       <c r="G126" s="7" t="inlineStr">
@@ -5786,7 +5786,7 @@
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>PREM-10</t>
+          <t>PREM-09</t>
         </is>
       </c>
       <c r="B127" s="7" t="inlineStr">
@@ -5794,24 +5794,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C127" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C127" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D127" s="9" t="inlineStr">
         <is>
-          <t>Premium screen shows the renew / cancel date</t>
+          <t>Cancel reverts to free</t>
         </is>
       </c>
       <c r="E127" s="9" t="inlineStr">
         <is>
-          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
+          <t>In the portal, cancel immediately, then return to the app.</t>
         </is>
       </c>
       <c r="F127" s="9" t="inlineStr">
         <is>
-          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
+          <t>Entitlement flips to free; the scrapbook is monthly-gated again; tenure (started_at) is preserved.</t>
         </is>
       </c>
       <c r="G127" s="7" t="inlineStr">
@@ -5826,7 +5826,7 @@
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>PREM-11</t>
+          <t>PREM-10</t>
         </is>
       </c>
       <c r="B128" s="7" t="inlineStr">
@@ -5834,29 +5834,29 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C128" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D128" s="9" t="inlineStr">
         <is>
-          <t>Comp allowlist: the owner email is always premium</t>
+          <t>Premium screen shows the renew / cancel date</t>
         </is>
       </c>
       <c r="E128" s="9" t="inlineStr">
         <is>
-          <t>Sign in with the comp email (the owner account listed in server/src/comp.ts), without ever paying.</t>
+          <t>As premium, open /premium; then schedule a cancel-at-period-end in the portal and reopen.</t>
         </is>
       </c>
       <c r="F128" s="9" t="inlineStr">
         <is>
-          <t>Premium is active immediately: Settings and the Lookback show the scrapbook unlocked and Scan works, with no Stripe charge. A non-allowlisted free account stays free. The allowlist is checked against a cryptographically verified token on the costed gate, so a forged token cannot claim premium compute.</t>
+          <t>Reads 'Renews &lt;date&gt;' when active, and 'Premium until &lt;date&gt;, then free' when a cancel is scheduled.</t>
         </is>
       </c>
       <c r="G128" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="H128" s="7" t="inlineStr"/>
@@ -5866,7 +5866,7 @@
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>PREM-12</t>
+          <t>PREM-11</t>
         </is>
       </c>
       <c r="B129" s="7" t="inlineStr">
@@ -5874,24 +5874,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C129" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="C129" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D129" s="9" t="inlineStr">
         <is>
-          <t>Lookback insights: the premium 'Your patterns' card</t>
+          <t>Comp allowlist: the owner email is always premium</t>
         </is>
       </c>
       <c r="E129" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), finish a few tasks across a couple of days this week including one big/dreaded one, then open the Lookback and scroll below the Scrapbook. Tap 'Reflect on this week'.</t>
+          <t>Sign in with the comp email (the owner account listed in server/src/comp.ts), without ever paying.</t>
         </is>
       </c>
       <c r="F129" s="9" t="inlineStr">
         <is>
-          <t>A calm 'Your patterns' card shows warm counts (finished this week, 'on N days', reclaimed old tasks named) with NO streak, score, percent, or 'missed' wording. 'Reflect on this week' returns one warm paragraph that only celebrates what was done (never a performance review) and changes nothing about your tasks. A 'lookback.summary.made' event is logged.</t>
+          <t>Premium is active immediately: Settings and the Lookback show the scrapbook unlocked and Scan works, with no Stripe charge. A non-allowlisted free account stays free. The allowlist is checked against a cryptographically verified token on the costed gate, so a forged token cannot claim premium compute.</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr">
@@ -5906,7 +5906,7 @@
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>PREM-13</t>
+          <t>PREM-12</t>
         </is>
       </c>
       <c r="B130" s="7" t="inlineStr">
@@ -5921,17 +5921,17 @@
       </c>
       <c r="D130" s="9" t="inlineStr">
         <is>
-          <t>Lookback insights: free sees a calm upsell, not a wall</t>
+          <t>Lookback insights: the premium 'Your patterns' card</t>
         </is>
       </c>
       <c r="E130" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open the Lookback and scroll below the Scrapbook, then tap the 'Your patterns' card.</t>
+          <t>As premium (or with the dev Premium override on), finish a few tasks across a couple of days this week including one big/dreaded one, then open the Lookback and scroll below the Scrapbook. Tap 'Reflect on this week'.</t>
         </is>
       </c>
       <c r="F130" s="9" t="inlineStr">
         <is>
-          <t>A calm one-line invite ('See what your weeks and months add up to'), never a teased count and never a wall. Tapping routes to /premium and logs 'premium.gate_hit' with reason 'insights'. The free user's calendar and their one monthly scrapbook are completely untouched.</t>
+          <t>A calm 'Your patterns' card shows warm counts (finished this week, 'on N days', reclaimed old tasks named) with NO streak, score, percent, or 'missed' wording. 'Reflect on this week' returns one warm paragraph that only celebrates what was done (never a performance review) and changes nothing about your tasks. A 'lookback.summary.made' event is logged.</t>
         </is>
       </c>
       <c r="G130" s="7" t="inlineStr">
@@ -5946,7 +5946,7 @@
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>PREM-14</t>
+          <t>PREM-13</t>
         </is>
       </c>
       <c r="B131" s="7" t="inlineStr">
@@ -5954,24 +5954,24 @@
           <t>Premium</t>
         </is>
       </c>
-      <c r="C131" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C131" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D131" s="9" t="inlineStr">
         <is>
-          <t>Premium: custom colour theme</t>
+          <t>Lookback insights: free sees a calm upsell, not a wall</t>
         </is>
       </c>
       <c r="E131" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), open Settings -&gt; Comfort -&gt; 'Colour theme' and tap each of Dusk / Sage / Slate / Heather / Fog / Honey / Rose, reloading after choosing one, in BOTH light and dark mode. Then as a FREE user, tap a preset.</t>
+          <t>As a free user, open the Lookback and scroll below the Scrapbook, then tap the 'Your patterns' card.</t>
         </is>
       </c>
       <c r="F131" s="9" t="inlineStr">
         <is>
-          <t>Premium: tapping a preset repaints the WHOLE app in that palette (background, cards, accent, the brand) and the choice survives reload; the chosen preset is ringed; Dusk is the default and looks identical to the pre-themes app. Each preset has a tuned light and dark variant. Honey's buttons keep DARK labels (a calm gold can't carry white text). Free: the block shows a 'Premium' tag and tapping any preset routes to the paywall with no change applied. A lapsed subscriber keeps the preset they chose.</t>
+          <t>A calm one-line invite ('See what your weeks and months add up to'), never a teased count and never a wall. Tapping routes to /premium and logs 'premium.gate_hit' with reason 'insights'. The free user's calendar and their one monthly scrapbook are completely untouched.</t>
         </is>
       </c>
       <c r="G131" s="7" t="inlineStr">
@@ -5986,7 +5986,7 @@
     <row r="132">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>PREM-15</t>
+          <t>PREM-14</t>
         </is>
       </c>
       <c r="B132" s="7" t="inlineStr">
@@ -6001,17 +6001,17 @@
       </c>
       <c r="D132" s="9" t="inlineStr">
         <is>
-          <t>Post-payment 'taking a while' recovery</t>
+          <t>Premium: custom colour theme</t>
         </is>
       </c>
       <c r="E132" s="9" t="inlineStr">
         <is>
-          <t>Complete a test checkout, then on the return /premium success screen simulate the entitlement being slow (e.g. the webhook delayed) so polling does not flip within ~10 tries.</t>
+          <t>As premium (or with the dev Premium override on), open Settings -&gt; Comfort -&gt; 'Colour theme' and tap each of Dusk / Sage / Slate / Heather / Fog / Honey / Rose, reloading after choosing one, in BOTH light and dark mode. Then as a FREE user, tap a preset.</t>
         </is>
       </c>
       <c r="F132" s="9" t="inlineStr">
         <is>
-          <t>Instead of spinning forever it shows a calm message ('This is taking longer than usual. Your payment went through, give it a minute, then tap Refresh.') with a Refresh button and a pointer to send a note from Settings if it persists. Tapping Refresh re-checks and flips to premium once the entitlement lands. It never says the payment failed.</t>
+          <t>Premium: tapping a preset repaints the WHOLE app in that palette (background, cards, accent, the brand) and the choice survives reload; the chosen preset is ringed; Dusk is the default and looks identical to the pre-themes app. Each preset has a tuned light and dark variant. Honey's buttons keep DARK labels (a calm gold can't carry white text). Free: the block shows a 'Premium' tag and tapping any preset routes to the paywall with no change applied. A lapsed subscriber keeps the preset they chose.</t>
         </is>
       </c>
       <c r="G132" s="7" t="inlineStr">
@@ -6026,7 +6026,7 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>PREM-16</t>
+          <t>PREM-15</t>
         </is>
       </c>
       <c r="B133" s="7" t="inlineStr">
@@ -6041,17 +6041,17 @@
       </c>
       <c r="D133" s="9" t="inlineStr">
         <is>
-          <t>Card-free 'Try Premium' one-month trial</t>
+          <t>Post-payment 'taking a while' recovery</t>
         </is>
       </c>
       <c r="E133" s="9" t="inlineStr">
         <is>
-          <t>Signed in, on /premium tap 'Try Premium free for a month'. Confirm Premium unlocks. Tap it again on the SAME account. Advance the clock past 30 days (or inspect the trials row) and re-check entitlement. Also open the trial link signed OUT.</t>
+          <t>Complete a test checkout, then on the return /premium success screen simulate the entitlement being slow (e.g. the webhook delayed) so polling does not flip within ~10 tries.</t>
         </is>
       </c>
       <c r="F133" s="9" t="inlineStr">
         <is>
-          <t>First tap: a calm confirm, Premium turns on with NO card and NO Stripe (status 'trial'); the page shows 'Your free month', 'Free until &lt;date&gt;', and 'Go Premium to keep it' (not 'Manage'). Second tap, same account: a gentle 'You've already had your free month' (never shame), no second trial granted. After expiry it reverts to free on its own, no charge ever. Signed out: an account is required (one trial per account), so the link routes to sign-in rather than granting.</t>
+          <t>Instead of spinning forever it shows a calm message ('This is taking longer than usual. Your payment went through, give it a minute, then tap Refresh.') with a Refresh button and a pointer to send a note from Settings if it persists. Tapping Refresh re-checks and flips to premium once the entitlement lands. It never says the payment failed.</t>
         </is>
       </c>
       <c r="G133" s="7" t="inlineStr">
@@ -6066,7 +6066,7 @@
     <row r="134">
       <c r="A134" s="6" t="inlineStr">
         <is>
-          <t>PREM-17</t>
+          <t>PREM-16</t>
         </is>
       </c>
       <c r="B134" s="7" t="inlineStr">
@@ -6081,17 +6081,17 @@
       </c>
       <c r="D134" s="9" t="inlineStr">
         <is>
-          <t>Annual vs monthly plan checkout</t>
+          <t>Card-free 'Try Premium' one-month trial</t>
         </is>
       </c>
       <c r="E134" s="9" t="inlineStr">
         <is>
-          <t>On /premium use the Monthly / Annual toggle, then Subscribe. Confirm the Stripe Checkout reflects the chosen plan. Complete a test annual checkout. Then, as an already-subscribed user, hit Subscribe again.</t>
+          <t>Signed in, on /premium tap 'Try Premium free for a month'. Confirm Premium unlocks. Tap it again on the SAME account. Advance the clock past 30 days (or inspect the trials row) and re-check entitlement. Also open the trial link signed OUT.</t>
         </is>
       </c>
       <c r="F134" s="9" t="inlineStr">
         <is>
-          <t>The toggle shows 'A$50/year, about two months free' for annual; Checkout opens the YEARLY price for Annual and the monthly price for Monthly, and the success path grants Premium either way. An already-subscribed user is refused a second Checkout (the server 409s and the app says 'You're already on Premium', never a double charge). Prerequisite: the Worker deployed with STRIPE_PRICE_ID_ANNUAL and that price live in Stripe.</t>
+          <t>First tap: a calm confirm, Premium turns on with NO card and NO Stripe (status 'trial'); the page shows 'Your free month', 'Free until &lt;date&gt;', and 'Go Premium to keep it' (not 'Manage'). Second tap, same account: a gentle 'You've already had your free month' (never shame), no second trial granted. After expiry it reverts to free on its own, no charge ever. Signed out: an account is required (one trial per account), so the link routes to sign-in rather than granting.</t>
         </is>
       </c>
       <c r="G134" s="7" t="inlineStr">
@@ -6106,32 +6106,32 @@
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>PIN-01</t>
+          <t>PREM-17</t>
         </is>
       </c>
       <c r="B135" s="7" t="inlineStr">
         <is>
-          <t>Pin</t>
-        </is>
-      </c>
-      <c r="C135" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C135" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D135" s="9" t="inlineStr">
         <is>
-          <t>Premium: pin a task as the day's one thing</t>
+          <t>Annual vs monthly plan checkout</t>
         </is>
       </c>
       <c r="E135" s="9" t="inlineStr">
         <is>
-          <t>As premium (or with the dev Premium override on), tap-and-hold a one-off task to select it, then tap 'Pin' in the select bar.</t>
+          <t>On /premium use the Monthly / Annual toggle, then Subscribe. Confirm the Stripe Checkout reflects the chosen plan. Complete a test annual checkout. Then, as an already-subscribed user, hit Subscribe again.</t>
         </is>
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>The task gets a calm mauve star and border and floats to the top of Today. 'Focus on one thing' then opens straight to it.</t>
+          <t>The toggle shows 'A$50/year, about two months free' for annual; Checkout opens the YEARLY price for Annual and the monthly price for Monthly, and the success path grants Premium either way. An already-subscribed user is refused a second Checkout (the server 409s and the app says 'You're already on Premium', never a double charge). Prerequisite: the Worker deployed with STRIPE_PRICE_ID_ANNUAL and that price live in Stripe.</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
@@ -6146,7 +6146,7 @@
     <row r="136">
       <c r="A136" s="6" t="inlineStr">
         <is>
-          <t>PIN-02</t>
+          <t>PIN-01</t>
         </is>
       </c>
       <c r="B136" s="7" t="inlineStr">
@@ -6161,17 +6161,17 @@
       </c>
       <c r="D136" s="9" t="inlineStr">
         <is>
-          <t>Free: Pin routes to the upsell, never pins</t>
+          <t>Premium: pin a task as the day's one thing</t>
         </is>
       </c>
       <c r="E136" s="9" t="inlineStr">
         <is>
-          <t>As a free user, select a single one-off task and tap the dimmed 'Pin' action.</t>
+          <t>As premium (or with the dev Premium override on), tap-and-hold a one-off task to select it, then tap 'Pin' in the select bar.</t>
         </is>
       </c>
       <c r="F136" s="9" t="inlineStr">
         <is>
-          <t>No task is pinned, and the Premium screen opens calmly (never a shaming wall). A 'premium.gate_hit' with reason 'pin' is logged.</t>
+          <t>The task gets a calm mauve star and border and floats to the top of Today. 'Focus on one thing' then opens straight to it.</t>
         </is>
       </c>
       <c r="G136" s="7" t="inlineStr">
@@ -6186,7 +6186,7 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>PIN-03</t>
+          <t>PIN-02</t>
         </is>
       </c>
       <c r="B137" s="7" t="inlineStr">
@@ -6194,24 +6194,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C137" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D137" s="9" t="inlineStr">
         <is>
-          <t>Only one task is pinned at a time</t>
+          <t>Free: Pin routes to the upsell, never pins</t>
         </is>
       </c>
       <c r="E137" s="9" t="inlineStr">
         <is>
-          <t>As premium, pin task A, then select task B and pin it.</t>
+          <t>As a free user, select a single one-off task and tap the dimmed 'Pin' action.</t>
         </is>
       </c>
       <c r="F137" s="9" t="inlineStr">
         <is>
-          <t>Task B is now pinned (starred, floated to the top), and task A is no longer pinned. At most one pin ever exists.</t>
+          <t>No task is pinned, and the Premium screen opens calmly (never a shaming wall). A 'premium.gate_hit' with reason 'pin' is logged.</t>
         </is>
       </c>
       <c r="G137" s="7" t="inlineStr">
@@ -6226,7 +6226,7 @@
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>PIN-04</t>
+          <t>PIN-03</t>
         </is>
       </c>
       <c r="B138" s="7" t="inlineStr">
@@ -6241,17 +6241,17 @@
       </c>
       <c r="D138" s="9" t="inlineStr">
         <is>
-          <t>A pin syncs across devices</t>
+          <t>Only one task is pinned at a time</t>
         </is>
       </c>
       <c r="E138" s="9" t="inlineStr">
         <is>
-          <t>As premium and signed in, pin a task, then sign out and back in (or open a second device).</t>
+          <t>As premium, pin task A, then select task B and pin it.</t>
         </is>
       </c>
       <c r="F138" s="9" t="inlineStr">
         <is>
-          <t>The task is still pinned after the sync round-trip (the star and float persist). Needs the pinned_at column applied in Supabase.</t>
+          <t>Task B is now pinned (starred, floated to the top), and task A is no longer pinned. At most one pin ever exists.</t>
         </is>
       </c>
       <c r="G138" s="7" t="inlineStr">
@@ -6266,7 +6266,7 @@
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>PIN-05</t>
+          <t>PIN-04</t>
         </is>
       </c>
       <c r="B139" s="7" t="inlineStr">
@@ -6274,24 +6274,24 @@
           <t>Pin</t>
         </is>
       </c>
-      <c r="C139" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C139" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D139" s="9" t="inlineStr">
         <is>
-          <t>Pin is offered only on one-off Today rows</t>
+          <t>A pin syncs across devices</t>
         </is>
       </c>
       <c r="E139" s="9" t="inlineStr">
         <is>
-          <t>Select a recurring task, then separately look at a task in the 'Later' list.</t>
+          <t>As premium and signed in, pin a task, then sign out and back in (or open a second device).</t>
         </is>
       </c>
       <c r="F139" s="9" t="inlineStr">
         <is>
-          <t>No 'Pin' action appears for a recurring task, and Later rows carry no pin affordance (pinning is Today-only and one-offs only).</t>
+          <t>The task is still pinned after the sync round-trip (the star and float persist). Needs the pinned_at column applied in Supabase.</t>
         </is>
       </c>
       <c r="G139" s="7" t="inlineStr">
@@ -6306,32 +6306,32 @@
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>OCR-01</t>
+          <t>PIN-05</t>
         </is>
       </c>
       <c r="B140" s="7" t="inlineStr">
         <is>
-          <t>Scan</t>
-        </is>
-      </c>
-      <c r="C140" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Pin</t>
+        </is>
+      </c>
+      <c r="C140" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D140" s="9" t="inlineStr">
         <is>
-          <t>Premium: the Scan button opens the camera</t>
+          <t>Pin is offered only on one-off Today rows</t>
         </is>
       </c>
       <c r="E140" s="9" t="inlineStr">
         <is>
-          <t>As premium, open the add panel and tap the Scan (camera) pill beside Speak.</t>
+          <t>Select a recurring task, then separately look at a task in the 'Later' list.</t>
         </is>
       </c>
       <c r="F140" s="9" t="inlineStr">
         <is>
-          <t>The camera screen opens: a live viewfinder with a shutter and a Photos shortcut on a device, or a 'Choose a photo' prompt on web. No paywall.</t>
+          <t>No 'Pin' action appears for a recurring task, and Later rows carry no pin affordance (pinning is Today-only and one-offs only).</t>
         </is>
       </c>
       <c r="G140" s="7" t="inlineStr">
@@ -6346,7 +6346,7 @@
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>OCR-02</t>
+          <t>OCR-01</t>
         </is>
       </c>
       <c r="B141" s="7" t="inlineStr">
@@ -6361,17 +6361,17 @@
       </c>
       <c r="D141" s="9" t="inlineStr">
         <is>
-          <t>Free: Scan routes to the upsell, never opens the camera</t>
+          <t>Premium: the Scan button opens the camera</t>
         </is>
       </c>
       <c r="E141" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open the add panel and tap the Scan pill.</t>
+          <t>As premium, open the add panel and tap the Scan (camera) pill beside Speak.</t>
         </is>
       </c>
       <c r="F141" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium screen calmly (never a wall). A 'premium.gate_hit' with reason 'ocr' is logged. No camera opens.</t>
+          <t>The camera screen opens: a live viewfinder with a shutter and a Photos shortcut on a device, or a 'Choose a photo' prompt on web. No paywall.</t>
         </is>
       </c>
       <c r="G141" s="7" t="inlineStr">
@@ -6386,7 +6386,7 @@
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>OCR-03</t>
+          <t>OCR-02</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
@@ -6401,22 +6401,22 @@
       </c>
       <c r="D142" s="9" t="inlineStr">
         <is>
-          <t>Photograph a list and the tasks land in the box</t>
+          <t>Free: Scan routes to the upsell, never opens the camera</t>
         </is>
       </c>
       <c r="E142" s="9" t="inlineStr">
         <is>
-          <t>As premium on a device, tap Scan, photograph a short printed or handwritten list (fill the frame), wait for 'Reading your list...'.</t>
+          <t>As a free user, open the add panel and tap the Scan pill.</t>
         </is>
       </c>
       <c r="F142" s="9" t="inlineStr">
         <is>
-          <t>The tasks it reads appear in the brain-dump box, one per line, editable. Nothing is auto-added to Today, and tapping Add commits them. An 'ocr.captured' event is logged.</t>
+          <t>Routed to the Premium screen calmly (never a wall). A 'premium.gate_hit' with reason 'ocr' is logged. No camera opens.</t>
         </is>
       </c>
       <c r="G142" s="7" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr"/>
@@ -6426,7 +6426,7 @@
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>OCR-04</t>
+          <t>OCR-03</t>
         </is>
       </c>
       <c r="B143" s="7" t="inlineStr">
@@ -6434,29 +6434,29 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C143" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C143" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D143" s="9" t="inlineStr">
         <is>
-          <t>Gallery fallback reads an existing photo</t>
+          <t>Photograph a list and the tasks land in the box</t>
         </is>
       </c>
       <c r="E143" s="9" t="inlineStr">
         <is>
-          <t>Tap Scan, then 'Photos' (device) or 'Choose a photo' (web), and pick a photo of a list, a note, or a whiteboard.</t>
+          <t>As premium on a device, tap Scan, photograph a short printed or handwritten list (fill the frame), wait for 'Reading your list...'.</t>
         </is>
       </c>
       <c r="F143" s="9" t="inlineStr">
         <is>
-          <t>Same result: the read tasks land in the box for review. Covers a screenshot of a texted list, or a photo taken earlier.</t>
+          <t>The tasks it reads appear in the brain-dump box, one per line, editable. Nothing is auto-added to Today, and tapping Add commits them. An 'ocr.captured' event is logged.</t>
         </is>
       </c>
       <c r="G143" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr"/>
@@ -6466,7 +6466,7 @@
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>OCR-05</t>
+          <t>OCR-04</t>
         </is>
       </c>
       <c r="B144" s="7" t="inlineStr">
@@ -6481,17 +6481,17 @@
       </c>
       <c r="D144" s="9" t="inlineStr">
         <is>
-          <t>An unreadable photo fails calmly</t>
+          <t>Gallery fallback reads an existing photo</t>
         </is>
       </c>
       <c r="E144" s="9" t="inlineStr">
         <is>
-          <t>Scan a blank, blurry, or list-free image.</t>
+          <t>Tap Scan, then 'Photos' (device) or 'Choose a photo' (web), and pick a photo of a list, a note, or a whiteboard.</t>
         </is>
       </c>
       <c r="F144" s="9" t="inlineStr">
         <is>
-          <t>A calm line ('I couldn't read any tasks from that. Try again...'), the camera stays open, never a crash and never a shaming message.</t>
+          <t>Same result: the read tasks land in the box for review. Covers a screenshot of a texted list, or a photo taken earlier.</t>
         </is>
       </c>
       <c r="G144" s="7" t="inlineStr">
@@ -6506,7 +6506,7 @@
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>OCR-06</t>
+          <t>OCR-05</t>
         </is>
       </c>
       <c r="B145" s="7" t="inlineStr">
@@ -6521,22 +6521,22 @@
       </c>
       <c r="D145" s="9" t="inlineStr">
         <is>
-          <t>Camera denial is never a dead end</t>
+          <t>An unreadable photo fails calmly</t>
         </is>
       </c>
       <c r="E145" s="9" t="inlineStr">
         <is>
-          <t>On a device, deny the camera permission when prompted.</t>
+          <t>Scan a blank, blurry, or list-free image.</t>
         </is>
       </c>
       <c r="F145" s="9" t="inlineStr">
         <is>
-          <t>A calm screen offers 'Allow camera' and 'Choose from photos instead', and the gallery path still reads a list.</t>
+          <t>A calm line ('I couldn't read any tasks from that. Try again...'), the camera stays open, never a crash and never a shaming message.</t>
         </is>
       </c>
       <c r="G145" s="7" t="inlineStr">
         <is>
-          <t>Device</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="H145" s="7" t="inlineStr"/>
@@ -6546,7 +6546,7 @@
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
         <is>
-          <t>OCR-07</t>
+          <t>OCR-06</t>
         </is>
       </c>
       <c r="B146" s="7" t="inlineStr">
@@ -6554,29 +6554,29 @@
           <t>Scan</t>
         </is>
       </c>
-      <c r="C146" s="11" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="C146" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D146" s="9" t="inlineStr">
         <is>
-          <t>AI egress is disclosed at the point of use</t>
+          <t>Camera denial is never a dead end</t>
         </is>
       </c>
       <c r="E146" s="9" t="inlineStr">
         <is>
-          <t>Open the Scan screen (device or web).</t>
+          <t>On a device, deny the camera permission when prompted.</t>
         </is>
       </c>
       <c r="F146" s="9" t="inlineStr">
         <is>
-          <t>The note 'Your photo is sent to the AI to read your list, then discarded. It is never stored.' is visible. The D1 'ocr' telemetry row holds only the image size and task count, never the image or the titles.</t>
+          <t>A calm screen offers 'Allow camera' and 'Choose from photos instead', and the gallery path still reads a list.</t>
         </is>
       </c>
       <c r="G146" s="7" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="H146" s="7" t="inlineStr"/>
@@ -6586,32 +6586,32 @@
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>CHART-01</t>
+          <t>OCR-07</t>
         </is>
       </c>
       <c r="B147" s="7" t="inlineStr">
         <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C147" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Scan</t>
+        </is>
+      </c>
+      <c r="C147" s="11" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D147" s="9" t="inlineStr">
         <is>
-          <t>Premium: chart a course toward a goal</t>
+          <t>AI egress is disclosed at the point of use</t>
         </is>
       </c>
       <c r="E147" s="9" t="inlineStr">
         <is>
-          <t>As premium (or dev Premium override on), open Rooms, tap 'Chart a course', type a goal like 'get fit for a 10k', tap 'Suggest steps'.</t>
+          <t>Open the Scan screen (device or web).</t>
         </is>
       </c>
       <c r="F147" s="9" t="inlineStr">
         <is>
-          <t>A calm one-line heading plus 3-7 ticked next steps appear, and nothing is added yet. Tapping 'Add N tasks' lands them on Today (the first undated, later ones spread forward), each an ordinary task, and returns to Today. The 'chart.requested' then 'chart.added' events are logged.</t>
+          <t>The note 'Your photo is sent to the AI to read your list, then discarded. It is never stored.' is visible. The D1 'ocr' telemetry row holds only the image size and task count, never the image or the titles.</t>
         </is>
       </c>
       <c r="G147" s="7" t="inlineStr">
@@ -6626,7 +6626,7 @@
     <row r="148">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t>CHART-02</t>
+          <t>CHART-01</t>
         </is>
       </c>
       <c r="B148" s="7" t="inlineStr">
@@ -6641,17 +6641,17 @@
       </c>
       <c r="D148" s="9" t="inlineStr">
         <is>
-          <t>Free: charting routes to the upsell, never plans</t>
+          <t>Premium: chart a course toward a goal</t>
         </is>
       </c>
       <c r="E148" s="9" t="inlineStr">
         <is>
-          <t>As a free user, open Rooms, tap 'Chart a course', type a goal, tap 'Suggest steps'.</t>
+          <t>As premium (or dev Premium override on), open Rooms, tap 'Chart a course', type a goal like 'get fit for a 10k', tap 'Suggest steps'.</t>
         </is>
       </c>
       <c r="F148" s="9" t="inlineStr">
         <is>
-          <t>Routed to the Premium screen calmly (never a wall), and a 'premium.gate_hit' with reason 'chart' is logged. No plan is generated and nothing is added.</t>
+          <t>A calm one-line heading plus 3-7 ticked next steps appear, and nothing is added yet. Tapping 'Add N tasks' lands them on Today (the first undated, later ones spread forward), each an ordinary task, and returns to Today. The 'chart.requested' then 'chart.added' events are logged.</t>
         </is>
       </c>
       <c r="G148" s="7" t="inlineStr">
@@ -6666,7 +6666,7 @@
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>CHART-03</t>
+          <t>CHART-02</t>
         </is>
       </c>
       <c r="B149" s="7" t="inlineStr">
@@ -6674,24 +6674,24 @@
           <t>Chart</t>
         </is>
       </c>
-      <c r="C149" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D149" s="9" t="inlineStr">
         <is>
-          <t>Propose-then-accept: nothing auto-adds</t>
+          <t>Free: charting routes to the upsell, never plans</t>
         </is>
       </c>
       <c r="E149" s="9" t="inlineStr">
         <is>
-          <t>As premium, generate a plan, untick two steps, then tap 'Add'. Separately, generate a plan and back out with 'Not these, start over' or Back.</t>
+          <t>As a free user, open Rooms, tap 'Chart a course', type a goal, tap 'Suggest steps'.</t>
         </is>
       </c>
       <c r="F149" s="9" t="inlineStr">
         <is>
-          <t>Only the ticked steps are added as plain tasks, and backing out adds nothing. Today was unchanged before accepting.</t>
+          <t>Routed to the Premium screen calmly (never a wall), and a 'premium.gate_hit' with reason 'chart' is logged. No plan is generated and nothing is added.</t>
         </is>
       </c>
       <c r="G149" s="7" t="inlineStr">
@@ -6706,7 +6706,7 @@
     <row r="150">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t>CHART-04</t>
+          <t>CHART-03</t>
         </is>
       </c>
       <c r="B150" s="7" t="inlineStr">
@@ -6721,17 +6721,17 @@
       </c>
       <c r="D150" s="9" t="inlineStr">
         <is>
-          <t>A goal that cannot be mapped fails calmly</t>
+          <t>Propose-then-accept: nothing auto-adds</t>
         </is>
       </c>
       <c r="E150" s="9" t="inlineStr">
         <is>
-          <t>Enter an empty goal (the button is disabled), then a nonsensical goal and submit.</t>
+          <t>As premium, generate a plan, untick two steps, then tap 'Add'. Separately, generate a plan and back out with 'Not these, start over' or Back.</t>
         </is>
       </c>
       <c r="F150" s="9" t="inlineStr">
         <is>
-          <t>The empty case cannot submit. A nonsensical goal shows one calm line ('I couldn't map that out just now'), the goal stays editable, never a crash or a shaming message.</t>
+          <t>Only the ticked steps are added as plain tasks, and backing out adds nothing. Today was unchanged before accepting.</t>
         </is>
       </c>
       <c r="G150" s="7" t="inlineStr">
@@ -6746,7 +6746,7 @@
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>CHART-05</t>
+          <t>CHART-04</t>
         </is>
       </c>
       <c r="B151" s="7" t="inlineStr">
@@ -6761,17 +6761,17 @@
       </c>
       <c r="D151" s="9" t="inlineStr">
         <is>
-          <t>A deadline spreads the steps across the timeframe</t>
+          <t>A goal that cannot be mapped fails calmly</t>
         </is>
       </c>
       <c r="E151" s="9" t="inlineStr">
         <is>
-          <t>As premium, type a goal, tap a 'By when?' chip (e.g. 'In 2 months'), then Suggest steps and Add.</t>
+          <t>Enter an empty goal (the button is disabled), then a nonsensical goal and submit.</t>
         </is>
       </c>
       <c r="F151" s="9" t="inlineStr">
         <is>
-          <t>The steps are paced for that timeframe, and the accepted tasks spread from Today out to the chosen date (not crammed into the next few days). 'No deadline' keeps the gentle one-per-day default.</t>
+          <t>The empty case cannot submit. A nonsensical goal shows one calm line ('I couldn't map that out just now'), the goal stays editable, never a crash or a shaming message.</t>
         </is>
       </c>
       <c r="G151" s="7" t="inlineStr">
@@ -6786,32 +6786,32 @@
     <row r="152">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t>SEQ-01</t>
+          <t>CHART-05</t>
         </is>
       </c>
       <c r="B152" s="7" t="inlineStr">
         <is>
-          <t>Sequence</t>
-        </is>
-      </c>
-      <c r="C152" s="8" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C152" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D152" s="9" t="inlineStr">
         <is>
-          <t>Premium: Plan my day suggests a calm sequence</t>
+          <t>A deadline spreads the steps across the timeframe</t>
         </is>
       </c>
       <c r="E152" s="9" t="inlineStr">
         <is>
-          <t>As premium with 3+ open one-off tasks on Today, tap 'Plan my day'.</t>
+          <t>As premium, type a goal, tap a 'By when?' chip (e.g. 'In 2 months'), then Suggest steps and Add.</t>
         </is>
       </c>
       <c r="F152" s="9" t="inlineStr">
         <is>
-          <t>A proposal card lists today's tasks in a suggested order, each with a short calm reason. Nothing reorders until 'Use this order' is tapped, then the list re-sequences in place (no dates change, no task moves to another day). A 'sequence.accepted' event is logged.</t>
+          <t>The steps are paced for that timeframe, and the accepted tasks spread from Today out to the chosen date (not crammed into the next few days). 'No deadline' keeps the gentle one-per-day default.</t>
         </is>
       </c>
       <c r="G152" s="7" t="inlineStr">
@@ -6826,7 +6826,7 @@
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>SEQ-02</t>
+          <t>SEQ-01</t>
         </is>
       </c>
       <c r="B153" s="7" t="inlineStr">
@@ -6841,17 +6841,17 @@
       </c>
       <c r="D153" s="9" t="inlineStr">
         <is>
-          <t>Free: Plan my day routes to the upsell, never reorders</t>
+          <t>Premium: Plan my day suggests a calm sequence</t>
         </is>
       </c>
       <c r="E153" s="9" t="inlineStr">
         <is>
-          <t>As a free user with 2+ tasks on Today, tap 'Plan my day'.</t>
+          <t>As premium with 3+ open one-off tasks on Today, tap 'Plan my day'.</t>
         </is>
       </c>
       <c r="F153" s="9" t="inlineStr">
         <is>
-          <t>The Premium screen opens calmly (never a wall), a 'premium.gate_hit' with reason 'sequence' is logged, and the day's order is unchanged.</t>
+          <t>A proposal card lists today's tasks in a suggested order, each with a short calm reason. Nothing reorders until 'Use this order' is tapped, then the list re-sequences in place (no dates change, no task moves to another day). A 'sequence.accepted' event is logged.</t>
         </is>
       </c>
       <c r="G153" s="7" t="inlineStr">
@@ -6866,7 +6866,7 @@
     <row r="154">
       <c r="A154" s="6" t="inlineStr">
         <is>
-          <t>SEQ-03</t>
+          <t>SEQ-02</t>
         </is>
       </c>
       <c r="B154" s="7" t="inlineStr">
@@ -6874,24 +6874,24 @@
           <t>Sequence</t>
         </is>
       </c>
-      <c r="C154" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="C154" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D154" s="9" t="inlineStr">
         <is>
-          <t>'Not now' leaves the day untouched</t>
+          <t>Free: Plan my day routes to the upsell, never reorders</t>
         </is>
       </c>
       <c r="E154" s="9" t="inlineStr">
         <is>
-          <t>As premium, open the proposal, then tap 'Not now' or the backdrop.</t>
+          <t>As a free user with 2+ tasks on Today, tap 'Plan my day'.</t>
         </is>
       </c>
       <c r="F154" s="9" t="inlineStr">
         <is>
-          <t>The order is exactly as before, nothing reordered, and no manualOrder is written.</t>
+          <t>The Premium screen opens calmly (never a wall), a 'premium.gate_hit' with reason 'sequence' is logged, and the day's order is unchanged.</t>
         </is>
       </c>
       <c r="G154" s="7" t="